<commit_message>
Identified problem if 'max_crop_in_crop_prod' too close to 100%, added note in data sheet
</commit_message>
<xml_diff>
--- a/data/default/FeedMgmt.xlsx
+++ b/data/default/FeedMgmt.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1570" uniqueCount="647">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1561" uniqueCount="648">
   <si>
     <t>f_feed</t>
   </si>
@@ -1981,6 +1981,29 @@
   <si>
     <t>Crop residues</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Note:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Setting this parameter too close to 100% may cause problems.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -1989,7 +2012,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2177,6 +2200,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF00B0F0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2773,7 +2804,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R154"/>
+  <dimension ref="A1:R153"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="7" width="20.28515625" customWidth="1"/>
@@ -3886,35 +3917,13 @@
     </row>
     <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>19</v>
-      </c>
-      <c r="H69" t="s">
-        <v>319</v>
-      </c>
-      <c r="I69" t="s">
-        <v>28</v>
-      </c>
-      <c r="M69" t="s">
-        <v>320</v>
-      </c>
-      <c r="N69" s="3">
-        <v>90</v>
-      </c>
-      <c r="O69" t="s">
-        <v>23</v>
-      </c>
-      <c r="P69" s="3"/>
+        <v>647</v>
+      </c>
     </row>
     <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>19</v>
       </c>
-      <c r="B70" t="s">
-        <v>314</v>
-      </c>
-      <c r="E70" t="s">
-        <v>315</v>
-      </c>
       <c r="H70" t="s">
         <v>319</v>
       </c>
@@ -3925,7 +3934,7 @@
         <v>320</v>
       </c>
       <c r="N70" s="3">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="O70" t="s">
         <v>23</v>
@@ -3940,7 +3949,7 @@
         <v>314</v>
       </c>
       <c r="E71" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H71" t="s">
         <v>319</v>
@@ -3963,8 +3972,11 @@
       <c r="A72" t="s">
         <v>19</v>
       </c>
+      <c r="B72" t="s">
+        <v>314</v>
+      </c>
       <c r="E72" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H72" t="s">
         <v>319</v>
@@ -3976,7 +3988,7 @@
         <v>320</v>
       </c>
       <c r="N72" s="3">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O72" t="s">
         <v>23</v>
@@ -3987,11 +3999,8 @@
       <c r="A73" t="s">
         <v>19</v>
       </c>
-      <c r="B73" t="s">
-        <v>314</v>
-      </c>
       <c r="E73" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H73" t="s">
         <v>319</v>
@@ -4011,31 +4020,34 @@
       <c r="P73" s="3"/>
     </row>
     <row r="74" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N74" s="3"/>
+      <c r="A74" t="s">
+        <v>19</v>
+      </c>
+      <c r="B74" t="s">
+        <v>314</v>
+      </c>
+      <c r="E74" t="s">
+        <v>318</v>
+      </c>
+      <c r="H74" t="s">
+        <v>319</v>
+      </c>
+      <c r="I74" t="s">
+        <v>28</v>
+      </c>
+      <c r="M74" t="s">
+        <v>320</v>
+      </c>
+      <c r="N74" s="3">
+        <v>0</v>
+      </c>
+      <c r="O74" t="s">
+        <v>23</v>
+      </c>
       <c r="P74" s="3"/>
     </row>
     <row r="75" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>19</v>
-      </c>
-      <c r="H75" t="s">
-        <v>319</v>
-      </c>
-      <c r="I75" t="s">
-        <v>28</v>
-      </c>
-      <c r="L75">
-        <v>811</v>
-      </c>
-      <c r="M75" t="s">
-        <v>320</v>
-      </c>
-      <c r="N75" s="3">
-        <v>100</v>
-      </c>
-      <c r="O75" t="s">
-        <v>23</v>
-      </c>
+      <c r="N75" s="3"/>
       <c r="P75" s="3"/>
     </row>
     <row r="76" spans="1:17" x14ac:dyDescent="0.25">
@@ -4159,6 +4171,12 @@
       <c r="A80" t="s">
         <v>19</v>
       </c>
+      <c r="B80" t="s">
+        <v>314</v>
+      </c>
+      <c r="E80" t="s">
+        <v>315</v>
+      </c>
       <c r="H80" t="s">
         <v>319</v>
       </c>
@@ -4172,7 +4190,7 @@
         <v>320</v>
       </c>
       <c r="N80" s="3">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="O80" t="s">
         <v>23</v>
@@ -4187,7 +4205,7 @@
         <v>314</v>
       </c>
       <c r="E81" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="H81" t="s">
         <v>319</v>
@@ -4213,11 +4231,8 @@
       <c r="A82" t="s">
         <v>19</v>
       </c>
-      <c r="B82" t="s">
-        <v>314</v>
-      </c>
       <c r="E82" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H82" t="s">
         <v>319</v>
@@ -4232,7 +4247,7 @@
         <v>320</v>
       </c>
       <c r="N82" s="3">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="O82" t="s">
         <v>23</v>
@@ -4243,8 +4258,11 @@
       <c r="A83" t="s">
         <v>19</v>
       </c>
+      <c r="B83" t="s">
+        <v>314</v>
+      </c>
       <c r="E83" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="H83" t="s">
         <v>319</v>
@@ -4267,88 +4285,72 @@
       <c r="P83" s="3"/>
     </row>
     <row r="84" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>19</v>
-      </c>
-      <c r="B84" t="s">
-        <v>314</v>
-      </c>
-      <c r="E84" t="s">
-        <v>318</v>
-      </c>
-      <c r="H84" t="s">
+      <c r="N84" s="3"/>
+      <c r="P84" s="3"/>
+    </row>
+    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>377</v>
+      </c>
+      <c r="H85" t="s">
         <v>319</v>
       </c>
-      <c r="I84" t="s">
+      <c r="I85" t="s">
         <v>28</v>
       </c>
-      <c r="L84">
-        <v>812</v>
-      </c>
-      <c r="M84" t="s">
+      <c r="M85" t="s">
         <v>320</v>
       </c>
-      <c r="N84" s="3">
-        <v>0</v>
-      </c>
-      <c r="O84" t="s">
+      <c r="N85" s="3">
+        <v>10</v>
+      </c>
+      <c r="O85" t="s">
         <v>23</v>
       </c>
-      <c r="P84" s="3"/>
-    </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N85" s="3"/>
       <c r="P85" s="3"/>
     </row>
     <row r="86" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>377</v>
-      </c>
-      <c r="H86" t="s">
-        <v>319</v>
-      </c>
-      <c r="I86" t="s">
-        <v>28</v>
-      </c>
-      <c r="M86" t="s">
-        <v>320</v>
-      </c>
-      <c r="N86" s="3">
-        <v>10</v>
-      </c>
-      <c r="O86" t="s">
+      <c r="N86" s="3"/>
+      <c r="P86" s="3"/>
+    </row>
+    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A87" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="B87" s="1"/>
+      <c r="C87" s="1"/>
+      <c r="D87" s="1"/>
+      <c r="E87" s="2"/>
+      <c r="F87" s="2"/>
+      <c r="G87" s="2"/>
+      <c r="H87" s="2"/>
+      <c r="I87" s="2"/>
+      <c r="J87" s="2"/>
+      <c r="K87" s="2"/>
+      <c r="L87" s="2"/>
+      <c r="M87" s="2"/>
+      <c r="N87" s="2"/>
+      <c r="O87" s="2"/>
+      <c r="P87" s="2"/>
+      <c r="Q87" s="2"/>
+    </row>
+    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M88" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="N88" s="6">
+        <v>0</v>
+      </c>
+      <c r="O88" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="P86" s="3"/>
-    </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N87" s="3"/>
-      <c r="P87" s="3"/>
-    </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A88" s="1" t="s">
-        <v>380</v>
-      </c>
-      <c r="B88" s="1"/>
-      <c r="C88" s="1"/>
-      <c r="D88" s="1"/>
-      <c r="E88" s="2"/>
-      <c r="F88" s="2"/>
-      <c r="G88" s="2"/>
-      <c r="H88" s="2"/>
-      <c r="I88" s="2"/>
-      <c r="J88" s="2"/>
-      <c r="K88" s="2"/>
-      <c r="L88" s="2"/>
-      <c r="M88" s="2"/>
-      <c r="N88" s="2"/>
-      <c r="O88" s="2"/>
-      <c r="P88" s="2"/>
-      <c r="Q88" s="2"/>
+      <c r="P88" s="6" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="M89" s="6" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="N89" s="6">
         <v>0</v>
@@ -4361,29 +4363,39 @@
       </c>
     </row>
     <row r="90" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M90" s="6" t="s">
-        <v>379</v>
-      </c>
-      <c r="N90" s="6">
-        <v>0</v>
-      </c>
-      <c r="O90" s="6" t="s">
+      <c r="A90" t="s">
+        <v>19</v>
+      </c>
+      <c r="B90" t="s">
+        <v>314</v>
+      </c>
+      <c r="E90" t="s">
+        <v>315</v>
+      </c>
+      <c r="G90" t="s">
+        <v>632</v>
+      </c>
+      <c r="M90" s="21" t="s">
+        <v>378</v>
+      </c>
+      <c r="N90" s="21">
+        <f>(0.8*20+0.2*2)</f>
+        <v>16.399999999999999</v>
+      </c>
+      <c r="O90" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="P90" s="6" t="s">
-        <v>29</v>
+      <c r="P90" s="21" t="s">
+        <v>382</v>
+      </c>
+      <c r="Q90" t="s">
+        <v>639</v>
       </c>
     </row>
     <row r="91" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>19</v>
       </c>
-      <c r="B91" t="s">
-        <v>314</v>
-      </c>
-      <c r="E91" t="s">
-        <v>315</v>
-      </c>
       <c r="G91" t="s">
         <v>632</v>
       </c>
@@ -4391,14 +4403,14 @@
         <v>378</v>
       </c>
       <c r="N91" s="21">
-        <f>(0.8*20+0.2*2)</f>
-        <v>16.399999999999999</v>
+        <f>(0.6*20+0.4*2)</f>
+        <v>12.8</v>
       </c>
       <c r="O91" s="21" t="s">
         <v>23</v>
       </c>
       <c r="P91" s="21" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="Q91" t="s">
         <v>639</v>
@@ -4406,7 +4418,7 @@
     </row>
     <row r="92" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>19</v>
+        <v>381</v>
       </c>
       <c r="G92" t="s">
         <v>632</v>
@@ -4415,14 +4427,13 @@
         <v>378</v>
       </c>
       <c r="N92" s="21">
-        <f>(0.6*20+0.4*2)</f>
-        <v>12.8</v>
+        <v>2</v>
       </c>
       <c r="O92" s="21" t="s">
         <v>23</v>
       </c>
       <c r="P92" s="21" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="Q92" t="s">
         <v>639</v>
@@ -4430,7 +4441,7 @@
     </row>
     <row r="93" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="G93" t="s">
         <v>632</v>
@@ -4453,22 +4464,28 @@
     </row>
     <row r="94" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>377</v>
+        <v>19</v>
+      </c>
+      <c r="B94" t="s">
+        <v>314</v>
+      </c>
+      <c r="E94" t="s">
+        <v>315</v>
       </c>
       <c r="G94" t="s">
         <v>632</v>
       </c>
       <c r="M94" s="21" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="N94" s="21">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O94" s="21" t="s">
         <v>23</v>
       </c>
       <c r="P94" s="21" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="Q94" t="s">
         <v>639</v>
@@ -4478,11 +4495,8 @@
       <c r="A95" t="s">
         <v>19</v>
       </c>
-      <c r="B95" t="s">
-        <v>314</v>
-      </c>
       <c r="E95" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="G95" t="s">
         <v>632</v>
@@ -4507,9 +4521,6 @@
       <c r="A96" t="s">
         <v>19</v>
       </c>
-      <c r="E96" t="s">
-        <v>317</v>
-      </c>
       <c r="G96" t="s">
         <v>632</v>
       </c>
@@ -4517,13 +4528,14 @@
         <v>379</v>
       </c>
       <c r="N96" s="21">
-        <v>5</v>
+        <f>0.9*5+0.1*15</f>
+        <v>6</v>
       </c>
       <c r="O96" s="21" t="s">
         <v>23</v>
       </c>
       <c r="P96" s="21" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="Q96" t="s">
         <v>639</v>
@@ -4531,7 +4543,7 @@
     </row>
     <row r="97" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>19</v>
+        <v>381</v>
       </c>
       <c r="G97" t="s">
         <v>632</v>
@@ -4540,22 +4552,19 @@
         <v>379</v>
       </c>
       <c r="N97" s="21">
-        <f>0.9*5+0.1*15</f>
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="O97" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="P97" s="21" t="s">
-        <v>386</v>
-      </c>
+      <c r="P97" s="21"/>
       <c r="Q97" t="s">
         <v>639</v>
       </c>
     </row>
     <row r="98" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="G98" t="s">
         <v>632</v>
@@ -4575,17 +4584,17 @@
       </c>
     </row>
     <row r="99" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>377</v>
-      </c>
+      <c r="A99" s="22"/>
+      <c r="B99" s="22"/>
+      <c r="E99" s="22"/>
       <c r="G99" t="s">
-        <v>632</v>
+        <v>301</v>
       </c>
       <c r="M99" s="21" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="N99" s="21">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="O99" s="21" t="s">
         <v>23</v>
@@ -4596,44 +4605,56 @@
       </c>
     </row>
     <row r="100" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A100" s="22"/>
-      <c r="B100" s="22"/>
-      <c r="E100" s="22"/>
+      <c r="A100" s="22" t="str">
+        <f>A94</f>
+        <v>cattle</v>
+      </c>
+      <c r="B100" s="22" t="str">
+        <f>B94</f>
+        <v>dairy</v>
+      </c>
+      <c r="E100" s="22" t="str">
+        <f t="shared" ref="E100:E101" si="0">E94</f>
+        <v>cows</v>
+      </c>
       <c r="G100" t="s">
         <v>301</v>
       </c>
-      <c r="M100" s="21" t="s">
-        <v>378</v>
-      </c>
-      <c r="N100" s="21">
+      <c r="M100" s="22" t="str">
+        <f t="shared" ref="M100:Q104" si="1">M94</f>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N100" s="22">
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="O100" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="P100" s="21"/>
-      <c r="Q100" t="s">
-        <v>639</v>
+      <c r="O100" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="P100" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="Q100" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="101" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="22" t="str">
-        <f>A95</f>
+        <f t="shared" ref="A101:A104" si="2">A95</f>
         <v>cattle</v>
       </c>
-      <c r="B101" s="22" t="str">
-        <f>B95</f>
-        <v>dairy</v>
-      </c>
       <c r="E101" s="22" t="str">
-        <f t="shared" ref="E101:E102" si="0">E95</f>
-        <v>cows</v>
+        <f t="shared" si="0"/>
+        <v>bulls</v>
       </c>
       <c r="G101" t="s">
         <v>301</v>
       </c>
       <c r="M101" s="22" t="str">
-        <f t="shared" ref="M101:Q105" si="1">M95</f>
+        <f t="shared" si="1"/>
         <v>feeding_losses</v>
       </c>
       <c r="N101" s="22">
@@ -4655,12 +4676,8 @@
     </row>
     <row r="102" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="22" t="str">
-        <f t="shared" ref="A102:A105" si="2">A96</f>
+        <f t="shared" si="2"/>
         <v>cattle</v>
-      </c>
-      <c r="E102" s="22" t="str">
-        <f t="shared" si="0"/>
-        <v>bulls</v>
       </c>
       <c r="G102" t="s">
         <v>301</v>
@@ -4671,7 +4688,7 @@
       </c>
       <c r="N102" s="22">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O102" s="22" t="str">
         <f t="shared" si="1"/>
@@ -4679,7 +4696,7 @@
       </c>
       <c r="P102" s="22" t="str">
         <f t="shared" si="1"/>
-        <v>No feeding on pasture</v>
+        <v>10% feeding on pasture</v>
       </c>
       <c r="Q102" s="22" t="str">
         <f t="shared" si="1"/>
@@ -4689,7 +4706,7 @@
     <row r="103" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="22" t="str">
         <f t="shared" si="2"/>
-        <v>cattle</v>
+        <v>sheep</v>
       </c>
       <c r="G103" t="s">
         <v>301</v>
@@ -4700,16 +4717,13 @@
       </c>
       <c r="N103" s="22">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="O103" s="22" t="str">
         <f t="shared" si="1"/>
         <v>%</v>
       </c>
-      <c r="P103" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>10% feeding on pasture</v>
-      </c>
+      <c r="P103" s="22"/>
       <c r="Q103" s="22" t="str">
         <f t="shared" si="1"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
@@ -4718,7 +4732,7 @@
     <row r="104" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="22" t="str">
         <f t="shared" si="2"/>
-        <v>sheep</v>
+        <v>horses</v>
       </c>
       <c r="G104" t="s">
         <v>301</v>
@@ -4742,67 +4756,74 @@
       </c>
     </row>
     <row r="105" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A105" s="22" t="str">
-        <f t="shared" si="2"/>
-        <v>horses</v>
-      </c>
       <c r="G105" t="s">
-        <v>301</v>
-      </c>
-      <c r="M105" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N105" s="22">
-        <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-      <c r="O105" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>%</v>
-      </c>
-      <c r="P105" s="22"/>
-      <c r="Q105" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
+        <v>633</v>
+      </c>
+      <c r="M105" s="21" t="s">
+        <v>378</v>
+      </c>
+      <c r="N105" s="21">
+        <v>5</v>
+      </c>
+      <c r="O105" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="P105" s="21"/>
+      <c r="Q105" t="s">
+        <v>639</v>
       </c>
     </row>
     <row r="106" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A106" s="22" t="str">
+        <f>A94</f>
+        <v>cattle</v>
+      </c>
+      <c r="B106" s="22" t="str">
+        <f>B94</f>
+        <v>dairy</v>
+      </c>
+      <c r="E106" s="22" t="str">
+        <f t="shared" ref="E106:E107" si="3">E94</f>
+        <v>cows</v>
+      </c>
       <c r="G106" t="s">
         <v>633</v>
       </c>
-      <c r="M106" s="21" t="s">
-        <v>378</v>
-      </c>
-      <c r="N106" s="21">
+      <c r="M106" s="22" t="str">
+        <f t="shared" ref="M106:Q110" si="4">M94</f>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N106" s="22">
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="O106" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="P106" s="21"/>
-      <c r="Q106" t="s">
-        <v>639</v>
+      <c r="O106" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="P106" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="Q106" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="107" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="22" t="str">
-        <f>A95</f>
+        <f t="shared" ref="A107:A110" si="5">A95</f>
         <v>cattle</v>
       </c>
-      <c r="B107" s="22" t="str">
-        <f>B95</f>
-        <v>dairy</v>
-      </c>
       <c r="E107" s="22" t="str">
-        <f t="shared" ref="E107:E108" si="3">E95</f>
-        <v>cows</v>
+        <f t="shared" si="3"/>
+        <v>bulls</v>
       </c>
       <c r="G107" t="s">
         <v>633</v>
       </c>
       <c r="M107" s="22" t="str">
-        <f t="shared" ref="M107:Q111" si="4">M95</f>
+        <f t="shared" si="4"/>
         <v>feeding_losses</v>
       </c>
       <c r="N107" s="22">
@@ -4824,12 +4845,8 @@
     </row>
     <row r="108" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="22" t="str">
-        <f t="shared" ref="A108:A111" si="5">A96</f>
+        <f t="shared" si="5"/>
         <v>cattle</v>
-      </c>
-      <c r="E108" s="22" t="str">
-        <f t="shared" si="3"/>
-        <v>bulls</v>
       </c>
       <c r="G108" t="s">
         <v>633</v>
@@ -4840,7 +4857,7 @@
       </c>
       <c r="N108" s="22">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O108" s="22" t="str">
         <f t="shared" si="4"/>
@@ -4848,7 +4865,7 @@
       </c>
       <c r="P108" s="22" t="str">
         <f t="shared" si="4"/>
-        <v>No feeding on pasture</v>
+        <v>10% feeding on pasture</v>
       </c>
       <c r="Q108" s="22" t="str">
         <f t="shared" si="4"/>
@@ -4858,7 +4875,7 @@
     <row r="109" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="22" t="str">
         <f t="shared" si="5"/>
-        <v>cattle</v>
+        <v>sheep</v>
       </c>
       <c r="G109" t="s">
         <v>633</v>
@@ -4869,25 +4886,22 @@
       </c>
       <c r="N109" s="22">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="O109" s="22" t="str">
         <f t="shared" si="4"/>
         <v>%</v>
       </c>
-      <c r="P109" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>10% feeding on pasture</v>
-      </c>
+      <c r="P109" s="21"/>
       <c r="Q109" s="22" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="Q109:Q110" si="6">Q97</f>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="110" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="22" t="str">
         <f t="shared" si="5"/>
-        <v>sheep</v>
+        <v>horses</v>
       </c>
       <c r="G110" t="s">
         <v>633</v>
@@ -4906,39 +4920,26 @@
       </c>
       <c r="P110" s="21"/>
       <c r="Q110" s="22" t="str">
-        <f t="shared" ref="Q110:Q111" si="6">Q98</f>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A111" s="22" t="str">
-        <f t="shared" si="5"/>
-        <v>horses</v>
-      </c>
-      <c r="G111" t="s">
-        <v>633</v>
-      </c>
-      <c r="M111" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N111" s="22">
-        <f t="shared" si="4"/>
-        <v>15</v>
-      </c>
-      <c r="O111" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>%</v>
-      </c>
-      <c r="P111" s="21"/>
-      <c r="Q111" s="22" t="str">
         <f t="shared" si="6"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
+    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N111" s="3"/>
+      <c r="P111" s="21"/>
+    </row>
     <row r="112" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N112" s="3"/>
-      <c r="P112" s="21"/>
+      <c r="A112" s="3"/>
+      <c r="G112" t="s">
+        <v>634</v>
+      </c>
+      <c r="M112" s="21" t="s">
+        <v>378</v>
+      </c>
+      <c r="N112" s="21"/>
+      <c r="P112" s="3" t="s">
+        <v>636</v>
+      </c>
     </row>
     <row r="113" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A113" s="3"/>
@@ -4946,32 +4947,32 @@
         <v>634</v>
       </c>
       <c r="M113" s="21" t="s">
-        <v>378</v>
-      </c>
-      <c r="N113" s="21"/>
+        <v>379</v>
+      </c>
+      <c r="N113" s="21">
+        <v>2</v>
+      </c>
+      <c r="O113" s="21" t="s">
+        <v>23</v>
+      </c>
       <c r="P113" s="3" t="s">
-        <v>636</v>
+        <v>640</v>
+      </c>
+      <c r="Q113" t="s">
+        <v>638</v>
       </c>
     </row>
     <row r="114" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A114" s="3"/>
       <c r="G114" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="M114" s="21" t="s">
-        <v>379</v>
-      </c>
-      <c r="N114" s="21">
-        <v>2</v>
-      </c>
-      <c r="O114" s="21" t="s">
-        <v>23</v>
-      </c>
+        <v>378</v>
+      </c>
+      <c r="N114" s="21"/>
       <c r="P114" s="3" t="s">
-        <v>640</v>
-      </c>
-      <c r="Q114" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
     </row>
     <row r="115" spans="1:17" x14ac:dyDescent="0.25">
@@ -4980,67 +4981,82 @@
         <v>635</v>
       </c>
       <c r="M115" s="21" t="s">
-        <v>378</v>
-      </c>
-      <c r="N115" s="21"/>
+        <v>379</v>
+      </c>
+      <c r="N115" s="21">
+        <v>3</v>
+      </c>
+      <c r="O115" s="21" t="s">
+        <v>23</v>
+      </c>
       <c r="P115" s="3" t="s">
-        <v>636</v>
+        <v>640</v>
+      </c>
+      <c r="Q115" t="s">
+        <v>638</v>
       </c>
     </row>
     <row r="116" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A116" s="3"/>
-      <c r="G116" t="s">
-        <v>635</v>
-      </c>
-      <c r="M116" s="21" t="s">
-        <v>379</v>
-      </c>
-      <c r="N116" s="21">
-        <v>3</v>
-      </c>
-      <c r="O116" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="P116" s="3" t="s">
-        <v>640</v>
-      </c>
-      <c r="Q116" t="s">
-        <v>638</v>
-      </c>
+      <c r="N116" s="3"/>
+      <c r="P116" s="21"/>
     </row>
     <row r="117" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N117" s="3"/>
-      <c r="P117" s="21"/>
+      <c r="A117" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="B117" s="1"/>
+      <c r="C117" s="1"/>
+      <c r="D117" s="1"/>
+      <c r="E117" s="2"/>
+      <c r="F117" s="2"/>
+      <c r="G117" s="2"/>
+      <c r="H117" s="2"/>
+      <c r="I117" s="2"/>
+      <c r="J117" s="2"/>
+      <c r="K117" s="2"/>
+      <c r="L117" s="2"/>
+      <c r="M117" s="2"/>
+      <c r="N117" s="2"/>
+      <c r="O117" s="2"/>
+      <c r="P117" s="2"/>
+      <c r="Q117" s="2"/>
     </row>
     <row r="118" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A118" s="1" t="s">
-        <v>600</v>
-      </c>
-      <c r="B118" s="1"/>
-      <c r="C118" s="1"/>
-      <c r="D118" s="1"/>
-      <c r="E118" s="2"/>
-      <c r="F118" s="2"/>
-      <c r="G118" s="2"/>
-      <c r="H118" s="2"/>
-      <c r="I118" s="2"/>
-      <c r="J118" s="2"/>
-      <c r="K118" s="2"/>
-      <c r="L118" s="2"/>
-      <c r="M118" s="2"/>
-      <c r="N118" s="2"/>
-      <c r="O118" s="2"/>
-      <c r="P118" s="2"/>
-      <c r="Q118" s="2"/>
+      <c r="A118" t="s">
+        <v>19</v>
+      </c>
+      <c r="N118" s="21"/>
+      <c r="P118" s="21" t="s">
+        <v>601</v>
+      </c>
     </row>
     <row r="119" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>19</v>
-      </c>
-      <c r="N119" s="21"/>
-      <c r="P119" s="21" t="s">
-        <v>601</v>
-      </c>
+      <c r="A119" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="B119" s="3"/>
+      <c r="C119" s="3"/>
+      <c r="D119" s="3"/>
+      <c r="E119" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="F119" s="3"/>
+      <c r="G119" s="3"/>
+      <c r="H119" s="3"/>
+      <c r="I119" s="3"/>
+      <c r="J119" s="3"/>
+      <c r="K119" s="3"/>
+      <c r="L119" s="3"/>
+      <c r="M119" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="N119" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="O119" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="P119" s="3"/>
     </row>
     <row r="120" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="s">
@@ -5049,9 +5065,7 @@
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
       <c r="D120" s="3"/>
-      <c r="E120" s="3" t="s">
-        <v>485</v>
-      </c>
+      <c r="E120" s="3"/>
       <c r="F120" s="3"/>
       <c r="G120" s="3"/>
       <c r="H120" s="3"/>
@@ -5063,7 +5077,7 @@
         <v>486</v>
       </c>
       <c r="N120" s="3">
-        <v>4.5</v>
+        <v>6.5</v>
       </c>
       <c r="O120" s="3" t="s">
         <v>487</v>
@@ -5071,40 +5085,32 @@
       <c r="P120" s="3"/>
     </row>
     <row r="121" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A121" s="3" t="s">
-        <v>381</v>
-      </c>
-      <c r="B121" s="3"/>
-      <c r="C121" s="3"/>
-      <c r="D121" s="3"/>
-      <c r="E121" s="3"/>
-      <c r="F121" s="3"/>
-      <c r="G121" s="3"/>
-      <c r="H121" s="3"/>
-      <c r="I121" s="3"/>
-      <c r="J121" s="3"/>
-      <c r="K121" s="3"/>
-      <c r="L121" s="3"/>
-      <c r="M121" s="3" t="s">
-        <v>486</v>
-      </c>
-      <c r="N121" s="3">
-        <v>6.5</v>
-      </c>
-      <c r="O121" s="3" t="s">
-        <v>487</v>
+      <c r="A121" t="s">
+        <v>377</v>
+      </c>
+      <c r="M121" t="s">
+        <v>488</v>
+      </c>
+      <c r="N121" s="21">
+        <v>18</v>
+      </c>
+      <c r="O121" t="s">
+        <v>489</v>
       </c>
       <c r="P121" s="3"/>
+      <c r="Q121" t="s">
+        <v>490</v>
+      </c>
     </row>
     <row r="122" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>377</v>
+        <v>20</v>
       </c>
       <c r="M122" t="s">
         <v>488</v>
       </c>
       <c r="N122" s="21">
-        <v>18</v>
+        <v>1.5</v>
       </c>
       <c r="O122" t="s">
         <v>489</v>
@@ -5116,13 +5122,13 @@
     </row>
     <row r="123" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>20</v>
+        <v>374</v>
       </c>
       <c r="M123" t="s">
         <v>488</v>
       </c>
       <c r="N123" s="21">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="O123" t="s">
         <v>489</v>
@@ -5133,28 +5139,28 @@
       </c>
     </row>
     <row r="124" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
-        <v>374</v>
-      </c>
-      <c r="M124" t="s">
-        <v>488</v>
-      </c>
-      <c r="N124" s="21">
-        <v>0</v>
-      </c>
-      <c r="O124" t="s">
-        <v>489</v>
-      </c>
+      <c r="N124" s="21"/>
       <c r="P124" s="3"/>
-      <c r="Q124" t="s">
-        <v>490</v>
-      </c>
     </row>
     <row r="125" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N125" s="21"/>
-      <c r="P125" s="3"/>
+      <c r="M125" t="s">
+        <v>602</v>
+      </c>
+      <c r="N125" s="21">
+        <v>1</v>
+      </c>
+      <c r="O125" s="21" t="s">
+        <v>603</v>
+      </c>
+      <c r="P125" s="21" t="s">
+        <v>604</v>
+      </c>
+      <c r="Q125" s="21"/>
     </row>
     <row r="126" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>19</v>
+      </c>
       <c r="M126" t="s">
         <v>602</v>
       </c>
@@ -5164,15 +5170,19 @@
       <c r="O126" s="21" t="s">
         <v>603</v>
       </c>
-      <c r="P126" s="21" t="s">
-        <v>604</v>
-      </c>
+      <c r="P126" s="21"/>
       <c r="Q126" s="21"/>
     </row>
     <row r="127" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>19</v>
       </c>
+      <c r="B127" t="s">
+        <v>314</v>
+      </c>
+      <c r="E127" t="s">
+        <v>315</v>
+      </c>
       <c r="M127" t="s">
         <v>602</v>
       </c>
@@ -5193,7 +5203,7 @@
         <v>314</v>
       </c>
       <c r="E128" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="M128" t="s">
         <v>602</v>
@@ -5212,7 +5222,7 @@
         <v>19</v>
       </c>
       <c r="B129" t="s">
-        <v>314</v>
+        <v>605</v>
       </c>
       <c r="E129" t="s">
         <v>317</v>
@@ -5230,86 +5240,72 @@
       <c r="Q129" s="21"/>
     </row>
     <row r="130" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A130" t="s">
-        <v>19</v>
-      </c>
-      <c r="B130" t="s">
-        <v>605</v>
-      </c>
-      <c r="E130" t="s">
-        <v>317</v>
-      </c>
-      <c r="M130" t="s">
-        <v>602</v>
-      </c>
-      <c r="N130" s="21">
-        <v>1</v>
-      </c>
-      <c r="O130" s="21" t="s">
-        <v>603</v>
-      </c>
-      <c r="P130" s="21"/>
-      <c r="Q130" s="21"/>
+      <c r="N130" s="3"/>
+      <c r="P130" s="3"/>
     </row>
     <row r="131" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N131" s="3"/>
-      <c r="P131" s="3"/>
+      <c r="A131" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B131" s="1"/>
+      <c r="C131" s="1"/>
+      <c r="D131" s="1"/>
+      <c r="E131" s="2"/>
+      <c r="F131" s="2"/>
+      <c r="G131" s="2"/>
+      <c r="H131" s="2"/>
+      <c r="I131" s="2"/>
+      <c r="J131" s="2"/>
+      <c r="K131" s="2"/>
+      <c r="L131" s="2"/>
+      <c r="M131" s="2"/>
+      <c r="N131" s="2"/>
+      <c r="O131" s="2"/>
+      <c r="P131" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="Q131" s="2"/>
     </row>
     <row r="132" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A132" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B132" s="1"/>
-      <c r="C132" s="1"/>
-      <c r="D132" s="1"/>
-      <c r="E132" s="2"/>
-      <c r="F132" s="2"/>
-      <c r="G132" s="2"/>
-      <c r="H132" s="2"/>
-      <c r="I132" s="2"/>
-      <c r="J132" s="2"/>
-      <c r="K132" s="2"/>
-      <c r="L132" s="2"/>
-      <c r="M132" s="2"/>
-      <c r="N132" s="2"/>
-      <c r="O132" s="2"/>
-      <c r="P132" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="Q132" s="2"/>
+      <c r="L132" s="103" t="s">
+        <v>617</v>
+      </c>
     </row>
     <row r="133" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="L133" s="103" t="s">
-        <v>617</v>
-      </c>
+      <c r="M133" t="s">
+        <v>375</v>
+      </c>
+      <c r="N133" s="21" t="s">
+        <v>614</v>
+      </c>
+      <c r="O133" t="s">
+        <v>598</v>
+      </c>
+      <c r="P133" s="3"/>
     </row>
     <row r="134" spans="1:17" x14ac:dyDescent="0.25">
       <c r="M134" t="s">
-        <v>375</v>
+        <v>476</v>
       </c>
       <c r="N134" s="21" t="s">
         <v>614</v>
       </c>
       <c r="O134" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="P134" s="3"/>
     </row>
     <row r="135" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M135" t="s">
-        <v>476</v>
+      <c r="M135" s="37" t="s">
+        <v>608</v>
       </c>
       <c r="N135" s="21" t="s">
         <v>614</v>
       </c>
-      <c r="O135" t="s">
-        <v>597</v>
-      </c>
-      <c r="P135" s="3"/>
     </row>
     <row r="136" spans="1:17" x14ac:dyDescent="0.25">
       <c r="M136" s="37" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="N136" s="21" t="s">
         <v>614</v>
@@ -5317,7 +5313,7 @@
     </row>
     <row r="137" spans="1:17" x14ac:dyDescent="0.25">
       <c r="M137" s="37" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="N137" s="21" t="s">
         <v>614</v>
@@ -5325,175 +5321,167 @@
     </row>
     <row r="138" spans="1:17" x14ac:dyDescent="0.25">
       <c r="M138" s="37" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="N138" s="21" t="s">
         <v>614</v>
       </c>
+      <c r="P138" s="3"/>
     </row>
     <row r="139" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M139" s="37" t="s">
-        <v>611</v>
-      </c>
-      <c r="N139" s="21" t="s">
-        <v>614</v>
-      </c>
-      <c r="P139" s="3"/>
+      <c r="L139" s="103" t="s">
+        <v>616</v>
+      </c>
     </row>
     <row r="140" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="L140" s="103" t="s">
-        <v>616</v>
+      <c r="M140" t="s">
+        <v>17</v>
+      </c>
+      <c r="N140" s="21" t="s">
+        <v>615</v>
+      </c>
+      <c r="O140" t="s">
+        <v>622</v>
+      </c>
+      <c r="P140" s="21" t="s">
+        <v>595</v>
       </c>
     </row>
     <row r="141" spans="1:17" x14ac:dyDescent="0.25">
       <c r="M141" t="s">
-        <v>17</v>
+        <v>588</v>
       </c>
       <c r="N141" s="21" t="s">
         <v>615</v>
       </c>
       <c r="O141" t="s">
-        <v>622</v>
-      </c>
-      <c r="P141" s="21" t="s">
-        <v>595</v>
-      </c>
+        <v>596</v>
+      </c>
+      <c r="P141" s="3"/>
     </row>
     <row r="142" spans="1:17" x14ac:dyDescent="0.25">
       <c r="M142" t="s">
-        <v>588</v>
+        <v>477</v>
       </c>
       <c r="N142" s="21" t="s">
         <v>615</v>
       </c>
       <c r="O142" t="s">
-        <v>596</v>
-      </c>
-      <c r="P142" s="3"/>
+        <v>478</v>
+      </c>
+      <c r="P142" s="21" t="s">
+        <v>479</v>
+      </c>
     </row>
     <row r="143" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M143" t="s">
-        <v>477</v>
-      </c>
-      <c r="N143" s="21" t="s">
-        <v>615</v>
-      </c>
-      <c r="O143" t="s">
-        <v>478</v>
-      </c>
-      <c r="P143" s="21" t="s">
-        <v>479</v>
+      <c r="L143" s="103" t="s">
+        <v>618</v>
       </c>
     </row>
     <row r="144" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="L144" s="103" t="s">
-        <v>618</v>
+      <c r="M144" t="s">
+        <v>17</v>
+      </c>
+      <c r="N144" s="21" t="s">
+        <v>625</v>
+      </c>
+      <c r="O144" t="s">
+        <v>622</v>
+      </c>
+      <c r="P144" s="21" t="s">
+        <v>595</v>
       </c>
     </row>
     <row r="145" spans="12:16" x14ac:dyDescent="0.25">
       <c r="M145" t="s">
-        <v>17</v>
+        <v>588</v>
       </c>
       <c r="N145" s="21" t="s">
         <v>625</v>
       </c>
       <c r="O145" t="s">
+        <v>596</v>
+      </c>
+      <c r="P145" s="3"/>
+    </row>
+    <row r="146" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L146" s="103" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="147" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="M147" t="s">
+        <v>17</v>
+      </c>
+      <c r="N147" s="21" t="s">
+        <v>626</v>
+      </c>
+      <c r="O147" t="s">
         <v>622</v>
       </c>
-      <c r="P145" s="21" t="s">
+      <c r="P147" s="21" t="s">
         <v>595</v>
-      </c>
-    </row>
-    <row r="146" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="M146" t="s">
-        <v>588</v>
-      </c>
-      <c r="N146" s="21" t="s">
-        <v>625</v>
-      </c>
-      <c r="O146" t="s">
-        <v>596</v>
-      </c>
-      <c r="P146" s="3"/>
-    </row>
-    <row r="147" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="L147" s="103" t="s">
-        <v>619</v>
       </c>
     </row>
     <row r="148" spans="12:16" x14ac:dyDescent="0.25">
       <c r="M148" t="s">
-        <v>17</v>
+        <v>588</v>
       </c>
       <c r="N148" s="21" t="s">
         <v>626</v>
       </c>
       <c r="O148" t="s">
-        <v>622</v>
-      </c>
-      <c r="P148" s="21" t="s">
+        <v>596</v>
+      </c>
+      <c r="P148" s="3"/>
+    </row>
+    <row r="149" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L149" s="103" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="150" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="M150" t="s">
+        <v>17</v>
+      </c>
+      <c r="N150" s="21" t="s">
+        <v>627</v>
+      </c>
+      <c r="O150" t="s">
+        <v>623</v>
+      </c>
+      <c r="P150" s="21" t="s">
         <v>595</v>
-      </c>
-    </row>
-    <row r="149" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="M149" t="s">
-        <v>588</v>
-      </c>
-      <c r="N149" s="21" t="s">
-        <v>626</v>
-      </c>
-      <c r="O149" t="s">
-        <v>596</v>
-      </c>
-      <c r="P149" s="3"/>
-    </row>
-    <row r="150" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="L150" s="103" t="s">
-        <v>620</v>
       </c>
     </row>
     <row r="151" spans="12:16" x14ac:dyDescent="0.25">
       <c r="M151" t="s">
-        <v>17</v>
+        <v>588</v>
       </c>
       <c r="N151" s="21" t="s">
         <v>627</v>
       </c>
       <c r="O151" t="s">
-        <v>623</v>
-      </c>
-      <c r="P151" s="21" t="s">
-        <v>595</v>
-      </c>
+        <v>596</v>
+      </c>
+      <c r="P151" s="3"/>
     </row>
     <row r="152" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="M152" t="s">
-        <v>588</v>
-      </c>
-      <c r="N152" s="21" t="s">
-        <v>627</v>
-      </c>
-      <c r="O152" t="s">
-        <v>596</v>
-      </c>
-      <c r="P152" s="3"/>
+      <c r="L152" s="103" t="s">
+        <v>621</v>
+      </c>
     </row>
     <row r="153" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="L153" s="103" t="s">
-        <v>621</v>
-      </c>
-    </row>
-    <row r="154" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="M154" t="s">
+      <c r="M153" t="s">
         <v>613</v>
       </c>
-      <c r="N154" s="21" t="s">
+      <c r="N153" s="21" t="s">
         <v>628</v>
       </c>
-      <c r="O154" t="s">
+      <c r="O153" t="s">
         <v>624</v>
       </c>
-      <c r="P154" s="21"/>
+      <c r="P153" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Finnished implementation of SheepHerd and added necessary data
</commit_message>
<xml_diff>
--- a/data/default/FeedMgmt.xlsx
+++ b/data/default/FeedMgmt.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1561" uniqueCount="648">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1566" uniqueCount="648">
   <si>
     <t>f_feed</t>
   </si>
@@ -2804,7 +2804,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R153"/>
+  <dimension ref="A1:R158"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="7" width="20.28515625" customWidth="1"/>
@@ -4310,47 +4310,54 @@
       <c r="P85" s="3"/>
     </row>
     <row r="86" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N86" s="3"/>
+      <c r="A86" t="s">
+        <v>381</v>
+      </c>
+      <c r="H86" t="s">
+        <v>319</v>
+      </c>
+      <c r="I86" t="s">
+        <v>28</v>
+      </c>
+      <c r="M86" t="s">
+        <v>320</v>
+      </c>
+      <c r="N86" s="3">
+        <v>90</v>
+      </c>
+      <c r="O86" t="s">
+        <v>23</v>
+      </c>
       <c r="P86" s="3"/>
     </row>
     <row r="87" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A87" s="1" t="s">
+      <c r="N87" s="3"/>
+      <c r="P87" s="3"/>
+    </row>
+    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A88" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="B87" s="1"/>
-      <c r="C87" s="1"/>
-      <c r="D87" s="1"/>
-      <c r="E87" s="2"/>
-      <c r="F87" s="2"/>
-      <c r="G87" s="2"/>
-      <c r="H87" s="2"/>
-      <c r="I87" s="2"/>
-      <c r="J87" s="2"/>
-      <c r="K87" s="2"/>
-      <c r="L87" s="2"/>
-      <c r="M87" s="2"/>
-      <c r="N87" s="2"/>
-      <c r="O87" s="2"/>
-      <c r="P87" s="2"/>
-      <c r="Q87" s="2"/>
-    </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M88" s="6" t="s">
-        <v>378</v>
-      </c>
-      <c r="N88" s="6">
-        <v>0</v>
-      </c>
-      <c r="O88" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="P88" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="B88" s="1"/>
+      <c r="C88" s="1"/>
+      <c r="D88" s="1"/>
+      <c r="E88" s="2"/>
+      <c r="F88" s="2"/>
+      <c r="G88" s="2"/>
+      <c r="H88" s="2"/>
+      <c r="I88" s="2"/>
+      <c r="J88" s="2"/>
+      <c r="K88" s="2"/>
+      <c r="L88" s="2"/>
+      <c r="M88" s="2"/>
+      <c r="N88" s="2"/>
+      <c r="O88" s="2"/>
+      <c r="P88" s="2"/>
+      <c r="Q88" s="2"/>
     </row>
     <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="M89" s="6" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="N89" s="6">
         <v>0</v>
@@ -4363,39 +4370,29 @@
       </c>
     </row>
     <row r="90" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>19</v>
-      </c>
-      <c r="B90" t="s">
-        <v>314</v>
-      </c>
-      <c r="E90" t="s">
-        <v>315</v>
-      </c>
-      <c r="G90" t="s">
-        <v>632</v>
-      </c>
-      <c r="M90" s="21" t="s">
-        <v>378</v>
-      </c>
-      <c r="N90" s="21">
-        <f>(0.8*20+0.2*2)</f>
-        <v>16.399999999999999</v>
-      </c>
-      <c r="O90" s="21" t="s">
+      <c r="M90" s="6" t="s">
+        <v>379</v>
+      </c>
+      <c r="N90" s="6">
+        <v>0</v>
+      </c>
+      <c r="O90" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="P90" s="21" t="s">
-        <v>382</v>
-      </c>
-      <c r="Q90" t="s">
-        <v>639</v>
+      <c r="P90" s="6" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="91" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>19</v>
       </c>
+      <c r="B91" t="s">
+        <v>314</v>
+      </c>
+      <c r="E91" t="s">
+        <v>315</v>
+      </c>
       <c r="G91" t="s">
         <v>632</v>
       </c>
@@ -4403,37 +4400,38 @@
         <v>378</v>
       </c>
       <c r="N91" s="21">
+        <f>(0.8*20+0.2*2)</f>
+        <v>16.399999999999999</v>
+      </c>
+      <c r="O91" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="P91" s="21" t="s">
+        <v>382</v>
+      </c>
+      <c r="Q91" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>19</v>
+      </c>
+      <c r="G92" t="s">
+        <v>632</v>
+      </c>
+      <c r="M92" s="21" t="s">
+        <v>378</v>
+      </c>
+      <c r="N92" s="21">
         <f>(0.6*20+0.4*2)</f>
         <v>12.8</v>
       </c>
-      <c r="O91" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="P91" s="21" t="s">
-        <v>383</v>
-      </c>
-      <c r="Q91" t="s">
-        <v>639</v>
-      </c>
-    </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>381</v>
-      </c>
-      <c r="G92" t="s">
-        <v>632</v>
-      </c>
-      <c r="M92" s="21" t="s">
-        <v>378</v>
-      </c>
-      <c r="N92" s="21">
-        <v>2</v>
-      </c>
       <c r="O92" s="21" t="s">
         <v>23</v>
       </c>
       <c r="P92" s="21" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="Q92" t="s">
         <v>639</v>
@@ -4441,7 +4439,7 @@
     </row>
     <row r="93" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="G93" t="s">
         <v>632</v>
@@ -4464,63 +4462,43 @@
     </row>
     <row r="94" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>19</v>
-      </c>
-      <c r="B94" t="s">
-        <v>314</v>
-      </c>
-      <c r="E94" t="s">
-        <v>315</v>
+        <v>377</v>
       </c>
       <c r="G94" t="s">
         <v>632</v>
       </c>
       <c r="M94" s="21" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="N94" s="21">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O94" s="21" t="s">
         <v>23</v>
       </c>
       <c r="P94" s="21" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="Q94" t="s">
         <v>639</v>
       </c>
     </row>
     <row r="95" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>19</v>
-      </c>
-      <c r="E95" t="s">
-        <v>317</v>
-      </c>
-      <c r="G95" t="s">
-        <v>632</v>
-      </c>
-      <c r="M95" s="21" t="s">
-        <v>379</v>
-      </c>
-      <c r="N95" s="21">
-        <v>5</v>
-      </c>
-      <c r="O95" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="P95" s="21" t="s">
-        <v>385</v>
-      </c>
-      <c r="Q95" t="s">
-        <v>639</v>
-      </c>
+      <c r="M95" s="21"/>
+      <c r="N95" s="21"/>
+      <c r="O95" s="21"/>
+      <c r="P95" s="21"/>
     </row>
     <row r="96" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>19</v>
       </c>
+      <c r="B96" t="s">
+        <v>314</v>
+      </c>
+      <c r="E96" t="s">
+        <v>315</v>
+      </c>
       <c r="G96" t="s">
         <v>632</v>
       </c>
@@ -4528,73 +4506,80 @@
         <v>379</v>
       </c>
       <c r="N96" s="21">
+        <v>5</v>
+      </c>
+      <c r="O96" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="P96" s="21" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q96" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>19</v>
+      </c>
+      <c r="E97" t="s">
+        <v>317</v>
+      </c>
+      <c r="G97" t="s">
+        <v>632</v>
+      </c>
+      <c r="M97" s="21" t="s">
+        <v>379</v>
+      </c>
+      <c r="N97" s="21">
+        <v>5</v>
+      </c>
+      <c r="O97" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="P97" s="21" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q97" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>19</v>
+      </c>
+      <c r="G98" t="s">
+        <v>632</v>
+      </c>
+      <c r="M98" s="21" t="s">
+        <v>379</v>
+      </c>
+      <c r="N98" s="21">
         <f>0.9*5+0.1*15</f>
         <v>6</v>
       </c>
-      <c r="O96" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="P96" s="21" t="s">
-        <v>386</v>
-      </c>
-      <c r="Q96" t="s">
-        <v>639</v>
-      </c>
-    </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>381</v>
-      </c>
-      <c r="G97" t="s">
-        <v>632</v>
-      </c>
-      <c r="M97" s="21" t="s">
-        <v>379</v>
-      </c>
-      <c r="N97" s="21">
-        <v>15</v>
-      </c>
-      <c r="O97" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="P97" s="21"/>
-      <c r="Q97" t="s">
-        <v>639</v>
-      </c>
-    </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>377</v>
-      </c>
-      <c r="G98" t="s">
-        <v>632</v>
-      </c>
-      <c r="M98" s="21" t="s">
-        <v>379</v>
-      </c>
-      <c r="N98" s="21">
-        <v>15</v>
-      </c>
       <c r="O98" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="P98" s="21"/>
+      <c r="P98" s="21" t="s">
+        <v>386</v>
+      </c>
       <c r="Q98" t="s">
         <v>639</v>
       </c>
     </row>
     <row r="99" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A99" s="22"/>
-      <c r="B99" s="22"/>
-      <c r="E99" s="22"/>
+      <c r="A99" t="s">
+        <v>381</v>
+      </c>
       <c r="G99" t="s">
-        <v>301</v>
+        <v>632</v>
       </c>
       <c r="M99" s="21" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="N99" s="21">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="O99" s="21" t="s">
         <v>23</v>
@@ -4605,125 +4590,85 @@
       </c>
     </row>
     <row r="100" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A100" s="22" t="str">
-        <f>A94</f>
+      <c r="A100" t="s">
+        <v>377</v>
+      </c>
+      <c r="G100" t="s">
+        <v>632</v>
+      </c>
+      <c r="M100" s="21" t="s">
+        <v>379</v>
+      </c>
+      <c r="N100" s="21">
+        <v>15</v>
+      </c>
+      <c r="O100" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="P100" s="21"/>
+      <c r="Q100" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M101" s="21"/>
+      <c r="N101" s="21"/>
+      <c r="O101" s="21"/>
+      <c r="P101" s="21"/>
+    </row>
+    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A102" s="22"/>
+      <c r="B102" s="22"/>
+      <c r="E102" s="22"/>
+      <c r="G102" t="s">
+        <v>301</v>
+      </c>
+      <c r="M102" s="21" t="s">
+        <v>378</v>
+      </c>
+      <c r="N102" s="21">
+        <v>5</v>
+      </c>
+      <c r="O102" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="P102" s="21"/>
+      <c r="Q102" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A103" s="22" t="str">
+        <f>A96</f>
         <v>cattle</v>
       </c>
-      <c r="B100" s="22" t="str">
-        <f>B94</f>
+      <c r="B103" s="22" t="str">
+        <f>B96</f>
         <v>dairy</v>
       </c>
-      <c r="E100" s="22" t="str">
-        <f t="shared" ref="E100:E101" si="0">E94</f>
+      <c r="E103" s="22" t="str">
+        <f t="shared" ref="E103:E104" si="0">E96</f>
         <v>cows</v>
       </c>
-      <c r="G100" t="s">
+      <c r="G103" t="s">
         <v>301</v>
       </c>
-      <c r="M100" s="22" t="str">
-        <f t="shared" ref="M100:Q104" si="1">M94</f>
+      <c r="M103" s="22" t="str">
+        <f t="shared" ref="M103:Q107" si="1">M96</f>
         <v>feeding_losses</v>
       </c>
-      <c r="N100" s="22">
+      <c r="N103" s="22">
         <f t="shared" si="1"/>
         <v>5</v>
-      </c>
-      <c r="O100" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>%</v>
-      </c>
-      <c r="P100" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="Q100" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A101" s="22" t="str">
-        <f t="shared" ref="A101:A104" si="2">A95</f>
-        <v>cattle</v>
-      </c>
-      <c r="E101" s="22" t="str">
-        <f t="shared" si="0"/>
-        <v>bulls</v>
-      </c>
-      <c r="G101" t="s">
-        <v>301</v>
-      </c>
-      <c r="M101" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N101" s="22">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="O101" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>%</v>
-      </c>
-      <c r="P101" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="Q101" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A102" s="22" t="str">
-        <f t="shared" si="2"/>
-        <v>cattle</v>
-      </c>
-      <c r="G102" t="s">
-        <v>301</v>
-      </c>
-      <c r="M102" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N102" s="22">
-        <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="O102" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>%</v>
-      </c>
-      <c r="P102" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>10% feeding on pasture</v>
-      </c>
-      <c r="Q102" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A103" s="22" t="str">
-        <f t="shared" si="2"/>
-        <v>sheep</v>
-      </c>
-      <c r="G103" t="s">
-        <v>301</v>
-      </c>
-      <c r="M103" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N103" s="22">
-        <f t="shared" si="1"/>
-        <v>15</v>
       </c>
       <c r="O103" s="22" t="str">
         <f t="shared" si="1"/>
         <v>%</v>
       </c>
-      <c r="P103" s="22"/>
+      <c r="P103" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>No feeding on pasture</v>
+      </c>
       <c r="Q103" s="22" t="str">
         <f t="shared" si="1"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
@@ -4731,8 +4676,12 @@
     </row>
     <row r="104" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="22" t="str">
-        <f t="shared" si="2"/>
-        <v>horses</v>
+        <f t="shared" ref="A104:A107" si="2">A97</f>
+        <v>cattle</v>
+      </c>
+      <c r="E104" s="22" t="str">
+        <f t="shared" si="0"/>
+        <v>bulls</v>
       </c>
       <c r="G104" t="s">
         <v>301</v>
@@ -4743,745 +4692,844 @@
       </c>
       <c r="N104" s="22">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="O104" s="22" t="str">
         <f t="shared" si="1"/>
         <v>%</v>
       </c>
-      <c r="P104" s="22"/>
+      <c r="P104" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>No feeding on pasture</v>
+      </c>
       <c r="Q104" s="22" t="str">
         <f t="shared" si="1"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="105" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A105" s="22" t="str">
+        <f t="shared" si="2"/>
+        <v>cattle</v>
+      </c>
       <c r="G105" t="s">
-        <v>633</v>
-      </c>
-      <c r="M105" s="21" t="s">
-        <v>378</v>
-      </c>
-      <c r="N105" s="21">
-        <v>5</v>
-      </c>
-      <c r="O105" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="P105" s="21"/>
-      <c r="Q105" t="s">
-        <v>639</v>
+        <v>301</v>
+      </c>
+      <c r="M105" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N105" s="22">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="O105" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="P105" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>10% feeding on pasture</v>
+      </c>
+      <c r="Q105" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="106" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="22" t="str">
-        <f>A94</f>
+        <f t="shared" si="2"/>
+        <v>sheep</v>
+      </c>
+      <c r="G106" t="s">
+        <v>301</v>
+      </c>
+      <c r="M106" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N106" s="22">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="O106" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="P106" s="22"/>
+      <c r="Q106" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A107" s="22" t="str">
+        <f t="shared" si="2"/>
+        <v>horses</v>
+      </c>
+      <c r="G107" t="s">
+        <v>301</v>
+      </c>
+      <c r="M107" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N107" s="22">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="O107" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="P107" s="22"/>
+      <c r="Q107" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A108" s="22"/>
+      <c r="M108" s="22"/>
+      <c r="N108" s="22"/>
+      <c r="O108" s="22"/>
+      <c r="P108" s="22"/>
+      <c r="Q108" s="22"/>
+    </row>
+    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="G109" t="s">
+        <v>633</v>
+      </c>
+      <c r="M109" s="21" t="s">
+        <v>378</v>
+      </c>
+      <c r="N109" s="21">
+        <v>5</v>
+      </c>
+      <c r="O109" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="P109" s="21"/>
+      <c r="Q109" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A110" s="22" t="str">
+        <f>A96</f>
         <v>cattle</v>
       </c>
-      <c r="B106" s="22" t="str">
-        <f>B94</f>
+      <c r="B110" s="22" t="str">
+        <f>B96</f>
         <v>dairy</v>
       </c>
-      <c r="E106" s="22" t="str">
-        <f t="shared" ref="E106:E107" si="3">E94</f>
+      <c r="E110" s="22" t="str">
+        <f t="shared" ref="E110:E111" si="3">E96</f>
         <v>cows</v>
       </c>
-      <c r="G106" t="s">
+      <c r="G110" t="s">
         <v>633</v>
       </c>
-      <c r="M106" s="22" t="str">
-        <f t="shared" ref="M106:Q110" si="4">M94</f>
+      <c r="M110" s="22" t="str">
+        <f t="shared" ref="M110:Q114" si="4">M96</f>
         <v>feeding_losses</v>
       </c>
-      <c r="N106" s="22">
+      <c r="N110" s="22">
         <f t="shared" si="4"/>
         <v>5</v>
-      </c>
-      <c r="O106" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>%</v>
-      </c>
-      <c r="P106" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="Q106" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A107" s="22" t="str">
-        <f t="shared" ref="A107:A110" si="5">A95</f>
-        <v>cattle</v>
-      </c>
-      <c r="E107" s="22" t="str">
-        <f t="shared" si="3"/>
-        <v>bulls</v>
-      </c>
-      <c r="G107" t="s">
-        <v>633</v>
-      </c>
-      <c r="M107" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N107" s="22">
-        <f t="shared" si="4"/>
-        <v>5</v>
-      </c>
-      <c r="O107" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>%</v>
-      </c>
-      <c r="P107" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="Q107" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A108" s="22" t="str">
-        <f t="shared" si="5"/>
-        <v>cattle</v>
-      </c>
-      <c r="G108" t="s">
-        <v>633</v>
-      </c>
-      <c r="M108" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N108" s="22">
-        <f t="shared" si="4"/>
-        <v>6</v>
-      </c>
-      <c r="O108" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>%</v>
-      </c>
-      <c r="P108" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>10% feeding on pasture</v>
-      </c>
-      <c r="Q108" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A109" s="22" t="str">
-        <f t="shared" si="5"/>
-        <v>sheep</v>
-      </c>
-      <c r="G109" t="s">
-        <v>633</v>
-      </c>
-      <c r="M109" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N109" s="22">
-        <f t="shared" si="4"/>
-        <v>15</v>
-      </c>
-      <c r="O109" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>%</v>
-      </c>
-      <c r="P109" s="21"/>
-      <c r="Q109" s="22" t="str">
-        <f t="shared" ref="Q109:Q110" si="6">Q97</f>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A110" s="22" t="str">
-        <f t="shared" si="5"/>
-        <v>horses</v>
-      </c>
-      <c r="G110" t="s">
-        <v>633</v>
-      </c>
-      <c r="M110" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N110" s="22">
-        <f t="shared" si="4"/>
-        <v>15</v>
       </c>
       <c r="O110" s="22" t="str">
         <f t="shared" si="4"/>
         <v>%</v>
       </c>
-      <c r="P110" s="21"/>
+      <c r="P110" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>No feeding on pasture</v>
+      </c>
       <c r="Q110" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A111" s="22" t="str">
+        <f t="shared" ref="A111:A114" si="5">A97</f>
+        <v>cattle</v>
+      </c>
+      <c r="E111" s="22" t="str">
+        <f t="shared" si="3"/>
+        <v>bulls</v>
+      </c>
+      <c r="G111" t="s">
+        <v>633</v>
+      </c>
+      <c r="M111" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N111" s="22">
+        <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="O111" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="P111" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="Q111" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A112" s="22" t="str">
+        <f t="shared" si="5"/>
+        <v>cattle</v>
+      </c>
+      <c r="G112" t="s">
+        <v>633</v>
+      </c>
+      <c r="M112" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N112" s="22">
+        <f t="shared" si="4"/>
+        <v>6</v>
+      </c>
+      <c r="O112" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="P112" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>10% feeding on pasture</v>
+      </c>
+      <c r="Q112" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A113" s="22" t="str">
+        <f t="shared" si="5"/>
+        <v>sheep</v>
+      </c>
+      <c r="G113" t="s">
+        <v>633</v>
+      </c>
+      <c r="M113" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N113" s="22">
+        <f t="shared" si="4"/>
+        <v>15</v>
+      </c>
+      <c r="O113" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="P113" s="21"/>
+      <c r="Q113" s="22" t="str">
+        <f t="shared" ref="Q113:Q114" si="6">Q99</f>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A114" s="22" t="str">
+        <f t="shared" si="5"/>
+        <v>horses</v>
+      </c>
+      <c r="G114" t="s">
+        <v>633</v>
+      </c>
+      <c r="M114" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N114" s="22">
+        <f t="shared" si="4"/>
+        <v>15</v>
+      </c>
+      <c r="O114" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="P114" s="21"/>
+      <c r="Q114" s="22" t="str">
         <f t="shared" si="6"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N111" s="3"/>
-      <c r="P111" s="21"/>
-    </row>
-    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A112" s="3"/>
-      <c r="G112" t="s">
+    <row r="115" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N115" s="3"/>
+      <c r="P115" s="21"/>
+    </row>
+    <row r="116" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A116" s="3"/>
+      <c r="G116" t="s">
         <v>634</v>
       </c>
-      <c r="M112" s="21" t="s">
+      <c r="M116" s="21" t="s">
         <v>378</v>
       </c>
-      <c r="N112" s="21"/>
-      <c r="P112" s="3" t="s">
+      <c r="N116" s="21"/>
+      <c r="P116" s="3" t="s">
         <v>636</v>
       </c>
     </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A113" s="3"/>
-      <c r="G113" t="s">
+    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A117" s="3"/>
+      <c r="G117" t="s">
         <v>634</v>
       </c>
-      <c r="M113" s="21" t="s">
+      <c r="M117" s="21" t="s">
         <v>379</v>
       </c>
-      <c r="N113" s="21">
+      <c r="N117" s="21">
         <v>2</v>
       </c>
-      <c r="O113" s="21" t="s">
+      <c r="O117" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="P113" s="3" t="s">
+      <c r="P117" s="3" t="s">
         <v>640</v>
       </c>
-      <c r="Q113" t="s">
+      <c r="Q117" t="s">
         <v>638</v>
       </c>
     </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A114" s="3"/>
-      <c r="G114" t="s">
+    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A118" s="3"/>
+      <c r="M118" s="21"/>
+      <c r="N118" s="21"/>
+      <c r="O118" s="21"/>
+      <c r="P118" s="3"/>
+    </row>
+    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A119" s="3"/>
+      <c r="G119" t="s">
         <v>635</v>
       </c>
-      <c r="M114" s="21" t="s">
+      <c r="M119" s="21" t="s">
         <v>378</v>
       </c>
-      <c r="N114" s="21"/>
-      <c r="P114" s="3" t="s">
+      <c r="N119" s="21"/>
+      <c r="P119" s="3" t="s">
         <v>636</v>
       </c>
     </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A115" s="3"/>
-      <c r="G115" t="s">
+    <row r="120" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A120" s="3"/>
+      <c r="G120" t="s">
         <v>635</v>
       </c>
-      <c r="M115" s="21" t="s">
+      <c r="M120" s="21" t="s">
         <v>379</v>
       </c>
-      <c r="N115" s="21">
+      <c r="N120" s="21">
         <v>3</v>
       </c>
-      <c r="O115" s="21" t="s">
+      <c r="O120" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="P115" s="3" t="s">
+      <c r="P120" s="3" t="s">
         <v>640</v>
       </c>
-      <c r="Q115" t="s">
+      <c r="Q120" t="s">
         <v>638</v>
       </c>
     </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N116" s="3"/>
-      <c r="P116" s="21"/>
-    </row>
-    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A117" s="1" t="s">
+    <row r="121" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N121" s="3"/>
+      <c r="P121" s="21"/>
+    </row>
+    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A122" s="1" t="s">
         <v>600</v>
       </c>
-      <c r="B117" s="1"/>
-      <c r="C117" s="1"/>
-      <c r="D117" s="1"/>
-      <c r="E117" s="2"/>
-      <c r="F117" s="2"/>
-      <c r="G117" s="2"/>
-      <c r="H117" s="2"/>
-      <c r="I117" s="2"/>
-      <c r="J117" s="2"/>
-      <c r="K117" s="2"/>
-      <c r="L117" s="2"/>
-      <c r="M117" s="2"/>
-      <c r="N117" s="2"/>
-      <c r="O117" s="2"/>
-      <c r="P117" s="2"/>
-      <c r="Q117" s="2"/>
-    </row>
-    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>19</v>
-      </c>
-      <c r="N118" s="21"/>
-      <c r="P118" s="21" t="s">
-        <v>601</v>
-      </c>
-    </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A119" s="3" t="s">
-        <v>381</v>
-      </c>
-      <c r="B119" s="3"/>
-      <c r="C119" s="3"/>
-      <c r="D119" s="3"/>
-      <c r="E119" s="3" t="s">
-        <v>485</v>
-      </c>
-      <c r="F119" s="3"/>
-      <c r="G119" s="3"/>
-      <c r="H119" s="3"/>
-      <c r="I119" s="3"/>
-      <c r="J119" s="3"/>
-      <c r="K119" s="3"/>
-      <c r="L119" s="3"/>
-      <c r="M119" s="3" t="s">
-        <v>486</v>
-      </c>
-      <c r="N119" s="3">
-        <v>4.5</v>
-      </c>
-      <c r="O119" s="3" t="s">
-        <v>487</v>
-      </c>
-      <c r="P119" s="3"/>
-    </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A120" s="3" t="s">
-        <v>381</v>
-      </c>
-      <c r="B120" s="3"/>
-      <c r="C120" s="3"/>
-      <c r="D120" s="3"/>
-      <c r="E120" s="3"/>
-      <c r="F120" s="3"/>
-      <c r="G120" s="3"/>
-      <c r="H120" s="3"/>
-      <c r="I120" s="3"/>
-      <c r="J120" s="3"/>
-      <c r="K120" s="3"/>
-      <c r="L120" s="3"/>
-      <c r="M120" s="3" t="s">
-        <v>486</v>
-      </c>
-      <c r="N120" s="3">
-        <v>6.5</v>
-      </c>
-      <c r="O120" s="3" t="s">
-        <v>487</v>
-      </c>
-      <c r="P120" s="3"/>
-    </row>
-    <row r="121" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>377</v>
-      </c>
-      <c r="M121" t="s">
-        <v>488</v>
-      </c>
-      <c r="N121" s="21">
-        <v>18</v>
-      </c>
-      <c r="O121" t="s">
-        <v>489</v>
-      </c>
-      <c r="P121" s="3"/>
-      <c r="Q121" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>20</v>
-      </c>
-      <c r="M122" t="s">
-        <v>488</v>
-      </c>
-      <c r="N122" s="21">
-        <v>1.5</v>
-      </c>
-      <c r="O122" t="s">
-        <v>489</v>
-      </c>
-      <c r="P122" s="3"/>
-      <c r="Q122" t="s">
-        <v>490</v>
-      </c>
+      <c r="B122" s="1"/>
+      <c r="C122" s="1"/>
+      <c r="D122" s="1"/>
+      <c r="E122" s="2"/>
+      <c r="F122" s="2"/>
+      <c r="G122" s="2"/>
+      <c r="H122" s="2"/>
+      <c r="I122" s="2"/>
+      <c r="J122" s="2"/>
+      <c r="K122" s="2"/>
+      <c r="L122" s="2"/>
+      <c r="M122" s="2"/>
+      <c r="N122" s="2"/>
+      <c r="O122" s="2"/>
+      <c r="P122" s="2"/>
+      <c r="Q122" s="2"/>
     </row>
     <row r="123" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>374</v>
-      </c>
-      <c r="M123" t="s">
-        <v>488</v>
-      </c>
-      <c r="N123" s="21">
-        <v>0</v>
-      </c>
-      <c r="O123" t="s">
-        <v>489</v>
-      </c>
-      <c r="P123" s="3"/>
-      <c r="Q123" t="s">
-        <v>490</v>
+        <v>19</v>
+      </c>
+      <c r="N123" s="21"/>
+      <c r="P123" s="21" t="s">
+        <v>601</v>
       </c>
     </row>
     <row r="124" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N124" s="21"/>
+      <c r="A124" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="B124" s="3"/>
+      <c r="C124" s="3"/>
+      <c r="D124" s="3"/>
+      <c r="E124" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="F124" s="3"/>
+      <c r="G124" s="3"/>
+      <c r="H124" s="3"/>
+      <c r="I124" s="3"/>
+      <c r="J124" s="3"/>
+      <c r="K124" s="3"/>
+      <c r="L124" s="3"/>
+      <c r="M124" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="N124" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="O124" s="3" t="s">
+        <v>487</v>
+      </c>
       <c r="P124" s="3"/>
     </row>
     <row r="125" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M125" t="s">
-        <v>602</v>
-      </c>
-      <c r="N125" s="21">
-        <v>1</v>
-      </c>
-      <c r="O125" s="21" t="s">
-        <v>603</v>
-      </c>
-      <c r="P125" s="21" t="s">
-        <v>604</v>
-      </c>
-      <c r="Q125" s="21"/>
+      <c r="A125" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="B125" s="3"/>
+      <c r="C125" s="3"/>
+      <c r="D125" s="3"/>
+      <c r="E125" s="3"/>
+      <c r="F125" s="3"/>
+      <c r="G125" s="3"/>
+      <c r="H125" s="3"/>
+      <c r="I125" s="3"/>
+      <c r="J125" s="3"/>
+      <c r="K125" s="3"/>
+      <c r="L125" s="3"/>
+      <c r="M125" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="N125" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="O125" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="P125" s="3"/>
     </row>
     <row r="126" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>19</v>
+        <v>377</v>
       </c>
       <c r="M126" t="s">
-        <v>602</v>
+        <v>488</v>
       </c>
       <c r="N126" s="21">
-        <v>1</v>
-      </c>
-      <c r="O126" s="21" t="s">
-        <v>603</v>
-      </c>
-      <c r="P126" s="21"/>
-      <c r="Q126" s="21"/>
+        <v>18</v>
+      </c>
+      <c r="O126" t="s">
+        <v>489</v>
+      </c>
+      <c r="P126" s="3"/>
+      <c r="Q126" t="s">
+        <v>490</v>
+      </c>
     </row>
     <row r="127" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>19</v>
-      </c>
-      <c r="B127" t="s">
-        <v>314</v>
-      </c>
-      <c r="E127" t="s">
-        <v>315</v>
+        <v>20</v>
       </c>
       <c r="M127" t="s">
-        <v>602</v>
+        <v>488</v>
       </c>
       <c r="N127" s="21">
-        <v>1</v>
-      </c>
-      <c r="O127" s="21" t="s">
-        <v>603</v>
-      </c>
-      <c r="P127" s="21"/>
-      <c r="Q127" s="21"/>
+        <v>1.5</v>
+      </c>
+      <c r="O127" t="s">
+        <v>489</v>
+      </c>
+      <c r="P127" s="3"/>
+      <c r="Q127" t="s">
+        <v>490</v>
+      </c>
     </row>
     <row r="128" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
+        <v>374</v>
+      </c>
+      <c r="M128" t="s">
+        <v>488</v>
+      </c>
+      <c r="N128" s="21">
+        <v>0</v>
+      </c>
+      <c r="O128" t="s">
+        <v>489</v>
+      </c>
+      <c r="P128" s="3"/>
+      <c r="Q128" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N129" s="21"/>
+      <c r="P129" s="3"/>
+    </row>
+    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M130" t="s">
+        <v>602</v>
+      </c>
+      <c r="N130" s="21">
+        <v>1</v>
+      </c>
+      <c r="O130" s="21" t="s">
+        <v>603</v>
+      </c>
+      <c r="P130" s="21" t="s">
+        <v>604</v>
+      </c>
+      <c r="Q130" s="21"/>
+    </row>
+    <row r="131" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
         <v>19</v>
       </c>
-      <c r="B128" t="s">
+      <c r="M131" t="s">
+        <v>602</v>
+      </c>
+      <c r="N131" s="21">
+        <v>1</v>
+      </c>
+      <c r="O131" s="21" t="s">
+        <v>603</v>
+      </c>
+      <c r="P131" s="21"/>
+      <c r="Q131" s="21"/>
+    </row>
+    <row r="132" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>19</v>
+      </c>
+      <c r="B132" t="s">
         <v>314</v>
       </c>
-      <c r="E128" t="s">
+      <c r="E132" t="s">
+        <v>315</v>
+      </c>
+      <c r="M132" t="s">
+        <v>602</v>
+      </c>
+      <c r="N132" s="21">
+        <v>1</v>
+      </c>
+      <c r="O132" s="21" t="s">
+        <v>603</v>
+      </c>
+      <c r="P132" s="21"/>
+      <c r="Q132" s="21"/>
+    </row>
+    <row r="133" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>19</v>
+      </c>
+      <c r="B133" t="s">
+        <v>314</v>
+      </c>
+      <c r="E133" t="s">
         <v>317</v>
       </c>
-      <c r="M128" t="s">
+      <c r="M133" t="s">
         <v>602</v>
       </c>
-      <c r="N128" s="21">
+      <c r="N133" s="21">
         <v>1</v>
       </c>
-      <c r="O128" s="21" t="s">
+      <c r="O133" s="21" t="s">
         <v>603</v>
       </c>
-      <c r="P128" s="21"/>
-      <c r="Q128" s="21"/>
-    </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
+      <c r="P133" s="21"/>
+      <c r="Q133" s="21"/>
+    </row>
+    <row r="134" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
         <v>19</v>
       </c>
-      <c r="B129" t="s">
+      <c r="B134" t="s">
         <v>605</v>
       </c>
-      <c r="E129" t="s">
+      <c r="E134" t="s">
         <v>317</v>
       </c>
-      <c r="M129" t="s">
+      <c r="M134" t="s">
         <v>602</v>
       </c>
-      <c r="N129" s="21">
+      <c r="N134" s="21">
         <v>1</v>
       </c>
-      <c r="O129" s="21" t="s">
+      <c r="O134" s="21" t="s">
         <v>603</v>
       </c>
-      <c r="P129" s="21"/>
-      <c r="Q129" s="21"/>
-    </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N130" s="3"/>
-      <c r="P130" s="3"/>
-    </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A131" s="1" t="s">
+      <c r="P134" s="21"/>
+      <c r="Q134" s="21"/>
+    </row>
+    <row r="135" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N135" s="3"/>
+      <c r="P135" s="3"/>
+    </row>
+    <row r="136" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A136" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B131" s="1"/>
-      <c r="C131" s="1"/>
-      <c r="D131" s="1"/>
-      <c r="E131" s="2"/>
-      <c r="F131" s="2"/>
-      <c r="G131" s="2"/>
-      <c r="H131" s="2"/>
-      <c r="I131" s="2"/>
-      <c r="J131" s="2"/>
-      <c r="K131" s="2"/>
-      <c r="L131" s="2"/>
-      <c r="M131" s="2"/>
-      <c r="N131" s="2"/>
-      <c r="O131" s="2"/>
-      <c r="P131" s="2" t="s">
+      <c r="B136" s="1"/>
+      <c r="C136" s="1"/>
+      <c r="D136" s="1"/>
+      <c r="E136" s="2"/>
+      <c r="F136" s="2"/>
+      <c r="G136" s="2"/>
+      <c r="H136" s="2"/>
+      <c r="I136" s="2"/>
+      <c r="J136" s="2"/>
+      <c r="K136" s="2"/>
+      <c r="L136" s="2"/>
+      <c r="M136" s="2"/>
+      <c r="N136" s="2"/>
+      <c r="O136" s="2"/>
+      <c r="P136" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="Q131" s="2"/>
-    </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="L132" s="103" t="s">
+      <c r="Q136" s="2"/>
+    </row>
+    <row r="137" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="L137" s="103" t="s">
         <v>617</v>
       </c>
     </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M133" t="s">
+    <row r="138" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M138" t="s">
         <v>375</v>
-      </c>
-      <c r="N133" s="21" t="s">
-        <v>614</v>
-      </c>
-      <c r="O133" t="s">
-        <v>598</v>
-      </c>
-      <c r="P133" s="3"/>
-    </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M134" t="s">
-        <v>476</v>
-      </c>
-      <c r="N134" s="21" t="s">
-        <v>614</v>
-      </c>
-      <c r="O134" t="s">
-        <v>597</v>
-      </c>
-      <c r="P134" s="3"/>
-    </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M135" s="37" t="s">
-        <v>608</v>
-      </c>
-      <c r="N135" s="21" t="s">
-        <v>614</v>
-      </c>
-    </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M136" s="37" t="s">
-        <v>609</v>
-      </c>
-      <c r="N136" s="21" t="s">
-        <v>614</v>
-      </c>
-    </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M137" s="37" t="s">
-        <v>610</v>
-      </c>
-      <c r="N137" s="21" t="s">
-        <v>614</v>
-      </c>
-    </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M138" s="37" t="s">
-        <v>611</v>
       </c>
       <c r="N138" s="21" t="s">
         <v>614</v>
       </c>
+      <c r="O138" t="s">
+        <v>598</v>
+      </c>
       <c r="P138" s="3"/>
     </row>
     <row r="139" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="L139" s="103" t="s">
+      <c r="M139" t="s">
+        <v>476</v>
+      </c>
+      <c r="N139" s="21" t="s">
+        <v>614</v>
+      </c>
+      <c r="O139" t="s">
+        <v>597</v>
+      </c>
+      <c r="P139" s="3"/>
+    </row>
+    <row r="140" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M140" s="37" t="s">
+        <v>608</v>
+      </c>
+      <c r="N140" s="21" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M141" s="37" t="s">
+        <v>609</v>
+      </c>
+      <c r="N141" s="21" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="142" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M142" s="37" t="s">
+        <v>610</v>
+      </c>
+      <c r="N142" s="21" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="143" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M143" s="37" t="s">
+        <v>611</v>
+      </c>
+      <c r="N143" s="21" t="s">
+        <v>614</v>
+      </c>
+      <c r="P143" s="3"/>
+    </row>
+    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="L144" s="103" t="s">
         <v>616</v>
-      </c>
-    </row>
-    <row r="140" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M140" t="s">
-        <v>17</v>
-      </c>
-      <c r="N140" s="21" t="s">
-        <v>615</v>
-      </c>
-      <c r="O140" t="s">
-        <v>622</v>
-      </c>
-      <c r="P140" s="21" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M141" t="s">
-        <v>588</v>
-      </c>
-      <c r="N141" s="21" t="s">
-        <v>615</v>
-      </c>
-      <c r="O141" t="s">
-        <v>596</v>
-      </c>
-      <c r="P141" s="3"/>
-    </row>
-    <row r="142" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M142" t="s">
-        <v>477</v>
-      </c>
-      <c r="N142" s="21" t="s">
-        <v>615</v>
-      </c>
-      <c r="O142" t="s">
-        <v>478</v>
-      </c>
-      <c r="P142" s="21" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="L143" s="103" t="s">
-        <v>618</v>
-      </c>
-    </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M144" t="s">
-        <v>17</v>
-      </c>
-      <c r="N144" s="21" t="s">
-        <v>625</v>
-      </c>
-      <c r="O144" t="s">
-        <v>622</v>
-      </c>
-      <c r="P144" s="21" t="s">
-        <v>595</v>
       </c>
     </row>
     <row r="145" spans="12:16" x14ac:dyDescent="0.25">
       <c r="M145" t="s">
+        <v>17</v>
+      </c>
+      <c r="N145" s="21" t="s">
+        <v>615</v>
+      </c>
+      <c r="O145" t="s">
+        <v>622</v>
+      </c>
+      <c r="P145" s="21" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="146" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="M146" t="s">
         <v>588</v>
       </c>
-      <c r="N145" s="21" t="s">
-        <v>625</v>
-      </c>
-      <c r="O145" t="s">
+      <c r="N146" s="21" t="s">
+        <v>615</v>
+      </c>
+      <c r="O146" t="s">
         <v>596</v>
       </c>
-      <c r="P145" s="3"/>
-    </row>
-    <row r="146" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="L146" s="103" t="s">
-        <v>619</v>
-      </c>
+      <c r="P146" s="3"/>
     </row>
     <row r="147" spans="12:16" x14ac:dyDescent="0.25">
       <c r="M147" t="s">
+        <v>477</v>
+      </c>
+      <c r="N147" s="21" t="s">
+        <v>615</v>
+      </c>
+      <c r="O147" t="s">
+        <v>478</v>
+      </c>
+      <c r="P147" s="21" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="148" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L148" s="103" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="149" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="M149" t="s">
         <v>17</v>
       </c>
-      <c r="N147" s="21" t="s">
-        <v>626</v>
-      </c>
-      <c r="O147" t="s">
+      <c r="N149" s="21" t="s">
+        <v>625</v>
+      </c>
+      <c r="O149" t="s">
         <v>622</v>
       </c>
-      <c r="P147" s="21" t="s">
+      <c r="P149" s="21" t="s">
         <v>595</v>
-      </c>
-    </row>
-    <row r="148" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="M148" t="s">
-        <v>588</v>
-      </c>
-      <c r="N148" s="21" t="s">
-        <v>626</v>
-      </c>
-      <c r="O148" t="s">
-        <v>596</v>
-      </c>
-      <c r="P148" s="3"/>
-    </row>
-    <row r="149" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="L149" s="103" t="s">
-        <v>620</v>
       </c>
     </row>
     <row r="150" spans="12:16" x14ac:dyDescent="0.25">
       <c r="M150" t="s">
+        <v>588</v>
+      </c>
+      <c r="N150" s="21" t="s">
+        <v>625</v>
+      </c>
+      <c r="O150" t="s">
+        <v>596</v>
+      </c>
+      <c r="P150" s="3"/>
+    </row>
+    <row r="151" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L151" s="103" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="152" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="M152" t="s">
         <v>17</v>
       </c>
-      <c r="N150" s="21" t="s">
-        <v>627</v>
-      </c>
-      <c r="O150" t="s">
-        <v>623</v>
-      </c>
-      <c r="P150" s="21" t="s">
+      <c r="N152" s="21" t="s">
+        <v>626</v>
+      </c>
+      <c r="O152" t="s">
+        <v>622</v>
+      </c>
+      <c r="P152" s="21" t="s">
         <v>595</v>
-      </c>
-    </row>
-    <row r="151" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="M151" t="s">
-        <v>588</v>
-      </c>
-      <c r="N151" s="21" t="s">
-        <v>627</v>
-      </c>
-      <c r="O151" t="s">
-        <v>596</v>
-      </c>
-      <c r="P151" s="3"/>
-    </row>
-    <row r="152" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="L152" s="103" t="s">
-        <v>621</v>
       </c>
     </row>
     <row r="153" spans="12:16" x14ac:dyDescent="0.25">
       <c r="M153" t="s">
+        <v>588</v>
+      </c>
+      <c r="N153" s="21" t="s">
+        <v>626</v>
+      </c>
+      <c r="O153" t="s">
+        <v>596</v>
+      </c>
+      <c r="P153" s="3"/>
+    </row>
+    <row r="154" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L154" s="103" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="155" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="M155" t="s">
+        <v>17</v>
+      </c>
+      <c r="N155" s="21" t="s">
+        <v>627</v>
+      </c>
+      <c r="O155" t="s">
+        <v>623</v>
+      </c>
+      <c r="P155" s="21" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="156" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="M156" t="s">
+        <v>588</v>
+      </c>
+      <c r="N156" s="21" t="s">
+        <v>627</v>
+      </c>
+      <c r="O156" t="s">
+        <v>596</v>
+      </c>
+      <c r="P156" s="3"/>
+    </row>
+    <row r="157" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L157" s="103" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="158" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="M158" t="s">
         <v>613</v>
       </c>
-      <c r="N153" s="21" t="s">
+      <c r="N158" s="21" t="s">
         <v>628</v>
       </c>
-      <c r="O153" t="s">
+      <c r="O158" t="s">
         <v>624</v>
       </c>
-      <c r="P153" s="21"/>
+      <c r="P158" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Removed handling of by-product imports from FeedMgmt module
</commit_message>
<xml_diff>
--- a/data/default/FeedMgmt.xlsx
+++ b/data/default/FeedMgmt.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1519" uniqueCount="658">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1513" uniqueCount="658">
   <si>
     <t>f_feed</t>
   </si>
@@ -5491,7 +5491,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R153"/>
+  <dimension ref="A1:R151"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="7" width="20.28515625" customWidth="1"/>
@@ -6589,92 +6589,121 @@
       <c r="P70" s="6"/>
     </row>
     <row r="71" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="J71" t="s">
-        <v>38</v>
+      <c r="I71" t="s">
+        <v>37</v>
       </c>
       <c r="M71" t="s">
         <v>25</v>
       </c>
-      <c r="N71" s="21">
+      <c r="N71" s="3">
         <v>100</v>
       </c>
-      <c r="O71" s="21" t="s">
+      <c r="O71" t="s">
         <v>23</v>
       </c>
-      <c r="P71" s="6"/>
+      <c r="P71" s="3" t="s">
+        <v>293</v>
+      </c>
     </row>
     <row r="72" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="J72" t="s">
-        <v>30</v>
+      <c r="I72" t="s">
+        <v>34</v>
       </c>
       <c r="M72" t="s">
         <v>25</v>
       </c>
-      <c r="N72" s="21">
-        <v>61</v>
+      <c r="N72" s="3">
+        <v>50</v>
       </c>
       <c r="O72" t="s">
         <v>23</v>
       </c>
+      <c r="P72" s="3" t="s">
+        <v>372</v>
+      </c>
     </row>
     <row r="73" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="I73" t="s">
-        <v>37</v>
-      </c>
-      <c r="M73" t="s">
-        <v>25</v>
-      </c>
-      <c r="N73" s="3">
-        <v>100</v>
-      </c>
-      <c r="O73" t="s">
+      <c r="A73" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B73" s="1"/>
+      <c r="C73" s="1"/>
+      <c r="D73" s="1"/>
+      <c r="E73" s="2"/>
+      <c r="F73" s="2"/>
+      <c r="G73" s="2"/>
+      <c r="H73" s="2"/>
+      <c r="I73" s="2"/>
+      <c r="J73" s="2"/>
+      <c r="K73" s="2"/>
+      <c r="L73" s="2"/>
+      <c r="M73" s="2"/>
+      <c r="N73" s="2"/>
+      <c r="O73" s="2"/>
+      <c r="P73" s="2"/>
+      <c r="Q73" s="2"/>
+    </row>
+    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>19</v>
+      </c>
+      <c r="H75" t="s">
+        <v>315</v>
+      </c>
+      <c r="I75" t="s">
+        <v>27</v>
+      </c>
+      <c r="M75" t="s">
+        <v>316</v>
+      </c>
+      <c r="N75" s="21">
+        <v>85</v>
+      </c>
+      <c r="O75" t="s">
         <v>23</v>
       </c>
-      <c r="P73" s="3" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="I74" t="s">
-        <v>34</v>
-      </c>
-      <c r="M74" t="s">
-        <v>25</v>
-      </c>
-      <c r="N74" s="3">
-        <v>50</v>
-      </c>
-      <c r="O74" t="s">
+      <c r="P75" s="21" t="s">
+        <v>656</v>
+      </c>
+      <c r="Q75" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>19</v>
+      </c>
+      <c r="B76" t="s">
+        <v>312</v>
+      </c>
+      <c r="E76" t="s">
+        <v>313</v>
+      </c>
+      <c r="H76" t="s">
+        <v>315</v>
+      </c>
+      <c r="I76" t="s">
+        <v>27</v>
+      </c>
+      <c r="M76" t="s">
+        <v>316</v>
+      </c>
+      <c r="N76" s="21">
+        <v>20</v>
+      </c>
+      <c r="O76" t="s">
         <v>23</v>
       </c>
-      <c r="P74" s="3" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A75" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="B75" s="1"/>
-      <c r="C75" s="1"/>
-      <c r="D75" s="1"/>
-      <c r="E75" s="2"/>
-      <c r="F75" s="2"/>
-      <c r="G75" s="2"/>
-      <c r="H75" s="2"/>
-      <c r="I75" s="2"/>
-      <c r="J75" s="2"/>
-      <c r="K75" s="2"/>
-      <c r="L75" s="2"/>
-      <c r="M75" s="2"/>
-      <c r="N75" s="2"/>
-      <c r="O75" s="2"/>
-      <c r="P75" s="2"/>
-      <c r="Q75" s="2"/>
+      <c r="P76" s="21" t="s">
+        <v>657</v>
+      </c>
+      <c r="Q76" t="s">
+        <v>652</v>
+      </c>
     </row>
     <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>19</v>
+        <v>373</v>
       </c>
       <c r="H77" t="s">
         <v>315</v>
@@ -6686,27 +6715,19 @@
         <v>316</v>
       </c>
       <c r="N77" s="21">
-        <v>85</v>
+        <v>14.5</v>
       </c>
       <c r="O77" t="s">
         <v>23</v>
       </c>
-      <c r="P77" s="21" t="s">
-        <v>656</v>
-      </c>
+      <c r="P77" s="3"/>
       <c r="Q77" t="s">
-        <v>655</v>
+        <v>635</v>
       </c>
     </row>
     <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>19</v>
-      </c>
-      <c r="B78" t="s">
-        <v>312</v>
-      </c>
-      <c r="E78" t="s">
-        <v>313</v>
+        <v>377</v>
       </c>
       <c r="H78" t="s">
         <v>315</v>
@@ -6718,21 +6739,25 @@
         <v>316</v>
       </c>
       <c r="N78" s="21">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="O78" t="s">
         <v>23</v>
       </c>
-      <c r="P78" s="21" t="s">
-        <v>657</v>
-      </c>
+      <c r="P78" s="3"/>
       <c r="Q78" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
     </row>
     <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>373</v>
+        <v>377</v>
+      </c>
+      <c r="D79" t="s">
+        <v>647</v>
+      </c>
+      <c r="E79" t="s">
+        <v>481</v>
       </c>
       <c r="H79" t="s">
         <v>315</v>
@@ -6744,132 +6769,126 @@
         <v>316</v>
       </c>
       <c r="N79" s="21">
-        <v>14.5</v>
+        <v>69</v>
       </c>
       <c r="O79" t="s">
         <v>23</v>
       </c>
       <c r="P79" s="3"/>
       <c r="Q79" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N80" s="3"/>
+      <c r="P80" s="3"/>
+    </row>
+    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A81" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="B81" s="1"/>
+      <c r="C81" s="1"/>
+      <c r="D81" s="1"/>
+      <c r="E81" s="2"/>
+      <c r="F81" s="2"/>
+      <c r="G81" s="2"/>
+      <c r="H81" s="2"/>
+      <c r="I81" s="2"/>
+      <c r="J81" s="2"/>
+      <c r="K81" s="2"/>
+      <c r="L81" s="2"/>
+      <c r="M81" s="2"/>
+      <c r="N81" s="2"/>
+      <c r="O81" s="2"/>
+      <c r="P81" s="2"/>
+      <c r="Q81" s="2"/>
+    </row>
+    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M82" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="N82" s="6">
+        <v>0</v>
+      </c>
+      <c r="O82" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="P82" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M83" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="N83" s="6">
+        <v>0</v>
+      </c>
+      <c r="O83" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="P83" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>19</v>
+      </c>
+      <c r="B84" t="s">
+        <v>312</v>
+      </c>
+      <c r="E84" t="s">
+        <v>313</v>
+      </c>
+      <c r="G84" t="s">
+        <v>628</v>
+      </c>
+      <c r="M84" s="21" t="s">
+        <v>374</v>
+      </c>
+      <c r="N84" s="21">
+        <f>(0.8*20+0.2*2)</f>
+        <v>16.399999999999999</v>
+      </c>
+      <c r="O84" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="P84" s="21" t="s">
+        <v>378</v>
+      </c>
+      <c r="Q84" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
-        <v>377</v>
-      </c>
-      <c r="H80" t="s">
-        <v>315</v>
-      </c>
-      <c r="I80" t="s">
-        <v>27</v>
-      </c>
-      <c r="M80" t="s">
-        <v>316</v>
-      </c>
-      <c r="N80" s="21">
-        <v>100</v>
-      </c>
-      <c r="O80" t="s">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>19</v>
+      </c>
+      <c r="G85" t="s">
+        <v>628</v>
+      </c>
+      <c r="M85" s="21" t="s">
+        <v>374</v>
+      </c>
+      <c r="N85" s="21">
+        <f>(0.6*20+0.4*2)</f>
+        <v>12.8</v>
+      </c>
+      <c r="O85" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="P80" s="3"/>
-      <c r="Q80" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>377</v>
-      </c>
-      <c r="D81" t="s">
-        <v>647</v>
-      </c>
-      <c r="E81" t="s">
-        <v>481</v>
-      </c>
-      <c r="H81" t="s">
-        <v>315</v>
-      </c>
-      <c r="I81" t="s">
-        <v>27</v>
-      </c>
-      <c r="M81" t="s">
-        <v>316</v>
-      </c>
-      <c r="N81" s="21">
-        <v>69</v>
-      </c>
-      <c r="O81" t="s">
-        <v>23</v>
-      </c>
-      <c r="P81" s="3"/>
-      <c r="Q81" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N82" s="3"/>
-      <c r="P82" s="3"/>
-    </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A83" s="1" t="s">
-        <v>376</v>
-      </c>
-      <c r="B83" s="1"/>
-      <c r="C83" s="1"/>
-      <c r="D83" s="1"/>
-      <c r="E83" s="2"/>
-      <c r="F83" s="2"/>
-      <c r="G83" s="2"/>
-      <c r="H83" s="2"/>
-      <c r="I83" s="2"/>
-      <c r="J83" s="2"/>
-      <c r="K83" s="2"/>
-      <c r="L83" s="2"/>
-      <c r="M83" s="2"/>
-      <c r="N83" s="2"/>
-      <c r="O83" s="2"/>
-      <c r="P83" s="2"/>
-      <c r="Q83" s="2"/>
-    </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M84" s="6" t="s">
-        <v>374</v>
-      </c>
-      <c r="N84" s="6">
-        <v>0</v>
-      </c>
-      <c r="O84" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="P84" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M85" s="6" t="s">
-        <v>375</v>
-      </c>
-      <c r="N85" s="6">
-        <v>0</v>
-      </c>
-      <c r="O85" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="P85" s="6" t="s">
-        <v>28</v>
+      <c r="P85" s="21" t="s">
+        <v>379</v>
+      </c>
+      <c r="Q85" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="86" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>19</v>
-      </c>
-      <c r="B86" t="s">
-        <v>312</v>
-      </c>
-      <c r="E86" t="s">
-        <v>313</v>
+        <v>377</v>
       </c>
       <c r="G86" t="s">
         <v>628</v>
@@ -6878,14 +6897,13 @@
         <v>374</v>
       </c>
       <c r="N86" s="21">
-        <f>(0.8*20+0.2*2)</f>
-        <v>16.399999999999999</v>
+        <v>2</v>
       </c>
       <c r="O86" s="21" t="s">
         <v>23</v>
       </c>
       <c r="P86" s="21" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="Q86" t="s">
         <v>635</v>
@@ -6893,7 +6911,7 @@
     </row>
     <row r="87" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>19</v>
+        <v>373</v>
       </c>
       <c r="G87" t="s">
         <v>628</v>
@@ -6902,81 +6920,83 @@
         <v>374</v>
       </c>
       <c r="N87" s="21">
-        <f>(0.6*20+0.4*2)</f>
-        <v>12.8</v>
+        <v>2</v>
       </c>
       <c r="O87" s="21" t="s">
         <v>23</v>
       </c>
       <c r="P87" s="21" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="Q87" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="88" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>377</v>
-      </c>
-      <c r="G88" t="s">
-        <v>628</v>
-      </c>
-      <c r="M88" s="21" t="s">
-        <v>374</v>
-      </c>
-      <c r="N88" s="21">
-        <v>2</v>
-      </c>
-      <c r="O88" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="P88" s="21" t="s">
-        <v>380</v>
-      </c>
-      <c r="Q88" t="s">
-        <v>635</v>
-      </c>
+      <c r="M88" s="21"/>
+      <c r="N88" s="21"/>
+      <c r="O88" s="21"/>
+      <c r="P88" s="21"/>
     </row>
     <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>373</v>
+        <v>19</v>
+      </c>
+      <c r="B89" t="s">
+        <v>312</v>
+      </c>
+      <c r="E89" t="s">
+        <v>313</v>
       </c>
       <c r="G89" t="s">
         <v>628</v>
       </c>
       <c r="M89" s="21" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="N89" s="21">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O89" s="21" t="s">
         <v>23</v>
       </c>
       <c r="P89" s="21" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="Q89" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="90" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M90" s="21"/>
-      <c r="N90" s="21"/>
-      <c r="O90" s="21"/>
-      <c r="P90" s="21"/>
+      <c r="A90" t="s">
+        <v>19</v>
+      </c>
+      <c r="E90" t="s">
+        <v>314</v>
+      </c>
+      <c r="G90" t="s">
+        <v>628</v>
+      </c>
+      <c r="M90" s="21" t="s">
+        <v>375</v>
+      </c>
+      <c r="N90" s="21">
+        <v>5</v>
+      </c>
+      <c r="O90" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="P90" s="21" t="s">
+        <v>381</v>
+      </c>
+      <c r="Q90" t="s">
+        <v>635</v>
+      </c>
     </row>
     <row r="91" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>19</v>
       </c>
-      <c r="B91" t="s">
-        <v>312</v>
-      </c>
-      <c r="E91" t="s">
-        <v>313</v>
-      </c>
       <c r="G91" t="s">
         <v>628</v>
       </c>
@@ -6984,13 +7004,14 @@
         <v>375</v>
       </c>
       <c r="N91" s="21">
-        <v>5</v>
+        <f>0.9*5+0.1*15</f>
+        <v>6</v>
       </c>
       <c r="O91" s="21" t="s">
         <v>23</v>
       </c>
       <c r="P91" s="21" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="Q91" t="s">
         <v>635</v>
@@ -6998,10 +7019,7 @@
     </row>
     <row r="92" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>19</v>
-      </c>
-      <c r="E92" t="s">
-        <v>314</v>
+        <v>377</v>
       </c>
       <c r="G92" t="s">
         <v>628</v>
@@ -7010,21 +7028,19 @@
         <v>375</v>
       </c>
       <c r="N92" s="21">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="O92" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="P92" s="21" t="s">
-        <v>381</v>
-      </c>
+      <c r="P92" s="21"/>
       <c r="Q92" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="93" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>19</v>
+        <v>373</v>
       </c>
       <c r="G93" t="s">
         <v>628</v>
@@ -7033,52 +7049,34 @@
         <v>375</v>
       </c>
       <c r="N93" s="21">
-        <f>0.9*5+0.1*15</f>
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="O93" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="P93" s="21" t="s">
-        <v>382</v>
-      </c>
+      <c r="P93" s="21"/>
       <c r="Q93" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="94" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>377</v>
-      </c>
-      <c r="G94" t="s">
-        <v>628</v>
-      </c>
-      <c r="M94" s="21" t="s">
-        <v>375</v>
-      </c>
-      <c r="N94" s="21">
-        <v>15</v>
-      </c>
-      <c r="O94" s="21" t="s">
-        <v>23</v>
-      </c>
+      <c r="M94" s="21"/>
+      <c r="N94" s="21"/>
+      <c r="O94" s="21"/>
       <c r="P94" s="21"/>
-      <c r="Q94" t="s">
-        <v>635</v>
-      </c>
     </row>
     <row r="95" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>373</v>
-      </c>
+      <c r="A95" s="22"/>
+      <c r="B95" s="22"/>
+      <c r="E95" s="22"/>
       <c r="G95" t="s">
-        <v>628</v>
+        <v>300</v>
       </c>
       <c r="M95" s="21" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="N95" s="21">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="O95" s="21" t="s">
         <v>23</v>
@@ -7089,55 +7087,90 @@
       </c>
     </row>
     <row r="96" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M96" s="21"/>
-      <c r="N96" s="21"/>
-      <c r="O96" s="21"/>
-      <c r="P96" s="21"/>
+      <c r="A96" s="22" t="str">
+        <f>A89</f>
+        <v>cattle</v>
+      </c>
+      <c r="B96" s="22" t="str">
+        <f>B89</f>
+        <v>dairy</v>
+      </c>
+      <c r="E96" s="22" t="str">
+        <f t="shared" ref="E96:E97" si="0">E89</f>
+        <v>cows</v>
+      </c>
+      <c r="G96" t="s">
+        <v>300</v>
+      </c>
+      <c r="M96" s="22" t="str">
+        <f t="shared" ref="M96:Q100" si="1">M89</f>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N96" s="22">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="O96" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="P96" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="Q96" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
     </row>
     <row r="97" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A97" s="22"/>
-      <c r="B97" s="22"/>
-      <c r="E97" s="22"/>
+      <c r="A97" s="22" t="str">
+        <f t="shared" ref="A97:A100" si="2">A90</f>
+        <v>cattle</v>
+      </c>
+      <c r="E97" s="22" t="str">
+        <f t="shared" si="0"/>
+        <v>bulls</v>
+      </c>
       <c r="G97" t="s">
         <v>300</v>
       </c>
-      <c r="M97" s="21" t="s">
-        <v>374</v>
-      </c>
-      <c r="N97" s="21">
+      <c r="M97" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N97" s="22">
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="O97" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="P97" s="21"/>
-      <c r="Q97" t="s">
-        <v>635</v>
+      <c r="O97" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="P97" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="Q97" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="98" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="22" t="str">
-        <f>A91</f>
+        <f t="shared" si="2"/>
         <v>cattle</v>
-      </c>
-      <c r="B98" s="22" t="str">
-        <f>B91</f>
-        <v>dairy</v>
-      </c>
-      <c r="E98" s="22" t="str">
-        <f t="shared" ref="E98:E99" si="0">E91</f>
-        <v>cows</v>
       </c>
       <c r="G98" t="s">
         <v>300</v>
       </c>
       <c r="M98" s="22" t="str">
-        <f t="shared" ref="M98:Q102" si="1">M91</f>
+        <f t="shared" si="1"/>
         <v>feeding_losses</v>
       </c>
       <c r="N98" s="22">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O98" s="22" t="str">
         <f t="shared" si="1"/>
@@ -7145,7 +7178,7 @@
       </c>
       <c r="P98" s="22" t="str">
         <f t="shared" si="1"/>
-        <v>No feeding on pasture</v>
+        <v>10% feeding on pasture</v>
       </c>
       <c r="Q98" s="22" t="str">
         <f t="shared" si="1"/>
@@ -7154,12 +7187,8 @@
     </row>
     <row r="99" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="22" t="str">
-        <f t="shared" ref="A99:A102" si="2">A92</f>
-        <v>cattle</v>
-      </c>
-      <c r="E99" s="22" t="str">
-        <f t="shared" si="0"/>
-        <v>bulls</v>
+        <f t="shared" si="2"/>
+        <v>sheep</v>
       </c>
       <c r="G99" t="s">
         <v>300</v>
@@ -7170,16 +7199,13 @@
       </c>
       <c r="N99" s="22">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="O99" s="22" t="str">
         <f t="shared" si="1"/>
         <v>%</v>
       </c>
-      <c r="P99" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>No feeding on pasture</v>
-      </c>
+      <c r="P99" s="22"/>
       <c r="Q99" s="22" t="str">
         <f t="shared" si="1"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
@@ -7188,7 +7214,7 @@
     <row r="100" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="22" t="str">
         <f t="shared" si="2"/>
-        <v>cattle</v>
+        <v>horses</v>
       </c>
       <c r="G100" t="s">
         <v>300</v>
@@ -7199,122 +7225,129 @@
       </c>
       <c r="N100" s="22">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="O100" s="22" t="str">
         <f t="shared" si="1"/>
         <v>%</v>
       </c>
-      <c r="P100" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>10% feeding on pasture</v>
-      </c>
+      <c r="P100" s="22"/>
       <c r="Q100" s="22" t="str">
         <f t="shared" si="1"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="101" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A101" s="22" t="str">
-        <f t="shared" si="2"/>
-        <v>sheep</v>
-      </c>
-      <c r="G101" t="s">
-        <v>300</v>
-      </c>
-      <c r="M101" s="22" t="str">
-        <f t="shared" si="1"/>
+      <c r="A101" s="22"/>
+      <c r="M101" s="22"/>
+      <c r="N101" s="22"/>
+      <c r="O101" s="22"/>
+      <c r="P101" s="22"/>
+      <c r="Q101" s="22"/>
+    </row>
+    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="G102" t="s">
+        <v>629</v>
+      </c>
+      <c r="M102" s="21" t="s">
+        <v>374</v>
+      </c>
+      <c r="N102" s="21">
+        <v>5</v>
+      </c>
+      <c r="O102" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="P102" s="21"/>
+      <c r="Q102" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A103" s="22" t="str">
+        <f>A89</f>
+        <v>cattle</v>
+      </c>
+      <c r="B103" s="22" t="str">
+        <f>B89</f>
+        <v>dairy</v>
+      </c>
+      <c r="E103" s="22" t="str">
+        <f t="shared" ref="E103:E104" si="3">E89</f>
+        <v>cows</v>
+      </c>
+      <c r="G103" t="s">
+        <v>629</v>
+      </c>
+      <c r="M103" s="22" t="str">
+        <f t="shared" ref="M103:Q107" si="4">M89</f>
         <v>feeding_losses</v>
       </c>
-      <c r="N101" s="22">
-        <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-      <c r="O101" s="22" t="str">
-        <f t="shared" si="1"/>
+      <c r="N103" s="22">
+        <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="O103" s="22" t="str">
+        <f t="shared" si="4"/>
         <v>%</v>
       </c>
-      <c r="P101" s="22"/>
-      <c r="Q101" s="22" t="str">
-        <f t="shared" si="1"/>
+      <c r="P103" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="Q103" s="22" t="str">
+        <f t="shared" si="4"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A102" s="22" t="str">
-        <f t="shared" si="2"/>
-        <v>horses</v>
-      </c>
-      <c r="G102" t="s">
-        <v>300</v>
-      </c>
-      <c r="M102" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N102" s="22">
-        <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-      <c r="O102" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>%</v>
-      </c>
-      <c r="P102" s="22"/>
-      <c r="Q102" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A103" s="22"/>
-      <c r="M103" s="22"/>
-      <c r="N103" s="22"/>
-      <c r="O103" s="22"/>
-      <c r="P103" s="22"/>
-      <c r="Q103" s="22"/>
-    </row>
     <row r="104" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A104" s="22" t="str">
+        <f t="shared" ref="A104:A107" si="5">A90</f>
+        <v>cattle</v>
+      </c>
+      <c r="E104" s="22" t="str">
+        <f t="shared" si="3"/>
+        <v>bulls</v>
+      </c>
       <c r="G104" t="s">
         <v>629</v>
       </c>
-      <c r="M104" s="21" t="s">
-        <v>374</v>
-      </c>
-      <c r="N104" s="21">
+      <c r="M104" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N104" s="22">
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="O104" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="P104" s="21"/>
-      <c r="Q104" t="s">
-        <v>635</v>
+      <c r="O104" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="P104" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="Q104" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="105" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="22" t="str">
-        <f>A91</f>
+        <f t="shared" si="5"/>
         <v>cattle</v>
-      </c>
-      <c r="B105" s="22" t="str">
-        <f>B91</f>
-        <v>dairy</v>
-      </c>
-      <c r="E105" s="22" t="str">
-        <f t="shared" ref="E105:E106" si="3">E91</f>
-        <v>cows</v>
       </c>
       <c r="G105" t="s">
         <v>629</v>
       </c>
       <c r="M105" s="22" t="str">
-        <f t="shared" ref="M105:Q109" si="4">M91</f>
+        <f t="shared" si="4"/>
         <v>feeding_losses</v>
       </c>
       <c r="N105" s="22">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O105" s="22" t="str">
         <f t="shared" si="4"/>
@@ -7322,7 +7355,7 @@
       </c>
       <c r="P105" s="22" t="str">
         <f t="shared" si="4"/>
-        <v>No feeding on pasture</v>
+        <v>10% feeding on pasture</v>
       </c>
       <c r="Q105" s="22" t="str">
         <f t="shared" si="4"/>
@@ -7331,12 +7364,8 @@
     </row>
     <row r="106" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="22" t="str">
-        <f t="shared" ref="A106:A109" si="5">A92</f>
-        <v>cattle</v>
-      </c>
-      <c r="E106" s="22" t="str">
-        <f t="shared" si="3"/>
-        <v>bulls</v>
+        <f t="shared" si="5"/>
+        <v>sheep</v>
       </c>
       <c r="G106" t="s">
         <v>629</v>
@@ -7347,25 +7376,22 @@
       </c>
       <c r="N106" s="22">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="O106" s="22" t="str">
         <f t="shared" si="4"/>
         <v>%</v>
       </c>
-      <c r="P106" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>No feeding on pasture</v>
-      </c>
+      <c r="P106" s="21"/>
       <c r="Q106" s="22" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="Q106:Q107" si="6">Q92</f>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="107" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="22" t="str">
         <f t="shared" si="5"/>
-        <v>cattle</v>
+        <v>horses</v>
       </c>
       <c r="G107" t="s">
         <v>629</v>
@@ -7376,249 +7402,230 @@
       </c>
       <c r="N107" s="22">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="O107" s="22" t="str">
         <f t="shared" si="4"/>
         <v>%</v>
       </c>
-      <c r="P107" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>10% feeding on pasture</v>
-      </c>
+      <c r="P107" s="21"/>
       <c r="Q107" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A108" s="22" t="str">
-        <f t="shared" si="5"/>
-        <v>sheep</v>
-      </c>
-      <c r="G108" t="s">
-        <v>629</v>
-      </c>
-      <c r="M108" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N108" s="22">
-        <f t="shared" si="4"/>
-        <v>15</v>
-      </c>
-      <c r="O108" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>%</v>
-      </c>
-      <c r="P108" s="21"/>
-      <c r="Q108" s="22" t="str">
-        <f t="shared" ref="Q108:Q109" si="6">Q94</f>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A109" s="22" t="str">
-        <f t="shared" si="5"/>
-        <v>horses</v>
-      </c>
-      <c r="G109" t="s">
-        <v>629</v>
-      </c>
-      <c r="M109" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N109" s="22">
-        <f t="shared" si="4"/>
-        <v>15</v>
-      </c>
-      <c r="O109" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>%</v>
-      </c>
-      <c r="P109" s="21"/>
-      <c r="Q109" s="22" t="str">
         <f t="shared" si="6"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
+    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N108" s="3"/>
+      <c r="P108" s="21"/>
+    </row>
+    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A109" s="3"/>
+      <c r="G109" t="s">
+        <v>630</v>
+      </c>
+      <c r="M109" s="21" t="s">
+        <v>374</v>
+      </c>
+      <c r="N109" s="21"/>
+      <c r="P109" s="3" t="s">
+        <v>632</v>
+      </c>
+    </row>
     <row r="110" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N110" s="3"/>
-      <c r="P110" s="21"/>
+      <c r="A110" s="3"/>
+      <c r="G110" t="s">
+        <v>630</v>
+      </c>
+      <c r="M110" s="21" t="s">
+        <v>375</v>
+      </c>
+      <c r="N110" s="21">
+        <v>2</v>
+      </c>
+      <c r="O110" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="P110" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="Q110" t="s">
+        <v>634</v>
+      </c>
     </row>
     <row r="111" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A111" s="3"/>
-      <c r="G111" t="s">
-        <v>630</v>
-      </c>
-      <c r="M111" s="21" t="s">
-        <v>374</v>
-      </c>
+      <c r="M111" s="21"/>
       <c r="N111" s="21"/>
-      <c r="P111" s="3" t="s">
-        <v>632</v>
-      </c>
+      <c r="O111" s="21"/>
+      <c r="P111" s="3"/>
     </row>
     <row r="112" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A112" s="3"/>
       <c r="G112" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="M112" s="21" t="s">
-        <v>375</v>
-      </c>
-      <c r="N112" s="21">
-        <v>2</v>
-      </c>
-      <c r="O112" s="21" t="s">
-        <v>23</v>
-      </c>
+        <v>374</v>
+      </c>
+      <c r="N112" s="21"/>
       <c r="P112" s="3" t="s">
-        <v>636</v>
-      </c>
-      <c r="Q112" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
     </row>
     <row r="113" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A113" s="3"/>
-      <c r="M113" s="21"/>
-      <c r="N113" s="21"/>
-      <c r="O113" s="21"/>
-      <c r="P113" s="3"/>
+      <c r="G113" t="s">
+        <v>631</v>
+      </c>
+      <c r="M113" s="21" t="s">
+        <v>375</v>
+      </c>
+      <c r="N113" s="21">
+        <v>3</v>
+      </c>
+      <c r="O113" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="P113" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="Q113" t="s">
+        <v>634</v>
+      </c>
     </row>
     <row r="114" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A114" s="3"/>
-      <c r="G114" t="s">
-        <v>631</v>
-      </c>
-      <c r="M114" s="21" t="s">
-        <v>374</v>
-      </c>
-      <c r="N114" s="21"/>
-      <c r="P114" s="3" t="s">
-        <v>632</v>
-      </c>
+      <c r="N114" s="3"/>
+      <c r="P114" s="21"/>
     </row>
     <row r="115" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A115" s="3"/>
-      <c r="G115" t="s">
-        <v>631</v>
-      </c>
-      <c r="M115" s="21" t="s">
-        <v>375</v>
-      </c>
-      <c r="N115" s="21">
-        <v>3</v>
-      </c>
-      <c r="O115" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="P115" s="3" t="s">
-        <v>636</v>
-      </c>
-      <c r="Q115" t="s">
-        <v>634</v>
-      </c>
+      <c r="A115" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="B115" s="1"/>
+      <c r="C115" s="1"/>
+      <c r="D115" s="1"/>
+      <c r="E115" s="2"/>
+      <c r="F115" s="2"/>
+      <c r="G115" s="2"/>
+      <c r="H115" s="2"/>
+      <c r="I115" s="2"/>
+      <c r="J115" s="2"/>
+      <c r="K115" s="2"/>
+      <c r="L115" s="2"/>
+      <c r="M115" s="2"/>
+      <c r="N115" s="2"/>
+      <c r="O115" s="2"/>
+      <c r="P115" s="2"/>
+      <c r="Q115" s="2"/>
     </row>
     <row r="116" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N116" s="3"/>
-      <c r="P116" s="21"/>
+      <c r="A116" t="s">
+        <v>19</v>
+      </c>
+      <c r="N116" s="21"/>
+      <c r="P116" s="21" t="s">
+        <v>597</v>
+      </c>
     </row>
     <row r="117" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A117" s="1" t="s">
-        <v>596</v>
-      </c>
-      <c r="B117" s="1"/>
-      <c r="C117" s="1"/>
-      <c r="D117" s="1"/>
-      <c r="E117" s="2"/>
-      <c r="F117" s="2"/>
-      <c r="G117" s="2"/>
-      <c r="H117" s="2"/>
-      <c r="I117" s="2"/>
-      <c r="J117" s="2"/>
-      <c r="K117" s="2"/>
-      <c r="L117" s="2"/>
-      <c r="M117" s="2"/>
-      <c r="N117" s="2"/>
-      <c r="O117" s="2"/>
-      <c r="P117" s="2"/>
-      <c r="Q117" s="2"/>
+      <c r="A117" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="B117" s="3"/>
+      <c r="C117" s="3"/>
+      <c r="D117" s="3"/>
+      <c r="E117" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="F117" s="3"/>
+      <c r="G117" s="3"/>
+      <c r="H117" s="3"/>
+      <c r="I117" s="3"/>
+      <c r="J117" s="3"/>
+      <c r="K117" s="3"/>
+      <c r="L117" s="3"/>
+      <c r="M117" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="N117" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="O117" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="P117" s="3"/>
     </row>
     <row r="118" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>19</v>
-      </c>
-      <c r="N118" s="21"/>
-      <c r="P118" s="21" t="s">
-        <v>597</v>
-      </c>
+      <c r="A118" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="B118" s="3"/>
+      <c r="C118" s="3"/>
+      <c r="D118" s="3"/>
+      <c r="E118" s="3"/>
+      <c r="F118" s="3"/>
+      <c r="G118" s="3"/>
+      <c r="H118" s="3"/>
+      <c r="I118" s="3"/>
+      <c r="J118" s="3"/>
+      <c r="K118" s="3"/>
+      <c r="L118" s="3"/>
+      <c r="M118" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="N118" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="O118" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="P118" s="3"/>
     </row>
     <row r="119" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A119" s="3" t="s">
-        <v>377</v>
-      </c>
-      <c r="B119" s="3"/>
-      <c r="C119" s="3"/>
-      <c r="D119" s="3"/>
-      <c r="E119" s="3" t="s">
-        <v>481</v>
-      </c>
-      <c r="F119" s="3"/>
-      <c r="G119" s="3"/>
-      <c r="H119" s="3"/>
-      <c r="I119" s="3"/>
-      <c r="J119" s="3"/>
-      <c r="K119" s="3"/>
-      <c r="L119" s="3"/>
-      <c r="M119" s="3" t="s">
-        <v>482</v>
-      </c>
-      <c r="N119" s="3">
-        <v>4.5</v>
-      </c>
-      <c r="O119" s="3" t="s">
-        <v>483</v>
+      <c r="A119" t="s">
+        <v>373</v>
+      </c>
+      <c r="M119" t="s">
+        <v>484</v>
+      </c>
+      <c r="N119" s="21">
+        <v>18</v>
+      </c>
+      <c r="O119" t="s">
+        <v>485</v>
       </c>
       <c r="P119" s="3"/>
+      <c r="Q119" t="s">
+        <v>486</v>
+      </c>
     </row>
     <row r="120" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A120" s="3" t="s">
-        <v>377</v>
-      </c>
-      <c r="B120" s="3"/>
-      <c r="C120" s="3"/>
-      <c r="D120" s="3"/>
-      <c r="E120" s="3"/>
-      <c r="F120" s="3"/>
-      <c r="G120" s="3"/>
-      <c r="H120" s="3"/>
-      <c r="I120" s="3"/>
-      <c r="J120" s="3"/>
-      <c r="K120" s="3"/>
-      <c r="L120" s="3"/>
-      <c r="M120" s="3" t="s">
-        <v>482</v>
-      </c>
-      <c r="N120" s="3">
-        <v>6.5</v>
-      </c>
-      <c r="O120" s="3" t="s">
-        <v>483</v>
+      <c r="A120" t="s">
+        <v>20</v>
+      </c>
+      <c r="M120" t="s">
+        <v>484</v>
+      </c>
+      <c r="N120" s="21">
+        <v>1.5</v>
+      </c>
+      <c r="O120" t="s">
+        <v>485</v>
       </c>
       <c r="P120" s="3"/>
+      <c r="Q120" t="s">
+        <v>486</v>
+      </c>
     </row>
     <row r="121" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="M121" t="s">
         <v>484</v>
       </c>
       <c r="N121" s="21">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="O121" t="s">
         <v>485</v>
@@ -7629,46 +7636,50 @@
       </c>
     </row>
     <row r="122" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>20</v>
-      </c>
-      <c r="M122" t="s">
-        <v>484</v>
-      </c>
-      <c r="N122" s="21">
-        <v>1.5</v>
-      </c>
-      <c r="O122" t="s">
-        <v>485</v>
-      </c>
+      <c r="N122" s="21"/>
       <c r="P122" s="3"/>
-      <c r="Q122" t="s">
-        <v>486</v>
-      </c>
     </row>
     <row r="123" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
-        <v>370</v>
-      </c>
       <c r="M123" t="s">
-        <v>484</v>
+        <v>598</v>
       </c>
       <c r="N123" s="21">
-        <v>0</v>
-      </c>
-      <c r="O123" t="s">
-        <v>485</v>
-      </c>
-      <c r="P123" s="3"/>
-      <c r="Q123" t="s">
-        <v>486</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="O123" s="21" t="s">
+        <v>599</v>
+      </c>
+      <c r="P123" s="21" t="s">
+        <v>600</v>
+      </c>
+      <c r="Q123" s="21"/>
     </row>
     <row r="124" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N124" s="21"/>
-      <c r="P124" s="3"/>
+      <c r="A124" t="s">
+        <v>19</v>
+      </c>
+      <c r="M124" t="s">
+        <v>598</v>
+      </c>
+      <c r="N124" s="21">
+        <v>1</v>
+      </c>
+      <c r="O124" s="21" t="s">
+        <v>599</v>
+      </c>
+      <c r="P124" s="21"/>
+      <c r="Q124" s="21"/>
     </row>
     <row r="125" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>19</v>
+      </c>
+      <c r="B125" t="s">
+        <v>312</v>
+      </c>
+      <c r="E125" t="s">
+        <v>313</v>
+      </c>
       <c r="M125" t="s">
         <v>598</v>
       </c>
@@ -7678,15 +7689,19 @@
       <c r="O125" s="21" t="s">
         <v>599</v>
       </c>
-      <c r="P125" s="21" t="s">
-        <v>600</v>
-      </c>
+      <c r="P125" s="21"/>
       <c r="Q125" s="21"/>
     </row>
     <row r="126" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>19</v>
       </c>
+      <c r="B126" t="s">
+        <v>312</v>
+      </c>
+      <c r="E126" t="s">
+        <v>314</v>
+      </c>
       <c r="M126" t="s">
         <v>598</v>
       </c>
@@ -7704,10 +7719,10 @@
         <v>19</v>
       </c>
       <c r="B127" t="s">
-        <v>312</v>
+        <v>601</v>
       </c>
       <c r="E127" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="M127" t="s">
         <v>598</v>
@@ -7722,108 +7737,80 @@
       <c r="Q127" s="21"/>
     </row>
     <row r="128" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
-        <v>19</v>
-      </c>
-      <c r="B128" t="s">
-        <v>312</v>
-      </c>
-      <c r="E128" t="s">
-        <v>314</v>
-      </c>
-      <c r="M128" t="s">
-        <v>598</v>
-      </c>
-      <c r="N128" s="21">
-        <v>1</v>
-      </c>
-      <c r="O128" s="21" t="s">
-        <v>599</v>
-      </c>
-      <c r="P128" s="21"/>
-      <c r="Q128" s="21"/>
+      <c r="N128" s="3"/>
+      <c r="P128" s="3"/>
     </row>
     <row r="129" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
-        <v>19</v>
-      </c>
-      <c r="B129" t="s">
-        <v>601</v>
-      </c>
-      <c r="E129" t="s">
-        <v>314</v>
-      </c>
-      <c r="M129" t="s">
-        <v>598</v>
-      </c>
-      <c r="N129" s="21">
-        <v>1</v>
-      </c>
-      <c r="O129" s="21" t="s">
-        <v>599</v>
-      </c>
-      <c r="P129" s="21"/>
-      <c r="Q129" s="21"/>
+      <c r="A129" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B129" s="1"/>
+      <c r="C129" s="1"/>
+      <c r="D129" s="1"/>
+      <c r="E129" s="2"/>
+      <c r="F129" s="2"/>
+      <c r="G129" s="2"/>
+      <c r="H129" s="2"/>
+      <c r="I129" s="2"/>
+      <c r="J129" s="2"/>
+      <c r="K129" s="2"/>
+      <c r="L129" s="2"/>
+      <c r="M129" s="2"/>
+      <c r="N129" s="2"/>
+      <c r="O129" s="2"/>
+      <c r="P129" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="Q129" s="2"/>
     </row>
     <row r="130" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N130" s="3"/>
-      <c r="P130" s="3"/>
+      <c r="L130" s="103" t="s">
+        <v>613</v>
+      </c>
     </row>
     <row r="131" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A131" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B131" s="1"/>
-      <c r="C131" s="1"/>
-      <c r="D131" s="1"/>
-      <c r="E131" s="2"/>
-      <c r="F131" s="2"/>
-      <c r="G131" s="2"/>
-      <c r="H131" s="2"/>
-      <c r="I131" s="2"/>
-      <c r="J131" s="2"/>
-      <c r="K131" s="2"/>
-      <c r="L131" s="2"/>
-      <c r="M131" s="2"/>
-      <c r="N131" s="2"/>
-      <c r="O131" s="2"/>
-      <c r="P131" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="Q131" s="2"/>
+      <c r="M131" t="s">
+        <v>371</v>
+      </c>
+      <c r="N131" s="21" t="s">
+        <v>610</v>
+      </c>
+      <c r="O131" t="s">
+        <v>594</v>
+      </c>
+      <c r="P131" s="3"/>
     </row>
     <row r="132" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="L132" s="103" t="s">
-        <v>613</v>
-      </c>
+      <c r="M132" t="s">
+        <v>472</v>
+      </c>
+      <c r="N132" s="21" t="s">
+        <v>610</v>
+      </c>
+      <c r="O132" t="s">
+        <v>593</v>
+      </c>
+      <c r="P132" s="3"/>
     </row>
     <row r="133" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M133" t="s">
-        <v>371</v>
+      <c r="M133" s="37" t="s">
+        <v>604</v>
       </c>
       <c r="N133" s="21" t="s">
         <v>610</v>
       </c>
-      <c r="O133" t="s">
-        <v>594</v>
-      </c>
-      <c r="P133" s="3"/>
     </row>
     <row r="134" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M134" t="s">
-        <v>472</v>
+      <c r="M134" s="37" t="s">
+        <v>605</v>
       </c>
       <c r="N134" s="21" t="s">
         <v>610</v>
       </c>
-      <c r="O134" t="s">
-        <v>593</v>
-      </c>
-      <c r="P134" s="3"/>
     </row>
     <row r="135" spans="1:17" x14ac:dyDescent="0.25">
       <c r="M135" s="37" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="N135" s="21" t="s">
         <v>610</v>
@@ -7831,183 +7818,167 @@
     </row>
     <row r="136" spans="1:17" x14ac:dyDescent="0.25">
       <c r="M136" s="37" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="N136" s="21" t="s">
         <v>610</v>
       </c>
+      <c r="P136" s="3"/>
     </row>
     <row r="137" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M137" s="37" t="s">
-        <v>606</v>
-      </c>
-      <c r="N137" s="21" t="s">
-        <v>610</v>
+      <c r="L137" s="103" t="s">
+        <v>612</v>
       </c>
     </row>
     <row r="138" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M138" s="37" t="s">
-        <v>607</v>
+      <c r="M138" t="s">
+        <v>17</v>
       </c>
       <c r="N138" s="21" t="s">
-        <v>610</v>
-      </c>
-      <c r="P138" s="3"/>
+        <v>611</v>
+      </c>
+      <c r="O138" t="s">
+        <v>618</v>
+      </c>
+      <c r="P138" s="21" t="s">
+        <v>591</v>
+      </c>
     </row>
     <row r="139" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="L139" s="103" t="s">
-        <v>612</v>
-      </c>
+      <c r="M139" t="s">
+        <v>584</v>
+      </c>
+      <c r="N139" s="21" t="s">
+        <v>611</v>
+      </c>
+      <c r="O139" t="s">
+        <v>592</v>
+      </c>
+      <c r="P139" s="3"/>
     </row>
     <row r="140" spans="1:17" x14ac:dyDescent="0.25">
       <c r="M140" t="s">
-        <v>17</v>
+        <v>473</v>
       </c>
       <c r="N140" s="21" t="s">
         <v>611</v>
       </c>
       <c r="O140" t="s">
-        <v>618</v>
+        <v>474</v>
       </c>
       <c r="P140" s="21" t="s">
-        <v>591</v>
+        <v>475</v>
       </c>
     </row>
     <row r="141" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M141" t="s">
-        <v>584</v>
-      </c>
-      <c r="N141" s="21" t="s">
-        <v>611</v>
-      </c>
-      <c r="O141" t="s">
-        <v>592</v>
-      </c>
-      <c r="P141" s="3"/>
+      <c r="L141" s="103" t="s">
+        <v>614</v>
+      </c>
     </row>
     <row r="142" spans="1:17" x14ac:dyDescent="0.25">
       <c r="M142" t="s">
-        <v>473</v>
+        <v>17</v>
       </c>
       <c r="N142" s="21" t="s">
-        <v>611</v>
+        <v>621</v>
       </c>
       <c r="O142" t="s">
-        <v>474</v>
+        <v>618</v>
       </c>
       <c r="P142" s="21" t="s">
-        <v>475</v>
+        <v>591</v>
       </c>
     </row>
     <row r="143" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="L143" s="103" t="s">
-        <v>614</v>
-      </c>
+      <c r="M143" t="s">
+        <v>584</v>
+      </c>
+      <c r="N143" s="21" t="s">
+        <v>621</v>
+      </c>
+      <c r="O143" t="s">
+        <v>592</v>
+      </c>
+      <c r="P143" s="3"/>
     </row>
     <row r="144" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M144" t="s">
-        <v>17</v>
-      </c>
-      <c r="N144" s="21" t="s">
-        <v>621</v>
-      </c>
-      <c r="O144" t="s">
-        <v>618</v>
-      </c>
-      <c r="P144" s="21" t="s">
-        <v>591</v>
+      <c r="L144" s="103" t="s">
+        <v>615</v>
       </c>
     </row>
     <row r="145" spans="12:16" x14ac:dyDescent="0.25">
       <c r="M145" t="s">
+        <v>17</v>
+      </c>
+      <c r="N145" s="21" t="s">
+        <v>622</v>
+      </c>
+      <c r="O145" t="s">
+        <v>618</v>
+      </c>
+      <c r="P145" s="21" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="146" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="M146" t="s">
         <v>584</v>
       </c>
-      <c r="N145" s="21" t="s">
-        <v>621</v>
-      </c>
-      <c r="O145" t="s">
+      <c r="N146" s="21" t="s">
+        <v>622</v>
+      </c>
+      <c r="O146" t="s">
         <v>592</v>
       </c>
-      <c r="P145" s="3"/>
-    </row>
-    <row r="146" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="L146" s="103" t="s">
-        <v>615</v>
-      </c>
+      <c r="P146" s="3"/>
     </row>
     <row r="147" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="M147" t="s">
-        <v>17</v>
-      </c>
-      <c r="N147" s="21" t="s">
-        <v>622</v>
-      </c>
-      <c r="O147" t="s">
-        <v>618</v>
-      </c>
-      <c r="P147" s="21" t="s">
-        <v>591</v>
+      <c r="L147" s="103" t="s">
+        <v>616</v>
       </c>
     </row>
     <row r="148" spans="12:16" x14ac:dyDescent="0.25">
       <c r="M148" t="s">
+        <v>17</v>
+      </c>
+      <c r="N148" s="21" t="s">
+        <v>623</v>
+      </c>
+      <c r="O148" t="s">
+        <v>619</v>
+      </c>
+      <c r="P148" s="21" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="149" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="M149" t="s">
         <v>584</v>
       </c>
-      <c r="N148" s="21" t="s">
-        <v>622</v>
-      </c>
-      <c r="O148" t="s">
+      <c r="N149" s="21" t="s">
+        <v>623</v>
+      </c>
+      <c r="O149" t="s">
         <v>592</v>
       </c>
-      <c r="P148" s="3"/>
-    </row>
-    <row r="149" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="L149" s="103" t="s">
-        <v>616</v>
-      </c>
+      <c r="P149" s="3"/>
     </row>
     <row r="150" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="M150" t="s">
-        <v>17</v>
-      </c>
-      <c r="N150" s="21" t="s">
-        <v>623</v>
-      </c>
-      <c r="O150" t="s">
-        <v>619</v>
-      </c>
-      <c r="P150" s="21" t="s">
-        <v>591</v>
+      <c r="L150" s="103" t="s">
+        <v>617</v>
       </c>
     </row>
     <row r="151" spans="12:16" x14ac:dyDescent="0.25">
       <c r="M151" t="s">
-        <v>584</v>
+        <v>609</v>
       </c>
       <c r="N151" s="21" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="O151" t="s">
-        <v>592</v>
-      </c>
-      <c r="P151" s="3"/>
-    </row>
-    <row r="152" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="L152" s="103" t="s">
-        <v>617</v>
-      </c>
-    </row>
-    <row r="153" spans="12:16" x14ac:dyDescent="0.25">
-      <c r="M153" t="s">
-        <v>609</v>
-      </c>
-      <c r="N153" s="21" t="s">
-        <v>624</v>
-      </c>
-      <c r="O153" t="s">
         <v>620</v>
       </c>
-      <c r="P153" s="21"/>
+      <c r="P151" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
N/P/K in mineral feed
</commit_message>
<xml_diff>
--- a/data/default/FeedMgmt.xlsx
+++ b/data/default/FeedMgmt.xlsx
@@ -145,7 +145,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1542" uniqueCount="677">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1543" uniqueCount="678">
   <si>
     <t>f_feed</t>
   </si>
@@ -2234,6 +2234,9 @@
   </si>
   <si>
     <t>FeedMgmt-feed_pars.csv</t>
+  </si>
+  <si>
+    <t>Around 4% P seems common in mineral feed</t>
   </si>
 </sst>
 </file>
@@ -2652,7 +2655,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -2799,6 +2802,7 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -12315,9 +12319,18 @@
         <f t="shared" si="3"/>
         <v>100</v>
       </c>
-      <c r="F48" s="82"/>
-      <c r="G48" s="83"/>
-      <c r="H48" s="84"/>
+      <c r="F48" s="82">
+        <f t="shared" ref="F48" si="63">AVERAGE(W48,AL48)</f>
+        <v>0</v>
+      </c>
+      <c r="G48" s="83">
+        <f t="shared" ref="G48" si="64">AVERAGE(X48,AM48)</f>
+        <v>4</v>
+      </c>
+      <c r="H48" s="84">
+        <f t="shared" ref="H48" si="65">AVERAGE(Y48,AN48)</f>
+        <v>0</v>
+      </c>
       <c r="I48" s="85"/>
       <c r="J48" s="85"/>
       <c r="K48" s="20"/>
@@ -12343,15 +12356,27 @@
       <c r="S48" s="88">
         <v>0</v>
       </c>
-      <c r="T48" s="88"/>
-      <c r="U48" s="88"/>
+      <c r="T48" s="88">
+        <v>0</v>
+      </c>
+      <c r="U48" s="88">
+        <v>0</v>
+      </c>
       <c r="V48" s="89">
         <v>1000</v>
       </c>
-      <c r="W48" s="88"/>
-      <c r="X48" s="88"/>
-      <c r="Y48" s="89"/>
-      <c r="Z48" s="78"/>
+      <c r="W48" s="88">
+        <v>0</v>
+      </c>
+      <c r="X48" s="88">
+        <v>4</v>
+      </c>
+      <c r="Y48" s="89">
+        <v>0</v>
+      </c>
+      <c r="Z48" s="118" t="s">
+        <v>677</v>
+      </c>
       <c r="AA48" s="73"/>
       <c r="AB48" s="20"/>
       <c r="AC48" s="86">
@@ -12369,9 +12394,15 @@
       <c r="AG48" s="87">
         <v>0</v>
       </c>
-      <c r="AH48" s="86"/>
-      <c r="AI48" s="87"/>
-      <c r="AJ48" s="88"/>
+      <c r="AH48" s="86">
+        <v>0</v>
+      </c>
+      <c r="AI48" s="87">
+        <v>0</v>
+      </c>
+      <c r="AJ48" s="88">
+        <v>0</v>
+      </c>
       <c r="AK48" s="91">
         <v>1000</v>
       </c>
@@ -18554,17 +18585,17 @@
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A45,'feed pars'!$B$6:$B$48,0),E$1)&lt;&gt;"",E$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A45,'feed pars'!$B$6:$B$48,0),E$1), "")</f>
         <v>100</v>
       </c>
-      <c r="F45" s="57" t="str">
+      <c r="F45" s="57">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A45,'feed pars'!$B$6:$B$48,0),F$1)&lt;&gt;"",F$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A45,'feed pars'!$B$6:$B$48,0),F$1), "")</f>
-        <v/>
-      </c>
-      <c r="G45" s="57" t="str">
+        <v>0</v>
+      </c>
+      <c r="G45" s="57">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A45,'feed pars'!$B$6:$B$48,0),G$1)&lt;&gt;"",G$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A45,'feed pars'!$B$6:$B$48,0),G$1), "")</f>
-        <v/>
-      </c>
-      <c r="H45" s="57" t="str">
+        <v>4</v>
+      </c>
+      <c r="H45" s="57">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A45,'feed pars'!$B$6:$B$48,0),H$1)&lt;&gt;"",H$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A45,'feed pars'!$B$6:$B$48,0),H$1), "")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J45" s="57" t="str">
         <f>'feed pars'!$B48</f>

</xml_diff>

<commit_message>
Refinements to maximum shares sng in grazing
</commit_message>
<xml_diff>
--- a/data/default/FeedMgmt.xlsx
+++ b/data/default/FeedMgmt.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="5100" firstSheet="1" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="5100" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="references" sheetId="9" r:id="rId1"/>
@@ -17,7 +17,7 @@
     <sheet name="horses" sheetId="7" r:id="rId8"/>
     <sheet name="poultry" sheetId="5" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -145,7 +145,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1543" uniqueCount="678">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1566" uniqueCount="679">
   <si>
     <t>f_feed</t>
   </si>
@@ -2158,21 +2158,12 @@
     </r>
   </si>
   <si>
-    <t>Hessle &amp; Danielsson (2023)</t>
-  </si>
-  <si>
-    <t>Hessle, A. &amp; Danielsson, R. (2023) Number of cattle required to obtain good ecological status in Swedish grasslands and livestock’s methane emissions. Swedish University of Agricultural Sciences. Department of Animal Environment and Health. Section of Production systems</t>
-  </si>
-  <si>
     <t>Ahlgren, S., Behaderovic, D., Wirsenius, S., Carlsson, A., Hessle, A. Toräng, P., Seeman, A., den Braver, T. &amp;  et al. Kvarnbäck, O. (2022) Miljöpåverkan av svensk nöt- och lammköttsproduktion. RISE</t>
   </si>
   <si>
     <t>Ahlgren et al. (2022)</t>
   </si>
   <si>
-    <t>Suckler cows and all young animals</t>
-  </si>
-  <si>
     <t>Based on 4 weeks grazing for cows with dry period coinciding with grazing period</t>
   </si>
   <si>
@@ -2237,6 +2228,18 @@
   </si>
   <si>
     <t>Around 4% P seems common in mineral feed</t>
+  </si>
+  <si>
+    <t>Hessle, A. &amp; Danielsson, R. (2024). Cattle population required for favorable conservation status of management-dependent semi-natural grasslands and forests, and associated increase in enteric methane emissions. Journal for Nature Conservation, 78, 126571. https://doi.org/10.1016/j.jnc.2024.126571</t>
+  </si>
+  <si>
+    <t>Hessle &amp; Danielsson (2024)</t>
+  </si>
+  <si>
+    <t>calves, suckling</t>
+  </si>
+  <si>
+    <t>same as suckler cows</t>
   </si>
 </sst>
 </file>
@@ -2246,7 +2249,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="30" x14ac:knownFonts="1">
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2467,6 +2470,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -2655,7 +2665,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -2803,6 +2813,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3106,12 +3117,12 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>652</v>
+        <v>675</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
     </row>
   </sheetData>
@@ -3121,7 +3132,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R153"/>
+  <dimension ref="A1:R156"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="7" width="20.28515625" customWidth="1"/>
@@ -4292,6 +4303,12 @@
       <c r="A76" t="s">
         <v>19</v>
       </c>
+      <c r="B76" t="s">
+        <v>311</v>
+      </c>
+      <c r="E76" t="s">
+        <v>312</v>
+      </c>
       <c r="H76" t="s">
         <v>314</v>
       </c>
@@ -4302,16 +4319,16 @@
         <v>315</v>
       </c>
       <c r="N76" s="21">
-        <v>85</v>
+        <v>28</v>
       </c>
       <c r="O76" t="s">
         <v>22</v>
       </c>
       <c r="P76" s="21" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="Q76" t="s">
-        <v>654</v>
+        <v>676</v>
       </c>
     </row>
     <row r="77" spans="1:17" x14ac:dyDescent="0.25">
@@ -4319,7 +4336,7 @@
         <v>19</v>
       </c>
       <c r="B77" t="s">
-        <v>311</v>
+        <v>600</v>
       </c>
       <c r="E77" t="s">
         <v>312</v>
@@ -4334,21 +4351,25 @@
         <v>315</v>
       </c>
       <c r="N77" s="21">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="O77" t="s">
         <v>22</v>
       </c>
-      <c r="P77" s="21" t="s">
-        <v>656</v>
-      </c>
+      <c r="P77" s="21"/>
       <c r="Q77" t="s">
-        <v>651</v>
+        <v>676</v>
       </c>
     </row>
     <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>372</v>
+        <v>19</v>
+      </c>
+      <c r="B78" t="s">
+        <v>600</v>
+      </c>
+      <c r="E78" t="s">
+        <v>677</v>
       </c>
       <c r="H78" t="s">
         <v>314</v>
@@ -4359,20 +4380,23 @@
       <c r="M78" t="s">
         <v>315</v>
       </c>
-      <c r="N78" s="21">
-        <v>14.5</v>
+      <c r="N78" s="119">
+        <f>N77</f>
+        <v>100</v>
       </c>
       <c r="O78" t="s">
         <v>22</v>
       </c>
-      <c r="P78" s="3"/>
+      <c r="P78" s="21" t="s">
+        <v>678</v>
+      </c>
       <c r="Q78" t="s">
-        <v>634</v>
+        <v>676</v>
       </c>
     </row>
     <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>376</v>
+        <v>19</v>
       </c>
       <c r="H79" t="s">
         <v>314</v>
@@ -4384,25 +4408,19 @@
         <v>315</v>
       </c>
       <c r="N79" s="21">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="O79" t="s">
         <v>22</v>
       </c>
-      <c r="P79" s="3"/>
+      <c r="P79" s="21"/>
       <c r="Q79" t="s">
-        <v>654</v>
+        <v>676</v>
       </c>
     </row>
     <row r="80" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>376</v>
-      </c>
-      <c r="D80" t="s">
-        <v>646</v>
-      </c>
-      <c r="E80" t="s">
-        <v>480</v>
+        <v>372</v>
       </c>
       <c r="H80" t="s">
         <v>314</v>
@@ -4414,199 +4432,222 @@
         <v>315</v>
       </c>
       <c r="N80" s="21">
-        <v>69</v>
+        <v>14.5</v>
       </c>
       <c r="O80" t="s">
         <v>22</v>
       </c>
       <c r="P80" s="3"/>
       <c r="Q80" t="s">
-        <v>654</v>
+        <v>634</v>
       </c>
     </row>
     <row r="81" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N81" s="3"/>
+      <c r="A81" t="s">
+        <v>376</v>
+      </c>
+      <c r="H81" t="s">
+        <v>314</v>
+      </c>
+      <c r="I81" t="s">
+        <v>26</v>
+      </c>
+      <c r="M81" t="s">
+        <v>315</v>
+      </c>
+      <c r="N81" s="21">
+        <v>100</v>
+      </c>
+      <c r="O81" t="s">
+        <v>22</v>
+      </c>
       <c r="P81" s="3"/>
+      <c r="Q81" t="s">
+        <v>652</v>
+      </c>
     </row>
     <row r="82" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A82" s="1" t="s">
+      <c r="A82" t="s">
+        <v>376</v>
+      </c>
+      <c r="D82" t="s">
+        <v>646</v>
+      </c>
+      <c r="H82" t="s">
+        <v>314</v>
+      </c>
+      <c r="I82" t="s">
+        <v>26</v>
+      </c>
+      <c r="M82" t="s">
+        <v>315</v>
+      </c>
+      <c r="N82" s="21">
+        <v>66</v>
+      </c>
+      <c r="O82" t="s">
+        <v>22</v>
+      </c>
+      <c r="P82" s="3"/>
+      <c r="Q82" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>376</v>
+      </c>
+      <c r="D83" t="s">
+        <v>646</v>
+      </c>
+      <c r="E83" t="s">
+        <v>480</v>
+      </c>
+      <c r="H83" t="s">
+        <v>314</v>
+      </c>
+      <c r="I83" t="s">
+        <v>26</v>
+      </c>
+      <c r="M83" t="s">
+        <v>315</v>
+      </c>
+      <c r="N83" s="21">
+        <v>69</v>
+      </c>
+      <c r="O83" t="s">
+        <v>22</v>
+      </c>
+      <c r="P83" s="3"/>
+      <c r="Q83" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N84" s="3"/>
+      <c r="P84" s="3"/>
+    </row>
+    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A85" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="B82" s="1"/>
-      <c r="C82" s="1"/>
-      <c r="D82" s="1"/>
-      <c r="E82" s="2"/>
-      <c r="F82" s="2"/>
-      <c r="G82" s="2"/>
-      <c r="H82" s="2"/>
-      <c r="I82" s="2"/>
-      <c r="J82" s="2"/>
-      <c r="K82" s="2"/>
-      <c r="L82" s="2"/>
-      <c r="M82" s="2"/>
-      <c r="N82" s="2"/>
-      <c r="O82" s="2"/>
-      <c r="P82" s="2"/>
-      <c r="Q82" s="2"/>
-    </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M83" s="6" t="s">
+      <c r="B85" s="1"/>
+      <c r="C85" s="1"/>
+      <c r="D85" s="1"/>
+      <c r="E85" s="2"/>
+      <c r="F85" s="2"/>
+      <c r="G85" s="2"/>
+      <c r="H85" s="2"/>
+      <c r="I85" s="2"/>
+      <c r="J85" s="2"/>
+      <c r="K85" s="2"/>
+      <c r="L85" s="2"/>
+      <c r="M85" s="2"/>
+      <c r="N85" s="2"/>
+      <c r="O85" s="2"/>
+      <c r="P85" s="2"/>
+      <c r="Q85" s="2"/>
+    </row>
+    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M86" s="6" t="s">
         <v>373</v>
       </c>
-      <c r="N83" s="6">
-        <v>0</v>
-      </c>
-      <c r="O83" s="6" t="s">
+      <c r="N86" s="6">
+        <v>0</v>
+      </c>
+      <c r="O86" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="P83" s="6" t="s">
+      <c r="P86" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M84" s="6" t="s">
+    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M87" s="6" t="s">
         <v>374</v>
       </c>
-      <c r="N84" s="6">
-        <v>0</v>
-      </c>
-      <c r="O84" s="6" t="s">
+      <c r="N87" s="6">
+        <v>0</v>
+      </c>
+      <c r="O87" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="P84" s="6" t="s">
+      <c r="P87" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
+    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>19</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B88" t="s">
         <v>311</v>
       </c>
-      <c r="E85" t="s">
+      <c r="E88" t="s">
         <v>312</v>
       </c>
-      <c r="G85" t="s">
+      <c r="G88" t="s">
         <v>627</v>
       </c>
-      <c r="M85" s="21" t="s">
+      <c r="M88" s="21" t="s">
         <v>373</v>
       </c>
-      <c r="N85" s="21">
+      <c r="N88" s="21">
         <f>(0.8*20+0.2*2)</f>
         <v>16.399999999999999</v>
       </c>
-      <c r="O85" s="21" t="s">
+      <c r="O88" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="P85" s="21" t="s">
+      <c r="P88" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="Q85" t="s">
+      <c r="Q88" t="s">
         <v>634</v>
       </c>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
+    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>19</v>
       </c>
-      <c r="G86" t="s">
+      <c r="G89" t="s">
         <v>627</v>
       </c>
-      <c r="M86" s="21" t="s">
+      <c r="M89" s="21" t="s">
         <v>373</v>
       </c>
-      <c r="N86" s="21">
+      <c r="N89" s="21">
         <f>(0.6*20+0.4*2)</f>
         <v>12.8</v>
       </c>
-      <c r="O86" s="21" t="s">
+      <c r="O89" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="P86" s="21" t="s">
+      <c r="P89" s="21" t="s">
         <v>378</v>
       </c>
-      <c r="Q86" t="s">
+      <c r="Q89" t="s">
         <v>634</v>
       </c>
-    </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>376</v>
-      </c>
-      <c r="G87" t="s">
-        <v>627</v>
-      </c>
-      <c r="M87" s="21" t="s">
-        <v>373</v>
-      </c>
-      <c r="N87" s="21">
-        <v>2</v>
-      </c>
-      <c r="O87" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="P87" s="21" t="s">
-        <v>379</v>
-      </c>
-      <c r="Q87" t="s">
-        <v>634</v>
-      </c>
-    </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>372</v>
-      </c>
-      <c r="G88" t="s">
-        <v>627</v>
-      </c>
-      <c r="M88" s="21" t="s">
-        <v>373</v>
-      </c>
-      <c r="N88" s="21">
-        <v>2</v>
-      </c>
-      <c r="O88" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="P88" s="21" t="s">
-        <v>379</v>
-      </c>
-      <c r="Q88" t="s">
-        <v>634</v>
-      </c>
-    </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M89" s="21"/>
-      <c r="N89" s="21"/>
-      <c r="O89" s="21"/>
-      <c r="P89" s="21"/>
     </row>
     <row r="90" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>19</v>
-      </c>
-      <c r="B90" t="s">
-        <v>311</v>
-      </c>
-      <c r="E90" t="s">
-        <v>312</v>
+        <v>376</v>
       </c>
       <c r="G90" t="s">
         <v>627</v>
       </c>
       <c r="M90" s="21" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="N90" s="21">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O90" s="21" t="s">
         <v>22</v>
       </c>
       <c r="P90" s="21" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="Q90" t="s">
         <v>634</v>
@@ -4614,114 +4655,124 @@
     </row>
     <row r="91" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>19</v>
-      </c>
-      <c r="E91" t="s">
-        <v>313</v>
+        <v>372</v>
       </c>
       <c r="G91" t="s">
         <v>627</v>
       </c>
       <c r="M91" s="21" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="N91" s="21">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O91" s="21" t="s">
         <v>22</v>
       </c>
       <c r="P91" s="21" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="Q91" t="s">
         <v>634</v>
       </c>
     </row>
     <row r="92" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
+      <c r="M92" s="21"/>
+      <c r="N92" s="21"/>
+      <c r="O92" s="21"/>
+      <c r="P92" s="21"/>
+    </row>
+    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>19</v>
       </c>
-      <c r="G92" t="s">
+      <c r="B93" t="s">
+        <v>311</v>
+      </c>
+      <c r="E93" t="s">
+        <v>312</v>
+      </c>
+      <c r="G93" t="s">
         <v>627</v>
       </c>
-      <c r="M92" s="21" t="s">
+      <c r="M93" s="21" t="s">
         <v>374</v>
       </c>
-      <c r="N92" s="21">
+      <c r="N93" s="21">
+        <v>5</v>
+      </c>
+      <c r="O93" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="P93" s="21" t="s">
+        <v>380</v>
+      </c>
+      <c r="Q93" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>19</v>
+      </c>
+      <c r="E94" t="s">
+        <v>313</v>
+      </c>
+      <c r="G94" t="s">
+        <v>627</v>
+      </c>
+      <c r="M94" s="21" t="s">
+        <v>374</v>
+      </c>
+      <c r="N94" s="21">
+        <v>5</v>
+      </c>
+      <c r="O94" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="P94" s="21" t="s">
+        <v>380</v>
+      </c>
+      <c r="Q94" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="95" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>19</v>
+      </c>
+      <c r="G95" t="s">
+        <v>627</v>
+      </c>
+      <c r="M95" s="21" t="s">
+        <v>374</v>
+      </c>
+      <c r="N95" s="21">
         <f>0.9*5+0.1*15</f>
         <v>6</v>
       </c>
-      <c r="O92" s="21" t="s">
+      <c r="O95" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="P92" s="21" t="s">
+      <c r="P95" s="21" t="s">
         <v>381</v>
       </c>
-      <c r="Q92" t="s">
+      <c r="Q95" t="s">
         <v>634</v>
       </c>
     </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
+    <row r="96" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
         <v>376</v>
       </c>
-      <c r="G93" t="s">
+      <c r="G96" t="s">
         <v>627</v>
       </c>
-      <c r="M93" s="21" t="s">
+      <c r="M96" s="21" t="s">
         <v>374</v>
       </c>
-      <c r="N93" s="21">
+      <c r="N96" s="21">
         <v>15</v>
-      </c>
-      <c r="O93" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="P93" s="21"/>
-      <c r="Q93" t="s">
-        <v>634</v>
-      </c>
-    </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>372</v>
-      </c>
-      <c r="G94" t="s">
-        <v>627</v>
-      </c>
-      <c r="M94" s="21" t="s">
-        <v>374</v>
-      </c>
-      <c r="N94" s="21">
-        <v>15</v>
-      </c>
-      <c r="O94" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="P94" s="21"/>
-      <c r="Q94" t="s">
-        <v>634</v>
-      </c>
-    </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M95" s="21"/>
-      <c r="N95" s="21"/>
-      <c r="O95" s="21"/>
-      <c r="P95" s="21"/>
-    </row>
-    <row r="96" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A96" s="22"/>
-      <c r="B96" s="22"/>
-      <c r="E96" s="22"/>
-      <c r="G96" t="s">
-        <v>299</v>
-      </c>
-      <c r="M96" s="21" t="s">
-        <v>373</v>
-      </c>
-      <c r="N96" s="21">
-        <v>5</v>
       </c>
       <c r="O96" s="21" t="s">
         <v>22</v>
@@ -4732,125 +4783,85 @@
       </c>
     </row>
     <row r="97" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A97" s="22" t="str">
-        <f>A90</f>
+      <c r="A97" t="s">
+        <v>372</v>
+      </c>
+      <c r="G97" t="s">
+        <v>627</v>
+      </c>
+      <c r="M97" s="21" t="s">
+        <v>374</v>
+      </c>
+      <c r="N97" s="21">
+        <v>15</v>
+      </c>
+      <c r="O97" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="P97" s="21"/>
+      <c r="Q97" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M98" s="21"/>
+      <c r="N98" s="21"/>
+      <c r="O98" s="21"/>
+      <c r="P98" s="21"/>
+    </row>
+    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A99" s="22"/>
+      <c r="B99" s="22"/>
+      <c r="E99" s="22"/>
+      <c r="G99" t="s">
+        <v>299</v>
+      </c>
+      <c r="M99" s="21" t="s">
+        <v>373</v>
+      </c>
+      <c r="N99" s="21">
+        <v>5</v>
+      </c>
+      <c r="O99" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="P99" s="21"/>
+      <c r="Q99" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A100" s="22" t="str">
+        <f>A93</f>
         <v>cattle</v>
       </c>
-      <c r="B97" s="22" t="str">
-        <f>B90</f>
+      <c r="B100" s="22" t="str">
+        <f>B93</f>
         <v>dairy</v>
       </c>
-      <c r="E97" s="22" t="str">
-        <f t="shared" ref="E97:E98" si="0">E90</f>
+      <c r="E100" s="22" t="str">
+        <f t="shared" ref="E100:E101" si="0">E93</f>
         <v>cows</v>
       </c>
-      <c r="G97" t="s">
+      <c r="G100" t="s">
         <v>299</v>
       </c>
-      <c r="M97" s="22" t="str">
-        <f t="shared" ref="M97:Q101" si="1">M90</f>
+      <c r="M100" s="22" t="str">
+        <f t="shared" ref="M100:Q104" si="1">M93</f>
         <v>feeding_losses</v>
       </c>
-      <c r="N97" s="22">
+      <c r="N100" s="22">
         <f t="shared" si="1"/>
         <v>5</v>
-      </c>
-      <c r="O97" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>%</v>
-      </c>
-      <c r="P97" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="Q97" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A98" s="22" t="str">
-        <f t="shared" ref="A98:A101" si="2">A91</f>
-        <v>cattle</v>
-      </c>
-      <c r="E98" s="22" t="str">
-        <f t="shared" si="0"/>
-        <v>bulls</v>
-      </c>
-      <c r="G98" t="s">
-        <v>299</v>
-      </c>
-      <c r="M98" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N98" s="22">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="O98" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>%</v>
-      </c>
-      <c r="P98" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="Q98" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A99" s="22" t="str">
-        <f t="shared" si="2"/>
-        <v>cattle</v>
-      </c>
-      <c r="G99" t="s">
-        <v>299</v>
-      </c>
-      <c r="M99" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N99" s="22">
-        <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="O99" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>%</v>
-      </c>
-      <c r="P99" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>10% feeding on pasture</v>
-      </c>
-      <c r="Q99" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A100" s="22" t="str">
-        <f t="shared" si="2"/>
-        <v>sheep</v>
-      </c>
-      <c r="G100" t="s">
-        <v>299</v>
-      </c>
-      <c r="M100" s="22" t="str">
-        <f t="shared" si="1"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N100" s="22">
-        <f t="shared" si="1"/>
-        <v>15</v>
       </c>
       <c r="O100" s="22" t="str">
         <f t="shared" si="1"/>
         <v>%</v>
       </c>
-      <c r="P100" s="22"/>
+      <c r="P100" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>No feeding on pasture</v>
+      </c>
       <c r="Q100" s="22" t="str">
         <f t="shared" si="1"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
@@ -4858,8 +4869,12 @@
     </row>
     <row r="101" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="22" t="str">
-        <f t="shared" si="2"/>
-        <v>horses</v>
+        <f t="shared" ref="A101:A104" si="2">A94</f>
+        <v>cattle</v>
+      </c>
+      <c r="E101" s="22" t="str">
+        <f t="shared" si="0"/>
+        <v>bulls</v>
       </c>
       <c r="G101" t="s">
         <v>299</v>
@@ -4870,173 +4885,173 @@
       </c>
       <c r="N101" s="22">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="O101" s="22" t="str">
         <f t="shared" si="1"/>
         <v>%</v>
       </c>
-      <c r="P101" s="22"/>
+      <c r="P101" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>No feeding on pasture</v>
+      </c>
       <c r="Q101" s="22" t="str">
         <f t="shared" si="1"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="102" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A102" s="22"/>
-      <c r="M102" s="22"/>
-      <c r="N102" s="22"/>
-      <c r="O102" s="22"/>
-      <c r="P102" s="22"/>
-      <c r="Q102" s="22"/>
+      <c r="A102" s="22" t="str">
+        <f t="shared" si="2"/>
+        <v>cattle</v>
+      </c>
+      <c r="G102" t="s">
+        <v>299</v>
+      </c>
+      <c r="M102" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N102" s="22">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="O102" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="P102" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>10% feeding on pasture</v>
+      </c>
+      <c r="Q102" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
     </row>
     <row r="103" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A103" s="22" t="str">
+        <f t="shared" si="2"/>
+        <v>sheep</v>
+      </c>
       <c r="G103" t="s">
-        <v>628</v>
-      </c>
-      <c r="M103" s="21" t="s">
-        <v>373</v>
-      </c>
-      <c r="N103" s="21">
-        <v>5</v>
-      </c>
-      <c r="O103" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="P103" s="21"/>
-      <c r="Q103" t="s">
-        <v>634</v>
+        <v>299</v>
+      </c>
+      <c r="M103" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N103" s="22">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="O103" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="P103" s="22"/>
+      <c r="Q103" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="104" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="22" t="str">
-        <f>A90</f>
+        <f t="shared" si="2"/>
+        <v>horses</v>
+      </c>
+      <c r="G104" t="s">
+        <v>299</v>
+      </c>
+      <c r="M104" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N104" s="22">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="O104" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="P104" s="22"/>
+      <c r="Q104" s="22" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A105" s="22"/>
+      <c r="M105" s="22"/>
+      <c r="N105" s="22"/>
+      <c r="O105" s="22"/>
+      <c r="P105" s="22"/>
+      <c r="Q105" s="22"/>
+    </row>
+    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="G106" t="s">
+        <v>628</v>
+      </c>
+      <c r="M106" s="21" t="s">
+        <v>373</v>
+      </c>
+      <c r="N106" s="21">
+        <v>5</v>
+      </c>
+      <c r="O106" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="P106" s="21"/>
+      <c r="Q106" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A107" s="22" t="str">
+        <f>A93</f>
         <v>cattle</v>
       </c>
-      <c r="B104" s="22" t="str">
-        <f>B90</f>
+      <c r="B107" s="22" t="str">
+        <f>B93</f>
         <v>dairy</v>
       </c>
-      <c r="E104" s="22" t="str">
-        <f t="shared" ref="E104:E105" si="3">E90</f>
+      <c r="E107" s="22" t="str">
+        <f t="shared" ref="E107:E108" si="3">E93</f>
         <v>cows</v>
       </c>
-      <c r="G104" t="s">
+      <c r="G107" t="s">
         <v>628</v>
       </c>
-      <c r="M104" s="22" t="str">
-        <f t="shared" ref="M104:Q108" si="4">M90</f>
+      <c r="M107" s="22" t="str">
+        <f t="shared" ref="M107:Q111" si="4">M93</f>
         <v>feeding_losses</v>
       </c>
-      <c r="N104" s="22">
+      <c r="N107" s="22">
         <f t="shared" si="4"/>
         <v>5</v>
-      </c>
-      <c r="O104" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>%</v>
-      </c>
-      <c r="P104" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="Q104" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A105" s="22" t="str">
-        <f t="shared" ref="A105:A108" si="5">A91</f>
-        <v>cattle</v>
-      </c>
-      <c r="E105" s="22" t="str">
-        <f t="shared" si="3"/>
-        <v>bulls</v>
-      </c>
-      <c r="G105" t="s">
-        <v>628</v>
-      </c>
-      <c r="M105" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N105" s="22">
-        <f t="shared" si="4"/>
-        <v>5</v>
-      </c>
-      <c r="O105" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>%</v>
-      </c>
-      <c r="P105" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="Q105" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A106" s="22" t="str">
-        <f t="shared" si="5"/>
-        <v>cattle</v>
-      </c>
-      <c r="G106" t="s">
-        <v>628</v>
-      </c>
-      <c r="M106" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N106" s="22">
-        <f t="shared" si="4"/>
-        <v>6</v>
-      </c>
-      <c r="O106" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>%</v>
-      </c>
-      <c r="P106" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>10% feeding on pasture</v>
-      </c>
-      <c r="Q106" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A107" s="22" t="str">
-        <f t="shared" si="5"/>
-        <v>sheep</v>
-      </c>
-      <c r="G107" t="s">
-        <v>628</v>
-      </c>
-      <c r="M107" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N107" s="22">
-        <f t="shared" si="4"/>
-        <v>15</v>
       </c>
       <c r="O107" s="22" t="str">
         <f t="shared" si="4"/>
         <v>%</v>
       </c>
-      <c r="P107" s="21"/>
+      <c r="P107" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>No feeding on pasture</v>
+      </c>
       <c r="Q107" s="22" t="str">
-        <f t="shared" ref="Q107:Q108" si="6">Q93</f>
+        <f t="shared" si="4"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="108" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="22" t="str">
-        <f t="shared" si="5"/>
-        <v>horses</v>
+        <f t="shared" ref="A108:A111" si="5">A94</f>
+        <v>cattle</v>
+      </c>
+      <c r="E108" s="22" t="str">
+        <f t="shared" si="3"/>
+        <v>bulls</v>
       </c>
       <c r="G108" t="s">
         <v>628</v>
@@ -5047,67 +5062,110 @@
       </c>
       <c r="N108" s="22">
         <f t="shared" si="4"/>
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="O108" s="22" t="str">
         <f t="shared" si="4"/>
         <v>%</v>
       </c>
-      <c r="P108" s="21"/>
+      <c r="P108" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>No feeding on pasture</v>
+      </c>
       <c r="Q108" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A109" s="22" t="str">
+        <f t="shared" si="5"/>
+        <v>cattle</v>
+      </c>
+      <c r="G109" t="s">
+        <v>628</v>
+      </c>
+      <c r="M109" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N109" s="22">
+        <f t="shared" si="4"/>
+        <v>6</v>
+      </c>
+      <c r="O109" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="P109" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>10% feeding on pasture</v>
+      </c>
+      <c r="Q109" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A110" s="22" t="str">
+        <f t="shared" si="5"/>
+        <v>sheep</v>
+      </c>
+      <c r="G110" t="s">
+        <v>628</v>
+      </c>
+      <c r="M110" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N110" s="22">
+        <f t="shared" si="4"/>
+        <v>15</v>
+      </c>
+      <c r="O110" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="P110" s="21"/>
+      <c r="Q110" s="22" t="str">
+        <f t="shared" ref="Q110:Q111" si="6">Q96</f>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A111" s="22" t="str">
+        <f t="shared" si="5"/>
+        <v>horses</v>
+      </c>
+      <c r="G111" t="s">
+        <v>628</v>
+      </c>
+      <c r="M111" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N111" s="22">
+        <f t="shared" si="4"/>
+        <v>15</v>
+      </c>
+      <c r="O111" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="P111" s="21"/>
+      <c r="Q111" s="22" t="str">
         <f t="shared" si="6"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N109" s="3"/>
-      <c r="P109" s="21"/>
-    </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A110" s="3"/>
-      <c r="G110" t="s">
-        <v>629</v>
-      </c>
-      <c r="M110" s="21" t="s">
-        <v>373</v>
-      </c>
-      <c r="N110" s="21"/>
-      <c r="P110" s="3" t="s">
-        <v>631</v>
-      </c>
-    </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A111" s="3"/>
-      <c r="G111" t="s">
-        <v>629</v>
-      </c>
-      <c r="M111" s="21" t="s">
-        <v>374</v>
-      </c>
-      <c r="N111" s="21">
-        <v>2</v>
-      </c>
-      <c r="O111" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="P111" s="3" t="s">
-        <v>635</v>
-      </c>
-      <c r="Q111" t="s">
-        <v>633</v>
-      </c>
-    </row>
     <row r="112" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A112" s="3"/>
-      <c r="M112" s="21"/>
-      <c r="N112" s="21"/>
-      <c r="O112" s="21"/>
-      <c r="P112" s="3"/>
+      <c r="N112" s="3"/>
+      <c r="P112" s="21"/>
     </row>
     <row r="113" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A113" s="3"/>
       <c r="G113" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="M113" s="21" t="s">
         <v>373</v>
@@ -5120,13 +5178,13 @@
     <row r="114" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A114" s="3"/>
       <c r="G114" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="M114" s="21" t="s">
         <v>374</v>
       </c>
       <c r="N114" s="21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O114" s="21" t="s">
         <v>22</v>
@@ -5139,189 +5197,168 @@
       </c>
     </row>
     <row r="115" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N115" s="3"/>
-      <c r="P115" s="21"/>
+      <c r="A115" s="3"/>
+      <c r="M115" s="21"/>
+      <c r="N115" s="21"/>
+      <c r="O115" s="21"/>
+      <c r="P115" s="3"/>
     </row>
     <row r="116" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A116" s="1" t="s">
+      <c r="A116" s="3"/>
+      <c r="G116" t="s">
+        <v>630</v>
+      </c>
+      <c r="M116" s="21" t="s">
+        <v>373</v>
+      </c>
+      <c r="N116" s="21"/>
+      <c r="P116" s="3" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A117" s="3"/>
+      <c r="G117" t="s">
+        <v>630</v>
+      </c>
+      <c r="M117" s="21" t="s">
+        <v>374</v>
+      </c>
+      <c r="N117" s="21">
+        <v>3</v>
+      </c>
+      <c r="O117" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="P117" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="Q117" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N118" s="3"/>
+      <c r="P118" s="21"/>
+    </row>
+    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A119" s="1" t="s">
         <v>595</v>
       </c>
-      <c r="B116" s="1"/>
-      <c r="C116" s="1"/>
-      <c r="D116" s="1"/>
-      <c r="E116" s="2"/>
-      <c r="F116" s="2"/>
-      <c r="G116" s="2"/>
-      <c r="H116" s="2"/>
-      <c r="I116" s="2"/>
-      <c r="J116" s="2"/>
-      <c r="K116" s="2"/>
-      <c r="L116" s="2"/>
-      <c r="M116" s="2"/>
-      <c r="N116" s="2"/>
-      <c r="O116" s="2"/>
-      <c r="P116" s="2"/>
-      <c r="Q116" s="2"/>
-    </row>
-    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>19</v>
-      </c>
-      <c r="N117" s="21"/>
-      <c r="P117" s="21" t="s">
-        <v>596</v>
-      </c>
-    </row>
-    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A118" s="21" t="s">
-        <v>376</v>
-      </c>
-      <c r="B118" s="3"/>
-      <c r="C118" s="3"/>
-      <c r="D118" s="3"/>
-      <c r="E118" s="3"/>
-      <c r="F118" s="3"/>
-      <c r="G118" s="3"/>
-      <c r="H118" s="3"/>
-      <c r="I118" s="3"/>
-      <c r="J118" s="3"/>
-      <c r="K118" s="3"/>
-      <c r="L118" s="3"/>
-      <c r="M118" s="21" t="s">
-        <v>481</v>
-      </c>
-      <c r="N118" s="21">
-        <v>6.7</v>
-      </c>
-      <c r="O118" s="21" t="s">
-        <v>482</v>
-      </c>
-      <c r="P118" s="3"/>
-      <c r="Q118" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>372</v>
-      </c>
-      <c r="M119" t="s">
-        <v>483</v>
-      </c>
-      <c r="N119" s="21">
-        <v>18</v>
-      </c>
-      <c r="O119" t="s">
-        <v>484</v>
-      </c>
-      <c r="P119" s="3"/>
-      <c r="Q119" t="s">
-        <v>485</v>
-      </c>
+      <c r="B119" s="1"/>
+      <c r="C119" s="1"/>
+      <c r="D119" s="1"/>
+      <c r="E119" s="2"/>
+      <c r="F119" s="2"/>
+      <c r="G119" s="2"/>
+      <c r="H119" s="2"/>
+      <c r="I119" s="2"/>
+      <c r="J119" s="2"/>
+      <c r="K119" s="2"/>
+      <c r="L119" s="2"/>
+      <c r="M119" s="2"/>
+      <c r="N119" s="2"/>
+      <c r="O119" s="2"/>
+      <c r="P119" s="2"/>
+      <c r="Q119" s="2"/>
     </row>
     <row r="120" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>20</v>
-      </c>
-      <c r="M120" t="s">
-        <v>483</v>
-      </c>
-      <c r="N120" s="21">
-        <v>1.5</v>
-      </c>
-      <c r="O120" t="s">
-        <v>484</v>
-      </c>
-      <c r="P120" s="3"/>
-      <c r="Q120" t="s">
-        <v>485</v>
+        <v>19</v>
+      </c>
+      <c r="N120" s="21"/>
+      <c r="P120" s="21" t="s">
+        <v>596</v>
       </c>
     </row>
     <row r="121" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>369</v>
-      </c>
-      <c r="M121" t="s">
-        <v>483</v>
+      <c r="A121" s="21" t="s">
+        <v>376</v>
+      </c>
+      <c r="B121" s="3"/>
+      <c r="C121" s="3"/>
+      <c r="D121" s="3"/>
+      <c r="E121" s="3"/>
+      <c r="F121" s="3"/>
+      <c r="G121" s="3"/>
+      <c r="H121" s="3"/>
+      <c r="I121" s="3"/>
+      <c r="J121" s="3"/>
+      <c r="K121" s="3"/>
+      <c r="L121" s="3"/>
+      <c r="M121" s="21" t="s">
+        <v>481</v>
       </c>
       <c r="N121" s="21">
-        <v>0</v>
-      </c>
-      <c r="O121" t="s">
-        <v>484</v>
+        <v>6.7</v>
+      </c>
+      <c r="O121" s="21" t="s">
+        <v>482</v>
       </c>
       <c r="P121" s="3"/>
       <c r="Q121" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>372</v>
+      </c>
+      <c r="M122" t="s">
+        <v>483</v>
+      </c>
+      <c r="N122" s="21">
+        <v>18</v>
+      </c>
+      <c r="O122" t="s">
+        <v>484</v>
+      </c>
+      <c r="P122" s="3"/>
+      <c r="Q122" t="s">
         <v>485</v>
       </c>
     </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N122" s="21"/>
-      <c r="P122" s="3"/>
-    </row>
     <row r="123" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>20</v>
+      </c>
       <c r="M123" t="s">
-        <v>597</v>
+        <v>483</v>
       </c>
       <c r="N123" s="21">
-        <v>1</v>
-      </c>
-      <c r="O123" s="21" t="s">
-        <v>598</v>
-      </c>
-      <c r="P123" s="21" t="s">
-        <v>599</v>
-      </c>
-      <c r="Q123" s="21"/>
+        <v>1.5</v>
+      </c>
+      <c r="O123" t="s">
+        <v>484</v>
+      </c>
+      <c r="P123" s="3"/>
+      <c r="Q123" t="s">
+        <v>485</v>
+      </c>
     </row>
     <row r="124" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>19</v>
+        <v>369</v>
       </c>
       <c r="M124" t="s">
-        <v>597</v>
+        <v>483</v>
       </c>
       <c r="N124" s="21">
-        <v>1</v>
-      </c>
-      <c r="O124" s="21" t="s">
-        <v>598</v>
-      </c>
-      <c r="P124" s="21"/>
-      <c r="Q124" s="21"/>
+        <v>0</v>
+      </c>
+      <c r="O124" t="s">
+        <v>484</v>
+      </c>
+      <c r="P124" s="3"/>
+      <c r="Q124" t="s">
+        <v>485</v>
+      </c>
     </row>
     <row r="125" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
-        <v>19</v>
-      </c>
-      <c r="B125" t="s">
-        <v>311</v>
-      </c>
-      <c r="E125" t="s">
-        <v>312</v>
-      </c>
-      <c r="M125" t="s">
-        <v>597</v>
-      </c>
-      <c r="N125" s="21">
-        <v>1</v>
-      </c>
-      <c r="O125" s="21" t="s">
-        <v>598</v>
-      </c>
-      <c r="P125" s="21"/>
-      <c r="Q125" s="21"/>
+      <c r="N125" s="21"/>
+      <c r="P125" s="3"/>
     </row>
     <row r="126" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
-        <v>19</v>
-      </c>
-      <c r="B126" t="s">
-        <v>311</v>
-      </c>
-      <c r="E126" t="s">
-        <v>313</v>
-      </c>
       <c r="M126" t="s">
         <v>597</v>
       </c>
@@ -5331,19 +5368,15 @@
       <c r="O126" s="21" t="s">
         <v>598</v>
       </c>
-      <c r="P126" s="21"/>
+      <c r="P126" s="21" t="s">
+        <v>599</v>
+      </c>
       <c r="Q126" s="21"/>
     </row>
     <row r="127" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>19</v>
       </c>
-      <c r="B127" t="s">
-        <v>600</v>
-      </c>
-      <c r="E127" t="s">
-        <v>313</v>
-      </c>
       <c r="M127" t="s">
         <v>597</v>
       </c>
@@ -5357,102 +5390,97 @@
       <c r="Q127" s="21"/>
     </row>
     <row r="128" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N128" s="3"/>
-      <c r="P128" s="3"/>
+      <c r="A128" t="s">
+        <v>19</v>
+      </c>
+      <c r="B128" t="s">
+        <v>311</v>
+      </c>
+      <c r="E128" t="s">
+        <v>312</v>
+      </c>
+      <c r="M128" t="s">
+        <v>597</v>
+      </c>
+      <c r="N128" s="21">
+        <v>1</v>
+      </c>
+      <c r="O128" s="21" t="s">
+        <v>598</v>
+      </c>
+      <c r="P128" s="21"/>
+      <c r="Q128" s="21"/>
     </row>
     <row r="129" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A129" s="106" t="s">
-        <v>659</v>
-      </c>
-      <c r="B129" s="106"/>
-      <c r="C129" s="106"/>
-      <c r="D129" s="106"/>
-      <c r="E129" s="107"/>
-      <c r="F129" s="107"/>
-      <c r="G129" s="107"/>
-      <c r="H129" s="107"/>
-      <c r="I129" s="107"/>
-      <c r="J129" s="107"/>
-      <c r="K129" s="107"/>
-      <c r="L129" s="107"/>
-      <c r="M129" s="107"/>
-      <c r="N129" s="107"/>
-      <c r="O129" s="107"/>
-      <c r="P129" s="107" t="s">
+      <c r="A129" t="s">
+        <v>19</v>
+      </c>
+      <c r="B129" t="s">
+        <v>311</v>
+      </c>
+      <c r="E129" t="s">
+        <v>313</v>
+      </c>
+      <c r="M129" t="s">
+        <v>597</v>
+      </c>
+      <c r="N129" s="21">
+        <v>1</v>
+      </c>
+      <c r="O129" s="21" t="s">
+        <v>598</v>
+      </c>
+      <c r="P129" s="21"/>
+      <c r="Q129" s="21"/>
+    </row>
+    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>19</v>
+      </c>
+      <c r="B130" t="s">
+        <v>600</v>
+      </c>
+      <c r="E130" t="s">
+        <v>313</v>
+      </c>
+      <c r="M130" t="s">
+        <v>597</v>
+      </c>
+      <c r="N130" s="21">
+        <v>1</v>
+      </c>
+      <c r="O130" s="21" t="s">
+        <v>598</v>
+      </c>
+      <c r="P130" s="21"/>
+      <c r="Q130" s="21"/>
+    </row>
+    <row r="131" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N131" s="3"/>
+      <c r="P131" s="3"/>
+    </row>
+    <row r="132" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A132" s="106" t="s">
+        <v>656</v>
+      </c>
+      <c r="B132" s="106"/>
+      <c r="C132" s="106"/>
+      <c r="D132" s="106"/>
+      <c r="E132" s="107"/>
+      <c r="F132" s="107"/>
+      <c r="G132" s="107"/>
+      <c r="H132" s="107"/>
+      <c r="I132" s="107"/>
+      <c r="J132" s="107"/>
+      <c r="K132" s="107"/>
+      <c r="L132" s="107"/>
+      <c r="M132" s="107"/>
+      <c r="N132" s="107"/>
+      <c r="O132" s="107"/>
+      <c r="P132" s="107" t="s">
         <v>291</v>
       </c>
-      <c r="Q129" s="107"/>
-    </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A130" s="109"/>
-      <c r="B130" s="109"/>
-      <c r="C130" s="109"/>
-      <c r="D130" s="109"/>
-      <c r="E130" s="109"/>
-      <c r="F130" s="109"/>
-      <c r="G130" s="109"/>
-      <c r="H130" s="109"/>
-      <c r="I130" s="109"/>
-      <c r="J130" s="109"/>
-      <c r="K130" s="109"/>
-      <c r="L130" s="110" t="s">
-        <v>612</v>
-      </c>
-      <c r="M130" s="109"/>
-      <c r="N130" s="109"/>
-      <c r="O130" s="109"/>
-      <c r="P130" s="109"/>
-      <c r="Q130" s="109"/>
-    </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A131" s="109"/>
-      <c r="B131" s="109"/>
-      <c r="C131" s="109"/>
-      <c r="D131" s="109"/>
-      <c r="E131" s="109"/>
-      <c r="F131" s="109"/>
-      <c r="G131" s="109"/>
-      <c r="H131" s="109"/>
-      <c r="I131" s="109"/>
-      <c r="J131" s="109"/>
-      <c r="K131" s="109"/>
-      <c r="L131" s="109"/>
-      <c r="M131" s="109" t="s">
-        <v>370</v>
-      </c>
-      <c r="N131" s="111" t="s">
-        <v>609</v>
-      </c>
-      <c r="O131" s="109" t="s">
-        <v>593</v>
-      </c>
-      <c r="P131" s="112"/>
-      <c r="Q131" s="109"/>
-    </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A132" s="109"/>
-      <c r="B132" s="109"/>
-      <c r="C132" s="109"/>
-      <c r="D132" s="109"/>
-      <c r="E132" s="109"/>
-      <c r="F132" s="109"/>
-      <c r="G132" s="109"/>
-      <c r="H132" s="109"/>
-      <c r="I132" s="109"/>
-      <c r="J132" s="109"/>
-      <c r="K132" s="109"/>
-      <c r="L132" s="109"/>
-      <c r="M132" s="109" t="s">
-        <v>471</v>
-      </c>
-      <c r="N132" s="111" t="s">
-        <v>609</v>
-      </c>
-      <c r="O132" s="109" t="s">
-        <v>592</v>
-      </c>
-      <c r="P132" s="112"/>
-      <c r="Q132" s="109"/>
+      <c r="Q132" s="107"/>
     </row>
     <row r="133" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A133" s="109"/>
@@ -5466,13 +5494,11 @@
       <c r="I133" s="109"/>
       <c r="J133" s="109"/>
       <c r="K133" s="109"/>
-      <c r="L133" s="109"/>
-      <c r="M133" s="113" t="s">
-        <v>603</v>
-      </c>
-      <c r="N133" s="111" t="s">
-        <v>609</v>
-      </c>
+      <c r="L133" s="110" t="s">
+        <v>612</v>
+      </c>
+      <c r="M133" s="109"/>
+      <c r="N133" s="109"/>
       <c r="O133" s="109"/>
       <c r="P133" s="109"/>
       <c r="Q133" s="109"/>
@@ -5490,14 +5516,16 @@
       <c r="J134" s="109"/>
       <c r="K134" s="109"/>
       <c r="L134" s="109"/>
-      <c r="M134" s="113" t="s">
-        <v>604</v>
+      <c r="M134" s="109" t="s">
+        <v>370</v>
       </c>
       <c r="N134" s="111" t="s">
         <v>609</v>
       </c>
-      <c r="O134" s="109"/>
-      <c r="P134" s="109"/>
+      <c r="O134" s="109" t="s">
+        <v>593</v>
+      </c>
+      <c r="P134" s="112"/>
       <c r="Q134" s="109"/>
     </row>
     <row r="135" spans="1:17" x14ac:dyDescent="0.25">
@@ -5513,14 +5541,16 @@
       <c r="J135" s="109"/>
       <c r="K135" s="109"/>
       <c r="L135" s="109"/>
-      <c r="M135" s="113" t="s">
-        <v>605</v>
+      <c r="M135" s="109" t="s">
+        <v>471</v>
       </c>
       <c r="N135" s="111" t="s">
         <v>609</v>
       </c>
-      <c r="O135" s="109"/>
-      <c r="P135" s="109"/>
+      <c r="O135" s="109" t="s">
+        <v>592</v>
+      </c>
+      <c r="P135" s="112"/>
       <c r="Q135" s="109"/>
     </row>
     <row r="136" spans="1:17" x14ac:dyDescent="0.25">
@@ -5537,13 +5567,13 @@
       <c r="K136" s="109"/>
       <c r="L136" s="109"/>
       <c r="M136" s="113" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="N136" s="111" t="s">
         <v>609</v>
       </c>
       <c r="O136" s="109"/>
-      <c r="P136" s="112"/>
+      <c r="P136" s="109"/>
       <c r="Q136" s="109"/>
     </row>
     <row r="137" spans="1:17" x14ac:dyDescent="0.25">
@@ -5558,11 +5588,13 @@
       <c r="I137" s="109"/>
       <c r="J137" s="109"/>
       <c r="K137" s="109"/>
-      <c r="L137" s="110" t="s">
-        <v>611</v>
-      </c>
-      <c r="M137" s="109"/>
-      <c r="N137" s="109"/>
+      <c r="L137" s="109"/>
+      <c r="M137" s="113" t="s">
+        <v>604</v>
+      </c>
+      <c r="N137" s="111" t="s">
+        <v>609</v>
+      </c>
       <c r="O137" s="109"/>
       <c r="P137" s="109"/>
       <c r="Q137" s="109"/>
@@ -5580,18 +5612,14 @@
       <c r="J138" s="109"/>
       <c r="K138" s="109"/>
       <c r="L138" s="109"/>
-      <c r="M138" s="109" t="s">
-        <v>17</v>
+      <c r="M138" s="113" t="s">
+        <v>605</v>
       </c>
       <c r="N138" s="111" t="s">
-        <v>610</v>
-      </c>
-      <c r="O138" s="109" t="s">
-        <v>617</v>
-      </c>
-      <c r="P138" s="111" t="s">
-        <v>590</v>
-      </c>
+        <v>609</v>
+      </c>
+      <c r="O138" s="109"/>
+      <c r="P138" s="109"/>
       <c r="Q138" s="109"/>
     </row>
     <row r="139" spans="1:17" x14ac:dyDescent="0.25">
@@ -5607,15 +5635,13 @@
       <c r="J139" s="109"/>
       <c r="K139" s="109"/>
       <c r="L139" s="109"/>
-      <c r="M139" s="109" t="s">
-        <v>583</v>
+      <c r="M139" s="113" t="s">
+        <v>606</v>
       </c>
       <c r="N139" s="111" t="s">
-        <v>610</v>
-      </c>
-      <c r="O139" s="109" t="s">
-        <v>591</v>
-      </c>
+        <v>609</v>
+      </c>
+      <c r="O139" s="109"/>
       <c r="P139" s="112"/>
       <c r="Q139" s="109"/>
     </row>
@@ -5631,19 +5657,13 @@
       <c r="I140" s="109"/>
       <c r="J140" s="109"/>
       <c r="K140" s="109"/>
-      <c r="L140" s="109"/>
-      <c r="M140" s="109" t="s">
-        <v>472</v>
-      </c>
-      <c r="N140" s="111" t="s">
-        <v>610</v>
-      </c>
-      <c r="O140" s="109" t="s">
-        <v>473</v>
-      </c>
-      <c r="P140" s="111" t="s">
-        <v>474</v>
-      </c>
+      <c r="L140" s="110" t="s">
+        <v>611</v>
+      </c>
+      <c r="M140" s="109"/>
+      <c r="N140" s="109"/>
+      <c r="O140" s="109"/>
+      <c r="P140" s="109"/>
       <c r="Q140" s="109"/>
     </row>
     <row r="141" spans="1:17" x14ac:dyDescent="0.25">
@@ -5658,13 +5678,19 @@
       <c r="I141" s="109"/>
       <c r="J141" s="109"/>
       <c r="K141" s="109"/>
-      <c r="L141" s="110" t="s">
-        <v>613</v>
-      </c>
-      <c r="M141" s="109"/>
-      <c r="N141" s="109"/>
-      <c r="O141" s="109"/>
-      <c r="P141" s="109"/>
+      <c r="L141" s="109"/>
+      <c r="M141" s="109" t="s">
+        <v>17</v>
+      </c>
+      <c r="N141" s="111" t="s">
+        <v>610</v>
+      </c>
+      <c r="O141" s="109" t="s">
+        <v>617</v>
+      </c>
+      <c r="P141" s="111" t="s">
+        <v>590</v>
+      </c>
       <c r="Q141" s="109"/>
     </row>
     <row r="142" spans="1:17" x14ac:dyDescent="0.25">
@@ -5681,17 +5707,15 @@
       <c r="K142" s="109"/>
       <c r="L142" s="109"/>
       <c r="M142" s="109" t="s">
-        <v>17</v>
+        <v>583</v>
       </c>
       <c r="N142" s="111" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="O142" s="109" t="s">
-        <v>617</v>
-      </c>
-      <c r="P142" s="111" t="s">
-        <v>590</v>
-      </c>
+        <v>591</v>
+      </c>
+      <c r="P142" s="112"/>
       <c r="Q142" s="109"/>
     </row>
     <row r="143" spans="1:17" x14ac:dyDescent="0.25">
@@ -5708,15 +5732,17 @@
       <c r="K143" s="109"/>
       <c r="L143" s="109"/>
       <c r="M143" s="109" t="s">
-        <v>583</v>
+        <v>472</v>
       </c>
       <c r="N143" s="111" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="O143" s="109" t="s">
-        <v>591</v>
-      </c>
-      <c r="P143" s="112"/>
+        <v>473</v>
+      </c>
+      <c r="P143" s="111" t="s">
+        <v>474</v>
+      </c>
       <c r="Q143" s="109"/>
     </row>
     <row r="144" spans="1:17" x14ac:dyDescent="0.25">
@@ -5732,7 +5758,7 @@
       <c r="J144" s="109"/>
       <c r="K144" s="109"/>
       <c r="L144" s="110" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="M144" s="109"/>
       <c r="N144" s="109"/>
@@ -5757,7 +5783,7 @@
         <v>17</v>
       </c>
       <c r="N145" s="111" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="O145" s="109" t="s">
         <v>617</v>
@@ -5784,7 +5810,7 @@
         <v>583</v>
       </c>
       <c r="N146" s="111" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="O146" s="109" t="s">
         <v>591</v>
@@ -5805,7 +5831,7 @@
       <c r="J147" s="109"/>
       <c r="K147" s="109"/>
       <c r="L147" s="110" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="M147" s="109"/>
       <c r="N147" s="109"/>
@@ -5830,10 +5856,10 @@
         <v>17</v>
       </c>
       <c r="N148" s="111" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="O148" s="109" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="P148" s="111" t="s">
         <v>590</v>
@@ -5857,7 +5883,7 @@
         <v>583</v>
       </c>
       <c r="N149" s="111" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="O149" s="109" t="s">
         <v>591</v>
@@ -5878,7 +5904,7 @@
       <c r="J150" s="109"/>
       <c r="K150" s="109"/>
       <c r="L150" s="110" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="M150" s="109"/>
       <c r="N150" s="109"/>
@@ -5900,23 +5926,96 @@
       <c r="K151" s="109"/>
       <c r="L151" s="109"/>
       <c r="M151" s="109" t="s">
+        <v>17</v>
+      </c>
+      <c r="N151" s="111" t="s">
+        <v>622</v>
+      </c>
+      <c r="O151" s="109" t="s">
+        <v>618</v>
+      </c>
+      <c r="P151" s="111" t="s">
+        <v>590</v>
+      </c>
+      <c r="Q151" s="109"/>
+    </row>
+    <row r="152" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A152" s="109"/>
+      <c r="B152" s="109"/>
+      <c r="C152" s="109"/>
+      <c r="D152" s="109"/>
+      <c r="E152" s="109"/>
+      <c r="F152" s="109"/>
+      <c r="G152" s="109"/>
+      <c r="H152" s="109"/>
+      <c r="I152" s="109"/>
+      <c r="J152" s="109"/>
+      <c r="K152" s="109"/>
+      <c r="L152" s="109"/>
+      <c r="M152" s="109" t="s">
+        <v>583</v>
+      </c>
+      <c r="N152" s="111" t="s">
+        <v>622</v>
+      </c>
+      <c r="O152" s="109" t="s">
+        <v>591</v>
+      </c>
+      <c r="P152" s="112"/>
+      <c r="Q152" s="109"/>
+    </row>
+    <row r="153" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A153" s="109"/>
+      <c r="B153" s="109"/>
+      <c r="C153" s="109"/>
+      <c r="D153" s="109"/>
+      <c r="E153" s="109"/>
+      <c r="F153" s="109"/>
+      <c r="G153" s="109"/>
+      <c r="H153" s="109"/>
+      <c r="I153" s="109"/>
+      <c r="J153" s="109"/>
+      <c r="K153" s="109"/>
+      <c r="L153" s="110" t="s">
+        <v>616</v>
+      </c>
+      <c r="M153" s="109"/>
+      <c r="N153" s="109"/>
+      <c r="O153" s="109"/>
+      <c r="P153" s="109"/>
+      <c r="Q153" s="109"/>
+    </row>
+    <row r="154" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A154" s="109"/>
+      <c r="B154" s="109"/>
+      <c r="C154" s="109"/>
+      <c r="D154" s="109"/>
+      <c r="E154" s="109"/>
+      <c r="F154" s="109"/>
+      <c r="G154" s="109"/>
+      <c r="H154" s="109"/>
+      <c r="I154" s="109"/>
+      <c r="J154" s="109"/>
+      <c r="K154" s="109"/>
+      <c r="L154" s="109"/>
+      <c r="M154" s="109" t="s">
         <v>608</v>
       </c>
-      <c r="N151" s="111" t="s">
+      <c r="N154" s="111" t="s">
         <v>623</v>
       </c>
-      <c r="O151" s="109" t="s">
+      <c r="O154" s="109" t="s">
         <v>619</v>
       </c>
-      <c r="P151" s="111"/>
-      <c r="Q151" s="109"/>
-    </row>
-    <row r="153" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M153" s="5" t="s">
-        <v>675</v>
-      </c>
-      <c r="N153" s="108" t="s">
-        <v>676</v>
+      <c r="P154" s="111"/>
+      <c r="Q154" s="109"/>
+    </row>
+    <row r="156" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M156" s="5" t="s">
+        <v>672</v>
+      </c>
+      <c r="N156" s="108" t="s">
+        <v>673</v>
       </c>
     </row>
   </sheetData>
@@ -7810,7 +7909,7 @@
       </c>
       <c r="AO16" s="77"/>
       <c r="AP16" s="74" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="AQ16" t="s">
         <v>465</v>
@@ -12375,7 +12474,7 @@
         <v>0</v>
       </c>
       <c r="Z48" s="118" t="s">
-        <v>677</v>
+        <v>674</v>
       </c>
       <c r="AA48" s="73"/>
       <c r="AB48" s="20"/>
@@ -12430,7 +12529,7 @@
       <c r="J50" s="65"/>
       <c r="K50" s="66"/>
       <c r="O50" s="115" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
     </row>
     <row r="51" spans="4:19" x14ac:dyDescent="0.25">
@@ -12454,7 +12553,7 @@
         <v>29</v>
       </c>
       <c r="R51" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="S51" t="s">
         <v>41</v>
@@ -12504,7 +12603,7 @@
       <c r="J53" s="36"/>
       <c r="K53" s="39"/>
       <c r="O53" s="115" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
     </row>
     <row r="54" spans="4:19" x14ac:dyDescent="0.25">
@@ -12695,19 +12794,19 @@
         <v>15</v>
       </c>
       <c r="D2" s="36" t="s">
+        <v>660</v>
+      </c>
+      <c r="E2" s="36" t="s">
+        <v>661</v>
+      </c>
+      <c r="F2" s="36" t="s">
+        <v>662</v>
+      </c>
+      <c r="G2" s="36" t="s">
         <v>663</v>
       </c>
-      <c r="E2" s="36" t="s">
+      <c r="H2" s="36" t="s">
         <v>664</v>
-      </c>
-      <c r="F2" s="36" t="s">
-        <v>665</v>
-      </c>
-      <c r="G2" s="36" t="s">
-        <v>666</v>
-      </c>
-      <c r="H2" s="36" t="s">
-        <v>667</v>
       </c>
       <c r="I2" s="37"/>
       <c r="J2" s="36" t="s">
@@ -12720,19 +12819,19 @@
         <v>15</v>
       </c>
       <c r="M2" s="36" t="s">
+        <v>665</v>
+      </c>
+      <c r="N2" s="36" t="s">
+        <v>666</v>
+      </c>
+      <c r="O2" s="36" t="s">
+        <v>667</v>
+      </c>
+      <c r="P2" s="36" t="s">
+        <v>670</v>
+      </c>
+      <c r="Q2" s="36" t="s">
         <v>668</v>
-      </c>
-      <c r="N2" s="36" t="s">
-        <v>669</v>
-      </c>
-      <c r="O2" s="36" t="s">
-        <v>670</v>
-      </c>
-      <c r="P2" s="36" t="s">
-        <v>673</v>
-      </c>
-      <c r="Q2" s="36" t="s">
-        <v>671</v>
       </c>
       <c r="S2" s="36" t="s">
         <v>0</v>
@@ -12744,13 +12843,13 @@
         <v>15</v>
       </c>
       <c r="V2" s="36" t="s">
+        <v>665</v>
+      </c>
+      <c r="W2" s="36" t="s">
+        <v>670</v>
+      </c>
+      <c r="X2" s="36" t="s">
         <v>668</v>
-      </c>
-      <c r="W2" s="36" t="s">
-        <v>673</v>
-      </c>
-      <c r="X2" s="36" t="s">
-        <v>671</v>
       </c>
       <c r="Z2" s="36" t="s">
         <v>0</v>
@@ -12762,13 +12861,13 @@
         <v>15</v>
       </c>
       <c r="AC2" s="36" t="s">
+        <v>665</v>
+      </c>
+      <c r="AD2" s="36" t="s">
+        <v>670</v>
+      </c>
+      <c r="AE2" s="36" t="s">
         <v>668</v>
-      </c>
-      <c r="AD2" s="36" t="s">
-        <v>673</v>
-      </c>
-      <c r="AE2" s="36" t="s">
-        <v>671</v>
       </c>
       <c r="AG2" s="36" t="s">
         <v>0</v>
@@ -12780,10 +12879,10 @@
         <v>15</v>
       </c>
       <c r="AJ2" s="36" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="AK2" s="36" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
       <c r="AM2" s="36" t="s">
         <v>0</v>
@@ -12795,10 +12894,10 @@
         <v>15</v>
       </c>
       <c r="AP2" s="36" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="AQ2" s="36" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
       <c r="AS2" s="36" t="s">
         <v>0</v>
@@ -12810,7 +12909,7 @@
         <v>15</v>
       </c>
       <c r="AV2" s="101" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
     </row>
     <row r="3" spans="1:48" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Removed share_domestic=0 for 'sugare beet molasses'
</commit_message>
<xml_diff>
--- a/data/default/FeedMgmt.xlsx
+++ b/data/default/FeedMgmt.xlsx
@@ -146,7 +146,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1619" uniqueCount="682">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1615" uniqueCount="681">
   <si>
     <t>Statistics Netherlands (2012) Standardised calculation methods for animal manure and nutrients. Standard data 1990–2008</t>
   </si>
@@ -2267,9 +2267,6 @@
   </si>
   <si>
     <t>organic</t>
-  </si>
-  <si>
-    <t>&lt;-- BORDE INTE BEHÖVAS!</t>
   </si>
   <si>
     <t>No domestic organic sugar production</t>
@@ -3138,7 +3135,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R175"/>
+  <dimension ref="A1:R173"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="7" width="20.28515625" style="1" customWidth="1"/>
@@ -4294,20 +4291,18 @@
       <c r="H75"/>
       <c r="I75"/>
       <c r="J75" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="M75" s="1" t="s">
         <v>88</v>
       </c>
       <c r="N75" s="10">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="O75" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="P75" s="10" t="s">
-        <v>680</v>
-      </c>
+      <c r="P75" s="10"/>
       <c r="Q75"/>
     </row>
     <row r="76" spans="1:17" x14ac:dyDescent="0.25">
@@ -4315,8 +4310,18 @@
       <c r="G76"/>
       <c r="H76"/>
       <c r="I76"/>
-      <c r="J76"/>
-      <c r="N76" s="10"/>
+      <c r="J76" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="M76" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N76" s="10">
+        <v>42</v>
+      </c>
+      <c r="O76" s="1" t="s">
+        <v>82</v>
+      </c>
       <c r="P76" s="10"/>
       <c r="Q76"/>
     </row>
@@ -4325,14 +4330,14 @@
       <c r="G77"/>
       <c r="H77"/>
       <c r="I77"/>
-      <c r="J77" t="s">
-        <v>60</v>
+      <c r="J77" s="1" t="s">
+        <v>51</v>
       </c>
       <c r="M77" s="1" t="s">
         <v>88</v>
       </c>
       <c r="N77" s="10">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="O77" s="1" t="s">
         <v>82</v>
@@ -4346,13 +4351,13 @@
       <c r="H78"/>
       <c r="I78"/>
       <c r="J78" s="1" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="M78" s="1" t="s">
         <v>88</v>
       </c>
       <c r="N78" s="10">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="O78" s="1" t="s">
         <v>82</v>
@@ -4366,7 +4371,7 @@
       <c r="H79"/>
       <c r="I79"/>
       <c r="J79" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="M79" s="1" t="s">
         <v>88</v>
@@ -4386,7 +4391,7 @@
       <c r="H80"/>
       <c r="I80"/>
       <c r="J80" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="M80" s="1" t="s">
         <v>88</v>
@@ -4406,7 +4411,7 @@
       <c r="H81"/>
       <c r="I81"/>
       <c r="J81" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M81" s="1" t="s">
         <v>88</v>
@@ -4426,7 +4431,7 @@
       <c r="H82"/>
       <c r="I82"/>
       <c r="J82" s="1" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="M82" s="1" t="s">
         <v>88</v>
@@ -4441,38 +4446,22 @@
       <c r="Q82"/>
     </row>
     <row r="83" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="F83"/>
-      <c r="G83"/>
-      <c r="H83"/>
-      <c r="I83"/>
-      <c r="J83" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="M83" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="N83" s="10">
-        <v>0</v>
-      </c>
-      <c r="O83" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="N83" s="10"/>
       <c r="P83" s="10"/>
       <c r="Q83"/>
     </row>
     <row r="84" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="F84"/>
-      <c r="G84"/>
-      <c r="H84"/>
-      <c r="I84"/>
-      <c r="J84" s="1" t="s">
-        <v>76</v>
+      <c r="C84" t="s">
+        <v>679</v>
+      </c>
+      <c r="J84" t="s">
+        <v>60</v>
       </c>
       <c r="M84" s="1" t="s">
         <v>88</v>
       </c>
       <c r="N84" s="10">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="O84" s="1" t="s">
         <v>82</v>
@@ -4481,22 +4470,35 @@
       <c r="Q84"/>
     </row>
     <row r="85" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N85" s="10"/>
+      <c r="C85" t="s">
+        <v>679</v>
+      </c>
+      <c r="J85" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M85" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N85" s="10">
+        <v>4</v>
+      </c>
+      <c r="O85" s="1" t="s">
+        <v>82</v>
+      </c>
       <c r="P85" s="10"/>
-      <c r="Q85"/>
     </row>
     <row r="86" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C86" t="s">
         <v>679</v>
       </c>
       <c r="J86" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="M86" s="1" t="s">
         <v>88</v>
       </c>
       <c r="N86" s="10">
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="O86" s="1" t="s">
         <v>82</v>
@@ -4508,45 +4510,46 @@
       <c r="C87" t="s">
         <v>679</v>
       </c>
-      <c r="J87" s="1" t="s">
-        <v>54</v>
+      <c r="J87" t="s">
+        <v>70</v>
       </c>
       <c r="M87" s="1" t="s">
         <v>88</v>
       </c>
       <c r="N87" s="10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O87" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="P87" s="10"/>
+      <c r="P87" s="10" t="s">
+        <v>680</v>
+      </c>
     </row>
     <row r="88" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C88" t="s">
         <v>679</v>
       </c>
       <c r="J88" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="M88" s="1" t="s">
         <v>88</v>
       </c>
       <c r="N88" s="10">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O88" s="1" t="s">
         <v>82</v>
       </c>
       <c r="P88" s="10"/>
-      <c r="Q88"/>
     </row>
     <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C89" t="s">
         <v>679</v>
       </c>
-      <c r="J89" t="s">
-        <v>70</v>
+      <c r="J89" s="1" t="s">
+        <v>74</v>
       </c>
       <c r="M89" s="1" t="s">
         <v>88</v>
@@ -4557,80 +4560,104 @@
       <c r="O89" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="P89" s="10" t="s">
-        <v>681</v>
-      </c>
+      <c r="P89" s="10"/>
     </row>
     <row r="90" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C90" t="s">
-        <v>679</v>
-      </c>
-      <c r="J90" t="s">
-        <v>71</v>
-      </c>
-      <c r="M90" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="N90" s="10">
-        <v>0</v>
-      </c>
-      <c r="O90" s="1" t="s">
+      <c r="N90" s="10"/>
+      <c r="P90" s="10"/>
+    </row>
+    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A91" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B91" s="3"/>
+      <c r="C91" s="3"/>
+      <c r="D91" s="3"/>
+      <c r="E91" s="4"/>
+      <c r="F91" s="4"/>
+      <c r="G91" s="4"/>
+      <c r="H91" s="4"/>
+      <c r="I91" s="4"/>
+      <c r="J91" s="4"/>
+      <c r="K91" s="4"/>
+      <c r="L91" s="4"/>
+      <c r="M91" s="4"/>
+      <c r="N91" s="4"/>
+      <c r="O91" s="4"/>
+      <c r="P91" s="4"/>
+      <c r="Q91" s="4"/>
+    </row>
+    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A93" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H93" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I93" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M93" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="N93" s="12">
+        <v>28</v>
+      </c>
+      <c r="O93" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="P90" s="10"/>
-    </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C91" t="s">
-        <v>679</v>
-      </c>
-      <c r="J91" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="M91" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="N91" s="10">
-        <v>0</v>
-      </c>
-      <c r="O91" s="1" t="s">
+      <c r="P93" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q93" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A94" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H94" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I94" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M94" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="N94" s="12">
+        <v>100</v>
+      </c>
+      <c r="O94" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="P91" s="10"/>
-    </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N92" s="10"/>
-      <c r="P92" s="10"/>
-    </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A93" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B93" s="3"/>
-      <c r="C93" s="3"/>
-      <c r="D93" s="3"/>
-      <c r="E93" s="4"/>
-      <c r="F93" s="4"/>
-      <c r="G93" s="4"/>
-      <c r="H93" s="4"/>
-      <c r="I93" s="4"/>
-      <c r="J93" s="4"/>
-      <c r="K93" s="4"/>
-      <c r="L93" s="4"/>
-      <c r="M93" s="4"/>
-      <c r="N93" s="4"/>
-      <c r="O93" s="4"/>
-      <c r="P93" s="4"/>
-      <c r="Q93" s="4"/>
+      <c r="P94" s="12"/>
+      <c r="Q94" s="1" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="95" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="H95" s="1" t="s">
         <v>95</v>
@@ -4641,14 +4668,15 @@
       <c r="M95" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="N95" s="12">
-        <v>28</v>
+      <c r="N95" s="14">
+        <f>N94</f>
+        <v>100</v>
       </c>
       <c r="O95" s="1" t="s">
         <v>82</v>
       </c>
       <c r="P95" s="12" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="Q95" s="1" t="s">
         <v>98</v>
@@ -4658,12 +4686,6 @@
       <c r="A96" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B96" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="E96" s="1" t="s">
-        <v>94</v>
-      </c>
       <c r="H96" s="1" t="s">
         <v>95</v>
       </c>
@@ -4674,7 +4696,7 @@
         <v>96</v>
       </c>
       <c r="N96" s="12">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="O96" s="1" t="s">
         <v>82</v>
@@ -4686,13 +4708,7 @@
     </row>
     <row r="97" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B97" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="E97" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H97" s="1" t="s">
         <v>95</v>
@@ -4703,23 +4719,20 @@
       <c r="M97" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="N97" s="14">
-        <f>N96</f>
-        <v>100</v>
+      <c r="N97" s="12">
+        <v>14.5</v>
       </c>
       <c r="O97" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="P97" s="12" t="s">
-        <v>101</v>
-      </c>
+      <c r="P97" s="10"/>
       <c r="Q97" s="1" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="98" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="H98" s="1" t="s">
         <v>95</v>
@@ -4731,19 +4744,22 @@
         <v>96</v>
       </c>
       <c r="N98" s="12">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="O98" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="P98" s="12"/>
+      <c r="P98" s="10"/>
       <c r="Q98" s="1" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="99" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>106</v>
       </c>
       <c r="H99" s="1" t="s">
         <v>95</v>
@@ -4755,20 +4771,26 @@
         <v>96</v>
       </c>
       <c r="N99" s="12">
-        <v>14.5</v>
+        <v>66</v>
       </c>
       <c r="O99" s="1" t="s">
         <v>82</v>
       </c>
       <c r="P99" s="10"/>
       <c r="Q99" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="100" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>104</v>
       </c>
+      <c r="D100" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E100" s="1" t="s">
+        <v>107</v>
+      </c>
       <c r="H100" s="1" t="s">
         <v>95</v>
       </c>
@@ -4779,7 +4801,7 @@
         <v>96</v>
       </c>
       <c r="N100" s="12">
-        <v>100</v>
+        <v>69</v>
       </c>
       <c r="O100" s="1" t="s">
         <v>82</v>
@@ -4790,124 +4812,115 @@
       </c>
     </row>
     <row r="101" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A101" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D101" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="H101" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="I101" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="M101" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="N101" s="12">
-        <v>66</v>
-      </c>
-      <c r="O101" s="1" t="s">
+      <c r="N101" s="10"/>
+      <c r="P101" s="10"/>
+    </row>
+    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A102" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B102" s="3"/>
+      <c r="C102" s="3"/>
+      <c r="D102" s="3"/>
+      <c r="E102" s="4"/>
+      <c r="F102" s="4"/>
+      <c r="G102" s="4"/>
+      <c r="H102" s="4"/>
+      <c r="I102" s="4"/>
+      <c r="J102" s="4"/>
+      <c r="K102" s="4"/>
+      <c r="L102" s="4"/>
+      <c r="M102" s="4"/>
+      <c r="N102" s="4"/>
+      <c r="O102" s="4"/>
+      <c r="P102" s="4"/>
+      <c r="Q102" s="4"/>
+    </row>
+    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M103" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="N103" s="6">
+        <v>0</v>
+      </c>
+      <c r="O103" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="P101" s="10"/>
-      <c r="Q101" s="1" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A102" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D102" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="E102" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="H102" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="I102" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="M102" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="N102" s="12">
-        <v>69</v>
-      </c>
-      <c r="O102" s="1" t="s">
+      <c r="P103" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M104" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="N104" s="6">
+        <v>0</v>
+      </c>
+      <c r="O104" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="P102" s="10"/>
-      <c r="Q102" s="1" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N103" s="10"/>
-      <c r="P103" s="10"/>
-    </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A104" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="B104" s="3"/>
-      <c r="C104" s="3"/>
-      <c r="D104" s="3"/>
-      <c r="E104" s="4"/>
-      <c r="F104" s="4"/>
-      <c r="G104" s="4"/>
-      <c r="H104" s="4"/>
-      <c r="I104" s="4"/>
-      <c r="J104" s="4"/>
-      <c r="K104" s="4"/>
-      <c r="L104" s="4"/>
-      <c r="M104" s="4"/>
-      <c r="N104" s="4"/>
-      <c r="O104" s="4"/>
-      <c r="P104" s="4"/>
-      <c r="Q104" s="4"/>
+      <c r="P104" s="6" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="105" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M105" s="6" t="s">
+      <c r="A105" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G105" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="M105" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="N105" s="6">
-        <v>0</v>
-      </c>
-      <c r="O105" s="6" t="s">
+      <c r="N105" s="12">
+        <f>(0.8*20+0.2*2)</f>
+        <v>16.399999999999999</v>
+      </c>
+      <c r="O105" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="P105" s="6" t="s">
-        <v>25</v>
+      <c r="P105" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q105" s="1" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="106" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M106" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="N106" s="6">
-        <v>0</v>
-      </c>
-      <c r="O106" s="6" t="s">
+      <c r="A106" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G106" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="M106" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="N106" s="12">
+        <f>(0.6*20+0.4*2)</f>
+        <v>12.8</v>
+      </c>
+      <c r="O106" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="P106" s="6" t="s">
-        <v>25</v>
+      <c r="P106" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q106" s="1" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="107" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B107" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E107" s="1" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="G107" s="1" t="s">
         <v>111</v>
@@ -4916,14 +4929,13 @@
         <v>109</v>
       </c>
       <c r="N107" s="12">
-        <f>(0.8*20+0.2*2)</f>
-        <v>16.399999999999999</v>
+        <v>2</v>
       </c>
       <c r="O107" s="12" t="s">
         <v>82</v>
       </c>
       <c r="P107" s="12" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="Q107" s="1" t="s">
         <v>103</v>
@@ -4931,7 +4943,7 @@
     </row>
     <row r="108" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="G108" s="1" t="s">
         <v>111</v>
@@ -4940,81 +4952,83 @@
         <v>109</v>
       </c>
       <c r="N108" s="12">
-        <f>(0.6*20+0.4*2)</f>
-        <v>12.8</v>
+        <v>2</v>
       </c>
       <c r="O108" s="12" t="s">
         <v>82</v>
       </c>
       <c r="P108" s="12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="Q108" s="1" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="109" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A109" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="G109" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="M109" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="N109" s="12">
-        <v>2</v>
-      </c>
-      <c r="O109" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="P109" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="Q109" s="1" t="s">
-        <v>103</v>
-      </c>
+      <c r="M109" s="12"/>
+      <c r="N109" s="12"/>
+      <c r="O109" s="12"/>
+      <c r="P109" s="12"/>
     </row>
     <row r="110" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
-        <v>102</v>
+        <v>92</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E110" s="1" t="s">
+        <v>94</v>
       </c>
       <c r="G110" s="1" t="s">
         <v>111</v>
       </c>
       <c r="M110" s="12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N110" s="12">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O110" s="12" t="s">
         <v>82</v>
       </c>
       <c r="P110" s="12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q110" s="1" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="111" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M111" s="12"/>
-      <c r="N111" s="12"/>
-      <c r="O111" s="12"/>
-      <c r="P111" s="12"/>
+      <c r="A111" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="G111" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="M111" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="N111" s="12">
+        <v>5</v>
+      </c>
+      <c r="O111" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="P111" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q111" s="1" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="112" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B112" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E112" s="1" t="s">
-        <v>94</v>
-      </c>
       <c r="G112" s="1" t="s">
         <v>111</v>
       </c>
@@ -5022,13 +5036,14 @@
         <v>110</v>
       </c>
       <c r="N112" s="12">
-        <v>5</v>
+        <f>0.9*5+0.1*15</f>
+        <v>6</v>
       </c>
       <c r="O112" s="12" t="s">
         <v>82</v>
       </c>
       <c r="P112" s="12" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="Q112" s="1" t="s">
         <v>103</v>
@@ -5036,10 +5051,7 @@
     </row>
     <row r="113" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="E113" s="1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="G113" s="1" t="s">
         <v>111</v>
@@ -5048,21 +5060,19 @@
         <v>110</v>
       </c>
       <c r="N113" s="12">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="O113" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="P113" s="12" t="s">
-        <v>115</v>
-      </c>
+      <c r="P113" s="12"/>
       <c r="Q113" s="1" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="114" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="G114" s="1" t="s">
         <v>111</v>
@@ -5071,52 +5081,34 @@
         <v>110</v>
       </c>
       <c r="N114" s="12">
-        <f>0.9*5+0.1*15</f>
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="O114" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="P114" s="12" t="s">
-        <v>117</v>
-      </c>
+      <c r="P114" s="12"/>
       <c r="Q114" s="1" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="115" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A115" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="G115" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="M115" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="N115" s="12">
-        <v>15</v>
-      </c>
-      <c r="O115" s="12" t="s">
-        <v>82</v>
-      </c>
+      <c r="M115" s="12"/>
+      <c r="N115" s="12"/>
+      <c r="O115" s="12"/>
       <c r="P115" s="12"/>
-      <c r="Q115" s="1" t="s">
-        <v>103</v>
-      </c>
     </row>
     <row r="116" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A116" s="1" t="s">
-        <v>102</v>
-      </c>
+      <c r="A116" s="15"/>
+      <c r="B116" s="15"/>
+      <c r="E116" s="15"/>
       <c r="G116" s="1" t="s">
-        <v>111</v>
+        <v>30</v>
       </c>
       <c r="M116" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N116" s="12">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="O116" s="12" t="s">
         <v>82</v>
@@ -5127,30 +5119,73 @@
       </c>
     </row>
     <row r="117" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M117" s="12"/>
-      <c r="N117" s="12"/>
-      <c r="O117" s="12"/>
-      <c r="P117" s="12"/>
+      <c r="A117" s="15" t="str">
+        <f>A110</f>
+        <v>cattle</v>
+      </c>
+      <c r="B117" s="15" t="str">
+        <f>B110</f>
+        <v>dairy</v>
+      </c>
+      <c r="E117" s="15" t="str">
+        <f>E110</f>
+        <v>cows</v>
+      </c>
+      <c r="G117" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M117" s="15" t="str">
+        <f t="shared" ref="M117:Q119" si="0">M110</f>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N117" s="15">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="O117" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v>%</v>
+      </c>
+      <c r="P117" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="Q117" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
     </row>
     <row r="118" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A118" s="15"/>
-      <c r="B118" s="15"/>
-      <c r="E118" s="15"/>
+      <c r="A118" s="15" t="str">
+        <f>A111</f>
+        <v>cattle</v>
+      </c>
+      <c r="E118" s="15" t="str">
+        <f>E111</f>
+        <v>bulls</v>
+      </c>
       <c r="G118" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M118" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="N118" s="12">
+      <c r="M118" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N118" s="15">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="O118" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="P118" s="12"/>
-      <c r="Q118" s="1" t="s">
-        <v>103</v>
+      <c r="O118" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v>%</v>
+      </c>
+      <c r="P118" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="Q118" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="119" spans="1:17" x14ac:dyDescent="0.25">
@@ -5158,24 +5193,16 @@
         <f>A112</f>
         <v>cattle</v>
       </c>
-      <c r="B119" s="15" t="str">
-        <f>B112</f>
-        <v>dairy</v>
-      </c>
-      <c r="E119" s="15" t="str">
-        <f>E112</f>
-        <v>cows</v>
-      </c>
       <c r="G119" s="1" t="s">
         <v>30</v>
       </c>
       <c r="M119" s="15" t="str">
-        <f t="shared" ref="M119:Q121" si="0">M112</f>
+        <f t="shared" si="0"/>
         <v>feeding_losses</v>
       </c>
       <c r="N119" s="15">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O119" s="15" t="str">
         <f t="shared" si="0"/>
@@ -5183,7 +5210,7 @@
       </c>
       <c r="P119" s="15" t="str">
         <f t="shared" si="0"/>
-        <v>No feeding on pasture</v>
+        <v>10% feeding on pasture</v>
       </c>
       <c r="Q119" s="15" t="str">
         <f t="shared" si="0"/>
@@ -5193,141 +5220,149 @@
     <row r="120" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A120" s="15" t="str">
         <f>A113</f>
-        <v>cattle</v>
-      </c>
-      <c r="E120" s="15" t="str">
-        <f>E113</f>
-        <v>bulls</v>
+        <v>sheep</v>
       </c>
       <c r="G120" s="1" t="s">
         <v>30</v>
       </c>
       <c r="M120" s="15" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="M120:O121" si="1">M113</f>
         <v>feeding_losses</v>
       </c>
       <c r="N120" s="15">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <f t="shared" si="1"/>
+        <v>15</v>
       </c>
       <c r="O120" s="15" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>%</v>
       </c>
-      <c r="P120" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v>No feeding on pasture</v>
-      </c>
+      <c r="P120" s="15"/>
       <c r="Q120" s="15" t="str">
-        <f t="shared" si="0"/>
+        <f>Q113</f>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="121" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A121" s="15" t="str">
         <f>A114</f>
-        <v>cattle</v>
+        <v>horses</v>
       </c>
       <c r="G121" s="1" t="s">
         <v>30</v>
       </c>
       <c r="M121" s="15" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>feeding_losses</v>
       </c>
       <c r="N121" s="15">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="O121" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v>%</v>
-      </c>
-      <c r="P121" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v>10% feeding on pasture</v>
-      </c>
-      <c r="Q121" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A122" s="15" t="str">
-        <f>A115</f>
-        <v>sheep</v>
-      </c>
-      <c r="G122" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M122" s="15" t="str">
-        <f t="shared" ref="M122:O123" si="1">M115</f>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N122" s="15">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="O122" s="15" t="str">
+      <c r="O121" s="15" t="str">
         <f t="shared" si="1"/>
         <v>%</v>
       </c>
+      <c r="P121" s="15"/>
+      <c r="Q121" s="15" t="str">
+        <f>Q114</f>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A122" s="15"/>
+      <c r="M122" s="15"/>
+      <c r="N122" s="15"/>
+      <c r="O122" s="15"/>
       <c r="P122" s="15"/>
-      <c r="Q122" s="15" t="str">
-        <f>Q115</f>
+      <c r="Q122" s="15"/>
+    </row>
+    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="G123" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="M123" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="N123" s="12">
+        <v>5</v>
+      </c>
+      <c r="O123" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="P123" s="12"/>
+      <c r="Q123" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="124" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A124" s="15" t="str">
+        <f>A110</f>
+        <v>cattle</v>
+      </c>
+      <c r="B124" s="15" t="str">
+        <f>B110</f>
+        <v>dairy</v>
+      </c>
+      <c r="E124" s="15" t="str">
+        <f>E110</f>
+        <v>cows</v>
+      </c>
+      <c r="G124" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="M124" s="15" t="str">
+        <f t="shared" ref="M124:Q126" si="2">M110</f>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N124" s="15">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="O124" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v>%</v>
+      </c>
+      <c r="P124" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="Q124" s="15" t="str">
+        <f t="shared" si="2"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A123" s="15" t="str">
-        <f>A116</f>
-        <v>horses</v>
-      </c>
-      <c r="G123" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M123" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N123" s="15">
-        <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-      <c r="O123" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v>%</v>
-      </c>
-      <c r="P123" s="15"/>
-      <c r="Q123" s="15" t="str">
-        <f>Q116</f>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A124" s="15"/>
-      <c r="M124" s="15"/>
-      <c r="N124" s="15"/>
-      <c r="O124" s="15"/>
-      <c r="P124" s="15"/>
-      <c r="Q124" s="15"/>
-    </row>
     <row r="125" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A125" s="15" t="str">
+        <f>A111</f>
+        <v>cattle</v>
+      </c>
+      <c r="E125" s="15" t="str">
+        <f>E111</f>
+        <v>bulls</v>
+      </c>
       <c r="G125" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="M125" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="N125" s="12">
+      <c r="M125" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N125" s="15">
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="O125" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="P125" s="12"/>
-      <c r="Q125" s="1" t="s">
-        <v>103</v>
+      <c r="O125" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v>%</v>
+      </c>
+      <c r="P125" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="Q125" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="126" spans="1:17" x14ac:dyDescent="0.25">
@@ -5335,24 +5370,16 @@
         <f>A112</f>
         <v>cattle</v>
       </c>
-      <c r="B126" s="15" t="str">
-        <f>B112</f>
-        <v>dairy</v>
-      </c>
-      <c r="E126" s="15" t="str">
-        <f>E112</f>
-        <v>cows</v>
-      </c>
       <c r="G126" s="1" t="s">
         <v>118</v>
       </c>
       <c r="M126" s="15" t="str">
-        <f t="shared" ref="M126:Q128" si="2">M112</f>
+        <f t="shared" si="2"/>
         <v>feeding_losses</v>
       </c>
       <c r="N126" s="15">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O126" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5360,7 +5387,7 @@
       </c>
       <c r="P126" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>No feeding on pasture</v>
+        <v>10% feeding on pasture</v>
       </c>
       <c r="Q126" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5370,268 +5397,242 @@
     <row r="127" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A127" s="15" t="str">
         <f>A113</f>
-        <v>cattle</v>
-      </c>
-      <c r="E127" s="15" t="str">
-        <f>E113</f>
-        <v>bulls</v>
+        <v>sheep</v>
       </c>
       <c r="G127" s="1" t="s">
         <v>118</v>
       </c>
       <c r="M127" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="M127:O128" si="3">M113</f>
         <v>feeding_losses</v>
       </c>
       <c r="N127" s="15">
-        <f t="shared" si="2"/>
-        <v>5</v>
+        <f t="shared" si="3"/>
+        <v>15</v>
       </c>
       <c r="O127" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>%</v>
       </c>
-      <c r="P127" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>No feeding on pasture</v>
-      </c>
+      <c r="P127" s="12"/>
       <c r="Q127" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>Q113</f>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="128" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A128" s="15" t="str">
         <f>A114</f>
-        <v>cattle</v>
+        <v>horses</v>
       </c>
       <c r="G128" s="1" t="s">
         <v>118</v>
       </c>
       <c r="M128" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>feeding_losses</v>
       </c>
       <c r="N128" s="15">
-        <f t="shared" si="2"/>
-        <v>6</v>
-      </c>
-      <c r="O128" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>%</v>
-      </c>
-      <c r="P128" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>10% feeding on pasture</v>
-      </c>
-      <c r="Q128" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
-    </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A129" s="15" t="str">
-        <f>A115</f>
-        <v>sheep</v>
-      </c>
-      <c r="G129" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="M129" s="15" t="str">
-        <f t="shared" ref="M129:O130" si="3">M115</f>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N129" s="15">
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="O129" s="15" t="str">
+      <c r="O128" s="15" t="str">
         <f t="shared" si="3"/>
         <v>%</v>
       </c>
+      <c r="P128" s="12"/>
+      <c r="Q128" s="15" t="str">
+        <f>Q114</f>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N129" s="10"/>
       <c r="P129" s="12"/>
-      <c r="Q129" s="15" t="str">
-        <f>Q115</f>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
     </row>
     <row r="130" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A130" s="15" t="str">
-        <f>A116</f>
-        <v>horses</v>
-      </c>
+      <c r="A130" s="10"/>
       <c r="G130" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="M130" s="15" t="str">
-        <f t="shared" si="3"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N130" s="15">
-        <f t="shared" si="3"/>
-        <v>15</v>
-      </c>
-      <c r="O130" s="15" t="str">
-        <f t="shared" si="3"/>
-        <v>%</v>
-      </c>
-      <c r="P130" s="12"/>
-      <c r="Q130" s="15" t="str">
-        <f>Q116</f>
-        <v>Cederberg &amp; Henriksson (2020)</v>
+        <v>119</v>
+      </c>
+      <c r="M130" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="N130" s="12"/>
+      <c r="P130" s="10" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="131" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N131" s="10"/>
-      <c r="P131" s="12"/>
+      <c r="A131" s="10"/>
+      <c r="G131" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="M131" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="N131" s="12">
+        <v>2</v>
+      </c>
+      <c r="O131" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="P131" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q131" s="1" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="132" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A132" s="10"/>
-      <c r="G132" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="M132" s="12" t="s">
-        <v>109</v>
-      </c>
+      <c r="M132" s="12"/>
       <c r="N132" s="12"/>
-      <c r="P132" s="10" t="s">
-        <v>120</v>
-      </c>
+      <c r="O132" s="12"/>
+      <c r="P132" s="10"/>
     </row>
     <row r="133" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A133" s="10"/>
       <c r="G133" s="1" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="M133" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="N133" s="12">
-        <v>2</v>
-      </c>
-      <c r="O133" s="12" t="s">
-        <v>82</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="N133" s="12"/>
       <c r="P133" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="Q133" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="134" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A134" s="10"/>
-      <c r="M134" s="12"/>
-      <c r="N134" s="12"/>
-      <c r="O134" s="12"/>
-      <c r="P134" s="10"/>
+      <c r="G134" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="M134" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="N134" s="12">
+        <v>3</v>
+      </c>
+      <c r="O134" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="P134" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q134" s="1" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="135" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A135" s="10"/>
-      <c r="G135" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="M135" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="N135" s="12"/>
-      <c r="P135" s="10" t="s">
-        <v>120</v>
-      </c>
+      <c r="N135" s="10"/>
+      <c r="P135" s="12"/>
     </row>
     <row r="136" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A136" s="10"/>
-      <c r="G136" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="M136" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="N136" s="12">
-        <v>3</v>
-      </c>
-      <c r="O136" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="P136" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="Q136" s="1" t="s">
-        <v>122</v>
-      </c>
+      <c r="A136" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B136" s="3"/>
+      <c r="C136" s="3"/>
+      <c r="D136" s="3"/>
+      <c r="E136" s="4"/>
+      <c r="F136" s="4"/>
+      <c r="G136" s="4"/>
+      <c r="H136" s="4"/>
+      <c r="I136" s="4"/>
+      <c r="J136" s="4"/>
+      <c r="K136" s="4"/>
+      <c r="L136" s="4"/>
+      <c r="M136" s="4"/>
+      <c r="N136" s="4"/>
+      <c r="O136" s="4"/>
+      <c r="P136" s="4"/>
+      <c r="Q136" s="4"/>
     </row>
     <row r="137" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N137" s="10"/>
-      <c r="P137" s="12"/>
+      <c r="A137" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="N137" s="12"/>
+      <c r="P137" s="12" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="138" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A138" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="B138" s="3"/>
-      <c r="C138" s="3"/>
-      <c r="D138" s="3"/>
-      <c r="E138" s="4"/>
-      <c r="F138" s="4"/>
-      <c r="G138" s="4"/>
-      <c r="H138" s="4"/>
-      <c r="I138" s="4"/>
-      <c r="J138" s="4"/>
-      <c r="K138" s="4"/>
-      <c r="L138" s="4"/>
-      <c r="M138" s="4"/>
-      <c r="N138" s="4"/>
-      <c r="O138" s="4"/>
-      <c r="P138" s="4"/>
-      <c r="Q138" s="4"/>
+      <c r="A138" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="B138" s="10"/>
+      <c r="C138" s="10"/>
+      <c r="D138" s="10"/>
+      <c r="E138" s="10"/>
+      <c r="F138" s="10"/>
+      <c r="G138" s="10"/>
+      <c r="H138" s="10"/>
+      <c r="I138" s="10"/>
+      <c r="J138" s="10"/>
+      <c r="K138" s="10"/>
+      <c r="L138" s="10"/>
+      <c r="M138" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="N138" s="12">
+        <v>6.7</v>
+      </c>
+      <c r="O138" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="P138" s="10"/>
+      <c r="Q138" s="1" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="139" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="N139" s="12"/>
-      <c r="P139" s="12" t="s">
-        <v>125</v>
+        <v>102</v>
+      </c>
+      <c r="M139" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="N139" s="12">
+        <v>18</v>
+      </c>
+      <c r="O139" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="P139" s="10"/>
+      <c r="Q139" s="1" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="140" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A140" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="B140" s="10"/>
-      <c r="C140" s="10"/>
-      <c r="D140" s="10"/>
-      <c r="E140" s="10"/>
-      <c r="F140" s="10"/>
-      <c r="G140" s="10"/>
-      <c r="H140" s="10"/>
-      <c r="I140" s="10"/>
-      <c r="J140" s="10"/>
-      <c r="K140" s="10"/>
-      <c r="L140" s="10"/>
-      <c r="M140" s="12" t="s">
-        <v>126</v>
+      <c r="A140" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="M140" s="1" t="s">
+        <v>129</v>
       </c>
       <c r="N140" s="12">
-        <v>6.7</v>
-      </c>
-      <c r="O140" s="12" t="s">
-        <v>127</v>
+        <v>1.5</v>
+      </c>
+      <c r="O140" s="1" t="s">
+        <v>130</v>
       </c>
       <c r="P140" s="10"/>
       <c r="Q140" s="1" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="141" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="M141" s="1" t="s">
         <v>129</v>
       </c>
       <c r="N141" s="12">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="O141" s="1" t="s">
         <v>130</v>
@@ -5642,46 +5643,50 @@
       </c>
     </row>
     <row r="142" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A142" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="M142" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="N142" s="12">
-        <v>1.5</v>
-      </c>
-      <c r="O142" s="1" t="s">
-        <v>130</v>
-      </c>
+      <c r="N142" s="12"/>
       <c r="P142" s="10"/>
-      <c r="Q142" s="1" t="s">
-        <v>131</v>
-      </c>
     </row>
     <row r="143" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A143" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="M143" s="1" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="N143" s="12">
-        <v>0</v>
-      </c>
-      <c r="O143" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="P143" s="10"/>
-      <c r="Q143" s="1" t="s">
-        <v>131</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="O143" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="P143" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q143" s="12"/>
     </row>
     <row r="144" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N144" s="12"/>
-      <c r="P144" s="10"/>
+      <c r="A144" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M144" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="N144" s="12">
+        <v>1</v>
+      </c>
+      <c r="O144" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="P144" s="12"/>
+      <c r="Q144" s="12"/>
     </row>
     <row r="145" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A145" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B145" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E145" s="1" t="s">
+        <v>94</v>
+      </c>
       <c r="M145" s="1" t="s">
         <v>132</v>
       </c>
@@ -5691,15 +5696,19 @@
       <c r="O145" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="P145" s="12" t="s">
-        <v>134</v>
-      </c>
+      <c r="P145" s="12"/>
       <c r="Q145" s="12"/>
     </row>
     <row r="146" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>92</v>
       </c>
+      <c r="B146" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E146" s="1" t="s">
+        <v>116</v>
+      </c>
       <c r="M146" s="1" t="s">
         <v>132</v>
       </c>
@@ -5717,10 +5726,10 @@
         <v>92</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E147" s="1" t="s">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="M147" s="1" t="s">
         <v>132</v>
@@ -5735,75 +5744,77 @@
       <c r="Q147" s="12"/>
     </row>
     <row r="148" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A148" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B148" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E148" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="M148" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="N148" s="12">
-        <v>1</v>
-      </c>
-      <c r="O148" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="P148" s="12"/>
-      <c r="Q148" s="12"/>
+      <c r="N148" s="10"/>
+      <c r="P148" s="10"/>
     </row>
     <row r="149" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A149" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B149" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="E149" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="M149" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="N149" s="12">
-        <v>1</v>
-      </c>
-      <c r="O149" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="P149" s="12"/>
-      <c r="Q149" s="12"/>
+      <c r="A149" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="B149" s="16"/>
+      <c r="C149" s="16"/>
+      <c r="D149" s="16"/>
+      <c r="E149" s="17"/>
+      <c r="F149" s="17"/>
+      <c r="G149" s="17"/>
+      <c r="H149" s="17"/>
+      <c r="I149" s="17"/>
+      <c r="J149" s="17"/>
+      <c r="K149" s="17"/>
+      <c r="L149" s="17"/>
+      <c r="M149" s="17"/>
+      <c r="N149" s="17"/>
+      <c r="O149" s="17"/>
+      <c r="P149" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="Q149" s="17"/>
     </row>
     <row r="150" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N150" s="10"/>
-      <c r="P150" s="10"/>
+      <c r="A150" s="18"/>
+      <c r="B150" s="18"/>
+      <c r="C150" s="18"/>
+      <c r="D150" s="18"/>
+      <c r="E150" s="18"/>
+      <c r="F150" s="18"/>
+      <c r="G150" s="18"/>
+      <c r="H150" s="18"/>
+      <c r="I150" s="18"/>
+      <c r="J150" s="18"/>
+      <c r="K150" s="18"/>
+      <c r="L150" s="19" t="s">
+        <v>137</v>
+      </c>
+      <c r="M150" s="18"/>
+      <c r="N150" s="18"/>
+      <c r="O150" s="18"/>
+      <c r="P150" s="18"/>
+      <c r="Q150" s="18"/>
     </row>
     <row r="151" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A151" s="16" t="s">
-        <v>135</v>
-      </c>
-      <c r="B151" s="16"/>
-      <c r="C151" s="16"/>
-      <c r="D151" s="16"/>
-      <c r="E151" s="17"/>
-      <c r="F151" s="17"/>
-      <c r="G151" s="17"/>
-      <c r="H151" s="17"/>
-      <c r="I151" s="17"/>
-      <c r="J151" s="17"/>
-      <c r="K151" s="17"/>
-      <c r="L151" s="17"/>
-      <c r="M151" s="17"/>
-      <c r="N151" s="17"/>
-      <c r="O151" s="17"/>
-      <c r="P151" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="Q151" s="17"/>
+      <c r="A151" s="18"/>
+      <c r="B151" s="18"/>
+      <c r="C151" s="18"/>
+      <c r="D151" s="18"/>
+      <c r="E151" s="18"/>
+      <c r="F151" s="18"/>
+      <c r="G151" s="18"/>
+      <c r="H151" s="18"/>
+      <c r="I151" s="18"/>
+      <c r="J151" s="18"/>
+      <c r="K151" s="18"/>
+      <c r="L151" s="18"/>
+      <c r="M151" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="N151" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="O151" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="P151" s="21"/>
+      <c r="Q151" s="18"/>
     </row>
     <row r="152" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A152" s="18"/>
@@ -5817,13 +5828,17 @@
       <c r="I152" s="18"/>
       <c r="J152" s="18"/>
       <c r="K152" s="18"/>
-      <c r="L152" s="19" t="s">
-        <v>137</v>
-      </c>
-      <c r="M152" s="18"/>
-      <c r="N152" s="18"/>
-      <c r="O152" s="18"/>
-      <c r="P152" s="18"/>
+      <c r="L152" s="18"/>
+      <c r="M152" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="N152" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="O152" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="P152" s="21"/>
       <c r="Q152" s="18"/>
     </row>
     <row r="153" spans="1:17" x14ac:dyDescent="0.25">
@@ -5839,16 +5854,14 @@
       <c r="J153" s="18"/>
       <c r="K153" s="18"/>
       <c r="L153" s="18"/>
-      <c r="M153" s="18" t="s">
-        <v>138</v>
+      <c r="M153" s="22" t="s">
+        <v>143</v>
       </c>
       <c r="N153" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="O153" s="18" t="s">
-        <v>140</v>
-      </c>
-      <c r="P153" s="21"/>
+      <c r="O153" s="18"/>
+      <c r="P153" s="18"/>
       <c r="Q153" s="18"/>
     </row>
     <row r="154" spans="1:17" x14ac:dyDescent="0.25">
@@ -5864,16 +5877,14 @@
       <c r="J154" s="18"/>
       <c r="K154" s="18"/>
       <c r="L154" s="18"/>
-      <c r="M154" s="18" t="s">
-        <v>141</v>
+      <c r="M154" s="22" t="s">
+        <v>144</v>
       </c>
       <c r="N154" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="O154" s="18" t="s">
-        <v>142</v>
-      </c>
-      <c r="P154" s="21"/>
+      <c r="O154" s="18"/>
+      <c r="P154" s="18"/>
       <c r="Q154" s="18"/>
     </row>
     <row r="155" spans="1:17" x14ac:dyDescent="0.25">
@@ -5890,7 +5901,7 @@
       <c r="K155" s="18"/>
       <c r="L155" s="18"/>
       <c r="M155" s="22" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="N155" s="20" t="s">
         <v>139</v>
@@ -5913,13 +5924,13 @@
       <c r="K156" s="18"/>
       <c r="L156" s="18"/>
       <c r="M156" s="22" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="N156" s="20" t="s">
         <v>139</v>
       </c>
       <c r="O156" s="18"/>
-      <c r="P156" s="18"/>
+      <c r="P156" s="21"/>
       <c r="Q156" s="18"/>
     </row>
     <row r="157" spans="1:17" x14ac:dyDescent="0.25">
@@ -5934,13 +5945,11 @@
       <c r="I157" s="18"/>
       <c r="J157" s="18"/>
       <c r="K157" s="18"/>
-      <c r="L157" s="18"/>
-      <c r="M157" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="N157" s="20" t="s">
-        <v>139</v>
-      </c>
+      <c r="L157" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="M157" s="18"/>
+      <c r="N157" s="18"/>
       <c r="O157" s="18"/>
       <c r="P157" s="18"/>
       <c r="Q157" s="18"/>
@@ -5958,14 +5967,18 @@
       <c r="J158" s="18"/>
       <c r="K158" s="18"/>
       <c r="L158" s="18"/>
-      <c r="M158" s="22" t="s">
-        <v>146</v>
+      <c r="M158" s="18" t="s">
+        <v>148</v>
       </c>
       <c r="N158" s="20" t="s">
-        <v>139</v>
-      </c>
-      <c r="O158" s="18"/>
-      <c r="P158" s="21"/>
+        <v>149</v>
+      </c>
+      <c r="O158" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="P158" s="20" t="s">
+        <v>151</v>
+      </c>
       <c r="Q158" s="18"/>
     </row>
     <row r="159" spans="1:17" x14ac:dyDescent="0.25">
@@ -5980,13 +5993,17 @@
       <c r="I159" s="18"/>
       <c r="J159" s="18"/>
       <c r="K159" s="18"/>
-      <c r="L159" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="M159" s="18"/>
-      <c r="N159" s="18"/>
-      <c r="O159" s="18"/>
-      <c r="P159" s="18"/>
+      <c r="L159" s="18"/>
+      <c r="M159" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="N159" s="20" t="s">
+        <v>149</v>
+      </c>
+      <c r="O159" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="P159" s="21"/>
       <c r="Q159" s="18"/>
     </row>
     <row r="160" spans="1:17" x14ac:dyDescent="0.25">
@@ -6003,16 +6020,16 @@
       <c r="K160" s="18"/>
       <c r="L160" s="18"/>
       <c r="M160" s="18" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="N160" s="20" t="s">
         <v>149</v>
       </c>
       <c r="O160" s="18" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="P160" s="20" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="Q160" s="18"/>
     </row>
@@ -6028,17 +6045,13 @@
       <c r="I161" s="18"/>
       <c r="J161" s="18"/>
       <c r="K161" s="18"/>
-      <c r="L161" s="18"/>
-      <c r="M161" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="N161" s="20" t="s">
-        <v>149</v>
-      </c>
-      <c r="O161" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="P161" s="21"/>
+      <c r="L161" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="M161" s="18"/>
+      <c r="N161" s="18"/>
+      <c r="O161" s="18"/>
+      <c r="P161" s="18"/>
       <c r="Q161" s="18"/>
     </row>
     <row r="162" spans="1:17" x14ac:dyDescent="0.25">
@@ -6055,16 +6068,16 @@
       <c r="K162" s="18"/>
       <c r="L162" s="18"/>
       <c r="M162" s="18" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="N162" s="20" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="O162" s="18" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="P162" s="20" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="Q162" s="18"/>
     </row>
@@ -6080,13 +6093,17 @@
       <c r="I163" s="18"/>
       <c r="J163" s="18"/>
       <c r="K163" s="18"/>
-      <c r="L163" s="19" t="s">
-        <v>157</v>
-      </c>
-      <c r="M163" s="18"/>
-      <c r="N163" s="18"/>
-      <c r="O163" s="18"/>
-      <c r="P163" s="18"/>
+      <c r="L163" s="18"/>
+      <c r="M163" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="N163" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="O163" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="P163" s="21"/>
       <c r="Q163" s="18"/>
     </row>
     <row r="164" spans="1:17" x14ac:dyDescent="0.25">
@@ -6101,19 +6118,13 @@
       <c r="I164" s="18"/>
       <c r="J164" s="18"/>
       <c r="K164" s="18"/>
-      <c r="L164" s="18"/>
-      <c r="M164" s="18" t="s">
-        <v>148</v>
-      </c>
-      <c r="N164" s="20" t="s">
-        <v>158</v>
-      </c>
-      <c r="O164" s="18" t="s">
-        <v>150</v>
-      </c>
-      <c r="P164" s="20" t="s">
-        <v>151</v>
-      </c>
+      <c r="L164" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="M164" s="18"/>
+      <c r="N164" s="18"/>
+      <c r="O164" s="18"/>
+      <c r="P164" s="18"/>
       <c r="Q164" s="18"/>
     </row>
     <row r="165" spans="1:17" x14ac:dyDescent="0.25">
@@ -6130,15 +6141,17 @@
       <c r="K165" s="18"/>
       <c r="L165" s="18"/>
       <c r="M165" s="18" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="N165" s="20" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="O165" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="P165" s="21"/>
+        <v>150</v>
+      </c>
+      <c r="P165" s="20" t="s">
+        <v>151</v>
+      </c>
       <c r="Q165" s="18"/>
     </row>
     <row r="166" spans="1:17" x14ac:dyDescent="0.25">
@@ -6153,13 +6166,17 @@
       <c r="I166" s="18"/>
       <c r="J166" s="18"/>
       <c r="K166" s="18"/>
-      <c r="L166" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="M166" s="18"/>
-      <c r="N166" s="18"/>
-      <c r="O166" s="18"/>
-      <c r="P166" s="18"/>
+      <c r="L166" s="18"/>
+      <c r="M166" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="N166" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="O166" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="P166" s="21"/>
       <c r="Q166" s="18"/>
     </row>
     <row r="167" spans="1:17" x14ac:dyDescent="0.25">
@@ -6174,19 +6191,13 @@
       <c r="I167" s="18"/>
       <c r="J167" s="18"/>
       <c r="K167" s="18"/>
-      <c r="L167" s="18"/>
-      <c r="M167" s="18" t="s">
-        <v>148</v>
-      </c>
-      <c r="N167" s="20" t="s">
-        <v>160</v>
-      </c>
-      <c r="O167" s="18" t="s">
-        <v>150</v>
-      </c>
-      <c r="P167" s="20" t="s">
-        <v>151</v>
-      </c>
+      <c r="L167" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="M167" s="18"/>
+      <c r="N167" s="18"/>
+      <c r="O167" s="18"/>
+      <c r="P167" s="18"/>
       <c r="Q167" s="18"/>
     </row>
     <row r="168" spans="1:17" x14ac:dyDescent="0.25">
@@ -6203,15 +6214,17 @@
       <c r="K168" s="18"/>
       <c r="L168" s="18"/>
       <c r="M168" s="18" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="N168" s="20" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="O168" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="P168" s="21"/>
+        <v>163</v>
+      </c>
+      <c r="P168" s="20" t="s">
+        <v>151</v>
+      </c>
       <c r="Q168" s="18"/>
     </row>
     <row r="169" spans="1:17" x14ac:dyDescent="0.25">
@@ -6226,13 +6239,17 @@
       <c r="I169" s="18"/>
       <c r="J169" s="18"/>
       <c r="K169" s="18"/>
-      <c r="L169" s="19" t="s">
-        <v>161</v>
-      </c>
-      <c r="M169" s="18"/>
-      <c r="N169" s="18"/>
-      <c r="O169" s="18"/>
-      <c r="P169" s="18"/>
+      <c r="L169" s="18"/>
+      <c r="M169" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="N169" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="O169" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="P169" s="21"/>
       <c r="Q169" s="18"/>
     </row>
     <row r="170" spans="1:17" x14ac:dyDescent="0.25">
@@ -6247,19 +6264,13 @@
       <c r="I170" s="18"/>
       <c r="J170" s="18"/>
       <c r="K170" s="18"/>
-      <c r="L170" s="18"/>
-      <c r="M170" s="18" t="s">
-        <v>148</v>
-      </c>
-      <c r="N170" s="20" t="s">
-        <v>162</v>
-      </c>
-      <c r="O170" s="18" t="s">
-        <v>163</v>
-      </c>
-      <c r="P170" s="20" t="s">
-        <v>151</v>
-      </c>
+      <c r="L170" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="M170" s="18"/>
+      <c r="N170" s="18"/>
+      <c r="O170" s="18"/>
+      <c r="P170" s="18"/>
       <c r="Q170" s="18"/>
     </row>
     <row r="171" spans="1:17" x14ac:dyDescent="0.25">
@@ -6276,80 +6287,34 @@
       <c r="K171" s="18"/>
       <c r="L171" s="18"/>
       <c r="M171" s="18" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="N171" s="20" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="O171" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="P171" s="21"/>
+        <v>167</v>
+      </c>
+      <c r="P171" s="20"/>
       <c r="Q171" s="18"/>
     </row>
-    <row r="172" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A172" s="18"/>
-      <c r="B172" s="18"/>
-      <c r="C172" s="18"/>
-      <c r="D172" s="18"/>
-      <c r="E172" s="18"/>
-      <c r="F172" s="18"/>
-      <c r="G172" s="18"/>
-      <c r="H172" s="18"/>
-      <c r="I172" s="18"/>
-      <c r="J172" s="18"/>
-      <c r="K172" s="18"/>
-      <c r="L172" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="M172" s="18"/>
-      <c r="N172" s="18"/>
-      <c r="O172" s="18"/>
-      <c r="P172" s="18"/>
-      <c r="Q172" s="18"/>
-    </row>
     <row r="173" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A173" s="18"/>
-      <c r="B173" s="18"/>
-      <c r="C173" s="18"/>
-      <c r="D173" s="18"/>
-      <c r="E173" s="18"/>
-      <c r="F173" s="18"/>
-      <c r="G173" s="18"/>
-      <c r="H173" s="18"/>
-      <c r="I173" s="18"/>
-      <c r="J173" s="18"/>
-      <c r="K173" s="18"/>
-      <c r="L173" s="18"/>
-      <c r="M173" s="18" t="s">
-        <v>165</v>
-      </c>
-      <c r="N173" s="20" t="s">
-        <v>166</v>
-      </c>
-      <c r="O173" s="18" t="s">
-        <v>167</v>
-      </c>
-      <c r="P173" s="20"/>
-      <c r="Q173" s="18"/>
-    </row>
-    <row r="175" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="F175"/>
-      <c r="G175"/>
-      <c r="H175"/>
-      <c r="I175"/>
-      <c r="J175"/>
-      <c r="K175"/>
-      <c r="L175"/>
-      <c r="M175" s="1" t="s">
+      <c r="F173"/>
+      <c r="G173"/>
+      <c r="H173"/>
+      <c r="I173"/>
+      <c r="J173"/>
+      <c r="K173"/>
+      <c r="L173"/>
+      <c r="M173" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="N175" s="12" t="s">
+      <c r="N173" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="O175"/>
-      <c r="P175"/>
-      <c r="Q175"/>
+      <c r="O173"/>
+      <c r="P173"/>
+      <c r="Q173"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Added 'maize gluten meal' as a by-product and connected to feed
</commit_message>
<xml_diff>
--- a/data/default/FeedMgmt.xlsx
+++ b/data/default/FeedMgmt.xlsx
@@ -22,7 +22,7 @@
     <sheet name="horses" sheetId="8" r:id="rId8"/>
     <sheet name="poultry" sheetId="9" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -146,7 +146,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1615" uniqueCount="681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1621" uniqueCount="681">
   <si>
     <t>Statistics Netherlands (2012) Standardised calculation methods for animal manure and nutrients. Standard data 1990–2008</t>
   </si>
@@ -3135,7 +3135,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R173"/>
+  <dimension ref="A1:R175"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="7" width="20.28515625" style="1" customWidth="1"/>
@@ -3708,7 +3708,7 @@
         <v>1.1494252873563218</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F33" s="1" t="s">
         <v>61</v>
       </c>
@@ -3723,7 +3723,7 @@
         <v>1.1389521640091116</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F34" s="1" t="s">
         <v>62</v>
       </c>
@@ -3738,7 +3738,7 @@
         <v>1.1415525114155252</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F35" s="1" t="s">
         <v>64</v>
       </c>
@@ -3753,7 +3753,7 @@
         <v>1.1415525114155252</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F36" s="1" t="s">
         <v>65</v>
       </c>
@@ -3768,7 +3768,7 @@
         <v>1.1415525114155252</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F37" s="1" t="s">
         <v>66</v>
       </c>
@@ -3783,7 +3783,7 @@
         <v>1.1111111111111112</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F38" s="1" t="s">
         <v>68</v>
       </c>
@@ -3798,7 +3798,7 @@
         <v>1.1111111111111112</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F39" s="1" t="s">
         <v>69</v>
       </c>
@@ -3813,7 +3813,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F40" s="1" t="s">
         <v>70</v>
       </c>
@@ -3828,7 +3828,7 @@
         <v>1.3245033112582782</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F41" s="1" t="s">
         <v>71</v>
       </c>
@@ -3843,7 +3843,7 @@
         <v>1.1173184357541899</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F42" s="1" t="s">
         <v>72</v>
       </c>
@@ -3858,7 +3858,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F43" s="1" t="s">
         <v>73</v>
       </c>
@@ -3873,7 +3873,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F44" s="1" t="s">
         <v>74</v>
       </c>
@@ -3888,7 +3888,7 @@
         <v>1.0989010989010988</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F45" s="1" t="s">
         <v>75</v>
       </c>
@@ -3903,7 +3903,7 @@
         <v>4.3478260869565215</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F46" s="1" t="s">
         <v>76</v>
       </c>
@@ -3918,92 +3918,93 @@
         <v>1.0863661053775122</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N47" s="9"/>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A48" s="8" t="s">
+    <row r="47" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F47" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="J47" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="M47" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N47" s="9">
+        <f>1/INDEX('feed pars'!C$6:C$47/100,MATCH(F47,'feed pars'!B$6:B$47,0))</f>
+        <v>1.1152416356877324</v>
+      </c>
+    </row>
+    <row r="48" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="N48" s="9"/>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A49" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="N48" s="9"/>
-    </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="F49" s="1" t="s">
+      <c r="N49" s="9"/>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F50" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="K49" s="1" t="s">
+      <c r="K50" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="M49" s="1" t="s">
+      <c r="M50" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="N49" s="9">
+      <c r="N50" s="9">
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N50" s="9"/>
-    </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A51" s="3" t="s">
+      <c r="N51" s="9"/>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A52" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B51" s="3"/>
-      <c r="C51" s="3"/>
-      <c r="D51" s="3"/>
-      <c r="E51" s="4"/>
-      <c r="F51" s="4"/>
-      <c r="G51" s="4"/>
-      <c r="H51" s="4"/>
-      <c r="I51" s="4"/>
-      <c r="J51" s="4"/>
-      <c r="K51" s="4"/>
-      <c r="L51" s="4"/>
-      <c r="M51" s="4"/>
-      <c r="N51" s="4"/>
-      <c r="O51" s="4"/>
-      <c r="P51" s="4"/>
-      <c r="Q51" s="4"/>
-    </row>
-    <row r="52" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="13" t="s">
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+      <c r="H52" s="4"/>
+      <c r="I52" s="4"/>
+      <c r="J52" s="4"/>
+      <c r="K52" s="4"/>
+      <c r="L52" s="4"/>
+      <c r="M52" s="4"/>
+      <c r="N52" s="4"/>
+      <c r="O52" s="4"/>
+      <c r="P52" s="4"/>
+      <c r="Q52" s="4"/>
+    </row>
+    <row r="53" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="B52" s="8"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="8"/>
-    </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M53" s="6" t="s">
+      <c r="B53" s="8"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M54" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="N53" s="6">
-        <v>0</v>
-      </c>
-      <c r="O53" s="6" t="s">
+      <c r="N54" s="6">
+        <v>0</v>
+      </c>
+      <c r="O54" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="P53" s="6" t="s">
+      <c r="P54" s="6" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="I54" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="M54" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="N54" s="10">
-        <v>95</v>
-      </c>
-      <c r="O54" s="1" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I55" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="M55" s="1" t="s">
         <v>81</v>
@@ -4017,7 +4018,7 @@
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I56" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M56" s="1" t="s">
         <v>81</v>
@@ -4030,26 +4031,22 @@
       </c>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
-        <v>83</v>
-      </c>
       <c r="I57" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="M57" s="1" t="s">
         <v>81</v>
       </c>
       <c r="N57" s="10">
-        <v>30</v>
+        <v>95</v>
       </c>
       <c r="O57" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="P57" s="10"/>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I58" s="1" t="s">
         <v>36</v>
@@ -4067,10 +4064,10 @@
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M59" s="1" t="s">
         <v>81</v>
@@ -4085,7 +4082,7 @@
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I60" s="1" t="s">
         <v>35</v>
@@ -4103,10 +4100,10 @@
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="M61" s="1" t="s">
         <v>81</v>
@@ -4121,7 +4118,7 @@
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I62" s="1" t="s">
         <v>37</v>
@@ -4138,34 +4135,37 @@
       <c r="P62" s="10"/>
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N63" s="10"/>
+      <c r="A63" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="I63" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M63" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="N63" s="10">
+        <v>30</v>
+      </c>
+      <c r="O63" s="1" t="s">
+        <v>82</v>
+      </c>
       <c r="P63" s="10"/>
     </row>
     <row r="64" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A64" s="13" t="s">
-        <v>85</v>
-      </c>
       <c r="N64" s="10"/>
       <c r="P64" s="10"/>
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="I65" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="M65" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="N65" s="10">
-        <v>5</v>
-      </c>
-      <c r="O65" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="A65" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="N65" s="10"/>
       <c r="P65" s="10"/>
     </row>
     <row r="66" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I66" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="M66" s="1" t="s">
         <v>86</v>
@@ -4180,7 +4180,7 @@
     </row>
     <row r="67" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I67" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M67" s="1" t="s">
         <v>86</v>
@@ -4194,130 +4194,125 @@
       <c r="P67" s="10"/>
     </row>
     <row r="68" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N68" s="10"/>
+      <c r="I68" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M68" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="N68" s="10">
+        <v>5</v>
+      </c>
+      <c r="O68" s="1" t="s">
+        <v>82</v>
+      </c>
       <c r="P68" s="10"/>
     </row>
     <row r="69" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A69" s="3" t="s">
+      <c r="N69" s="10"/>
+      <c r="P69" s="10"/>
+    </row>
+    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A70" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B69" s="3"/>
-      <c r="C69" s="3"/>
-      <c r="D69" s="3"/>
-      <c r="E69" s="4"/>
-      <c r="F69" s="4"/>
-      <c r="G69" s="4"/>
-      <c r="H69" s="4"/>
-      <c r="I69" s="4"/>
-      <c r="J69" s="4"/>
-      <c r="K69" s="4"/>
-      <c r="L69" s="4"/>
-      <c r="M69" s="4"/>
-      <c r="N69" s="4"/>
-      <c r="O69" s="4"/>
-      <c r="P69" s="4"/>
-      <c r="Q69" s="4"/>
-    </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M70" s="6" t="s">
+      <c r="B70" s="3"/>
+      <c r="C70" s="3"/>
+      <c r="D70" s="3"/>
+      <c r="E70" s="4"/>
+      <c r="F70" s="4"/>
+      <c r="G70" s="4"/>
+      <c r="H70" s="4"/>
+      <c r="I70" s="4"/>
+      <c r="J70" s="4"/>
+      <c r="K70" s="4"/>
+      <c r="L70" s="4"/>
+      <c r="M70" s="4"/>
+      <c r="N70" s="4"/>
+      <c r="O70" s="4"/>
+      <c r="P70" s="4"/>
+      <c r="Q70" s="4"/>
+    </row>
+    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M71" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="N70" s="6">
+      <c r="N71" s="6">
         <v>100</v>
       </c>
-      <c r="O70" s="6" t="s">
+      <c r="O71" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="P70" s="6" t="s">
+      <c r="P71" s="6" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="I71" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="M71" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="N71" s="12">
-        <v>0</v>
-      </c>
-      <c r="O71" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="P71" s="6"/>
     </row>
     <row r="72" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I72" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="M72" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="N72" s="10">
-        <v>0</v>
-      </c>
-      <c r="O72" s="1" t="s">
+      <c r="N72" s="12">
+        <v>0</v>
+      </c>
+      <c r="O72" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="P72" s="10" t="s">
-        <v>89</v>
-      </c>
+      <c r="P72" s="6"/>
     </row>
     <row r="73" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I73" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="M73" s="1" t="s">
         <v>88</v>
       </c>
       <c r="N73" s="10">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="O73" s="1" t="s">
         <v>82</v>
       </c>
       <c r="P73" s="10" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="I74" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="M74" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N74" s="10">
+        <v>50</v>
+      </c>
+      <c r="O74" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="P74" s="10" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N74" s="10"/>
-      <c r="P74" s="10"/>
-    </row>
     <row r="75" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="F75"/>
-      <c r="G75"/>
-      <c r="H75"/>
-      <c r="I75"/>
-      <c r="J75" t="s">
-        <v>60</v>
-      </c>
-      <c r="M75" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="N75" s="10">
-        <v>80</v>
-      </c>
-      <c r="O75" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="N75" s="10"/>
       <c r="P75" s="10"/>
-      <c r="Q75"/>
     </row>
     <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F76"/>
       <c r="G76"/>
       <c r="H76"/>
       <c r="I76"/>
-      <c r="J76" s="1" t="s">
-        <v>46</v>
+      <c r="J76" t="s">
+        <v>60</v>
       </c>
       <c r="M76" s="1" t="s">
         <v>88</v>
       </c>
       <c r="N76" s="10">
-        <v>42</v>
+        <v>80</v>
       </c>
       <c r="O76" s="1" t="s">
         <v>82</v>
@@ -4331,13 +4326,13 @@
       <c r="H77"/>
       <c r="I77"/>
       <c r="J77" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="M77" s="1" t="s">
         <v>88</v>
       </c>
       <c r="N77" s="10">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="O77" s="1" t="s">
         <v>82</v>
@@ -4351,7 +4346,7 @@
       <c r="H78"/>
       <c r="I78"/>
       <c r="J78" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="M78" s="1" t="s">
         <v>88</v>
@@ -4371,7 +4366,7 @@
       <c r="H79"/>
       <c r="I79"/>
       <c r="J79" s="1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="M79" s="1" t="s">
         <v>88</v>
@@ -4391,7 +4386,7 @@
       <c r="H80"/>
       <c r="I80"/>
       <c r="J80" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M80" s="1" t="s">
         <v>88</v>
@@ -4411,7 +4406,7 @@
       <c r="H81"/>
       <c r="I81"/>
       <c r="J81" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M81" s="1" t="s">
         <v>88</v>
@@ -4431,7 +4426,7 @@
       <c r="H82"/>
       <c r="I82"/>
       <c r="J82" s="1" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="M82" s="1" t="s">
         <v>88</v>
@@ -4446,22 +4441,34 @@
       <c r="Q82"/>
     </row>
     <row r="83" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N83" s="10"/>
+      <c r="F83"/>
+      <c r="G83"/>
+      <c r="H83"/>
+      <c r="I83"/>
+      <c r="J83" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="M83" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N83" s="10">
+        <v>0</v>
+      </c>
+      <c r="O83" s="1" t="s">
+        <v>82</v>
+      </c>
       <c r="P83" s="10"/>
       <c r="Q83"/>
     </row>
     <row r="84" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C84" t="s">
-        <v>679</v>
-      </c>
-      <c r="J84" t="s">
-        <v>60</v>
+      <c r="J84" s="1" t="s">
+        <v>228</v>
       </c>
       <c r="M84" s="1" t="s">
         <v>88</v>
       </c>
       <c r="N84" s="10">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="O84" s="1" t="s">
         <v>82</v>
@@ -4470,35 +4477,22 @@
       <c r="Q84"/>
     </row>
     <row r="85" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C85" t="s">
-        <v>679</v>
-      </c>
-      <c r="J85" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="M85" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="N85" s="10">
-        <v>4</v>
-      </c>
-      <c r="O85" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="N85" s="10"/>
       <c r="P85" s="10"/>
+      <c r="Q85"/>
     </row>
     <row r="86" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C86" t="s">
         <v>679</v>
       </c>
       <c r="J86" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="M86" s="1" t="s">
         <v>88</v>
       </c>
       <c r="N86" s="10">
-        <v>10</v>
+        <v>85</v>
       </c>
       <c r="O86" s="1" t="s">
         <v>82</v>
@@ -4510,46 +4504,45 @@
       <c r="C87" t="s">
         <v>679</v>
       </c>
-      <c r="J87" t="s">
-        <v>70</v>
+      <c r="J87" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="M87" s="1" t="s">
         <v>88</v>
       </c>
       <c r="N87" s="10">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O87" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="P87" s="10" t="s">
-        <v>680</v>
-      </c>
+      <c r="P87" s="10"/>
     </row>
     <row r="88" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C88" t="s">
         <v>679</v>
       </c>
       <c r="J88" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="M88" s="1" t="s">
         <v>88</v>
       </c>
       <c r="N88" s="10">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O88" s="1" t="s">
         <v>82</v>
       </c>
       <c r="P88" s="10"/>
+      <c r="Q88"/>
     </row>
     <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C89" t="s">
         <v>679</v>
       </c>
-      <c r="J89" s="1" t="s">
-        <v>74</v>
+      <c r="J89" t="s">
+        <v>70</v>
       </c>
       <c r="M89" s="1" t="s">
         <v>88</v>
@@ -4560,104 +4553,80 @@
       <c r="O89" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="P89" s="10"/>
+      <c r="P89" s="10" t="s">
+        <v>680</v>
+      </c>
     </row>
     <row r="90" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N90" s="10"/>
+      <c r="C90" t="s">
+        <v>679</v>
+      </c>
+      <c r="J90" t="s">
+        <v>71</v>
+      </c>
+      <c r="M90" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N90" s="10">
+        <v>0</v>
+      </c>
+      <c r="O90" s="1" t="s">
+        <v>82</v>
+      </c>
       <c r="P90" s="10"/>
     </row>
     <row r="91" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A91" s="3" t="s">
+      <c r="C91" t="s">
+        <v>679</v>
+      </c>
+      <c r="J91" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="M91" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N91" s="10">
+        <v>0</v>
+      </c>
+      <c r="O91" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="P91" s="10"/>
+    </row>
+    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N92" s="10"/>
+      <c r="P92" s="10"/>
+    </row>
+    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A93" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B91" s="3"/>
-      <c r="C91" s="3"/>
-      <c r="D91" s="3"/>
-      <c r="E91" s="4"/>
-      <c r="F91" s="4"/>
-      <c r="G91" s="4"/>
-      <c r="H91" s="4"/>
-      <c r="I91" s="4"/>
-      <c r="J91" s="4"/>
-      <c r="K91" s="4"/>
-      <c r="L91" s="4"/>
-      <c r="M91" s="4"/>
-      <c r="N91" s="4"/>
-      <c r="O91" s="4"/>
-      <c r="P91" s="4"/>
-      <c r="Q91" s="4"/>
-    </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A93" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B93" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E93" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="H93" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="I93" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="M93" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="N93" s="12">
-        <v>28</v>
-      </c>
-      <c r="O93" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="P93" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q93" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A94" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B94" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="E94" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="H94" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="I94" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="M94" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="N94" s="12">
-        <v>100</v>
-      </c>
-      <c r="O94" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="P94" s="12"/>
-      <c r="Q94" s="1" t="s">
-        <v>98</v>
-      </c>
+      <c r="B93" s="3"/>
+      <c r="C93" s="3"/>
+      <c r="D93" s="3"/>
+      <c r="E93" s="4"/>
+      <c r="F93" s="4"/>
+      <c r="G93" s="4"/>
+      <c r="H93" s="4"/>
+      <c r="I93" s="4"/>
+      <c r="J93" s="4"/>
+      <c r="K93" s="4"/>
+      <c r="L93" s="4"/>
+      <c r="M93" s="4"/>
+      <c r="N93" s="4"/>
+      <c r="O93" s="4"/>
+      <c r="P93" s="4"/>
+      <c r="Q93" s="4"/>
     </row>
     <row r="95" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="H95" s="1" t="s">
         <v>95</v>
@@ -4668,15 +4637,14 @@
       <c r="M95" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="N95" s="14">
-        <f>N94</f>
-        <v>100</v>
+      <c r="N95" s="12">
+        <v>28</v>
       </c>
       <c r="O95" s="1" t="s">
         <v>82</v>
       </c>
       <c r="P95" s="12" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="Q95" s="1" t="s">
         <v>98</v>
@@ -4686,6 +4654,12 @@
       <c r="A96" s="1" t="s">
         <v>92</v>
       </c>
+      <c r="B96" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E96" s="1" t="s">
+        <v>94</v>
+      </c>
       <c r="H96" s="1" t="s">
         <v>95</v>
       </c>
@@ -4696,7 +4670,7 @@
         <v>96</v>
       </c>
       <c r="N96" s="12">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="O96" s="1" t="s">
         <v>82</v>
@@ -4708,7 +4682,13 @@
     </row>
     <row r="97" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
-        <v>102</v>
+        <v>92</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E97" s="1" t="s">
+        <v>100</v>
       </c>
       <c r="H97" s="1" t="s">
         <v>95</v>
@@ -4719,20 +4699,23 @@
       <c r="M97" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="N97" s="12">
-        <v>14.5</v>
+      <c r="N97" s="14">
+        <f>N96</f>
+        <v>100</v>
       </c>
       <c r="O97" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="P97" s="10"/>
+      <c r="P97" s="12" t="s">
+        <v>101</v>
+      </c>
       <c r="Q97" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="98" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="H98" s="1" t="s">
         <v>95</v>
@@ -4744,22 +4727,19 @@
         <v>96</v>
       </c>
       <c r="N98" s="12">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="O98" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="P98" s="10"/>
+      <c r="P98" s="12"/>
       <c r="Q98" s="1" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
     </row>
     <row r="99" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D99" s="1" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="H99" s="1" t="s">
         <v>95</v>
@@ -4771,26 +4751,20 @@
         <v>96</v>
       </c>
       <c r="N99" s="12">
-        <v>66</v>
+        <v>14.5</v>
       </c>
       <c r="O99" s="1" t="s">
         <v>82</v>
       </c>
       <c r="P99" s="10"/>
       <c r="Q99" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="100" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D100" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="E100" s="1" t="s">
-        <v>107</v>
-      </c>
       <c r="H100" s="1" t="s">
         <v>95</v>
       </c>
@@ -4801,7 +4775,7 @@
         <v>96</v>
       </c>
       <c r="N100" s="12">
-        <v>69</v>
+        <v>100</v>
       </c>
       <c r="O100" s="1" t="s">
         <v>82</v>
@@ -4812,223 +4786,231 @@
       </c>
     </row>
     <row r="101" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N101" s="10"/>
+      <c r="A101" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="H101" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I101" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M101" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="N101" s="12">
+        <v>66</v>
+      </c>
+      <c r="O101" s="1" t="s">
+        <v>82</v>
+      </c>
       <c r="P101" s="10"/>
+      <c r="Q101" s="1" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="102" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A102" s="3" t="s">
+      <c r="A102" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E102" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="H102" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I102" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M102" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="N102" s="12">
+        <v>69</v>
+      </c>
+      <c r="O102" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="P102" s="10"/>
+      <c r="Q102" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N103" s="10"/>
+      <c r="P103" s="10"/>
+    </row>
+    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A104" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="B102" s="3"/>
-      <c r="C102" s="3"/>
-      <c r="D102" s="3"/>
-      <c r="E102" s="4"/>
-      <c r="F102" s="4"/>
-      <c r="G102" s="4"/>
-      <c r="H102" s="4"/>
-      <c r="I102" s="4"/>
-      <c r="J102" s="4"/>
-      <c r="K102" s="4"/>
-      <c r="L102" s="4"/>
-      <c r="M102" s="4"/>
-      <c r="N102" s="4"/>
-      <c r="O102" s="4"/>
-      <c r="P102" s="4"/>
-      <c r="Q102" s="4"/>
-    </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M103" s="6" t="s">
+      <c r="B104" s="3"/>
+      <c r="C104" s="3"/>
+      <c r="D104" s="3"/>
+      <c r="E104" s="4"/>
+      <c r="F104" s="4"/>
+      <c r="G104" s="4"/>
+      <c r="H104" s="4"/>
+      <c r="I104" s="4"/>
+      <c r="J104" s="4"/>
+      <c r="K104" s="4"/>
+      <c r="L104" s="4"/>
+      <c r="M104" s="4"/>
+      <c r="N104" s="4"/>
+      <c r="O104" s="4"/>
+      <c r="P104" s="4"/>
+      <c r="Q104" s="4"/>
+    </row>
+    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M105" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="N103" s="6">
-        <v>0</v>
-      </c>
-      <c r="O103" s="6" t="s">
+      <c r="N105" s="6">
+        <v>0</v>
+      </c>
+      <c r="O105" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="P103" s="6" t="s">
+      <c r="P105" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M104" s="6" t="s">
+    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M106" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="N104" s="6">
-        <v>0</v>
-      </c>
-      <c r="O104" s="6" t="s">
+      <c r="N106" s="6">
+        <v>0</v>
+      </c>
+      <c r="O106" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="P104" s="6" t="s">
+      <c r="P106" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A105" s="1" t="s">
+    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A107" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B105" s="1" t="s">
+      <c r="B107" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E105" s="1" t="s">
+      <c r="E107" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="G105" s="1" t="s">
+      <c r="G107" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="M105" s="12" t="s">
+      <c r="M107" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="N105" s="12">
+      <c r="N107" s="12">
         <f>(0.8*20+0.2*2)</f>
         <v>16.399999999999999</v>
       </c>
-      <c r="O105" s="12" t="s">
+      <c r="O107" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="P105" s="12" t="s">
+      <c r="P107" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="Q105" s="1" t="s">
+      <c r="Q107" s="1" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A106" s="1" t="s">
+    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A108" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="G106" s="1" t="s">
+      <c r="G108" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="M106" s="12" t="s">
+      <c r="M108" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="N106" s="12">
+      <c r="N108" s="12">
         <f>(0.6*20+0.4*2)</f>
         <v>12.8</v>
       </c>
-      <c r="O106" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="P106" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q106" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A107" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="G107" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="M107" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="N107" s="12">
-        <v>2</v>
-      </c>
-      <c r="O107" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="P107" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="Q107" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A108" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="G108" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="M108" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="N108" s="12">
-        <v>2</v>
-      </c>
       <c r="O108" s="12" t="s">
         <v>82</v>
       </c>
       <c r="P108" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="Q108" s="1" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="109" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M109" s="12"/>
-      <c r="N109" s="12"/>
-      <c r="O109" s="12"/>
-      <c r="P109" s="12"/>
+      <c r="A109" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G109" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="M109" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="N109" s="12">
+        <v>2</v>
+      </c>
+      <c r="O109" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="P109" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q109" s="1" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="110" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B110" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E110" s="1" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="G110" s="1" t="s">
         <v>111</v>
       </c>
       <c r="M110" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N110" s="12">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O110" s="12" t="s">
         <v>82</v>
       </c>
       <c r="P110" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="Q110" s="1" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="111" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A111" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="E111" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="G111" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="M111" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="N111" s="12">
-        <v>5</v>
-      </c>
-      <c r="O111" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="P111" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="Q111" s="1" t="s">
-        <v>103</v>
-      </c>
+      <c r="M111" s="12"/>
+      <c r="N111" s="12"/>
+      <c r="O111" s="12"/>
+      <c r="P111" s="12"/>
     </row>
     <row r="112" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>92</v>
       </c>
+      <c r="B112" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E112" s="1" t="s">
+        <v>94</v>
+      </c>
       <c r="G112" s="1" t="s">
         <v>111</v>
       </c>
@@ -5036,79 +5018,101 @@
         <v>110</v>
       </c>
       <c r="N112" s="12">
+        <v>5</v>
+      </c>
+      <c r="O112" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="P112" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q112" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A113" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E113" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="G113" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="M113" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="N113" s="12">
+        <v>5</v>
+      </c>
+      <c r="O113" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="P113" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q113" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A114" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G114" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="M114" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="N114" s="12">
         <f>0.9*5+0.1*15</f>
         <v>6</v>
       </c>
-      <c r="O112" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="P112" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="Q112" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A113" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="G113" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="M113" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="N113" s="12">
-        <v>15</v>
-      </c>
-      <c r="O113" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="P113" s="12"/>
-      <c r="Q113" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A114" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="G114" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="M114" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="N114" s="12">
-        <v>15</v>
-      </c>
       <c r="O114" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="P114" s="12"/>
+      <c r="P114" s="12" t="s">
+        <v>117</v>
+      </c>
       <c r="Q114" s="1" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="115" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M115" s="12"/>
-      <c r="N115" s="12"/>
-      <c r="O115" s="12"/>
+      <c r="A115" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="M115" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="N115" s="12">
+        <v>15</v>
+      </c>
+      <c r="O115" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="P115" s="12"/>
+      <c r="Q115" s="1" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="116" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A116" s="15"/>
-      <c r="B116" s="15"/>
-      <c r="E116" s="15"/>
+      <c r="A116" s="1" t="s">
+        <v>102</v>
+      </c>
       <c r="G116" s="1" t="s">
-        <v>30</v>
+        <v>111</v>
       </c>
       <c r="M116" s="12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N116" s="12">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="O116" s="12" t="s">
         <v>82</v>
@@ -5119,73 +5123,30 @@
       </c>
     </row>
     <row r="117" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A117" s="15" t="str">
-        <f>A110</f>
-        <v>cattle</v>
-      </c>
-      <c r="B117" s="15" t="str">
-        <f>B110</f>
-        <v>dairy</v>
-      </c>
-      <c r="E117" s="15" t="str">
-        <f>E110</f>
-        <v>cows</v>
-      </c>
-      <c r="G117" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M117" s="15" t="str">
-        <f t="shared" ref="M117:Q119" si="0">M110</f>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N117" s="15">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="O117" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v>%</v>
-      </c>
-      <c r="P117" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="Q117" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
+      <c r="M117" s="12"/>
+      <c r="N117" s="12"/>
+      <c r="O117" s="12"/>
+      <c r="P117" s="12"/>
     </row>
     <row r="118" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A118" s="15" t="str">
-        <f>A111</f>
-        <v>cattle</v>
-      </c>
-      <c r="E118" s="15" t="str">
-        <f>E111</f>
-        <v>bulls</v>
-      </c>
+      <c r="A118" s="15"/>
+      <c r="B118" s="15"/>
+      <c r="E118" s="15"/>
       <c r="G118" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M118" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N118" s="15">
-        <f t="shared" si="0"/>
+      <c r="M118" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="N118" s="12">
         <v>5</v>
       </c>
-      <c r="O118" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v>%</v>
-      </c>
-      <c r="P118" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="Q118" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
+      <c r="O118" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="P118" s="12"/>
+      <c r="Q118" s="1" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="119" spans="1:17" x14ac:dyDescent="0.25">
@@ -5193,16 +5154,24 @@
         <f>A112</f>
         <v>cattle</v>
       </c>
+      <c r="B119" s="15" t="str">
+        <f>B112</f>
+        <v>dairy</v>
+      </c>
+      <c r="E119" s="15" t="str">
+        <f>E112</f>
+        <v>cows</v>
+      </c>
       <c r="G119" s="1" t="s">
         <v>30</v>
       </c>
       <c r="M119" s="15" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="M119:Q121" si="0">M112</f>
         <v>feeding_losses</v>
       </c>
       <c r="N119" s="15">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O119" s="15" t="str">
         <f t="shared" si="0"/>
@@ -5210,7 +5179,7 @@
       </c>
       <c r="P119" s="15" t="str">
         <f t="shared" si="0"/>
-        <v>10% feeding on pasture</v>
+        <v>No feeding on pasture</v>
       </c>
       <c r="Q119" s="15" t="str">
         <f t="shared" si="0"/>
@@ -5220,149 +5189,141 @@
     <row r="120" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A120" s="15" t="str">
         <f>A113</f>
-        <v>sheep</v>
+        <v>cattle</v>
+      </c>
+      <c r="E120" s="15" t="str">
+        <f>E113</f>
+        <v>bulls</v>
       </c>
       <c r="G120" s="1" t="s">
         <v>30</v>
       </c>
       <c r="M120" s="15" t="str">
-        <f t="shared" ref="M120:O121" si="1">M113</f>
+        <f t="shared" si="0"/>
         <v>feeding_losses</v>
       </c>
       <c r="N120" s="15">
-        <f t="shared" si="1"/>
-        <v>15</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="O120" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>%</v>
       </c>
-      <c r="P120" s="15"/>
+      <c r="P120" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v>No feeding on pasture</v>
+      </c>
       <c r="Q120" s="15" t="str">
-        <f>Q113</f>
+        <f t="shared" si="0"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="121" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A121" s="15" t="str">
         <f>A114</f>
-        <v>horses</v>
+        <v>cattle</v>
       </c>
       <c r="G121" s="1" t="s">
         <v>30</v>
       </c>
       <c r="M121" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N121" s="15">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="O121" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v>%</v>
+      </c>
+      <c r="P121" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v>10% feeding on pasture</v>
+      </c>
+      <c r="Q121" s="15" t="str">
+        <f t="shared" si="0"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A122" s="15" t="str">
+        <f>A115</f>
+        <v>sheep</v>
+      </c>
+      <c r="G122" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M122" s="15" t="str">
+        <f t="shared" ref="M122:O123" si="1">M115</f>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N122" s="15">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="O122" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="P122" s="15"/>
+      <c r="Q122" s="15" t="str">
+        <f>Q115</f>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A123" s="15" t="str">
+        <f>A116</f>
+        <v>horses</v>
+      </c>
+      <c r="G123" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M123" s="15" t="str">
         <f t="shared" si="1"/>
         <v>feeding_losses</v>
       </c>
-      <c r="N121" s="15">
+      <c r="N123" s="15">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="O121" s="15" t="str">
+      <c r="O123" s="15" t="str">
         <f t="shared" si="1"/>
         <v>%</v>
       </c>
-      <c r="P121" s="15"/>
-      <c r="Q121" s="15" t="str">
-        <f>Q114</f>
+      <c r="P123" s="15"/>
+      <c r="Q123" s="15" t="str">
+        <f>Q116</f>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A122" s="15"/>
-      <c r="M122" s="15"/>
-      <c r="N122" s="15"/>
-      <c r="O122" s="15"/>
-      <c r="P122" s="15"/>
-      <c r="Q122" s="15"/>
-    </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="G123" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="M123" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="N123" s="12">
-        <v>5</v>
-      </c>
-      <c r="O123" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="P123" s="12"/>
-      <c r="Q123" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
     <row r="124" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A124" s="15" t="str">
-        <f>A110</f>
-        <v>cattle</v>
-      </c>
-      <c r="B124" s="15" t="str">
-        <f>B110</f>
-        <v>dairy</v>
-      </c>
-      <c r="E124" s="15" t="str">
-        <f>E110</f>
-        <v>cows</v>
-      </c>
-      <c r="G124" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="M124" s="15" t="str">
-        <f t="shared" ref="M124:Q126" si="2">M110</f>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N124" s="15">
-        <f t="shared" si="2"/>
-        <v>5</v>
-      </c>
-      <c r="O124" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>%</v>
-      </c>
-      <c r="P124" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="Q124" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
-      </c>
+      <c r="A124" s="15"/>
+      <c r="M124" s="15"/>
+      <c r="N124" s="15"/>
+      <c r="O124" s="15"/>
+      <c r="P124" s="15"/>
+      <c r="Q124" s="15"/>
     </row>
     <row r="125" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A125" s="15" t="str">
-        <f>A111</f>
-        <v>cattle</v>
-      </c>
-      <c r="E125" s="15" t="str">
-        <f>E111</f>
-        <v>bulls</v>
-      </c>
       <c r="G125" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="M125" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N125" s="15">
-        <f t="shared" si="2"/>
+      <c r="M125" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="N125" s="12">
         <v>5</v>
       </c>
-      <c r="O125" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>%</v>
-      </c>
-      <c r="P125" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="Q125" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
+      <c r="O125" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="P125" s="12"/>
+      <c r="Q125" s="1" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="126" spans="1:17" x14ac:dyDescent="0.25">
@@ -5370,16 +5331,24 @@
         <f>A112</f>
         <v>cattle</v>
       </c>
+      <c r="B126" s="15" t="str">
+        <f>B112</f>
+        <v>dairy</v>
+      </c>
+      <c r="E126" s="15" t="str">
+        <f>E112</f>
+        <v>cows</v>
+      </c>
       <c r="G126" s="1" t="s">
         <v>118</v>
       </c>
       <c r="M126" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="M126:Q128" si="2">M112</f>
         <v>feeding_losses</v>
       </c>
       <c r="N126" s="15">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O126" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5387,7 +5356,7 @@
       </c>
       <c r="P126" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>10% feeding on pasture</v>
+        <v>No feeding on pasture</v>
       </c>
       <c r="Q126" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5397,242 +5366,268 @@
     <row r="127" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A127" s="15" t="str">
         <f>A113</f>
-        <v>sheep</v>
+        <v>cattle</v>
+      </c>
+      <c r="E127" s="15" t="str">
+        <f>E113</f>
+        <v>bulls</v>
       </c>
       <c r="G127" s="1" t="s">
         <v>118</v>
       </c>
       <c r="M127" s="15" t="str">
-        <f t="shared" ref="M127:O128" si="3">M113</f>
+        <f t="shared" si="2"/>
         <v>feeding_losses</v>
       </c>
       <c r="N127" s="15">
-        <f t="shared" si="3"/>
-        <v>15</v>
+        <f t="shared" si="2"/>
+        <v>5</v>
       </c>
       <c r="O127" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>%</v>
       </c>
-      <c r="P127" s="12"/>
+      <c r="P127" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v>No feeding on pasture</v>
+      </c>
       <c r="Q127" s="15" t="str">
-        <f>Q113</f>
+        <f t="shared" si="2"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="128" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A128" s="15" t="str">
         <f>A114</f>
-        <v>horses</v>
+        <v>cattle</v>
       </c>
       <c r="G128" s="1" t="s">
         <v>118</v>
       </c>
       <c r="M128" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N128" s="15">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="O128" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v>%</v>
+      </c>
+      <c r="P128" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v>10% feeding on pasture</v>
+      </c>
+      <c r="Q128" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A129" s="15" t="str">
+        <f>A115</f>
+        <v>sheep</v>
+      </c>
+      <c r="G129" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="M129" s="15" t="str">
+        <f t="shared" ref="M129:O130" si="3">M115</f>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N129" s="15">
+        <f t="shared" si="3"/>
+        <v>15</v>
+      </c>
+      <c r="O129" s="15" t="str">
+        <f t="shared" si="3"/>
+        <v>%</v>
+      </c>
+      <c r="P129" s="12"/>
+      <c r="Q129" s="15" t="str">
+        <f>Q115</f>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
+    </row>
+    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A130" s="15" t="str">
+        <f>A116</f>
+        <v>horses</v>
+      </c>
+      <c r="G130" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="M130" s="15" t="str">
         <f t="shared" si="3"/>
         <v>feeding_losses</v>
       </c>
-      <c r="N128" s="15">
+      <c r="N130" s="15">
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="O128" s="15" t="str">
+      <c r="O130" s="15" t="str">
         <f t="shared" si="3"/>
         <v>%</v>
       </c>
-      <c r="P128" s="12"/>
-      <c r="Q128" s="15" t="str">
-        <f>Q114</f>
+      <c r="P130" s="12"/>
+      <c r="Q130" s="15" t="str">
+        <f>Q116</f>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N129" s="10"/>
-      <c r="P129" s="12"/>
-    </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A130" s="10"/>
-      <c r="G130" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="M130" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="N130" s="12"/>
-      <c r="P130" s="10" t="s">
-        <v>120</v>
-      </c>
-    </row>
     <row r="131" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A131" s="10"/>
-      <c r="G131" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="M131" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="N131" s="12">
-        <v>2</v>
-      </c>
-      <c r="O131" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="P131" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="Q131" s="1" t="s">
-        <v>122</v>
-      </c>
+      <c r="N131" s="10"/>
+      <c r="P131" s="12"/>
     </row>
     <row r="132" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A132" s="10"/>
-      <c r="M132" s="12"/>
+      <c r="G132" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="M132" s="12" t="s">
+        <v>109</v>
+      </c>
       <c r="N132" s="12"/>
-      <c r="O132" s="12"/>
-      <c r="P132" s="10"/>
+      <c r="P132" s="10" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="133" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A133" s="10"/>
       <c r="G133" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M133" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="N133" s="12"/>
+        <v>110</v>
+      </c>
+      <c r="N133" s="12">
+        <v>2</v>
+      </c>
+      <c r="O133" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="P133" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
+      </c>
+      <c r="Q133" s="1" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="134" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A134" s="10"/>
-      <c r="G134" s="1" t="s">
+      <c r="M134" s="12"/>
+      <c r="N134" s="12"/>
+      <c r="O134" s="12"/>
+      <c r="P134" s="10"/>
+    </row>
+    <row r="135" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A135" s="10"/>
+      <c r="G135" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="M134" s="12" t="s">
+      <c r="M135" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="N135" s="12"/>
+      <c r="P135" s="10" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="136" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A136" s="10"/>
+      <c r="G136" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="M136" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="N134" s="12">
+      <c r="N136" s="12">
         <v>3</v>
       </c>
-      <c r="O134" s="12" t="s">
+      <c r="O136" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="P134" s="10" t="s">
+      <c r="P136" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="Q134" s="1" t="s">
+      <c r="Q136" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N135" s="10"/>
-      <c r="P135" s="12"/>
-    </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A136" s="3" t="s">
+    <row r="137" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N137" s="10"/>
+      <c r="P137" s="12"/>
+    </row>
+    <row r="138" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A138" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="B136" s="3"/>
-      <c r="C136" s="3"/>
-      <c r="D136" s="3"/>
-      <c r="E136" s="4"/>
-      <c r="F136" s="4"/>
-      <c r="G136" s="4"/>
-      <c r="H136" s="4"/>
-      <c r="I136" s="4"/>
-      <c r="J136" s="4"/>
-      <c r="K136" s="4"/>
-      <c r="L136" s="4"/>
-      <c r="M136" s="4"/>
-      <c r="N136" s="4"/>
-      <c r="O136" s="4"/>
-      <c r="P136" s="4"/>
-      <c r="Q136" s="4"/>
-    </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A137" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="N137" s="12"/>
-      <c r="P137" s="12" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A138" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="B138" s="10"/>
-      <c r="C138" s="10"/>
-      <c r="D138" s="10"/>
-      <c r="E138" s="10"/>
-      <c r="F138" s="10"/>
-      <c r="G138" s="10"/>
-      <c r="H138" s="10"/>
-      <c r="I138" s="10"/>
-      <c r="J138" s="10"/>
-      <c r="K138" s="10"/>
-      <c r="L138" s="10"/>
-      <c r="M138" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="N138" s="12">
-        <v>6.7</v>
-      </c>
-      <c r="O138" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="P138" s="10"/>
-      <c r="Q138" s="1" t="s">
-        <v>128</v>
-      </c>
+      <c r="B138" s="3"/>
+      <c r="C138" s="3"/>
+      <c r="D138" s="3"/>
+      <c r="E138" s="4"/>
+      <c r="F138" s="4"/>
+      <c r="G138" s="4"/>
+      <c r="H138" s="4"/>
+      <c r="I138" s="4"/>
+      <c r="J138" s="4"/>
+      <c r="K138" s="4"/>
+      <c r="L138" s="4"/>
+      <c r="M138" s="4"/>
+      <c r="N138" s="4"/>
+      <c r="O138" s="4"/>
+      <c r="P138" s="4"/>
+      <c r="Q138" s="4"/>
     </row>
     <row r="139" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="M139" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="N139" s="12">
-        <v>18</v>
-      </c>
-      <c r="O139" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="P139" s="10"/>
-      <c r="Q139" s="1" t="s">
-        <v>131</v>
+        <v>92</v>
+      </c>
+      <c r="N139" s="12"/>
+      <c r="P139" s="12" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="140" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A140" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="M140" s="1" t="s">
-        <v>129</v>
+      <c r="A140" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="B140" s="10"/>
+      <c r="C140" s="10"/>
+      <c r="D140" s="10"/>
+      <c r="E140" s="10"/>
+      <c r="F140" s="10"/>
+      <c r="G140" s="10"/>
+      <c r="H140" s="10"/>
+      <c r="I140" s="10"/>
+      <c r="J140" s="10"/>
+      <c r="K140" s="10"/>
+      <c r="L140" s="10"/>
+      <c r="M140" s="12" t="s">
+        <v>126</v>
       </c>
       <c r="N140" s="12">
-        <v>1.5</v>
-      </c>
-      <c r="O140" s="1" t="s">
-        <v>130</v>
+        <v>6.7</v>
+      </c>
+      <c r="O140" s="12" t="s">
+        <v>127</v>
       </c>
       <c r="P140" s="10"/>
       <c r="Q140" s="1" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="141" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="M141" s="1" t="s">
         <v>129</v>
       </c>
       <c r="N141" s="12">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="O141" s="1" t="s">
         <v>130</v>
@@ -5643,50 +5638,46 @@
       </c>
     </row>
     <row r="142" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N142" s="12"/>
+      <c r="A142" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="M142" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="N142" s="12">
+        <v>1.5</v>
+      </c>
+      <c r="O142" s="1" t="s">
+        <v>130</v>
+      </c>
       <c r="P142" s="10"/>
+      <c r="Q142" s="1" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="143" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A143" s="1" t="s">
+        <v>84</v>
+      </c>
       <c r="M143" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="N143" s="12">
-        <v>1</v>
-      </c>
-      <c r="O143" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="P143" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="Q143" s="12"/>
+        <v>0</v>
+      </c>
+      <c r="O143" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="P143" s="10"/>
+      <c r="Q143" s="1" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="144" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A144" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="M144" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="N144" s="12">
-        <v>1</v>
-      </c>
-      <c r="O144" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="P144" s="12"/>
-      <c r="Q144" s="12"/>
+      <c r="N144" s="12"/>
+      <c r="P144" s="10"/>
     </row>
     <row r="145" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A145" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B145" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E145" s="1" t="s">
-        <v>94</v>
-      </c>
       <c r="M145" s="1" t="s">
         <v>132</v>
       </c>
@@ -5696,19 +5687,15 @@
       <c r="O145" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="P145" s="12"/>
+      <c r="P145" s="12" t="s">
+        <v>134</v>
+      </c>
       <c r="Q145" s="12"/>
     </row>
     <row r="146" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B146" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E146" s="1" t="s">
-        <v>116</v>
-      </c>
       <c r="M146" s="1" t="s">
         <v>132</v>
       </c>
@@ -5726,10 +5713,10 @@
         <v>92</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="E147" s="1" t="s">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="M147" s="1" t="s">
         <v>132</v>
@@ -5744,77 +5731,75 @@
       <c r="Q147" s="12"/>
     </row>
     <row r="148" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N148" s="10"/>
-      <c r="P148" s="10"/>
+      <c r="A148" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B148" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E148" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="M148" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="N148" s="12">
+        <v>1</v>
+      </c>
+      <c r="O148" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="P148" s="12"/>
+      <c r="Q148" s="12"/>
     </row>
     <row r="149" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A149" s="16" t="s">
+      <c r="A149" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B149" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E149" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="M149" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="N149" s="12">
+        <v>1</v>
+      </c>
+      <c r="O149" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="P149" s="12"/>
+      <c r="Q149" s="12"/>
+    </row>
+    <row r="150" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N150" s="10"/>
+      <c r="P150" s="10"/>
+    </row>
+    <row r="151" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A151" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="B149" s="16"/>
-      <c r="C149" s="16"/>
-      <c r="D149" s="16"/>
-      <c r="E149" s="17"/>
-      <c r="F149" s="17"/>
-      <c r="G149" s="17"/>
-      <c r="H149" s="17"/>
-      <c r="I149" s="17"/>
-      <c r="J149" s="17"/>
-      <c r="K149" s="17"/>
-      <c r="L149" s="17"/>
-      <c r="M149" s="17"/>
-      <c r="N149" s="17"/>
-      <c r="O149" s="17"/>
-      <c r="P149" s="17" t="s">
+      <c r="B151" s="16"/>
+      <c r="C151" s="16"/>
+      <c r="D151" s="16"/>
+      <c r="E151" s="17"/>
+      <c r="F151" s="17"/>
+      <c r="G151" s="17"/>
+      <c r="H151" s="17"/>
+      <c r="I151" s="17"/>
+      <c r="J151" s="17"/>
+      <c r="K151" s="17"/>
+      <c r="L151" s="17"/>
+      <c r="M151" s="17"/>
+      <c r="N151" s="17"/>
+      <c r="O151" s="17"/>
+      <c r="P151" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="Q149" s="17"/>
-    </row>
-    <row r="150" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A150" s="18"/>
-      <c r="B150" s="18"/>
-      <c r="C150" s="18"/>
-      <c r="D150" s="18"/>
-      <c r="E150" s="18"/>
-      <c r="F150" s="18"/>
-      <c r="G150" s="18"/>
-      <c r="H150" s="18"/>
-      <c r="I150" s="18"/>
-      <c r="J150" s="18"/>
-      <c r="K150" s="18"/>
-      <c r="L150" s="19" t="s">
-        <v>137</v>
-      </c>
-      <c r="M150" s="18"/>
-      <c r="N150" s="18"/>
-      <c r="O150" s="18"/>
-      <c r="P150" s="18"/>
-      <c r="Q150" s="18"/>
-    </row>
-    <row r="151" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A151" s="18"/>
-      <c r="B151" s="18"/>
-      <c r="C151" s="18"/>
-      <c r="D151" s="18"/>
-      <c r="E151" s="18"/>
-      <c r="F151" s="18"/>
-      <c r="G151" s="18"/>
-      <c r="H151" s="18"/>
-      <c r="I151" s="18"/>
-      <c r="J151" s="18"/>
-      <c r="K151" s="18"/>
-      <c r="L151" s="18"/>
-      <c r="M151" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="N151" s="20" t="s">
-        <v>139</v>
-      </c>
-      <c r="O151" s="18" t="s">
-        <v>140</v>
-      </c>
-      <c r="P151" s="21"/>
-      <c r="Q151" s="18"/>
+      <c r="Q151" s="17"/>
     </row>
     <row r="152" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A152" s="18"/>
@@ -5828,17 +5813,13 @@
       <c r="I152" s="18"/>
       <c r="J152" s="18"/>
       <c r="K152" s="18"/>
-      <c r="L152" s="18"/>
-      <c r="M152" s="18" t="s">
-        <v>141</v>
-      </c>
-      <c r="N152" s="20" t="s">
-        <v>139</v>
-      </c>
-      <c r="O152" s="18" t="s">
-        <v>142</v>
-      </c>
-      <c r="P152" s="21"/>
+      <c r="L152" s="19" t="s">
+        <v>137</v>
+      </c>
+      <c r="M152" s="18"/>
+      <c r="N152" s="18"/>
+      <c r="O152" s="18"/>
+      <c r="P152" s="18"/>
       <c r="Q152" s="18"/>
     </row>
     <row r="153" spans="1:17" x14ac:dyDescent="0.25">
@@ -5854,14 +5835,16 @@
       <c r="J153" s="18"/>
       <c r="K153" s="18"/>
       <c r="L153" s="18"/>
-      <c r="M153" s="22" t="s">
-        <v>143</v>
+      <c r="M153" s="18" t="s">
+        <v>138</v>
       </c>
       <c r="N153" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="O153" s="18"/>
-      <c r="P153" s="18"/>
+      <c r="O153" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="P153" s="21"/>
       <c r="Q153" s="18"/>
     </row>
     <row r="154" spans="1:17" x14ac:dyDescent="0.25">
@@ -5877,14 +5860,16 @@
       <c r="J154" s="18"/>
       <c r="K154" s="18"/>
       <c r="L154" s="18"/>
-      <c r="M154" s="22" t="s">
-        <v>144</v>
+      <c r="M154" s="18" t="s">
+        <v>141</v>
       </c>
       <c r="N154" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="O154" s="18"/>
-      <c r="P154" s="18"/>
+      <c r="O154" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="P154" s="21"/>
       <c r="Q154" s="18"/>
     </row>
     <row r="155" spans="1:17" x14ac:dyDescent="0.25">
@@ -5901,7 +5886,7 @@
       <c r="K155" s="18"/>
       <c r="L155" s="18"/>
       <c r="M155" s="22" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="N155" s="20" t="s">
         <v>139</v>
@@ -5924,13 +5909,13 @@
       <c r="K156" s="18"/>
       <c r="L156" s="18"/>
       <c r="M156" s="22" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="N156" s="20" t="s">
         <v>139</v>
       </c>
       <c r="O156" s="18"/>
-      <c r="P156" s="21"/>
+      <c r="P156" s="18"/>
       <c r="Q156" s="18"/>
     </row>
     <row r="157" spans="1:17" x14ac:dyDescent="0.25">
@@ -5945,11 +5930,13 @@
       <c r="I157" s="18"/>
       <c r="J157" s="18"/>
       <c r="K157" s="18"/>
-      <c r="L157" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="M157" s="18"/>
-      <c r="N157" s="18"/>
+      <c r="L157" s="18"/>
+      <c r="M157" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="N157" s="20" t="s">
+        <v>139</v>
+      </c>
       <c r="O157" s="18"/>
       <c r="P157" s="18"/>
       <c r="Q157" s="18"/>
@@ -5967,18 +5954,14 @@
       <c r="J158" s="18"/>
       <c r="K158" s="18"/>
       <c r="L158" s="18"/>
-      <c r="M158" s="18" t="s">
-        <v>148</v>
+      <c r="M158" s="22" t="s">
+        <v>146</v>
       </c>
       <c r="N158" s="20" t="s">
-        <v>149</v>
-      </c>
-      <c r="O158" s="18" t="s">
-        <v>150</v>
-      </c>
-      <c r="P158" s="20" t="s">
-        <v>151</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="O158" s="18"/>
+      <c r="P158" s="21"/>
       <c r="Q158" s="18"/>
     </row>
     <row r="159" spans="1:17" x14ac:dyDescent="0.25">
@@ -5993,17 +5976,13 @@
       <c r="I159" s="18"/>
       <c r="J159" s="18"/>
       <c r="K159" s="18"/>
-      <c r="L159" s="18"/>
-      <c r="M159" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="N159" s="20" t="s">
-        <v>149</v>
-      </c>
-      <c r="O159" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="P159" s="21"/>
+      <c r="L159" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="M159" s="18"/>
+      <c r="N159" s="18"/>
+      <c r="O159" s="18"/>
+      <c r="P159" s="18"/>
       <c r="Q159" s="18"/>
     </row>
     <row r="160" spans="1:17" x14ac:dyDescent="0.25">
@@ -6020,16 +5999,16 @@
       <c r="K160" s="18"/>
       <c r="L160" s="18"/>
       <c r="M160" s="18" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="N160" s="20" t="s">
         <v>149</v>
       </c>
       <c r="O160" s="18" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="P160" s="20" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="Q160" s="18"/>
     </row>
@@ -6045,13 +6024,17 @@
       <c r="I161" s="18"/>
       <c r="J161" s="18"/>
       <c r="K161" s="18"/>
-      <c r="L161" s="19" t="s">
-        <v>157</v>
-      </c>
-      <c r="M161" s="18"/>
-      <c r="N161" s="18"/>
-      <c r="O161" s="18"/>
-      <c r="P161" s="18"/>
+      <c r="L161" s="18"/>
+      <c r="M161" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="N161" s="20" t="s">
+        <v>149</v>
+      </c>
+      <c r="O161" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="P161" s="21"/>
       <c r="Q161" s="18"/>
     </row>
     <row r="162" spans="1:17" x14ac:dyDescent="0.25">
@@ -6068,16 +6051,16 @@
       <c r="K162" s="18"/>
       <c r="L162" s="18"/>
       <c r="M162" s="18" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="N162" s="20" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="O162" s="18" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="P162" s="20" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="Q162" s="18"/>
     </row>
@@ -6093,17 +6076,13 @@
       <c r="I163" s="18"/>
       <c r="J163" s="18"/>
       <c r="K163" s="18"/>
-      <c r="L163" s="18"/>
-      <c r="M163" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="N163" s="20" t="s">
-        <v>158</v>
-      </c>
-      <c r="O163" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="P163" s="21"/>
+      <c r="L163" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="M163" s="18"/>
+      <c r="N163" s="18"/>
+      <c r="O163" s="18"/>
+      <c r="P163" s="18"/>
       <c r="Q163" s="18"/>
     </row>
     <row r="164" spans="1:17" x14ac:dyDescent="0.25">
@@ -6118,13 +6097,19 @@
       <c r="I164" s="18"/>
       <c r="J164" s="18"/>
       <c r="K164" s="18"/>
-      <c r="L164" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="M164" s="18"/>
-      <c r="N164" s="18"/>
-      <c r="O164" s="18"/>
-      <c r="P164" s="18"/>
+      <c r="L164" s="18"/>
+      <c r="M164" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="N164" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="O164" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="P164" s="20" t="s">
+        <v>151</v>
+      </c>
       <c r="Q164" s="18"/>
     </row>
     <row r="165" spans="1:17" x14ac:dyDescent="0.25">
@@ -6141,17 +6126,15 @@
       <c r="K165" s="18"/>
       <c r="L165" s="18"/>
       <c r="M165" s="18" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="N165" s="20" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="O165" s="18" t="s">
-        <v>150</v>
-      </c>
-      <c r="P165" s="20" t="s">
-        <v>151</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="P165" s="21"/>
       <c r="Q165" s="18"/>
     </row>
     <row r="166" spans="1:17" x14ac:dyDescent="0.25">
@@ -6166,17 +6149,13 @@
       <c r="I166" s="18"/>
       <c r="J166" s="18"/>
       <c r="K166" s="18"/>
-      <c r="L166" s="18"/>
-      <c r="M166" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="N166" s="20" t="s">
-        <v>160</v>
-      </c>
-      <c r="O166" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="P166" s="21"/>
+      <c r="L166" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="M166" s="18"/>
+      <c r="N166" s="18"/>
+      <c r="O166" s="18"/>
+      <c r="P166" s="18"/>
       <c r="Q166" s="18"/>
     </row>
     <row r="167" spans="1:17" x14ac:dyDescent="0.25">
@@ -6191,13 +6170,19 @@
       <c r="I167" s="18"/>
       <c r="J167" s="18"/>
       <c r="K167" s="18"/>
-      <c r="L167" s="19" t="s">
-        <v>161</v>
-      </c>
-      <c r="M167" s="18"/>
-      <c r="N167" s="18"/>
-      <c r="O167" s="18"/>
-      <c r="P167" s="18"/>
+      <c r="L167" s="18"/>
+      <c r="M167" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="N167" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="O167" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="P167" s="20" t="s">
+        <v>151</v>
+      </c>
       <c r="Q167" s="18"/>
     </row>
     <row r="168" spans="1:17" x14ac:dyDescent="0.25">
@@ -6214,17 +6199,15 @@
       <c r="K168" s="18"/>
       <c r="L168" s="18"/>
       <c r="M168" s="18" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="N168" s="20" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="O168" s="18" t="s">
-        <v>163</v>
-      </c>
-      <c r="P168" s="20" t="s">
-        <v>151</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="P168" s="21"/>
       <c r="Q168" s="18"/>
     </row>
     <row r="169" spans="1:17" x14ac:dyDescent="0.25">
@@ -6239,17 +6222,13 @@
       <c r="I169" s="18"/>
       <c r="J169" s="18"/>
       <c r="K169" s="18"/>
-      <c r="L169" s="18"/>
-      <c r="M169" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="N169" s="20" t="s">
-        <v>162</v>
-      </c>
-      <c r="O169" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="P169" s="21"/>
+      <c r="L169" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="M169" s="18"/>
+      <c r="N169" s="18"/>
+      <c r="O169" s="18"/>
+      <c r="P169" s="18"/>
       <c r="Q169" s="18"/>
     </row>
     <row r="170" spans="1:17" x14ac:dyDescent="0.25">
@@ -6264,13 +6243,19 @@
       <c r="I170" s="18"/>
       <c r="J170" s="18"/>
       <c r="K170" s="18"/>
-      <c r="L170" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="M170" s="18"/>
-      <c r="N170" s="18"/>
-      <c r="O170" s="18"/>
-      <c r="P170" s="18"/>
+      <c r="L170" s="18"/>
+      <c r="M170" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="N170" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="O170" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="P170" s="20" t="s">
+        <v>151</v>
+      </c>
       <c r="Q170" s="18"/>
     </row>
     <row r="171" spans="1:17" x14ac:dyDescent="0.25">
@@ -6287,34 +6272,80 @@
       <c r="K171" s="18"/>
       <c r="L171" s="18"/>
       <c r="M171" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="N171" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="O171" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="P171" s="21"/>
+      <c r="Q171" s="18"/>
+    </row>
+    <row r="172" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A172" s="18"/>
+      <c r="B172" s="18"/>
+      <c r="C172" s="18"/>
+      <c r="D172" s="18"/>
+      <c r="E172" s="18"/>
+      <c r="F172" s="18"/>
+      <c r="G172" s="18"/>
+      <c r="H172" s="18"/>
+      <c r="I172" s="18"/>
+      <c r="J172" s="18"/>
+      <c r="K172" s="18"/>
+      <c r="L172" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="M172" s="18"/>
+      <c r="N172" s="18"/>
+      <c r="O172" s="18"/>
+      <c r="P172" s="18"/>
+      <c r="Q172" s="18"/>
+    </row>
+    <row r="173" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A173" s="18"/>
+      <c r="B173" s="18"/>
+      <c r="C173" s="18"/>
+      <c r="D173" s="18"/>
+      <c r="E173" s="18"/>
+      <c r="F173" s="18"/>
+      <c r="G173" s="18"/>
+      <c r="H173" s="18"/>
+      <c r="I173" s="18"/>
+      <c r="J173" s="18"/>
+      <c r="K173" s="18"/>
+      <c r="L173" s="18"/>
+      <c r="M173" s="18" t="s">
         <v>165</v>
       </c>
-      <c r="N171" s="20" t="s">
+      <c r="N173" s="20" t="s">
         <v>166</v>
       </c>
-      <c r="O171" s="18" t="s">
+      <c r="O173" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="P171" s="20"/>
-      <c r="Q171" s="18"/>
-    </row>
-    <row r="173" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="F173"/>
-      <c r="G173"/>
-      <c r="H173"/>
-      <c r="I173"/>
-      <c r="J173"/>
-      <c r="K173"/>
-      <c r="L173"/>
-      <c r="M173" s="1" t="s">
+      <c r="P173" s="20"/>
+      <c r="Q173" s="18"/>
+    </row>
+    <row r="175" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F175"/>
+      <c r="G175"/>
+      <c r="H175"/>
+      <c r="I175"/>
+      <c r="J175"/>
+      <c r="K175"/>
+      <c r="L175"/>
+      <c r="M175" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="N173" s="12" t="s">
+      <c r="N175" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="O173"/>
-      <c r="P173"/>
-      <c r="Q173"/>
+      <c r="O175"/>
+      <c r="P175"/>
+      <c r="Q175"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Added AAT/PBV for maize and other silage
</commit_message>
<xml_diff>
--- a/data/default/FeedMgmt.xlsx
+++ b/data/default/FeedMgmt.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="references" sheetId="1" r:id="rId1"/>
@@ -838,12 +838,6 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>https://www.feedipedia.org/node/500, https://www.feedipedia.org/node/432</t>
-  </si>
-  <si>
-    <t>https://www.feedipedia.org/node/13883</t>
-  </si>
-  <si>
     <t>%DM accrding to harvest stat</t>
   </si>
   <si>
@@ -2270,6 +2264,12 @@
   </si>
   <si>
     <t>No domestic organic sugar production</t>
+  </si>
+  <si>
+    <t>https://www.feedipedia.org/node/13883, https://grovfoderverktyget.se/?p=31159</t>
+  </si>
+  <si>
+    <t>https://www.feedipedia.org/node/500, https://www.feedipedia.org/node/432, https://grovfoderverktyget.se/?p=31151</t>
   </si>
 </sst>
 </file>
@@ -3920,10 +3920,10 @@
     </row>
     <row r="47" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F47" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="M47" s="1" t="s">
         <v>24</v>
@@ -4462,7 +4462,7 @@
     </row>
     <row r="84" spans="1:17" x14ac:dyDescent="0.25">
       <c r="J84" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="M84" s="1" t="s">
         <v>88</v>
@@ -4483,7 +4483,7 @@
     </row>
     <row r="86" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C86" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="J86" t="s">
         <v>60</v>
@@ -4502,7 +4502,7 @@
     </row>
     <row r="87" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C87" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="J87" s="1" t="s">
         <v>54</v>
@@ -4520,7 +4520,7 @@
     </row>
     <row r="88" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C88" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="J88" t="s">
         <v>67</v>
@@ -4539,7 +4539,7 @@
     </row>
     <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C89" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="J89" t="s">
         <v>70</v>
@@ -4554,12 +4554,12 @@
         <v>82</v>
       </c>
       <c r="P89" s="10" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
     </row>
     <row r="90" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C90" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="J90" t="s">
         <v>71</v>
@@ -4577,7 +4577,7 @@
     </row>
     <row r="91" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C91" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="J91" s="1" t="s">
         <v>74</v>
@@ -7050,8 +7050,13 @@
         <f>(8.3+8.7)/2</f>
         <v>8.5</v>
       </c>
-      <c r="O8" s="55"/>
-      <c r="P8" s="55"/>
+      <c r="O8" s="55">
+        <v>61</v>
+      </c>
+      <c r="P8" s="67">
+        <f>P9</f>
+        <v>-19</v>
+      </c>
       <c r="Q8" s="55">
         <f>AVERAGE('ruminants, roughage'!H23:H24)</f>
         <v>10.75</v>
@@ -7086,7 +7091,7 @@
         <v>2.35</v>
       </c>
       <c r="Z8" s="51" t="s">
-        <v>203</v>
+        <v>680</v>
       </c>
       <c r="AA8" s="1" t="s">
         <v>202</v>
@@ -7253,8 +7258,12 @@
       <c r="N10" s="42">
         <v>11</v>
       </c>
-      <c r="O10" s="42"/>
-      <c r="P10" s="42"/>
+      <c r="O10" s="42">
+        <v>84</v>
+      </c>
+      <c r="P10" s="42">
+        <v>-44</v>
+      </c>
       <c r="Q10" s="42">
         <f>AVERAGE('ruminants, roughage'!H25:H26)</f>
         <v>12.3</v>
@@ -7288,7 +7297,7 @@
         <v>1.03</v>
       </c>
       <c r="Z10" s="51" t="s">
-        <v>204</v>
+        <v>679</v>
       </c>
       <c r="AA10" s="23" t="s">
         <v>202</v>
@@ -7445,7 +7454,7 @@
         <v>0.52500000000000002</v>
       </c>
       <c r="I12" s="61" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="K12" s="28">
         <f>MATCH($B12,ruminants!$A$3:$A$120,0)</f>
@@ -7565,7 +7574,7 @@
       </c>
       <c r="AO12" s="13"/>
       <c r="AP12" s="64" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="AQ12" s="1" t="s">
         <v>202</v>
@@ -7612,7 +7621,7 @@
         <v>0.58000000000000007</v>
       </c>
       <c r="I13" s="61" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="J13" s="2"/>
       <c r="K13" s="28">
@@ -7733,7 +7742,7 @@
       </c>
       <c r="AO13" s="13"/>
       <c r="AP13" s="64" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="AQ13" s="1" t="s">
         <v>202</v>
@@ -7780,7 +7789,7 @@
         <v>0.54</v>
       </c>
       <c r="I14" s="61" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="J14" s="2"/>
       <c r="K14" s="28">
@@ -7901,7 +7910,7 @@
       </c>
       <c r="AO14" s="13"/>
       <c r="AP14" s="64" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="AQ14" s="1" t="s">
         <v>202</v>
@@ -7948,7 +7957,7 @@
         <v>0.58000000000000007</v>
       </c>
       <c r="I15" s="61" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="J15" s="2"/>
       <c r="K15" s="28">
@@ -8069,7 +8078,7 @@
       </c>
       <c r="AO15" s="13"/>
       <c r="AP15" s="64" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="AQ15" s="1" t="s">
         <v>202</v>
@@ -8116,7 +8125,7 @@
         <v>0.55499999999999994</v>
       </c>
       <c r="I16" s="61" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="J16" s="2"/>
       <c r="K16" s="28">
@@ -8237,7 +8246,7 @@
       </c>
       <c r="AO16" s="13"/>
       <c r="AP16" s="64" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="AQ16" s="1" t="s">
         <v>202</v>
@@ -8284,7 +8293,7 @@
         <v>0.46500000000000002</v>
       </c>
       <c r="I17" s="61" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="J17" s="2"/>
       <c r="K17" s="28">
@@ -8403,7 +8412,7 @@
       </c>
       <c r="AO17" s="13"/>
       <c r="AP17" s="64" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="AQ17" s="1" t="s">
         <v>202</v>
@@ -8450,7 +8459,7 @@
         <v>1.155</v>
       </c>
       <c r="I18" s="61" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="J18" s="2"/>
       <c r="K18" s="28">
@@ -8568,7 +8577,7 @@
       </c>
       <c r="AO18" s="13"/>
       <c r="AP18" s="64" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="AQ18" s="1" t="s">
         <v>202</v>
@@ -8615,7 +8624,7 @@
         <v>1.375</v>
       </c>
       <c r="I19" s="61" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="J19" s="2"/>
       <c r="K19" s="28"/>
@@ -8670,7 +8679,7 @@
         <v>1.1499999999999999</v>
       </c>
       <c r="Z19" s="51" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="AA19" s="62"/>
       <c r="AB19" s="28">
@@ -8726,7 +8735,7 @@
       </c>
       <c r="AO19" s="13"/>
       <c r="AP19" s="64" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="AQ19" s="1" t="s">
         <v>202</v>
@@ -8764,7 +8773,7 @@
         <v>0.90999999999999992</v>
       </c>
       <c r="I20" s="61" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="J20" s="2"/>
       <c r="K20" s="28">
@@ -8882,7 +8891,7 @@
       </c>
       <c r="AO20" s="13"/>
       <c r="AP20" s="64" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="AQ20" s="1" t="s">
         <v>202</v>
@@ -8893,7 +8902,7 @@
         <v>16.8</v>
       </c>
       <c r="AU20" s="1" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="21" spans="2:47" x14ac:dyDescent="0.25">
@@ -8925,7 +8934,7 @@
         <v>0.89500000000000002</v>
       </c>
       <c r="I21" s="61" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="J21" s="2"/>
       <c r="K21" s="28">
@@ -9043,7 +9052,7 @@
       </c>
       <c r="AO21" s="13"/>
       <c r="AP21" s="64" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="AQ21" s="1" t="s">
         <v>202</v>
@@ -9131,7 +9140,7 @@
         <v>0</v>
       </c>
       <c r="Z22" s="51" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="AA22" s="62"/>
       <c r="AB22" s="28">
@@ -9187,7 +9196,7 @@
       </c>
       <c r="AO22" s="13"/>
       <c r="AP22" s="64" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="AQ22" s="1" t="s">
         <v>202</v>
@@ -9435,7 +9444,7 @@
         <v>16</v>
       </c>
       <c r="AU24" s="23" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="25" spans="2:47" x14ac:dyDescent="0.25">
@@ -9583,7 +9592,7 @@
       </c>
       <c r="AO25" s="13"/>
       <c r="AP25" s="64" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="AQ25" s="1" t="s">
         <v>202</v>
@@ -9683,7 +9692,7 @@
         <v>2.4300000000000002</v>
       </c>
       <c r="Z26" s="51" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="AA26" s="62"/>
       <c r="AB26" s="28">
@@ -9739,7 +9748,7 @@
       </c>
       <c r="AO26" s="13"/>
       <c r="AP26" s="64" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="AQ26" s="1" t="s">
         <v>202</v>
@@ -9893,7 +9902,7 @@
       </c>
       <c r="AO27" s="13"/>
       <c r="AP27" s="64" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="AQ27" s="1" t="s">
         <v>202</v>
@@ -10205,7 +10214,7 @@
       </c>
       <c r="AO29" s="13"/>
       <c r="AP29" s="64" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="AQ29" s="1" t="s">
         <v>202</v>
@@ -10216,7 +10225,7 @@
         <v>8.6</v>
       </c>
       <c r="AU29" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="30" spans="2:47" x14ac:dyDescent="0.25">
@@ -10450,7 +10459,7 @@
         <v>2.56</v>
       </c>
       <c r="Z31" s="51" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="AA31" s="62"/>
       <c r="AB31" s="28"/>
@@ -10620,7 +10629,7 @@
       </c>
       <c r="AO32" s="13"/>
       <c r="AP32" s="64" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="AQ32" s="1" t="s">
         <v>202</v>
@@ -10718,7 +10727,7 @@
         <v>0.62</v>
       </c>
       <c r="Z33" s="23" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="AA33" s="62"/>
       <c r="AB33" s="28">
@@ -10774,7 +10783,7 @@
       </c>
       <c r="AO33" s="13"/>
       <c r="AP33" s="64" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="AQ33" s="1" t="s">
         <v>202</v>
@@ -11264,7 +11273,7 @@
       </c>
       <c r="AO37" s="13"/>
       <c r="AP37" s="64" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="AQ37" s="1" t="s">
         <v>202</v>
@@ -11517,10 +11526,10 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="AO39" s="51" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="AP39" s="64" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="AQ39" s="1" t="s">
         <v>202</v>
@@ -11531,7 +11540,7 @@
     </row>
     <row r="40" spans="2:46" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C40" s="46">
         <f>AVERAGE(AC40,L40,AS40)</f>
@@ -11674,7 +11683,7 @@
       </c>
       <c r="AO40" s="51"/>
       <c r="AP40" s="64" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="AQ40" s="1" t="s">
         <v>202</v>
@@ -11837,7 +11846,7 @@
       </c>
       <c r="AO41" s="13"/>
       <c r="AP41" s="64" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="AQ41" s="1" t="s">
         <v>202</v>
@@ -11991,7 +12000,7 @@
       </c>
       <c r="AO42" s="13"/>
       <c r="AP42" s="64" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="AQ42" s="1" t="s">
         <v>202</v>
@@ -12235,7 +12244,7 @@
         <v>2.1</v>
       </c>
       <c r="Z44" s="51" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="AA44" s="62"/>
       <c r="AB44" s="28">
@@ -12291,7 +12300,7 @@
       </c>
       <c r="AO44" s="13"/>
       <c r="AP44" s="64" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="AQ44" s="1" t="s">
         <v>202</v>
@@ -12445,7 +12454,7 @@
       </c>
       <c r="AO45" s="13"/>
       <c r="AP45" s="64" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="AQ45" s="1" t="s">
         <v>202</v>
@@ -12655,7 +12664,7 @@
         <v>1.1900000000000002</v>
       </c>
       <c r="Z47" s="51" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="AA47" s="62"/>
       <c r="AB47" s="28">
@@ -12712,7 +12721,7 @@
       </c>
       <c r="AO47" s="13"/>
       <c r="AP47" s="64" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="AQ47" s="1" t="s">
         <v>202</v>
@@ -12732,7 +12741,7 @@
     </row>
     <row r="48" spans="2:46" x14ac:dyDescent="0.25">
       <c r="B48" s="10" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C48" s="73">
         <f t="shared" si="24"/>
@@ -12802,7 +12811,7 @@
         <v>0</v>
       </c>
       <c r="Z48" s="83" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="AA48" s="62"/>
       <c r="AB48" s="5"/>
@@ -12847,7 +12856,7 @@
     </row>
     <row r="50" spans="4:19" x14ac:dyDescent="0.25">
       <c r="D50" s="87" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E50" s="88"/>
       <c r="F50" s="89"/>
@@ -12857,12 +12866,12 @@
       <c r="J50" s="89"/>
       <c r="K50" s="90"/>
       <c r="O50" s="91" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="51" spans="4:19" x14ac:dyDescent="0.25">
       <c r="D51" s="39" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E51" s="52"/>
       <c r="F51" s="52"/>
@@ -12881,7 +12890,7 @@
         <v>46</v>
       </c>
       <c r="R51" s="1" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="S51" s="1" t="s">
         <v>59</v>
@@ -12889,7 +12898,7 @@
     </row>
     <row r="52" spans="4:19" x14ac:dyDescent="0.25">
       <c r="D52" s="92" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E52" s="23"/>
       <c r="F52" s="52"/>
@@ -12921,7 +12930,7 @@
     </row>
     <row r="53" spans="4:19" x14ac:dyDescent="0.25">
       <c r="D53" s="95" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="E53" s="96"/>
       <c r="F53" s="97"/>
@@ -12931,7 +12940,7 @@
       <c r="J53" s="97"/>
       <c r="K53" s="98"/>
       <c r="O53" s="91" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="54" spans="4:19" x14ac:dyDescent="0.25">
@@ -12959,7 +12968,7 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C1" r:id="rId1"/>
-    <hyperlink ref="Z10" r:id="rId2"/>
+    <hyperlink ref="Z10" r:id="rId2" display="https://www.feedipedia.org/node/13883"/>
     <hyperlink ref="AP12" r:id="rId3"/>
     <hyperlink ref="AP13" r:id="rId4"/>
     <hyperlink ref="AP14" r:id="rId5"/>
@@ -13014,7 +13023,7 @@
   <sheetData>
     <row r="1" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -13034,7 +13043,7 @@
         <v>6</v>
       </c>
       <c r="J1" s="27" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="K1" s="4"/>
       <c r="L1" s="4"/>
@@ -13054,7 +13063,7 @@
         <v>17</v>
       </c>
       <c r="S1" s="27" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="T1" s="4"/>
       <c r="U1" s="4"/>
@@ -13068,7 +13077,7 @@
         <v>17</v>
       </c>
       <c r="Z1" s="27" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="AA1" s="4"/>
       <c r="AB1" s="4"/>
@@ -13082,7 +13091,7 @@
         <v>17</v>
       </c>
       <c r="AG1" s="27" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="AH1" s="4"/>
       <c r="AI1" s="4"/>
@@ -13093,7 +13102,7 @@
         <v>29</v>
       </c>
       <c r="AM1" s="27" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="AN1" s="4"/>
       <c r="AO1" s="4"/>
@@ -13102,7 +13111,7 @@
       </c>
       <c r="AQ1" s="4"/>
       <c r="AS1" s="27" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="AT1" s="4"/>
       <c r="AU1" s="4"/>
@@ -13121,19 +13130,19 @@
         <v>8</v>
       </c>
       <c r="D2" s="97" t="s">
+        <v>249</v>
+      </c>
+      <c r="E2" s="97" t="s">
+        <v>250</v>
+      </c>
+      <c r="F2" s="97" t="s">
         <v>251</v>
       </c>
-      <c r="E2" s="97" t="s">
+      <c r="G2" s="97" t="s">
         <v>252</v>
       </c>
-      <c r="F2" s="97" t="s">
+      <c r="H2" s="97" t="s">
         <v>253</v>
-      </c>
-      <c r="G2" s="97" t="s">
-        <v>254</v>
-      </c>
-      <c r="H2" s="97" t="s">
-        <v>255</v>
       </c>
       <c r="I2" s="52"/>
       <c r="J2" s="97" t="s">
@@ -13146,19 +13155,19 @@
         <v>8</v>
       </c>
       <c r="M2" s="97" t="s">
+        <v>254</v>
+      </c>
+      <c r="N2" s="97" t="s">
+        <v>255</v>
+      </c>
+      <c r="O2" s="97" t="s">
         <v>256</v>
       </c>
-      <c r="N2" s="97" t="s">
+      <c r="P2" s="97" t="s">
         <v>257</v>
       </c>
-      <c r="O2" s="97" t="s">
+      <c r="Q2" s="97" t="s">
         <v>258</v>
-      </c>
-      <c r="P2" s="97" t="s">
-        <v>259</v>
-      </c>
-      <c r="Q2" s="97" t="s">
-        <v>260</v>
       </c>
       <c r="S2" s="97" t="s">
         <v>9</v>
@@ -13170,13 +13179,13 @@
         <v>8</v>
       </c>
       <c r="V2" s="97" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="W2" s="97" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="X2" s="97" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="Z2" s="97" t="s">
         <v>9</v>
@@ -13188,13 +13197,13 @@
         <v>8</v>
       </c>
       <c r="AC2" s="97" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="AD2" s="97" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="AE2" s="97" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="AG2" s="97" t="s">
         <v>9</v>
@@ -13206,10 +13215,10 @@
         <v>8</v>
       </c>
       <c r="AJ2" s="97" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="AK2" s="97" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="AM2" s="97" t="s">
         <v>9</v>
@@ -13221,10 +13230,10 @@
         <v>8</v>
       </c>
       <c r="AP2" s="97" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="AQ2" s="97" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="AS2" s="97" t="s">
         <v>9</v>
@@ -13236,7 +13245,7 @@
         <v>8</v>
       </c>
       <c r="AV2" s="99" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:48" x14ac:dyDescent="0.25">
@@ -13353,7 +13362,7 @@
         <v>83</v>
       </c>
       <c r="AO3" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP3" s="89" t="str">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A3,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A3,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -13489,7 +13498,7 @@
         <v>83</v>
       </c>
       <c r="AO4" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP4" s="52" t="str">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A4,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A4,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -13548,13 +13557,13 @@
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A5,'feed pars'!$B$6:$B$48,0),M$1)&lt;&gt;"",M$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A5,'feed pars'!$B$6:$B$48,0),M$1), "")</f>
         <v>8.5</v>
       </c>
-      <c r="N5" s="52" t="str">
+      <c r="N5" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A5,'feed pars'!$B$6:$B$48,0),N$1)&lt;&gt;"",N$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A5,'feed pars'!$B$6:$B$48,0),N$1), "")</f>
-        <v/>
-      </c>
-      <c r="O5" s="52" t="str">
+        <v>61</v>
+      </c>
+      <c r="O5" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A5,'feed pars'!$B$6:$B$48,0),O$1)&lt;&gt;"",O$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A5,'feed pars'!$B$6:$B$48,0),O$1), "")</f>
-        <v/>
+        <v>-19</v>
       </c>
       <c r="P5" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A5,'feed pars'!$B$6:$B$48,0),P$1)&lt;&gt;"",P$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A5,'feed pars'!$B$6:$B$48,0),P$1), "")</f>
@@ -13625,7 +13634,7 @@
         <v>83</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP5" s="52" t="str">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A5,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A5,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -13761,7 +13770,7 @@
         <v>83</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP6" s="52" t="str">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A6,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A6,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -13820,13 +13829,13 @@
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A7,'feed pars'!$B$6:$B$48,0),M$1)&lt;&gt;"",M$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A7,'feed pars'!$B$6:$B$48,0),M$1), "")</f>
         <v>11</v>
       </c>
-      <c r="N7" s="52" t="str">
+      <c r="N7" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A7,'feed pars'!$B$6:$B$48,0),N$1)&lt;&gt;"",N$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A7,'feed pars'!$B$6:$B$48,0),N$1), "")</f>
-        <v/>
-      </c>
-      <c r="O7" s="52" t="str">
+        <v>84</v>
+      </c>
+      <c r="O7" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A7,'feed pars'!$B$6:$B$48,0),O$1)&lt;&gt;"",O$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A7,'feed pars'!$B$6:$B$48,0),O$1), "")</f>
-        <v/>
+        <v>-44</v>
       </c>
       <c r="P7" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A7,'feed pars'!$B$6:$B$48,0),P$1)&lt;&gt;"",P$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A7,'feed pars'!$B$6:$B$48,0),P$1), "")</f>
@@ -13897,7 +13906,7 @@
         <v>83</v>
       </c>
       <c r="AO7" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP7" s="52" t="str">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A7,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A7,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -14033,7 +14042,7 @@
         <v>83</v>
       </c>
       <c r="AO8" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP8" s="52" t="str">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A8,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A8,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -14170,7 +14179,7 @@
         <v>83</v>
       </c>
       <c r="AO9" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP9" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A9,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A9,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -14307,7 +14316,7 @@
         <v>83</v>
       </c>
       <c r="AO10" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP10" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A10,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A10,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -14444,7 +14453,7 @@
         <v>83</v>
       </c>
       <c r="AO11" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP11" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A11,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A11,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -14581,7 +14590,7 @@
         <v>83</v>
       </c>
       <c r="AO12" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP12" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A12,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A12,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -14718,7 +14727,7 @@
         <v>83</v>
       </c>
       <c r="AO13" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP13" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A13,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A13,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -14855,7 +14864,7 @@
         <v>83</v>
       </c>
       <c r="AO14" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP14" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A14,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A14,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -14992,7 +15001,7 @@
         <v>83</v>
       </c>
       <c r="AO15" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP15" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A15,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A15,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -15129,7 +15138,7 @@
         <v>83</v>
       </c>
       <c r="AO16" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP16" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A16,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A16,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -15266,7 +15275,7 @@
         <v>83</v>
       </c>
       <c r="AO17" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP17" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A17,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A17,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -15403,7 +15412,7 @@
         <v>83</v>
       </c>
       <c r="AO18" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP18" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A18,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A18,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -15540,7 +15549,7 @@
         <v>83</v>
       </c>
       <c r="AO19" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP19" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A19,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A19,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -15677,7 +15686,7 @@
         <v>83</v>
       </c>
       <c r="AO20" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP20" s="52" t="str">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A20,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A20,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -15814,7 +15823,7 @@
         <v>83</v>
       </c>
       <c r="AO21" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP21" s="52" t="str">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A21,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A21,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -15951,7 +15960,7 @@
         <v>83</v>
       </c>
       <c r="AO22" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP22" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A22,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A22,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -16088,7 +16097,7 @@
         <v>83</v>
       </c>
       <c r="AO23" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP23" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A23,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A23,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -16225,7 +16234,7 @@
         <v>83</v>
       </c>
       <c r="AO24" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP24" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A24,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A24,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -16362,7 +16371,7 @@
         <v>83</v>
       </c>
       <c r="AO25" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP25" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A25,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A25,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -16499,7 +16508,7 @@
         <v>83</v>
       </c>
       <c r="AO26" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP26" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A26,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A26,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -16636,7 +16645,7 @@
         <v>83</v>
       </c>
       <c r="AO27" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP27" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A27,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A27,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -16773,7 +16782,7 @@
         <v>83</v>
       </c>
       <c r="AO28" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP28" s="52" t="str">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A28,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A28,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -16910,7 +16919,7 @@
         <v>83</v>
       </c>
       <c r="AO29" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP29" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A29,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A29,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -17047,7 +17056,7 @@
         <v>83</v>
       </c>
       <c r="AO30" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP30" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A30,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A30,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -17184,7 +17193,7 @@
         <v>83</v>
       </c>
       <c r="AO31" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP31" s="52" t="str">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A31,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A31,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -17321,7 +17330,7 @@
         <v>83</v>
       </c>
       <c r="AO32" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP32" s="52" t="str">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A32,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A32,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -17456,7 +17465,7 @@
         <v>83</v>
       </c>
       <c r="AO33" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP33" s="52" t="str">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A33,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A33,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -17593,7 +17602,7 @@
         <v>83</v>
       </c>
       <c r="AO34" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP34" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A34,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A34,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -17730,7 +17739,7 @@
         <v>83</v>
       </c>
       <c r="AO35" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP35" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A35,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A35,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -17867,7 +17876,7 @@
         <v>83</v>
       </c>
       <c r="AO36" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP36" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A36,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A36,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -18004,7 +18013,7 @@
         <v>83</v>
       </c>
       <c r="AO37" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP37" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A37,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A37,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -18141,7 +18150,7 @@
         <v>83</v>
       </c>
       <c r="AO38" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP38" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A38,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A38,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -18278,7 +18287,7 @@
         <v>83</v>
       </c>
       <c r="AO39" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP39" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A39,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A39,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -18415,7 +18424,7 @@
         <v>83</v>
       </c>
       <c r="AO40" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP40" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A40,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A40,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -18552,7 +18561,7 @@
         <v>83</v>
       </c>
       <c r="AO41" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP41" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A41,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A41,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -18689,7 +18698,7 @@
         <v>83</v>
       </c>
       <c r="AO42" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP42" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A42,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A42,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -18832,7 +18841,7 @@
         <v>83</v>
       </c>
       <c r="AO43" s="52" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP43" s="52" t="str">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A43,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A43,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -18973,7 +18982,7 @@
         <v>83</v>
       </c>
       <c r="AO44" s="42" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP44" s="52">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A44,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A44,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -19115,7 +19124,7 @@
         <v>83</v>
       </c>
       <c r="AO45" s="101" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="AP45" s="97">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A45,'feed pars'!$B$6:$B$48,0),AP$1)&lt;&gt;"",AP$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A45,'feed pars'!$B$6:$B$48,0),AP$1), "")</f>
@@ -19277,13 +19286,13 @@
         <v>178</v>
       </c>
       <c r="B2" s="103" t="s">
+        <v>262</v>
+      </c>
+      <c r="C2" s="103" t="s">
+        <v>263</v>
+      </c>
+      <c r="D2" s="103" t="s">
         <v>264</v>
-      </c>
-      <c r="C2" s="103" t="s">
-        <v>265</v>
-      </c>
-      <c r="D2" s="103" t="s">
-        <v>266</v>
       </c>
       <c r="E2" s="103" t="s">
         <v>197</v>
@@ -19292,109 +19301,109 @@
         <v>198</v>
       </c>
       <c r="G2" s="103" t="s">
+        <v>265</v>
+      </c>
+      <c r="H2" s="103" t="s">
+        <v>266</v>
+      </c>
+      <c r="I2" s="103" t="s">
         <v>267</v>
       </c>
-      <c r="H2" s="103" t="s">
+      <c r="J2" s="103" t="s">
         <v>268</v>
       </c>
-      <c r="I2" s="103" t="s">
+      <c r="K2" s="103" t="s">
         <v>269</v>
       </c>
-      <c r="J2" s="103" t="s">
+      <c r="L2" s="103" t="s">
         <v>270</v>
       </c>
-      <c r="K2" s="103" t="s">
+      <c r="M2" s="103" t="s">
         <v>271</v>
       </c>
-      <c r="L2" s="103" t="s">
+      <c r="N2" s="103" t="s">
         <v>272</v>
       </c>
-      <c r="M2" s="103" t="s">
+      <c r="O2" s="103" t="s">
         <v>273</v>
       </c>
-      <c r="N2" s="103" t="s">
+      <c r="P2" s="103" t="s">
         <v>274</v>
       </c>
-      <c r="O2" s="103" t="s">
+      <c r="Q2" s="103" t="s">
         <v>275</v>
       </c>
-      <c r="P2" s="103" t="s">
+      <c r="R2" s="103" t="s">
         <v>276</v>
       </c>
-      <c r="Q2" s="103" t="s">
+      <c r="S2" s="103" t="s">
         <v>277</v>
       </c>
-      <c r="R2" s="103" t="s">
+      <c r="T2" s="103" t="s">
         <v>278</v>
       </c>
-      <c r="S2" s="103" t="s">
+      <c r="U2" s="103" t="s">
         <v>279</v>
       </c>
-      <c r="T2" s="103" t="s">
+      <c r="V2" s="103" t="s">
         <v>280</v>
       </c>
-      <c r="U2" s="103" t="s">
+      <c r="W2" s="103" t="s">
         <v>281</v>
       </c>
-      <c r="V2" s="103" t="s">
+      <c r="X2" s="103" t="s">
         <v>282</v>
       </c>
-      <c r="W2" s="103" t="s">
+      <c r="Y2" s="103" t="s">
         <v>283</v>
       </c>
-      <c r="X2" s="103" t="s">
+      <c r="Z2" s="103" t="s">
         <v>284</v>
       </c>
-      <c r="Y2" s="103" t="s">
+      <c r="AA2" s="103" t="s">
         <v>285</v>
       </c>
-      <c r="Z2" s="103" t="s">
+      <c r="AB2" s="103" t="s">
         <v>286</v>
       </c>
-      <c r="AA2" s="103" t="s">
+      <c r="AC2" s="103" t="s">
         <v>287</v>
       </c>
-      <c r="AB2" s="103" t="s">
+      <c r="AD2" s="103" t="s">
         <v>288</v>
       </c>
-      <c r="AC2" s="103" t="s">
+      <c r="AE2" s="103" t="s">
         <v>289</v>
       </c>
-      <c r="AD2" s="103" t="s">
+      <c r="AF2" s="103" t="s">
         <v>290</v>
       </c>
-      <c r="AE2" s="103" t="s">
+      <c r="AG2" s="103" t="s">
         <v>291</v>
       </c>
-      <c r="AF2" s="103" t="s">
+      <c r="AH2" s="103" t="s">
         <v>292</v>
       </c>
-      <c r="AG2" s="103" t="s">
+      <c r="AI2" s="103" t="s">
         <v>293</v>
       </c>
-      <c r="AH2" s="103" t="s">
+      <c r="AJ2" s="103" t="s">
         <v>294</v>
       </c>
-      <c r="AI2" s="103" t="s">
+      <c r="AK2" s="103" t="s">
         <v>295</v>
       </c>
-      <c r="AJ2" s="103" t="s">
+      <c r="AL2" s="103" t="s">
         <v>296</v>
       </c>
-      <c r="AK2" s="103" t="s">
+      <c r="AM2" s="103" t="s">
         <v>297</v>
       </c>
-      <c r="AL2" s="103" t="s">
+      <c r="AN2" s="103" t="s">
         <v>298</v>
       </c>
-      <c r="AM2" s="103" t="s">
+      <c r="AO2" s="103" t="s">
         <v>299</v>
-      </c>
-      <c r="AN2" s="103" t="s">
-        <v>300</v>
-      </c>
-      <c r="AO2" s="103" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.25">
@@ -19405,7 +19414,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="105" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="D3" s="106">
         <v>11</v>
@@ -19507,7 +19516,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="108" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="D4" s="109">
         <v>28</v>
@@ -19616,7 +19625,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="105" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="D5" s="106">
         <v>90</v>
@@ -19727,7 +19736,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="108" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="D6" s="109">
         <v>89</v>
@@ -19849,7 +19858,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="105" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="D7" s="106">
         <v>8.1</v>
@@ -19959,7 +19968,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="108" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D8" s="109">
         <v>100</v>
@@ -20084,7 +20093,7 @@
         <v>7</v>
       </c>
       <c r="C9" s="105" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="D9" s="106">
         <v>92</v>
@@ -20206,7 +20215,7 @@
         <v>8</v>
       </c>
       <c r="C10" s="108" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="D10" s="109">
         <v>100</v>
@@ -20328,7 +20337,7 @@
         <v>9</v>
       </c>
       <c r="C11" s="105" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D11" s="106">
         <v>90</v>
@@ -20450,7 +20459,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="108" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D12" s="109">
         <v>91</v>
@@ -20571,7 +20580,7 @@
         <v>11</v>
       </c>
       <c r="C13" s="105" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D13" s="106">
         <v>87</v>
@@ -20693,7 +20702,7 @@
         <v>12</v>
       </c>
       <c r="C14" s="108" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D14" s="109">
         <v>87</v>
@@ -20802,7 +20811,7 @@
         <v>13</v>
       </c>
       <c r="C15" s="105" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="D15" s="106">
         <v>87</v>
@@ -20927,7 +20936,7 @@
         <v>14</v>
       </c>
       <c r="C16" s="108" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D16" s="109">
         <v>91</v>
@@ -21049,7 +21058,7 @@
         <v>15</v>
       </c>
       <c r="C17" s="105" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D17" s="106">
         <v>90</v>
@@ -21171,7 +21180,7 @@
         <v>16</v>
       </c>
       <c r="C18" s="108" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D18" s="109">
         <v>89</v>
@@ -21293,7 +21302,7 @@
         <v>17</v>
       </c>
       <c r="C19" s="105" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D19" s="106">
         <v>91</v>
@@ -21415,7 +21424,7 @@
         <v>18</v>
       </c>
       <c r="C20" s="108" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="D20" s="109">
         <v>99.5</v>
@@ -21540,7 +21549,7 @@
         <v>19</v>
       </c>
       <c r="C21" s="105" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D21" s="106">
         <v>87</v>
@@ -21662,7 +21671,7 @@
         <v>20</v>
       </c>
       <c r="C22" s="108" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D22" s="109">
         <v>88</v>
@@ -21784,7 +21793,7 @@
         <v>21</v>
       </c>
       <c r="C23" s="105" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D23" s="106">
         <v>88</v>
@@ -21903,13 +21912,13 @@
     </row>
     <row r="24" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B24" s="107">
         <v>22</v>
       </c>
       <c r="C24" s="108" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D24" s="109">
         <v>90</v>
@@ -22034,7 +22043,7 @@
         <v>23</v>
       </c>
       <c r="C25" s="105" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D25" s="106">
         <v>76</v>
@@ -22156,7 +22165,7 @@
         <v>24</v>
       </c>
       <c r="C26" s="108" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D26" s="109">
         <v>74</v>
@@ -22278,7 +22287,7 @@
         <v>25</v>
       </c>
       <c r="C27" s="105" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D27" s="106">
         <v>99.5</v>
@@ -22400,7 +22409,7 @@
         <v>26</v>
       </c>
       <c r="C28" s="108" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D28" s="109">
         <v>88</v>
@@ -22522,7 +22531,7 @@
         <v>27</v>
       </c>
       <c r="C29" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D29" s="106">
         <v>100</v>
@@ -22647,7 +22656,7 @@
         <v>28</v>
       </c>
       <c r="C30" s="108" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D30" s="109">
         <v>100</v>
@@ -22772,7 +22781,7 @@
         <v>29</v>
       </c>
       <c r="C31" s="105" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D31" s="106">
         <v>91</v>
@@ -22890,7 +22899,7 @@
         <v>30</v>
       </c>
       <c r="C32" s="108" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D32" s="109">
         <v>16.5</v>
@@ -23007,7 +23016,7 @@
         <v>31</v>
       </c>
       <c r="C33" s="105" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D33" s="106">
         <v>92</v>
@@ -23127,7 +23136,7 @@
         <v>32</v>
       </c>
       <c r="C34" s="108" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D34" s="109">
         <v>18</v>
@@ -23238,7 +23247,7 @@
         <v>33</v>
       </c>
       <c r="C35" s="105" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D35" s="106">
         <v>92</v>
@@ -23361,7 +23370,7 @@
         <v>34</v>
       </c>
       <c r="C36" s="108" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D36" s="109">
         <v>89</v>
@@ -23481,7 +23490,7 @@
         <v>35</v>
       </c>
       <c r="C37" s="105" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="D37" s="106">
         <v>89</v>
@@ -23606,7 +23615,7 @@
         <v>36</v>
       </c>
       <c r="C38" s="108" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D38" s="109">
         <v>89</v>
@@ -23728,7 +23737,7 @@
         <v>37</v>
       </c>
       <c r="C39" s="105" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="D39" s="106">
         <v>87</v>
@@ -23853,7 +23862,7 @@
         <v>38</v>
       </c>
       <c r="C40" s="108" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="D40" s="109">
         <v>87</v>
@@ -23978,7 +23987,7 @@
         <v>39</v>
       </c>
       <c r="C41" s="105" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="D41" s="106">
         <v>87</v>
@@ -24098,7 +24107,7 @@
         <v>40</v>
       </c>
       <c r="C42" s="108" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="D42" s="109">
         <v>100</v>
@@ -24220,7 +24229,7 @@
         <v>41</v>
       </c>
       <c r="C43" s="105" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D43" s="106">
         <v>95</v>
@@ -24342,7 +24351,7 @@
         <v>42</v>
       </c>
       <c r="C44" s="108" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D44" s="109">
         <v>88</v>
@@ -24461,7 +24470,7 @@
         <v>43</v>
       </c>
       <c r="C45" s="105" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D45" s="106">
         <v>88</v>
@@ -24583,7 +24592,7 @@
         <v>44</v>
       </c>
       <c r="C46" s="108" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D46" s="109">
         <v>88</v>
@@ -24708,7 +24717,7 @@
         <v>45</v>
       </c>
       <c r="C47" s="105" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="D47" s="106">
         <v>87</v>
@@ -24831,7 +24840,7 @@
         <v>46</v>
       </c>
       <c r="C48" s="108" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D48" s="109">
         <v>90</v>
@@ -24953,7 +24962,7 @@
         <v>47</v>
       </c>
       <c r="C49" s="105" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D49" s="106">
         <v>87</v>
@@ -25075,7 +25084,7 @@
         <v>48</v>
       </c>
       <c r="C50" s="108" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D50" s="109">
         <v>99</v>
@@ -25197,7 +25206,7 @@
         <v>49</v>
       </c>
       <c r="C51" s="105" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D51" s="106">
         <v>99</v>
@@ -25320,7 +25329,7 @@
         <v>50</v>
       </c>
       <c r="C52" s="108" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="D52" s="109">
         <v>5.5</v>
@@ -25442,7 +25451,7 @@
         <v>51</v>
       </c>
       <c r="C53" s="105" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D53" s="106">
         <v>98</v>
@@ -25567,7 +25576,7 @@
         <v>52</v>
       </c>
       <c r="C54" s="108" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="D54" s="109">
         <v>97</v>
@@ -25692,7 +25701,7 @@
         <v>53</v>
       </c>
       <c r="C55" s="105" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D55" s="106">
         <v>87</v>
@@ -25817,7 +25826,7 @@
         <v>54</v>
       </c>
       <c r="C56" s="108" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D56" s="109">
         <v>88</v>
@@ -25942,7 +25951,7 @@
         <v>55</v>
       </c>
       <c r="C57" s="105" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D57" s="106">
         <v>87</v>
@@ -26067,7 +26076,7 @@
         <v>56</v>
       </c>
       <c r="C58" s="108" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="D58" s="109">
         <v>87</v>
@@ -26190,7 +26199,7 @@
         <v>57</v>
       </c>
       <c r="C59" s="105" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="D59" s="106">
         <v>87</v>
@@ -26312,7 +26321,7 @@
         <v>58</v>
       </c>
       <c r="C60" s="108" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="D60" s="109">
         <v>12</v>
@@ -26594,16 +26603,16 @@
         <v>178</v>
       </c>
       <c r="B2" s="103" t="s">
+        <v>262</v>
+      </c>
+      <c r="C2" s="103" t="s">
+        <v>263</v>
+      </c>
+      <c r="D2" s="103" t="s">
         <v>264</v>
       </c>
-      <c r="C2" s="103" t="s">
-        <v>265</v>
-      </c>
-      <c r="D2" s="103" t="s">
-        <v>266</v>
-      </c>
       <c r="E2" s="103" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="F2" s="103" t="s">
         <v>189</v>
@@ -26612,85 +26621,85 @@
         <v>190</v>
       </c>
       <c r="H2" s="103" t="s">
+        <v>359</v>
+      </c>
+      <c r="I2" s="103" t="s">
+        <v>360</v>
+      </c>
+      <c r="J2" s="103" t="s">
         <v>361</v>
       </c>
-      <c r="I2" s="103" t="s">
-        <v>362</v>
-      </c>
-      <c r="J2" s="103" t="s">
-        <v>363</v>
-      </c>
       <c r="K2" s="103" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="L2" s="103" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="M2" s="103" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="N2" s="103" t="s">
         <v>195</v>
       </c>
       <c r="O2" s="103" t="s">
+        <v>362</v>
+      </c>
+      <c r="P2" s="103" t="s">
+        <v>363</v>
+      </c>
+      <c r="Q2" s="103" t="s">
         <v>364</v>
       </c>
-      <c r="P2" s="103" t="s">
+      <c r="R2" s="103" t="s">
         <v>365</v>
       </c>
-      <c r="Q2" s="103" t="s">
+      <c r="S2" s="103" t="s">
         <v>366</v>
       </c>
-      <c r="R2" s="103" t="s">
+      <c r="T2" s="103" t="s">
         <v>367</v>
       </c>
-      <c r="S2" s="103" t="s">
+      <c r="U2" s="103" t="s">
         <v>368</v>
       </c>
-      <c r="T2" s="103" t="s">
+      <c r="V2" s="103" t="s">
         <v>369</v>
       </c>
-      <c r="U2" s="103" t="s">
+      <c r="W2" s="103" t="s">
+        <v>272</v>
+      </c>
+      <c r="X2" s="103" t="s">
         <v>370</v>
       </c>
-      <c r="V2" s="103" t="s">
+      <c r="Y2" s="103" t="s">
+        <v>271</v>
+      </c>
+      <c r="Z2" s="103" t="s">
+        <v>269</v>
+      </c>
+      <c r="AA2" s="103" t="s">
         <v>371</v>
       </c>
-      <c r="W2" s="103" t="s">
-        <v>274</v>
-      </c>
-      <c r="X2" s="103" t="s">
+      <c r="AB2" s="103" t="s">
+        <v>289</v>
+      </c>
+      <c r="AC2" s="103" t="s">
+        <v>290</v>
+      </c>
+      <c r="AD2" s="103" t="s">
+        <v>291</v>
+      </c>
+      <c r="AE2" s="103" t="s">
+        <v>292</v>
+      </c>
+      <c r="AF2" s="103" t="s">
+        <v>293</v>
+      </c>
+      <c r="AG2" s="103" t="s">
         <v>372</v>
       </c>
-      <c r="Y2" s="103" t="s">
-        <v>273</v>
-      </c>
-      <c r="Z2" s="103" t="s">
-        <v>271</v>
-      </c>
-      <c r="AA2" s="103" t="s">
-        <v>373</v>
-      </c>
-      <c r="AB2" s="103" t="s">
-        <v>291</v>
-      </c>
-      <c r="AC2" s="103" t="s">
-        <v>292</v>
-      </c>
-      <c r="AD2" s="103" t="s">
+      <c r="AH2" s="103" t="s">
         <v>293</v>
-      </c>
-      <c r="AE2" s="103" t="s">
-        <v>294</v>
-      </c>
-      <c r="AF2" s="103" t="s">
-        <v>295</v>
-      </c>
-      <c r="AG2" s="103" t="s">
-        <v>374</v>
-      </c>
-      <c r="AH2" s="103" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -26698,7 +26707,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="106" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="D3" s="106">
         <v>50</v>
@@ -26769,7 +26778,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="109" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D4" s="109">
         <v>85</v>
@@ -26840,7 +26849,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="106" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="D5" s="106">
         <v>90</v>
@@ -26919,7 +26928,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="109" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="D6" s="109">
         <v>90</v>
@@ -26990,7 +26999,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="106" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="D7" s="106">
         <v>84</v>
@@ -27085,7 +27094,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="109" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="D8" s="109">
         <v>14</v>
@@ -27174,7 +27183,7 @@
         <v>7</v>
       </c>
       <c r="C9" s="106" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="D9" s="106">
         <v>85</v>
@@ -27245,7 +27254,7 @@
         <v>8</v>
       </c>
       <c r="C10" s="109" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="D10" s="109">
         <v>92</v>
@@ -27332,7 +27341,7 @@
         <v>9</v>
       </c>
       <c r="C11" s="106" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="D11" s="106">
         <v>92</v>
@@ -27431,7 +27440,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="109" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="D12" s="109">
         <v>92</v>
@@ -27514,7 +27523,7 @@
         <v>11</v>
       </c>
       <c r="C13" s="106" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D13" s="106">
         <v>92</v>
@@ -27597,7 +27606,7 @@
         <v>12</v>
       </c>
       <c r="C14" s="109" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="D14" s="109">
         <v>90</v>
@@ -27692,7 +27701,7 @@
         <v>13</v>
       </c>
       <c r="C15" s="106" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D15" s="106">
         <v>90</v>
@@ -27783,7 +27792,7 @@
         <v>14</v>
       </c>
       <c r="C16" s="109" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="D16" s="109">
         <v>99</v>
@@ -27862,7 +27871,7 @@
         <v>15</v>
       </c>
       <c r="C17" s="106" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="D17" s="106">
         <v>12</v>
@@ -27955,7 +27964,7 @@
         <v>16</v>
       </c>
       <c r="C18" s="109" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="D18" s="109">
         <v>90</v>
@@ -28030,7 +28039,7 @@
         <v>17</v>
       </c>
       <c r="C19" s="106" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D19" s="106">
         <v>15</v>
@@ -28119,7 +28128,7 @@
         <v>18</v>
       </c>
       <c r="C20" s="109" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="D20" s="109">
         <v>16</v>
@@ -28210,7 +28219,7 @@
         <v>19</v>
       </c>
       <c r="C21" s="106" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="D21" s="106">
         <v>90</v>
@@ -28301,7 +28310,7 @@
         <v>20</v>
       </c>
       <c r="C22" s="109" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="D22" s="109">
         <v>89</v>
@@ -28392,7 +28401,7 @@
         <v>21</v>
       </c>
       <c r="C23" s="106" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D23" s="106">
         <v>80</v>
@@ -28486,7 +28495,7 @@
         <v>22</v>
       </c>
       <c r="C24" s="109" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="D24" s="109">
         <v>85</v>
@@ -28585,7 +28594,7 @@
         <v>23</v>
       </c>
       <c r="C25" s="106" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="D25" s="106">
         <v>59</v>
@@ -28678,7 +28687,7 @@
         <v>24</v>
       </c>
       <c r="C26" s="109" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D26" s="109">
         <v>74</v>
@@ -28761,7 +28770,7 @@
         <v>25</v>
       </c>
       <c r="C27" s="106" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="D27" s="106">
         <v>93</v>
@@ -28832,7 +28841,7 @@
         <v>26</v>
       </c>
       <c r="C28" s="109" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="D28" s="109">
         <v>37</v>
@@ -28924,7 +28933,7 @@
         <v>27</v>
       </c>
       <c r="C29" s="106" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="D29" s="106">
         <v>87</v>
@@ -29006,7 +29015,7 @@
         <v>28</v>
       </c>
       <c r="C30" s="109" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="D30" s="109">
         <v>85</v>
@@ -29110,7 +29119,7 @@
         <v>29</v>
       </c>
       <c r="C31" s="106" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="D31" s="106">
         <v>87</v>
@@ -29197,7 +29206,7 @@
         <v>30</v>
       </c>
       <c r="C32" s="109" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D32" s="109">
         <v>87</v>
@@ -29288,7 +29297,7 @@
         <v>31</v>
       </c>
       <c r="C33" s="106" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="D33" s="106">
         <v>50</v>
@@ -29359,7 +29368,7 @@
         <v>32</v>
       </c>
       <c r="C34" s="109" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="D34" s="109">
         <v>82</v>
@@ -29446,7 +29455,7 @@
         <v>33</v>
       </c>
       <c r="C35" s="106" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="D35" s="106">
         <v>90</v>
@@ -29533,7 +29542,7 @@
         <v>34</v>
       </c>
       <c r="C36" s="109" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="D36" s="109">
         <v>88</v>
@@ -29624,7 +29633,7 @@
         <v>35</v>
       </c>
       <c r="C37" s="106" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="D37" s="106">
         <v>94</v>
@@ -29721,7 +29730,7 @@
         <v>36</v>
       </c>
       <c r="C38" s="109" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="D38" s="109">
         <v>92</v>
@@ -29814,7 +29823,7 @@
         <v>37</v>
       </c>
       <c r="C39" s="106" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="D39" s="106">
         <v>7</v>
@@ -29904,7 +29913,7 @@
         <v>38</v>
       </c>
       <c r="C40" s="109" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="D40" s="109">
         <v>90</v>
@@ -30001,7 +30010,7 @@
         <v>39</v>
       </c>
       <c r="C41" s="106" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="D41" s="106">
         <v>90</v>
@@ -30092,7 +30101,7 @@
         <v>40</v>
       </c>
       <c r="C42" s="109" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="D42" s="109">
         <v>37</v>
@@ -30189,7 +30198,7 @@
         <v>41</v>
       </c>
       <c r="C43" s="106" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="D43" s="106">
         <v>87</v>
@@ -30271,7 +30280,7 @@
         <v>42</v>
       </c>
       <c r="C44" s="109" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="D44" s="109">
         <v>87</v>
@@ -30372,7 +30381,7 @@
         <v>43</v>
       </c>
       <c r="C45" s="106" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D45" s="106">
         <v>86</v>
@@ -30469,7 +30478,7 @@
         <v>44</v>
       </c>
       <c r="C46" s="109" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D46" s="109">
         <v>12</v>
@@ -30567,7 +30576,7 @@
         <v>45</v>
       </c>
       <c r="C47" s="106" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D47" s="106">
         <v>93</v>
@@ -30660,7 +30669,7 @@
         <v>46</v>
       </c>
       <c r="C48" s="109" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="D48" s="109">
         <v>90</v>
@@ -30755,7 +30764,7 @@
         <v>47</v>
       </c>
       <c r="C49" s="106" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="D49" s="106">
         <v>90</v>
@@ -30848,7 +30857,7 @@
         <v>48</v>
       </c>
       <c r="C50" s="109" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D50" s="109">
         <v>87</v>
@@ -30941,7 +30950,7 @@
         <v>49</v>
       </c>
       <c r="C51" s="106" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D51" s="106">
         <v>13</v>
@@ -31027,13 +31036,13 @@
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B52" s="107">
         <v>50</v>
       </c>
       <c r="C52" s="109" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D52" s="109">
         <v>92</v>
@@ -31135,7 +31144,7 @@
         <v>51</v>
       </c>
       <c r="C53" s="106" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D53" s="106">
         <v>22</v>
@@ -31226,7 +31235,7 @@
         <v>52</v>
       </c>
       <c r="C54" s="109" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D54" s="109">
         <v>32</v>
@@ -31326,7 +31335,7 @@
         <v>53</v>
       </c>
       <c r="C55" s="106" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D55" s="106">
         <v>48</v>
@@ -31417,7 +31426,7 @@
         <v>54</v>
       </c>
       <c r="C56" s="109" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D56" s="109">
         <v>87</v>
@@ -31514,7 +31523,7 @@
         <v>55</v>
       </c>
       <c r="C57" s="106" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D57" s="106">
         <v>13</v>
@@ -31611,7 +31620,7 @@
         <v>56</v>
       </c>
       <c r="C58" s="109" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="D58" s="109">
         <v>8</v>
@@ -31705,7 +31714,7 @@
         <v>57</v>
       </c>
       <c r="C59" s="106" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="D59" s="106">
         <v>7</v>
@@ -31800,7 +31809,7 @@
         <v>58</v>
       </c>
       <c r="C60" s="109" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="D60" s="109">
         <v>6</v>
@@ -31895,7 +31904,7 @@
         <v>59</v>
       </c>
       <c r="C61" s="106" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="D61" s="106">
         <v>12</v>
@@ -31993,7 +32002,7 @@
         <v>60</v>
       </c>
       <c r="C62" s="109" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D62" s="109">
         <v>91</v>
@@ -32088,7 +32097,7 @@
         <v>61</v>
       </c>
       <c r="C63" s="106" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="D63" s="106">
         <v>91</v>
@@ -32181,7 +32190,7 @@
         <v>62</v>
       </c>
       <c r="C64" s="109" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="D64" s="109">
         <v>6</v>
@@ -32271,7 +32280,7 @@
         <v>63</v>
       </c>
       <c r="C65" s="106" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="D65" s="106">
         <v>23</v>
@@ -32370,7 +32379,7 @@
         <v>64</v>
       </c>
       <c r="C66" s="109" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="D66" s="109">
         <v>14</v>
@@ -32462,7 +32471,7 @@
         <v>65</v>
       </c>
       <c r="C67" s="106" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="D67" s="106">
         <v>90</v>
@@ -32554,7 +32563,7 @@
         <v>66</v>
       </c>
       <c r="C68" s="109" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="D68" s="109">
         <v>94</v>
@@ -32651,7 +32660,7 @@
         <v>67</v>
       </c>
       <c r="C69" s="106" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="D69" s="106">
         <v>94</v>
@@ -32750,7 +32759,7 @@
         <v>68</v>
       </c>
       <c r="C70" s="109" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="D70" s="109">
         <v>21</v>
@@ -32827,7 +32836,7 @@
         <v>69</v>
       </c>
       <c r="C71" s="106" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="D71" s="106">
         <v>90</v>
@@ -32929,7 +32938,7 @@
         <v>70</v>
       </c>
       <c r="C72" s="109" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="D72" s="109">
         <v>90</v>
@@ -33031,7 +33040,7 @@
         <v>71</v>
       </c>
       <c r="C73" s="106" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="D73" s="106">
         <v>93</v>
@@ -33130,7 +33139,7 @@
         <v>72</v>
       </c>
       <c r="C74" s="109" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="D74" s="109">
         <v>35</v>
@@ -33211,7 +33220,7 @@
         <v>73</v>
       </c>
       <c r="C75" s="106" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D75" s="106">
         <v>89</v>
@@ -33304,7 +33313,7 @@
         <v>74</v>
       </c>
       <c r="C76" s="109" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="D76" s="109">
         <v>87</v>
@@ -33399,7 +33408,7 @@
         <v>75</v>
       </c>
       <c r="C77" s="106" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="D77" s="106">
         <v>9</v>
@@ -33493,7 +33502,7 @@
         <v>76</v>
       </c>
       <c r="C78" s="109" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="D78" s="109">
         <v>87</v>
@@ -33587,7 +33596,7 @@
         <v>77</v>
       </c>
       <c r="C79" s="106" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="D79" s="106">
         <v>87</v>
@@ -33685,7 +33694,7 @@
         <v>78</v>
       </c>
       <c r="C80" s="109" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="D80" s="109">
         <v>87</v>
@@ -33782,7 +33791,7 @@
         <v>79</v>
       </c>
       <c r="C81" s="106" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="D81" s="106">
         <v>78</v>
@@ -33869,7 +33878,7 @@
         <v>80</v>
       </c>
       <c r="C82" s="109" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="D82" s="109">
         <v>93</v>
@@ -33940,7 +33949,7 @@
         <v>81</v>
       </c>
       <c r="C83" s="106" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="D83" s="106">
         <v>90</v>
@@ -34027,7 +34036,7 @@
         <v>82</v>
       </c>
       <c r="C84" s="109" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="D84" s="109">
         <v>94</v>
@@ -34098,7 +34107,7 @@
         <v>83</v>
       </c>
       <c r="C85" s="106" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="D85" s="106">
         <v>90</v>
@@ -34185,7 +34194,7 @@
         <v>84</v>
       </c>
       <c r="C86" s="109" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="D86" s="109">
         <v>90</v>
@@ -34268,7 +34277,7 @@
         <v>85</v>
       </c>
       <c r="C87" s="106" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="D87" s="106">
         <v>24</v>
@@ -34357,7 +34366,7 @@
         <v>86</v>
       </c>
       <c r="C88" s="109" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="D88" s="109">
         <v>14</v>
@@ -34442,7 +34451,7 @@
         <v>87</v>
       </c>
       <c r="C89" s="106" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="D89" s="106">
         <v>27</v>
@@ -34538,7 +34547,7 @@
         <v>88</v>
       </c>
       <c r="C90" s="109" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="D90" s="109">
         <v>75</v>
@@ -34623,7 +34632,7 @@
         <v>89</v>
       </c>
       <c r="C91" s="106" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="D91" s="106">
         <v>19</v>
@@ -34708,7 +34717,7 @@
         <v>90</v>
       </c>
       <c r="C92" s="109" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="D92" s="109">
         <v>91</v>
@@ -34808,7 +34817,7 @@
         <v>91</v>
       </c>
       <c r="C93" s="106" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="D93" s="106">
         <v>90</v>
@@ -34904,7 +34913,7 @@
         <v>92</v>
       </c>
       <c r="C94" s="109" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="D94" s="109">
         <v>87</v>
@@ -35000,7 +35009,7 @@
         <v>93</v>
       </c>
       <c r="C95" s="106" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D95" s="106">
         <v>87</v>
@@ -35097,7 +35106,7 @@
         <v>94</v>
       </c>
       <c r="C96" s="109" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="D96" s="109">
         <v>87</v>
@@ -35184,7 +35193,7 @@
         <v>95</v>
       </c>
       <c r="C97" s="106" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="D97" s="106">
         <v>92</v>
@@ -35277,7 +35286,7 @@
         <v>96</v>
       </c>
       <c r="C98" s="109" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="D98" s="109">
         <v>92</v>
@@ -35372,7 +35381,7 @@
         <v>97</v>
       </c>
       <c r="C99" s="106" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="D99" s="106">
         <v>93</v>
@@ -35463,7 +35472,7 @@
         <v>98</v>
       </c>
       <c r="C100" s="109" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="D100" s="109">
         <v>92</v>
@@ -35559,7 +35568,7 @@
         <v>99</v>
       </c>
       <c r="C101" s="106" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="D101" s="106">
         <v>92</v>
@@ -35654,7 +35663,7 @@
         <v>100</v>
       </c>
       <c r="C102" s="109" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="D102" s="109">
         <v>87</v>
@@ -35745,7 +35754,7 @@
         <v>101</v>
       </c>
       <c r="C103" s="106" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="D103" s="106">
         <v>50</v>
@@ -35824,7 +35833,7 @@
         <v>102</v>
       </c>
       <c r="C104" s="109" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="D104" s="109">
         <v>88</v>
@@ -35917,7 +35926,7 @@
         <v>103</v>
       </c>
       <c r="C105" s="106" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="D105" s="106">
         <v>50</v>
@@ -36002,7 +36011,7 @@
         <v>104</v>
       </c>
       <c r="C106" s="109" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="D106" s="109">
         <v>89</v>
@@ -36073,7 +36082,7 @@
         <v>105</v>
       </c>
       <c r="C107" s="106" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D107" s="106">
         <v>98</v>
@@ -36154,7 +36163,7 @@
         <v>106</v>
       </c>
       <c r="C108" s="109" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D108" s="109">
         <v>93</v>
@@ -36221,7 +36230,7 @@
         <v>107</v>
       </c>
       <c r="C109" s="106" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="D109" s="106">
         <v>90</v>
@@ -36292,7 +36301,7 @@
         <v>108</v>
       </c>
       <c r="C110" s="109" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D110" s="109">
         <v>85</v>
@@ -36366,7 +36375,7 @@
         <v>109</v>
       </c>
       <c r="C111" s="106" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="D111" s="106">
         <v>90</v>
@@ -36459,7 +36468,7 @@
         <v>110</v>
       </c>
       <c r="C112" s="109" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="D112" s="109">
         <v>87</v>
@@ -36549,7 +36558,7 @@
         <v>111</v>
       </c>
       <c r="C113" s="106" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="D113" s="106">
         <v>87</v>
@@ -36649,7 +36658,7 @@
         <v>112</v>
       </c>
       <c r="C114" s="109" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="D114" s="109">
         <v>87</v>
@@ -36748,7 +36757,7 @@
         <v>113</v>
       </c>
       <c r="C115" s="106" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="D115" s="106">
         <v>87</v>
@@ -36827,7 +36836,7 @@
         <v>114</v>
       </c>
       <c r="C116" s="109" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="D116" s="109">
         <v>19</v>
@@ -36925,7 +36934,7 @@
         <v>115</v>
       </c>
       <c r="C117" s="106" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="D117" s="106">
         <v>87</v>
@@ -37024,7 +37033,7 @@
         <v>116</v>
       </c>
       <c r="C118" s="109" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="D118" s="109">
         <v>31</v>
@@ -37107,7 +37116,7 @@
         <v>117</v>
       </c>
       <c r="C119" s="106" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D119" s="106">
         <v>31</v>
@@ -37190,7 +37199,7 @@
         <v>118</v>
       </c>
       <c r="C120" s="109" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="D120" s="109">
         <v>18</v>
@@ -37288,13 +37297,13 @@
   <sheetData>
     <row r="2" spans="2:31" ht="57.75" x14ac:dyDescent="0.25">
       <c r="B2" s="103" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C2" s="103" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D2" s="103" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="E2" s="103" t="s">
         <v>189</v>
@@ -37303,70 +37312,70 @@
         <v>190</v>
       </c>
       <c r="G2" s="103" t="s">
+        <v>491</v>
+      </c>
+      <c r="H2" s="103" t="s">
+        <v>492</v>
+      </c>
+      <c r="I2" s="103" t="s">
         <v>493</v>
       </c>
-      <c r="H2" s="103" t="s">
+      <c r="J2" s="103" t="s">
         <v>494</v>
       </c>
-      <c r="I2" s="103" t="s">
+      <c r="K2" s="103" t="s">
         <v>495</v>
       </c>
-      <c r="J2" s="103" t="s">
+      <c r="L2" s="103" t="s">
         <v>496</v>
       </c>
-      <c r="K2" s="103" t="s">
+      <c r="M2" s="103" t="s">
         <v>497</v>
       </c>
-      <c r="L2" s="103" t="s">
+      <c r="N2" s="103" t="s">
         <v>498</v>
       </c>
-      <c r="M2" s="103" t="s">
+      <c r="O2" s="103" t="s">
         <v>499</v>
       </c>
-      <c r="N2" s="103" t="s">
+      <c r="P2" s="103" t="s">
         <v>500</v>
       </c>
-      <c r="O2" s="103" t="s">
+      <c r="Q2" s="103" t="s">
         <v>501</v>
       </c>
-      <c r="P2" s="103" t="s">
+      <c r="R2" s="103" t="s">
         <v>502</v>
       </c>
-      <c r="Q2" s="103" t="s">
+      <c r="S2" s="103" t="s">
         <v>503</v>
       </c>
-      <c r="R2" s="103" t="s">
+      <c r="T2" s="103" t="s">
         <v>504</v>
       </c>
-      <c r="S2" s="103" t="s">
+      <c r="U2" s="103" t="s">
+        <v>269</v>
+      </c>
+      <c r="V2" s="103" t="s">
         <v>505</v>
       </c>
-      <c r="T2" s="103" t="s">
-        <v>506</v>
-      </c>
-      <c r="U2" s="103" t="s">
-        <v>271</v>
-      </c>
-      <c r="V2" s="103" t="s">
-        <v>507</v>
-      </c>
       <c r="W2" s="103" t="s">
+        <v>289</v>
+      </c>
+      <c r="X2" s="103" t="s">
+        <v>290</v>
+      </c>
+      <c r="Y2" s="103" t="s">
         <v>291</v>
       </c>
-      <c r="X2" s="103" t="s">
+      <c r="Z2" s="103" t="s">
         <v>292</v>
       </c>
-      <c r="Y2" s="103" t="s">
+      <c r="AA2" s="103" t="s">
         <v>293</v>
       </c>
-      <c r="Z2" s="103" t="s">
-        <v>294</v>
-      </c>
-      <c r="AA2" s="103" t="s">
-        <v>295</v>
-      </c>
       <c r="AB2" s="103" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="3" spans="2:31" x14ac:dyDescent="0.25">
@@ -37374,7 +37383,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="110" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="D3" s="106">
         <v>9.4</v>
@@ -37443,7 +37452,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="111" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="D4" s="109">
         <v>9.4</v>
@@ -37512,7 +37521,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="110" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="D5" s="106">
         <v>6.1</v>
@@ -37581,7 +37590,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="111" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="D6" s="109">
         <v>9.4</v>
@@ -37650,7 +37659,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="110" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="D7" s="106">
         <v>10.5</v>
@@ -37719,7 +37728,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="111" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="D8" s="109">
         <v>11.1</v>
@@ -37788,7 +37797,7 @@
         <v>7</v>
       </c>
       <c r="C9" s="110" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="D9" s="106">
         <v>11</v>
@@ -37862,7 +37871,7 @@
         <v>8</v>
       </c>
       <c r="C10" s="111" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="D10" s="109">
         <v>10.1</v>
@@ -37934,7 +37943,7 @@
         <v>9</v>
       </c>
       <c r="C11" s="110" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D11" s="106">
         <v>9.5</v>
@@ -38002,7 +38011,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="111" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D12" s="109">
         <v>10.5</v>
@@ -38078,7 +38087,7 @@
         <v>11</v>
       </c>
       <c r="C13" s="110" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D13" s="106">
         <v>10.8</v>
@@ -38152,7 +38161,7 @@
         <v>12</v>
       </c>
       <c r="C14" s="111" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="D14" s="109">
         <v>11.5</v>
@@ -38226,7 +38235,7 @@
         <v>13</v>
       </c>
       <c r="C15" s="110" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="D15" s="106">
         <v>9.8000000000000007</v>
@@ -38313,7 +38322,7 @@
         <v>14</v>
       </c>
       <c r="C16" s="111" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="D16" s="109">
         <v>9.8000000000000007</v>
@@ -38400,7 +38409,7 @@
         <v>15</v>
       </c>
       <c r="C17" s="110" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="D17" s="106">
         <v>9.3000000000000007</v>
@@ -38485,7 +38494,7 @@
         <v>16</v>
       </c>
       <c r="C18" s="111" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="D18" s="109">
         <v>9.3000000000000007</v>
@@ -38570,7 +38579,7 @@
         <v>17</v>
       </c>
       <c r="C19" s="110" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="D19" s="106">
         <v>10.199999999999999</v>
@@ -38655,7 +38664,7 @@
         <v>18</v>
       </c>
       <c r="C20" s="111" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="D20" s="109">
         <v>10.199999999999999</v>
@@ -38740,7 +38749,7 @@
         <v>19</v>
       </c>
       <c r="C21" s="110" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="D21" s="106">
         <v>10.9</v>
@@ -38823,7 +38832,7 @@
         <v>20</v>
       </c>
       <c r="C22" s="111" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="D22" s="109">
         <v>11.7</v>
@@ -38904,7 +38913,7 @@
         <v>21</v>
       </c>
       <c r="C23" s="110" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="D23" s="106">
         <v>8</v>
@@ -38983,7 +38992,7 @@
         <v>22</v>
       </c>
       <c r="C24" s="111" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="D24" s="109">
         <v>9.1999999999999993</v>
@@ -39066,7 +39075,7 @@
         <v>23</v>
       </c>
       <c r="C25" s="110" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="D25" s="106">
         <v>10.1</v>
@@ -39149,7 +39158,7 @@
         <v>24</v>
       </c>
       <c r="C26" s="111" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="D26" s="109">
         <v>10.3</v>
@@ -39232,7 +39241,7 @@
         <v>25</v>
       </c>
       <c r="C27" s="110" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="D27" s="106">
         <v>10.3</v>
@@ -39315,7 +39324,7 @@
         <v>26</v>
       </c>
       <c r="C28" s="111" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D28" s="109">
         <v>10.1</v>
@@ -39396,7 +39405,7 @@
         <v>27</v>
       </c>
       <c r="C29" s="110" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="D29" s="106">
         <v>10.199999999999999</v>
@@ -39477,7 +39486,7 @@
         <v>28</v>
       </c>
       <c r="C30" s="111" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="D30" s="109">
         <v>10.1</v>
@@ -39558,7 +39567,7 @@
         <v>29</v>
       </c>
       <c r="C31" s="110" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="D31" s="106">
         <v>10.199999999999999</v>
@@ -39641,7 +39650,7 @@
         <v>30</v>
       </c>
       <c r="C32" s="111" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="D32" s="109">
         <v>9.9</v>
@@ -39722,7 +39731,7 @@
         <v>31</v>
       </c>
       <c r="C33" s="110" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="D33" s="106">
         <v>9.1</v>
@@ -39803,7 +39812,7 @@
         <v>32</v>
       </c>
       <c r="C34" s="111" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="D34" s="109">
         <v>9.3000000000000007</v>
@@ -39884,7 +39893,7 @@
         <v>33</v>
       </c>
       <c r="C35" s="110" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="D35" s="106">
         <v>9.1999999999999993</v>
@@ -39965,7 +39974,7 @@
         <v>34</v>
       </c>
       <c r="C36" s="111" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="D36" s="109">
         <v>9.4</v>
@@ -40038,7 +40047,7 @@
         <v>35</v>
       </c>
       <c r="C37" s="110" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="D37" s="106">
         <v>10.199999999999999</v>
@@ -40125,7 +40134,7 @@
         <v>36</v>
       </c>
       <c r="C38" s="111" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="D38" s="109">
         <v>10.199999999999999</v>
@@ -40212,7 +40221,7 @@
         <v>37</v>
       </c>
       <c r="C39" s="110" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="D39" s="106">
         <v>9.8000000000000007</v>
@@ -40297,7 +40306,7 @@
         <v>38</v>
       </c>
       <c r="C40" s="111" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="D40" s="109">
         <v>9.8000000000000007</v>
@@ -40382,7 +40391,7 @@
         <v>39</v>
       </c>
       <c r="C41" s="110" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="D41" s="106">
         <v>10.7</v>
@@ -40467,7 +40476,7 @@
         <v>40</v>
       </c>
       <c r="C42" s="111" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="D42" s="109">
         <v>10.7</v>
@@ -40552,7 +40561,7 @@
         <v>41</v>
       </c>
       <c r="C43" s="110" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="D43" s="106">
         <v>9.9</v>
@@ -40637,7 +40646,7 @@
         <v>42</v>
       </c>
       <c r="C44" s="111" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="D44" s="109">
         <v>9.9</v>
@@ -40722,7 +40731,7 @@
         <v>43</v>
       </c>
       <c r="C45" s="110" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="D45" s="106">
         <v>9.5</v>
@@ -40807,7 +40816,7 @@
         <v>44</v>
       </c>
       <c r="C46" s="111" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="D46" s="109">
         <v>9.3000000000000007</v>
@@ -40892,7 +40901,7 @@
         <v>45</v>
       </c>
       <c r="C47" s="110" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="D47" s="106">
         <v>10.4</v>
@@ -40977,7 +40986,7 @@
         <v>46</v>
       </c>
       <c r="C48" s="111" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="D48" s="109">
         <v>10.4</v>
@@ -41062,7 +41071,7 @@
         <v>47</v>
       </c>
       <c r="C49" s="110" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="D49" s="106">
         <v>10.199999999999999</v>
@@ -41149,7 +41158,7 @@
         <v>48</v>
       </c>
       <c r="C50" s="111" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="D50" s="109">
         <v>10.199999999999999</v>
@@ -41236,7 +41245,7 @@
         <v>49</v>
       </c>
       <c r="C51" s="110" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="D51" s="106">
         <v>9.5</v>
@@ -41321,7 +41330,7 @@
         <v>50</v>
       </c>
       <c r="C52" s="111" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="D52" s="109">
         <v>9.5</v>
@@ -41406,7 +41415,7 @@
         <v>51</v>
       </c>
       <c r="C53" s="110" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="D53" s="106">
         <v>11</v>
@@ -41491,7 +41500,7 @@
         <v>52</v>
       </c>
       <c r="C54" s="111" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="D54" s="109">
         <v>11</v>
@@ -41576,7 +41585,7 @@
         <v>53</v>
       </c>
       <c r="C55" s="110" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="D55" s="106">
         <v>10.6</v>
@@ -41661,7 +41670,7 @@
         <v>54</v>
       </c>
       <c r="C56" s="111" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="D56" s="109">
         <v>10.6</v>
@@ -41746,7 +41755,7 @@
         <v>55</v>
       </c>
       <c r="C57" s="110" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="D57" s="106">
         <v>10.199999999999999</v>
@@ -41831,7 +41840,7 @@
         <v>56</v>
       </c>
       <c r="C58" s="111" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="D58" s="109">
         <v>10.199999999999999</v>
@@ -41916,7 +41925,7 @@
         <v>57</v>
       </c>
       <c r="C59" s="110" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="D59" s="106">
         <v>11</v>
@@ -42001,7 +42010,7 @@
         <v>58</v>
       </c>
       <c r="C60" s="111" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="D60" s="109">
         <v>11</v>
@@ -42086,7 +42095,7 @@
         <v>59</v>
       </c>
       <c r="C61" s="110" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="D61" s="106">
         <v>10.5</v>
@@ -42183,43 +42192,43 @@
         <v>178</v>
       </c>
       <c r="B2" s="103" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C2" s="103" t="s">
+        <v>565</v>
+      </c>
+      <c r="D2" s="103" t="s">
+        <v>566</v>
+      </c>
+      <c r="E2" s="103" t="s">
         <v>567</v>
       </c>
-      <c r="D2" s="103" t="s">
+      <c r="F2" s="103" t="s">
         <v>568</v>
       </c>
-      <c r="E2" s="103" t="s">
+      <c r="G2" s="103" t="s">
         <v>569</v>
       </c>
-      <c r="F2" s="103" t="s">
+      <c r="H2" s="103" t="s">
         <v>570</v>
       </c>
-      <c r="G2" s="103" t="s">
+      <c r="I2" s="103" t="s">
         <v>571</v>
       </c>
-      <c r="H2" s="103" t="s">
+      <c r="J2" s="103" t="s">
         <v>572</v>
       </c>
-      <c r="I2" s="103" t="s">
+      <c r="K2" s="103" t="s">
         <v>573</v>
       </c>
-      <c r="J2" s="103" t="s">
+      <c r="L2" s="103" t="s">
         <v>574</v>
       </c>
-      <c r="K2" s="103" t="s">
+      <c r="M2" s="103" t="s">
         <v>575</v>
       </c>
-      <c r="L2" s="103" t="s">
+      <c r="N2" s="103" t="s">
         <v>576</v>
-      </c>
-      <c r="M2" s="103" t="s">
-        <v>577</v>
-      </c>
-      <c r="N2" s="103" t="s">
-        <v>578</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -42227,7 +42236,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="106" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="D3" s="106">
         <v>50</v>
@@ -42266,7 +42275,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="109" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="D4" s="109">
         <v>85</v>
@@ -42305,7 +42314,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="106" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="D5" s="106">
         <v>90</v>
@@ -42346,7 +42355,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="109" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="D6" s="109">
         <v>90</v>
@@ -42387,7 +42396,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="106" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D7" s="106">
         <v>90</v>
@@ -42428,7 +42437,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="109" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="D8" s="109">
         <v>90</v>
@@ -42469,7 +42478,7 @@
         <v>7</v>
       </c>
       <c r="C9" s="106" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="D9" s="106">
         <v>8</v>
@@ -42510,7 +42519,7 @@
         <v>8</v>
       </c>
       <c r="C10" s="109" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="D10" s="109">
         <v>91</v>
@@ -42551,7 +42560,7 @@
         <v>9</v>
       </c>
       <c r="C11" s="106" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="D11" s="106">
         <v>94</v>
@@ -42592,7 +42601,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="109" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="D12" s="109">
         <v>91</v>
@@ -42633,7 +42642,7 @@
         <v>11</v>
       </c>
       <c r="C13" s="106" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="D13" s="106">
         <v>90</v>
@@ -42674,7 +42683,7 @@
         <v>12</v>
       </c>
       <c r="C14" s="109" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="D14" s="109">
         <v>87</v>
@@ -42713,7 +42722,7 @@
         <v>13</v>
       </c>
       <c r="C15" s="106" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="D15" s="106">
         <v>87</v>
@@ -42754,7 +42763,7 @@
         <v>14</v>
       </c>
       <c r="C16" s="109" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="D16" s="109">
         <v>87</v>
@@ -42795,7 +42804,7 @@
         <v>15</v>
       </c>
       <c r="C17" s="106" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="D17" s="106">
         <v>82</v>
@@ -42834,7 +42843,7 @@
         <v>16</v>
       </c>
       <c r="C18" s="109" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="D18" s="109">
         <v>87</v>
@@ -42869,7 +42878,7 @@
         <v>17</v>
       </c>
       <c r="C19" s="106" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="D19" s="106">
         <v>87</v>
@@ -42910,7 +42919,7 @@
         <v>18</v>
       </c>
       <c r="C20" s="109" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="D20" s="109">
         <v>93</v>
@@ -42951,7 +42960,7 @@
         <v>19</v>
       </c>
       <c r="C21" s="106" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="D21" s="106">
         <v>90</v>
@@ -42992,7 +43001,7 @@
         <v>20</v>
       </c>
       <c r="C22" s="109" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="D22" s="109">
         <v>87</v>
@@ -43033,7 +43042,7 @@
         <v>21</v>
       </c>
       <c r="C23" s="106" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="D23" s="106">
         <v>87</v>
@@ -43074,7 +43083,7 @@
         <v>22</v>
       </c>
       <c r="C24" s="109" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="D24" s="109">
         <v>92</v>
@@ -43115,7 +43124,7 @@
         <v>23</v>
       </c>
       <c r="C25" s="106" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="D25" s="106">
         <v>9</v>
@@ -43156,7 +43165,7 @@
         <v>24</v>
       </c>
       <c r="C26" s="109" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="D26" s="109">
         <v>12</v>
@@ -43197,7 +43206,7 @@
         <v>25</v>
       </c>
       <c r="C27" s="106" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="D27" s="106">
         <v>91</v>
@@ -43238,7 +43247,7 @@
         <v>26</v>
       </c>
       <c r="C28" s="109" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="D28" s="109">
         <v>90</v>
@@ -43279,7 +43288,7 @@
         <v>27</v>
       </c>
       <c r="C29" s="106" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="D29" s="106">
         <v>94</v>
@@ -43320,7 +43329,7 @@
         <v>28</v>
       </c>
       <c r="C30" s="109" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="D30" s="109">
         <v>94</v>
@@ -43361,7 +43370,7 @@
         <v>29</v>
       </c>
       <c r="C31" s="106" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="D31" s="106">
         <v>93</v>
@@ -43402,7 +43411,7 @@
         <v>30</v>
       </c>
       <c r="C32" s="109" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="D32" s="109">
         <v>87</v>
@@ -43443,7 +43452,7 @@
         <v>31</v>
       </c>
       <c r="C33" s="106" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="D33" s="106">
         <v>89</v>
@@ -43484,7 +43493,7 @@
         <v>32</v>
       </c>
       <c r="C34" s="109" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="D34" s="109">
         <v>87</v>
@@ -43525,7 +43534,7 @@
         <v>33</v>
       </c>
       <c r="C35" s="106" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="D35" s="106">
         <v>87</v>
@@ -43566,7 +43575,7 @@
         <v>34</v>
       </c>
       <c r="C36" s="109" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="D36" s="109">
         <v>87</v>
@@ -43607,7 +43616,7 @@
         <v>35</v>
       </c>
       <c r="C37" s="106" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="D37" s="106">
         <v>78</v>
@@ -43648,7 +43657,7 @@
         <v>36</v>
       </c>
       <c r="C38" s="109" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="D38" s="109">
         <v>75</v>
@@ -43689,7 +43698,7 @@
         <v>37</v>
       </c>
       <c r="C39" s="106" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="D39" s="106">
         <v>91</v>
@@ -43730,7 +43739,7 @@
         <v>38</v>
       </c>
       <c r="C40" s="109" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="D40" s="109">
         <v>90</v>
@@ -43771,7 +43780,7 @@
         <v>39</v>
       </c>
       <c r="C41" s="106" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="D41" s="106">
         <v>87</v>
@@ -43812,7 +43821,7 @@
         <v>40</v>
       </c>
       <c r="C42" s="109" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="D42" s="109">
         <v>87</v>
@@ -43853,7 +43862,7 @@
         <v>41</v>
       </c>
       <c r="C43" s="106" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="D43" s="106">
         <v>92</v>
@@ -43894,7 +43903,7 @@
         <v>42</v>
       </c>
       <c r="C44" s="109" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="D44" s="109">
         <v>92</v>
@@ -43935,7 +43944,7 @@
         <v>43</v>
       </c>
       <c r="C45" s="106" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="D45" s="106">
         <v>87</v>
@@ -43976,7 +43985,7 @@
         <v>44</v>
       </c>
       <c r="C46" s="109" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="D46" s="109">
         <v>90</v>
@@ -44017,7 +44026,7 @@
         <v>45</v>
       </c>
       <c r="C47" s="106" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="D47" s="106">
         <v>90</v>
@@ -44058,7 +44067,7 @@
         <v>46</v>
       </c>
       <c r="C48" s="109" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="D48" s="109">
         <v>88</v>
@@ -44099,7 +44108,7 @@
         <v>47</v>
       </c>
       <c r="C49" s="106" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="D49" s="106">
         <v>89</v>
@@ -44138,7 +44147,7 @@
         <v>48</v>
       </c>
       <c r="C50" s="109" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="D50" s="109">
         <v>100</v>
@@ -44179,7 +44188,7 @@
         <v>49</v>
       </c>
       <c r="C51" s="106" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="D51" s="106">
         <v>87</v>
@@ -44220,7 +44229,7 @@
         <v>50</v>
       </c>
       <c r="C52" s="109" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="D52" s="109">
         <v>87</v>
@@ -44261,7 +44270,7 @@
         <v>51</v>
       </c>
       <c r="C53" s="106" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="D53" s="106">
         <v>87</v>
@@ -44302,7 +44311,7 @@
         <v>52</v>
       </c>
       <c r="C54" s="109" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="D54" s="109">
         <v>87</v>
@@ -44341,7 +44350,7 @@
         <v>53</v>
       </c>
       <c r="C55" s="106" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D55" s="106">
         <v>87</v>
@@ -44382,7 +44391,7 @@
         <v>54</v>
       </c>
       <c r="C56" s="109" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="D56" s="109">
         <v>87</v>
@@ -44494,64 +44503,64 @@
         <v>178</v>
       </c>
       <c r="B2" s="103" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C2" s="103" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D2" s="103" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="E2" s="103" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="F2" s="103" t="s">
+        <v>628</v>
+      </c>
+      <c r="G2" s="103" t="s">
+        <v>629</v>
+      </c>
+      <c r="H2" s="103" t="s">
         <v>630</v>
       </c>
-      <c r="G2" s="103" t="s">
+      <c r="I2" s="103" t="s">
         <v>631</v>
       </c>
-      <c r="H2" s="103" t="s">
+      <c r="J2" s="103" t="s">
         <v>632</v>
       </c>
-      <c r="I2" s="103" t="s">
+      <c r="K2" s="103" t="s">
         <v>633</v>
       </c>
-      <c r="J2" s="103" t="s">
+      <c r="L2" s="103" t="s">
+        <v>271</v>
+      </c>
+      <c r="M2" s="103" t="s">
+        <v>272</v>
+      </c>
+      <c r="N2" s="103" t="s">
+        <v>268</v>
+      </c>
+      <c r="O2" s="103" t="s">
+        <v>289</v>
+      </c>
+      <c r="P2" s="103" t="s">
         <v>634</v>
       </c>
-      <c r="K2" s="103" t="s">
+      <c r="Q2" s="103" t="s">
         <v>635</v>
       </c>
-      <c r="L2" s="103" t="s">
-        <v>273</v>
-      </c>
-      <c r="M2" s="103" t="s">
-        <v>274</v>
-      </c>
-      <c r="N2" s="103" t="s">
-        <v>270</v>
-      </c>
-      <c r="O2" s="103" t="s">
-        <v>291</v>
-      </c>
-      <c r="P2" s="103" t="s">
+      <c r="R2" s="103" t="s">
+        <v>292</v>
+      </c>
+      <c r="S2" s="103" t="s">
+        <v>293</v>
+      </c>
+      <c r="T2" s="103" t="s">
         <v>636</v>
       </c>
-      <c r="Q2" s="103" t="s">
+      <c r="U2" s="103" t="s">
         <v>637</v>
-      </c>
-      <c r="R2" s="103" t="s">
-        <v>294</v>
-      </c>
-      <c r="S2" s="103" t="s">
-        <v>295</v>
-      </c>
-      <c r="T2" s="103" t="s">
-        <v>638</v>
-      </c>
-      <c r="U2" s="103" t="s">
-        <v>639</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
@@ -44562,7 +44571,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="106" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="D3" s="106">
         <v>99</v>
@@ -44624,7 +44633,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="109" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="D4" s="109">
         <v>99</v>
@@ -44686,7 +44695,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="106" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="D5" s="106">
         <v>100</v>
@@ -44748,7 +44757,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="109" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="D6" s="109">
         <v>100</v>
@@ -44810,7 +44819,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="106" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="D7" s="106">
         <v>100</v>
@@ -44875,7 +44884,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="109" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="D8" s="109">
         <v>92</v>
@@ -44937,7 +44946,7 @@
         <v>7</v>
       </c>
       <c r="C9" s="106" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="D9" s="106">
         <v>92</v>
@@ -44999,7 +45008,7 @@
         <v>8</v>
       </c>
       <c r="C10" s="109" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="D10" s="109">
         <v>92</v>
@@ -45061,7 +45070,7 @@
         <v>9</v>
       </c>
       <c r="C11" s="106" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="D11" s="106">
         <v>100</v>
@@ -45126,7 +45135,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="109" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="D12" s="109">
         <v>87</v>
@@ -45188,7 +45197,7 @@
         <v>11</v>
       </c>
       <c r="C13" s="106" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="D13" s="106">
         <v>87</v>
@@ -45250,7 +45259,7 @@
         <v>12</v>
       </c>
       <c r="C14" s="109" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D14" s="109">
         <v>87</v>
@@ -45312,7 +45321,7 @@
         <v>13</v>
       </c>
       <c r="C15" s="106" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D15" s="106">
         <v>87</v>
@@ -45374,7 +45383,7 @@
         <v>14</v>
       </c>
       <c r="C16" s="109" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="D16" s="109">
         <v>87</v>
@@ -45436,7 +45445,7 @@
         <v>15</v>
       </c>
       <c r="C17" s="106" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D17" s="106">
         <v>100</v>
@@ -45501,7 +45510,7 @@
         <v>16</v>
       </c>
       <c r="C18" s="109" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D18" s="109">
         <v>87</v>
@@ -45563,7 +45572,7 @@
         <v>17</v>
       </c>
       <c r="C19" s="106" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D19" s="106">
         <v>87</v>
@@ -45625,7 +45634,7 @@
         <v>18</v>
       </c>
       <c r="C20" s="109" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D20" s="109">
         <v>87</v>
@@ -45687,7 +45696,7 @@
         <v>19</v>
       </c>
       <c r="C21" s="106" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D21" s="106">
         <v>95</v>
@@ -45749,7 +45758,7 @@
         <v>20</v>
       </c>
       <c r="C22" s="109" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="D22" s="109">
         <v>93</v>
@@ -45811,7 +45820,7 @@
         <v>21</v>
       </c>
       <c r="C23" s="106" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="D23" s="106">
         <v>93</v>
@@ -45873,7 +45882,7 @@
         <v>22</v>
       </c>
       <c r="C24" s="109" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="D24" s="109">
         <v>90</v>
@@ -45935,7 +45944,7 @@
         <v>23</v>
       </c>
       <c r="C25" s="106" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D25" s="106">
         <v>100</v>
@@ -46000,7 +46009,7 @@
         <v>24</v>
       </c>
       <c r="C26" s="109" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="D26" s="109">
         <v>87</v>
@@ -46059,13 +46068,13 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B27" s="104">
         <v>25</v>
       </c>
       <c r="C27" s="106" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D27" s="106">
         <v>87</v>
@@ -46127,7 +46136,7 @@
         <v>26</v>
       </c>
       <c r="C28" s="109" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="D28" s="109">
         <v>100</v>
@@ -46189,7 +46198,7 @@
         <v>27</v>
       </c>
       <c r="C29" s="106" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="D29" s="106">
         <v>100</v>
@@ -46254,7 +46263,7 @@
         <v>28</v>
       </c>
       <c r="C30" s="109" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="D30" s="109">
         <v>90</v>
@@ -46319,7 +46328,7 @@
         <v>29</v>
       </c>
       <c r="C31" s="106" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="D31" s="106">
         <v>90</v>
@@ -46384,7 +46393,7 @@
         <v>30</v>
       </c>
       <c r="C32" s="109" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="D32" s="109">
         <v>87</v>
@@ -46449,7 +46458,7 @@
         <v>31</v>
       </c>
       <c r="C33" s="106" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="D33" s="106">
         <v>89</v>
@@ -46511,7 +46520,7 @@
         <v>32</v>
       </c>
       <c r="C34" s="109" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="D34" s="109">
         <v>99</v>
@@ -46576,7 +46585,7 @@
         <v>33</v>
       </c>
       <c r="C35" s="106" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="D35" s="106">
         <v>87</v>
@@ -46638,7 +46647,7 @@
         <v>34</v>
       </c>
       <c r="C36" s="109" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="D36" s="109">
         <v>99</v>
@@ -46703,7 +46712,7 @@
         <v>35</v>
       </c>
       <c r="C37" s="106" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="D37" s="106">
         <v>87</v>
@@ -46768,7 +46777,7 @@
         <v>36</v>
       </c>
       <c r="C38" s="109" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="D38" s="109">
         <v>87</v>
@@ -46830,7 +46839,7 @@
         <v>37</v>
       </c>
       <c r="C39" s="106" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="D39" s="106">
         <v>87</v>
@@ -46895,7 +46904,7 @@
         <v>38</v>
       </c>
       <c r="C40" s="109" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="D40" s="109">
         <v>87</v>
@@ -46960,7 +46969,7 @@
         <v>39</v>
       </c>
       <c r="C41" s="106" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="D41" s="106">
         <v>87</v>

</xml_diff>

<commit_message>
Added AME for rapeseed cake
</commit_message>
<xml_diff>
--- a/data/default/FeedMgmt.xlsx
+++ b/data/default/FeedMgmt.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="references" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="horses" sheetId="8" r:id="rId8"/>
     <sheet name="poultry" sheetId="9" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="162913" iterateDelta="1E-4"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -146,7 +146,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1621" uniqueCount="681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1622" uniqueCount="682">
   <si>
     <t>Statistics Netherlands (2012) Standardised calculation methods for animal manure and nutrients. Standard data 1990–2008</t>
   </si>
@@ -2270,6 +2270,9 @@
   </si>
   <si>
     <t>https://www.feedipedia.org/node/500, https://www.feedipedia.org/node/432, https://grovfoderverktyget.se/?p=31151</t>
+  </si>
+  <si>
+    <t>https://www.feedipedia.org/node/12502</t>
   </si>
 </sst>
 </file>
@@ -2697,7 +2700,7 @@
     <xf numFmtId="9" fontId="30" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
@@ -2841,6 +2844,7 @@
     <xf numFmtId="1" fontId="29" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -10067,7 +10071,12 @@
       <c r="AP28" s="64"/>
       <c r="AR28" s="28"/>
       <c r="AS28" s="39"/>
-      <c r="AT28" s="65"/>
+      <c r="AT28" s="65">
+        <v>10.5</v>
+      </c>
+      <c r="AU28" s="115" t="s">
+        <v>681</v>
+      </c>
     </row>
     <row r="29" spans="2:47" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
@@ -13003,10 +13012,11 @@
     <hyperlink ref="Z47" r:id="rId34"/>
     <hyperlink ref="AP47" r:id="rId35"/>
     <hyperlink ref="D52" r:id="rId36"/>
+    <hyperlink ref="AU28" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <legacyDrawing r:id="rId37"/>
+  <legacyDrawing r:id="rId38"/>
 </worksheet>
 </file>
 
@@ -13019,6 +13029,7 @@
     <col min="2" max="3" width="10.140625" style="1" customWidth="1"/>
     <col min="4" max="9" width="12.28515625" style="1" customWidth="1"/>
     <col min="10" max="24" width="8.85546875" style="1" customWidth="1"/>
+    <col min="45" max="45" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:48" x14ac:dyDescent="0.25">
@@ -16388,9 +16399,9 @@
       <c r="AT25" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="AV25" s="42" t="str">
+      <c r="AV25" s="42">
         <f>IF(AND(INDEX('feed pars'!$C$6:$AT$48,MATCH($A25,'feed pars'!$B$6:$B$48,0),AV$1)&lt;&gt;"",AV$1&lt;&gt;""), INDEX('feed pars'!$C$6:$AT$48,MATCH($A25,'feed pars'!$B$6:$B$48,0),AV$1), "")</f>
-        <v/>
+        <v>10.5</v>
       </c>
     </row>
     <row r="26" spans="1:48" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Data for rapeseed meal as a by-product of vegetable oils for feed
</commit_message>
<xml_diff>
--- a/data/default/FeedMgmt.xlsx
+++ b/data/default/FeedMgmt.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33D1DBCA-15B1-4B74-9490-01EE36603292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A19BF084-01D8-48DC-B211-7CE17313D69D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="14265" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1650" yWindow="2100" windowWidth="13710" windowHeight="8700" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="references" sheetId="1" r:id="rId1"/>
@@ -157,8 +157,30 @@
 </comments>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1621" uniqueCount="665">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1622" uniqueCount="667">
   <si>
     <t>Statistics Netherlands (2012) Standardised calculation methods for animal manure and nutrients. Standard data 1990–2008</t>
   </si>
@@ -2234,6 +2256,12 @@
   </si>
   <si>
     <t>https://doi.org/10.1080/09064702.2021.1993319</t>
+  </si>
+  <si>
+    <t>0.38 kg oil + 0.60 kg meal per kg rapeseed</t>
+  </si>
+  <si>
+    <t>See DemandAndConversions</t>
   </si>
 </sst>
 </file>
@@ -3126,7 +3154,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Q156"/>
+  <dimension ref="A1:Q157"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="7" width="20.28515625" customWidth="1"/>
@@ -3134,7 +3162,7 @@
     <col min="9" max="9" width="19.5703125" customWidth="1"/>
     <col min="10" max="11" width="20.140625" customWidth="1"/>
     <col min="12" max="12" width="9.7109375" customWidth="1"/>
-    <col min="13" max="13" width="16.42578125" customWidth="1"/>
+    <col min="13" max="13" width="17.28515625" customWidth="1"/>
     <col min="14" max="14" width="25.85546875" customWidth="1"/>
     <col min="15" max="15" width="12.7109375" customWidth="1"/>
     <col min="16" max="16" width="38.140625" customWidth="1"/>
@@ -3232,32 +3260,29 @@
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="M4" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="N4" s="6">
+        <v>0</v>
+      </c>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="M4" s="5"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="F5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I5" t="s">
-        <v>28</v>
-      </c>
-      <c r="M5" t="s">
-        <v>24</v>
-      </c>
-      <c r="N5" s="8">
-        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F5,'feed pars'!B$6:B$49,0))</f>
-        <v>1</v>
-      </c>
+      <c r="M5" s="5"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="5"/>
+      <c r="P5" s="5"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I6" t="s">
         <v>28</v>
@@ -3272,7 +3297,7 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I7" t="s">
         <v>28</v>
@@ -3287,7 +3312,7 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I8" t="s">
         <v>28</v>
@@ -3302,10 +3327,10 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I9" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="M9" t="s">
         <v>24</v>
@@ -3317,54 +3342,54 @@
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F10" t="s">
-        <v>653</v>
+        <v>32</v>
       </c>
       <c r="I10" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="M10" t="s">
         <v>24</v>
       </c>
       <c r="N10" s="8">
+        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F10,'feed pars'!B$6:B$49,0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F11" t="s">
-        <v>34</v>
+        <v>653</v>
       </c>
       <c r="I11" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="M11" t="s">
         <v>24</v>
       </c>
       <c r="N11" s="8">
-        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F11,'feed pars'!B$6:B$49,0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M12" t="s">
         <v>24</v>
       </c>
       <c r="N12" s="8">
         <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F12,'feed pars'!B$6:B$49,0))</f>
-        <v>1.1627906976744187</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="M13" t="s">
         <v>24</v>
@@ -3376,10 +3401,10 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M14" t="s">
         <v>24</v>
@@ -3391,10 +3416,10 @@
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M15" t="s">
         <v>24</v>
@@ -3406,10 +3431,10 @@
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M16" t="s">
         <v>24</v>
@@ -3419,12 +3444,12 @@
         <v>1.1627906976744187</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F17" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I17" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="M17" t="s">
         <v>24</v>
@@ -3434,24 +3459,24 @@
         <v>1.1627906976744187</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="M18" t="s">
         <v>24</v>
       </c>
       <c r="N18" s="8">
         <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F18,'feed pars'!B$6:B$49,0))</f>
-        <v>1.1764705882352942</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+        <v>1.1627906976744187</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F19" t="s">
-        <v>655</v>
+        <v>41</v>
       </c>
       <c r="I19" t="s">
         <v>41</v>
@@ -3460,71 +3485,69 @@
         <v>24</v>
       </c>
       <c r="N19" s="8">
-        <f>N18/0.2</f>
+        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F19,'feed pars'!B$6:B$49,0))</f>
+        <v>1.1764705882352942</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F20" t="s">
+        <v>655</v>
+      </c>
+      <c r="I20" t="s">
+        <v>41</v>
+      </c>
+      <c r="M20" t="s">
+        <v>24</v>
+      </c>
+      <c r="N20" s="8">
+        <f>N19/0.2</f>
         <v>5.8823529411764701</v>
       </c>
-      <c r="P19" t="s">
+      <c r="P20" t="s">
         <v>656</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="F20" s="9" t="s">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F21" s="9" t="s">
         <v>655</v>
       </c>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="J20" s="9" t="s">
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9" t="s">
         <v>657</v>
       </c>
-      <c r="K20" s="9"/>
-      <c r="L20" s="9"/>
-      <c r="M20" s="9" t="s">
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="N20" s="8"/>
-      <c r="P20" s="9" t="s">
+      <c r="N21" s="8"/>
+      <c r="P21" s="9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="F21" t="s">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F22" t="s">
         <v>42</v>
       </c>
-      <c r="I21" t="s">
+      <c r="I22" t="s">
         <v>42</v>
-      </c>
-      <c r="M21" t="s">
-        <v>24</v>
-      </c>
-      <c r="N21" s="8">
-        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F21,'feed pars'!B$6:B$49,0))</f>
-        <v>1.1764705882352942</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="F22" t="s">
-        <v>43</v>
-      </c>
-      <c r="I22" t="s">
-        <v>43</v>
       </c>
       <c r="M22" t="s">
         <v>24</v>
       </c>
       <c r="N22" s="8">
         <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F22,'feed pars'!B$6:B$49,0))</f>
-        <v>1.0989010989010988</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+        <v>1.1764705882352942</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="M23" t="s">
         <v>24</v>
@@ -3534,176 +3557,181 @@
         <v>1.0989010989010988</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="F24" s="9" t="s">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F24" t="s">
+        <v>44</v>
+      </c>
+      <c r="I24" t="s">
+        <v>44</v>
+      </c>
+      <c r="M24" t="s">
+        <v>24</v>
+      </c>
+      <c r="N24" s="8">
+        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F24,'feed pars'!B$6:B$49,0))</f>
+        <v>1.0989010989010988</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F25" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9" t="s">
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="J24" s="9"/>
-      <c r="K24" s="9"/>
-      <c r="L24" s="9"/>
-      <c r="M24" s="9" t="s">
+      <c r="J25" s="11"/>
+      <c r="K25" s="11"/>
+      <c r="L25" s="11"/>
+      <c r="M25" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="N24" s="10">
-        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F24,'feed pars'!B$6:B$49,0))*1/0.38</f>
+      <c r="N25" s="8">
+        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F25,'feed pars'!B$6:B$49,0))*1/0.38</f>
         <v>2.6315789473684212</v>
       </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="F25" s="9" t="s">
+      <c r="P25" t="s">
+        <v>665</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F26" s="11" t="s">
         <v>45</v>
-      </c>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="J25" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="K25" s="9"/>
-      <c r="L25" s="9"/>
-      <c r="M25" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="N25" s="8"/>
-      <c r="P25" s="9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="F26" s="11" t="s">
-        <v>49</v>
       </c>
       <c r="G26" s="11"/>
       <c r="H26" s="11"/>
-      <c r="I26" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="J26" s="11"/>
+      <c r="I26" s="11"/>
+      <c r="J26" s="11" t="s">
+        <v>46</v>
+      </c>
       <c r="K26" s="11"/>
       <c r="L26" s="11"/>
       <c r="M26" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="N26" s="8">
-        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F26,'feed pars'!B$6:B$49,0))</f>
-        <v>1.1494252873563218</v>
-      </c>
-      <c r="O26" s="11"/>
+        <v>47</v>
+      </c>
+      <c r="N26" s="8" cm="1">
+        <f t="array" ref="N26">1/_xlfn.SINGLE(INDEX('feed pars'!C$6:C$49/100,MATCH(F26,'feed pars'!B$6:B$49,0)))*1/0.6</f>
+        <v>1.6666666666666667</v>
+      </c>
       <c r="P26" s="9"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="F27" s="11"/>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F27" s="11" t="s">
+        <v>49</v>
+      </c>
       <c r="G27" s="11"/>
       <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
+      <c r="I27" s="11" t="s">
+        <v>49</v>
+      </c>
       <c r="J27" s="11"/>
       <c r="K27" s="11"/>
       <c r="L27" s="11"/>
-      <c r="M27" s="11"/>
-      <c r="N27" s="8"/>
+      <c r="M27" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="N27" s="8">
+        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F27,'feed pars'!B$6:B$49,0))</f>
+        <v>1.1494252873563218</v>
+      </c>
       <c r="O27" s="11"/>
       <c r="P27" s="9"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="F28" t="s">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
+      <c r="J28" s="11"/>
+      <c r="K28" s="11"/>
+      <c r="L28" s="11"/>
+      <c r="M28" s="11"/>
+      <c r="N28" s="8"/>
+      <c r="O28" s="11"/>
+      <c r="P28" s="9"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F29" t="s">
         <v>51</v>
       </c>
-      <c r="J28" t="s">
+      <c r="J29" t="s">
         <v>51</v>
       </c>
-      <c r="M28" t="s">
+      <c r="M29" t="s">
         <v>24</v>
       </c>
-      <c r="N28" s="8">
-        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F28,'feed pars'!B$6:B$49,0))</f>
-        <v>1.1428571428571428</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="F29" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="G29" s="9"/>
-      <c r="H29" s="9"/>
-      <c r="I29" s="9"/>
-      <c r="J29" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="K29" s="9"/>
-      <c r="L29" s="9"/>
-      <c r="M29" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="N29" s="10">
+      <c r="N29" s="8">
         <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F29,'feed pars'!B$6:B$49,0))</f>
         <v>1.1428571428571428</v>
       </c>
-      <c r="O29" s="9"/>
-      <c r="P29" s="9" t="s">
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F30" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
+      <c r="J30" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="K30" s="9"/>
+      <c r="L30" s="9"/>
+      <c r="M30" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="N30" s="10">
+        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F30,'feed pars'!B$6:B$49,0))</f>
+        <v>1.1428571428571428</v>
+      </c>
+      <c r="O30" s="9"/>
+      <c r="P30" s="9" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="F30" t="s">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F31" t="s">
         <v>46</v>
       </c>
-      <c r="J30" t="s">
+      <c r="J31" t="s">
         <v>46</v>
-      </c>
-      <c r="M30" t="s">
-        <v>24</v>
-      </c>
-      <c r="N30" s="8">
-        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F30,'feed pars'!B$6:B$49,0))</f>
-        <v>1.1173184357541899</v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="F31" t="s">
-        <v>54</v>
-      </c>
-      <c r="J31" t="s">
-        <v>54</v>
       </c>
       <c r="M31" t="s">
         <v>24</v>
       </c>
       <c r="N31" s="8">
         <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F31,'feed pars'!B$6:B$49,0))</f>
-        <v>1.0928961748633879</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+        <v>1.1173184357541899</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F32" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J32" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="M32" t="s">
         <v>24</v>
       </c>
       <c r="N32" s="8">
         <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F32,'feed pars'!B$6:B$49,0))</f>
-        <v>1.0989010989010988</v>
+        <v>1.0928961748633879</v>
       </c>
     </row>
     <row r="33" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F33" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J33" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M33" t="s">
         <v>24</v>
@@ -3714,47 +3742,47 @@
       </c>
     </row>
     <row r="34" spans="6:16" x14ac:dyDescent="0.25">
-      <c r="F34" s="9" t="s">
+      <c r="F34" t="s">
+        <v>56</v>
+      </c>
+      <c r="J34" t="s">
+        <v>56</v>
+      </c>
+      <c r="M34" t="s">
+        <v>24</v>
+      </c>
+      <c r="N34" s="8">
+        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F34,'feed pars'!B$6:B$49,0))</f>
+        <v>1.0989010989010988</v>
+      </c>
+    </row>
+    <row r="35" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="F35" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G34" s="9"/>
-      <c r="H34" s="9"/>
-      <c r="I34" s="9"/>
-      <c r="J34" s="9" t="s">
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="K34" s="9"/>
-      <c r="L34" s="9"/>
-      <c r="M34" s="9" t="s">
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="N34" s="10">
-        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F34,'feed pars'!B$6:B$49,0))</f>
+      <c r="N35" s="10">
+        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F35,'feed pars'!B$6:B$49,0))</f>
         <v>1.1111111111111112</v>
       </c>
-      <c r="O34" s="9"/>
-      <c r="P34" s="9" t="s">
+      <c r="O35" s="9"/>
+      <c r="P35" s="9" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="35" spans="6:16" x14ac:dyDescent="0.25">
-      <c r="F35" t="s">
-        <v>59</v>
-      </c>
-      <c r="J35" t="s">
-        <v>60</v>
-      </c>
-      <c r="M35" t="s">
-        <v>24</v>
-      </c>
-      <c r="N35" s="8">
-        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F35,'feed pars'!B$6:B$49,0))</f>
-        <v>1.1494252873563218</v>
       </c>
     </row>
     <row r="36" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F36" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="J36" t="s">
         <v>60</v>
@@ -3764,27 +3792,27 @@
       </c>
       <c r="N36" s="8">
         <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F36,'feed pars'!B$6:B$49,0))</f>
-        <v>1.1389521640091116</v>
+        <v>1.1494252873563218</v>
       </c>
     </row>
     <row r="37" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F37" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J37" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="M37" t="s">
         <v>24</v>
       </c>
       <c r="N37" s="8">
         <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F37,'feed pars'!B$6:B$49,0))</f>
-        <v>1.1415525114155252</v>
+        <v>1.1389521640091116</v>
       </c>
     </row>
     <row r="38" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F38" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="J38" t="s">
         <v>63</v>
@@ -3799,10 +3827,10 @@
     </row>
     <row r="39" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F39" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J39" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="M39" t="s">
         <v>24</v>
@@ -3814,22 +3842,22 @@
     </row>
     <row r="40" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F40" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J40" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="M40" t="s">
         <v>24</v>
       </c>
       <c r="N40" s="8">
         <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F40,'feed pars'!B$6:B$49,0))</f>
-        <v>1.1111111111111112</v>
+        <v>1.1415525114155252</v>
       </c>
     </row>
     <row r="41" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F41" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="J41" t="s">
         <v>67</v>
@@ -3838,73 +3866,73 @@
         <v>24</v>
       </c>
       <c r="N41" s="8">
-        <f>N40</f>
+        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F41,'feed pars'!B$6:B$49,0))</f>
         <v>1.1111111111111112</v>
       </c>
     </row>
     <row r="42" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F42" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J42" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M42" t="s">
         <v>24</v>
       </c>
-      <c r="N42" s="10">
+      <c r="N42" s="8">
+        <f>N41</f>
+        <v>1.1111111111111112</v>
+      </c>
+    </row>
+    <row r="43" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="F43" t="s">
+        <v>69</v>
+      </c>
+      <c r="J43" t="s">
+        <v>69</v>
+      </c>
+      <c r="M43" t="s">
+        <v>24</v>
+      </c>
+      <c r="N43" s="10">
         <f>1/0.25</f>
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="6:16" x14ac:dyDescent="0.25">
-      <c r="F43" t="s">
-        <v>70</v>
-      </c>
-      <c r="J43" t="s">
-        <v>70</v>
-      </c>
-      <c r="M43" t="s">
-        <v>24</v>
-      </c>
-      <c r="N43" s="8">
-        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F43,'feed pars'!B$6:B$49,0))</f>
-        <v>1.3245033112582782</v>
-      </c>
-    </row>
     <row r="44" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F44" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J44" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M44" t="s">
         <v>24</v>
       </c>
       <c r="N44" s="8">
         <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F44,'feed pars'!B$6:B$49,0))</f>
-        <v>1.1173184357541899</v>
+        <v>1.3245033112582782</v>
       </c>
     </row>
     <row r="45" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F45" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J45" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M45" t="s">
         <v>24</v>
       </c>
       <c r="N45" s="8">
         <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F45,'feed pars'!B$6:B$49,0))</f>
-        <v>16</v>
+        <v>1.1173184357541899</v>
       </c>
     </row>
     <row r="46" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F46" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J46" t="s">
         <v>72</v>
@@ -3912,171 +3940,172 @@
       <c r="M46" t="s">
         <v>24</v>
       </c>
-      <c r="N46" s="10">
-        <f>N45</f>
+      <c r="N46" s="8">
+        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F46,'feed pars'!B$6:B$49,0))</f>
         <v>16</v>
       </c>
     </row>
     <row r="47" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F47" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J47" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="M47" t="s">
         <v>24</v>
       </c>
-      <c r="N47" s="8">
-        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F47,'feed pars'!B$6:B$49,0))</f>
-        <v>1.0989010989010988</v>
+      <c r="N47" s="10">
+        <f>N46</f>
+        <v>16</v>
       </c>
     </row>
     <row r="48" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F48" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J48" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="M48" t="s">
         <v>24</v>
       </c>
       <c r="N48" s="8">
         <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F48,'feed pars'!B$6:B$49,0))</f>
-        <v>4.3478260869565215</v>
+        <v>1.0989010989010988</v>
       </c>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F49" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J49" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="M49" t="s">
         <v>24</v>
       </c>
       <c r="N49" s="8">
         <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F49,'feed pars'!B$6:B$49,0))</f>
-        <v>1.0863661053775122</v>
+        <v>4.3478260869565215</v>
       </c>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F50" t="s">
-        <v>658</v>
+        <v>76</v>
       </c>
       <c r="J50" t="s">
-        <v>659</v>
+        <v>76</v>
       </c>
       <c r="M50" t="s">
         <v>24</v>
       </c>
-      <c r="N50" s="10">
-        <v>1</v>
+      <c r="N50" s="8">
+        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F50,'feed pars'!B$6:B$49,0))</f>
+        <v>1.0863661053775122</v>
       </c>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F51" t="s">
-        <v>193</v>
+        <v>658</v>
       </c>
       <c r="J51" t="s">
-        <v>193</v>
+        <v>659</v>
       </c>
       <c r="M51" t="s">
         <v>24</v>
       </c>
-      <c r="N51" s="8">
-        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F51,'feed pars'!B$6:B$49,0))</f>
+      <c r="N51" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F52" t="s">
+        <v>193</v>
+      </c>
+      <c r="J52" t="s">
+        <v>193</v>
+      </c>
+      <c r="M52" t="s">
+        <v>24</v>
+      </c>
+      <c r="N52" s="8">
+        <f>1/INDEX('feed pars'!C$6:C$49/100,MATCH(F52,'feed pars'!B$6:B$49,0))</f>
         <v>1.1152416356877324</v>
       </c>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N52" s="8"/>
-    </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A53" s="7" t="s">
+      <c r="N53" s="8"/>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A54" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="N53" s="8"/>
-    </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="F54" t="s">
+      <c r="N54" s="8"/>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F55" t="s">
         <v>78</v>
       </c>
-      <c r="K54" t="s">
+      <c r="K55" t="s">
         <v>78</v>
       </c>
-      <c r="M54" t="s">
+      <c r="M55" t="s">
         <v>24</v>
       </c>
-      <c r="N54" s="8">
+      <c r="N55" s="8">
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N55" s="8"/>
-    </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A56" s="2" t="s">
+      <c r="N56" s="8"/>
+    </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A57" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="3"/>
-      <c r="F56" s="3"/>
-      <c r="G56" s="3"/>
-      <c r="H56" s="3"/>
-      <c r="I56" s="3"/>
-      <c r="J56" s="3"/>
-      <c r="K56" s="3"/>
-      <c r="L56" s="3"/>
-      <c r="M56" s="3"/>
-      <c r="N56" s="3"/>
-      <c r="O56" s="3"/>
-      <c r="P56" s="3"/>
-      <c r="Q56" s="3"/>
-    </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A57" s="12" t="s">
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3"/>
+      <c r="I57" s="3"/>
+      <c r="J57" s="3"/>
+      <c r="K57" s="3"/>
+      <c r="L57" s="3"/>
+      <c r="M57" s="3"/>
+      <c r="N57" s="3"/>
+      <c r="O57" s="3"/>
+      <c r="P57" s="3"/>
+      <c r="Q57" s="3"/>
+    </row>
+    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A58" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="B57" s="7"/>
-      <c r="C57" s="7"/>
-      <c r="D57" s="7"/>
-    </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M58" s="5" t="s">
+      <c r="B58" s="7"/>
+      <c r="C58" s="7"/>
+      <c r="D58" s="7"/>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M59" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="N58" s="5">
-        <v>0</v>
-      </c>
-      <c r="O58" s="5" t="s">
+      <c r="N59" s="5">
+        <v>0</v>
+      </c>
+      <c r="O59" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P58" s="5" t="s">
+      <c r="P59" s="5" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="I59" t="s">
-        <v>28</v>
-      </c>
-      <c r="M59" t="s">
-        <v>81</v>
-      </c>
-      <c r="N59" s="9">
-        <v>95</v>
-      </c>
-      <c r="O59" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I60" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="M60" t="s">
         <v>81</v>
@@ -4090,7 +4119,7 @@
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I61" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M61" t="s">
         <v>81</v>
@@ -4103,26 +4132,22 @@
       </c>
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>83</v>
-      </c>
       <c r="I62" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="M62" t="s">
         <v>81</v>
       </c>
       <c r="N62" s="9">
-        <v>30</v>
+        <v>95</v>
       </c>
       <c r="O62" t="s">
         <v>82</v>
       </c>
-      <c r="P62" s="9"/>
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I63" t="s">
         <v>36</v>
@@ -4140,10 +4165,10 @@
     </row>
     <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I64" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M64" t="s">
         <v>81</v>
@@ -4158,7 +4183,7 @@
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I65" t="s">
         <v>35</v>
@@ -4176,10 +4201,10 @@
     </row>
     <row r="66" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I66" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="M66" t="s">
         <v>81</v>
@@ -4194,7 +4219,7 @@
     </row>
     <row r="67" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I67" t="s">
         <v>37</v>
@@ -4211,34 +4236,37 @@
       <c r="P67" s="9"/>
     </row>
     <row r="68" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N68" s="9"/>
+      <c r="A68" t="s">
+        <v>84</v>
+      </c>
+      <c r="I68" t="s">
+        <v>37</v>
+      </c>
+      <c r="M68" t="s">
+        <v>81</v>
+      </c>
+      <c r="N68" s="9">
+        <v>30</v>
+      </c>
+      <c r="O68" t="s">
+        <v>82</v>
+      </c>
       <c r="P68" s="9"/>
     </row>
     <row r="69" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A69" s="12" t="s">
-        <v>85</v>
-      </c>
       <c r="N69" s="9"/>
       <c r="P69" s="9"/>
     </row>
     <row r="70" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="I70" t="s">
-        <v>28</v>
-      </c>
-      <c r="M70" t="s">
-        <v>86</v>
-      </c>
-      <c r="N70" s="9">
-        <v>5</v>
-      </c>
-      <c r="O70" t="s">
-        <v>82</v>
-      </c>
+      <c r="A70" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="N70" s="9"/>
       <c r="P70" s="9"/>
     </row>
     <row r="71" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I71" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="M71" t="s">
         <v>86</v>
@@ -4253,7 +4281,7 @@
     </row>
     <row r="72" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I72" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M72" t="s">
         <v>86</v>
@@ -4267,121 +4295,121 @@
       <c r="P72" s="9"/>
     </row>
     <row r="73" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N73" s="9"/>
+      <c r="I73" t="s">
+        <v>34</v>
+      </c>
+      <c r="M73" t="s">
+        <v>86</v>
+      </c>
+      <c r="N73" s="9">
+        <v>5</v>
+      </c>
+      <c r="O73" t="s">
+        <v>82</v>
+      </c>
       <c r="P73" s="9"/>
     </row>
     <row r="74" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A74" s="2" t="s">
+      <c r="N74" s="9"/>
+      <c r="P74" s="9"/>
+    </row>
+    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A75" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B74" s="2"/>
-      <c r="C74" s="2"/>
-      <c r="D74" s="2"/>
-      <c r="E74" s="3"/>
-      <c r="F74" s="3"/>
-      <c r="G74" s="3"/>
-      <c r="H74" s="3"/>
-      <c r="I74" s="3"/>
-      <c r="J74" s="3"/>
-      <c r="K74" s="3"/>
-      <c r="L74" s="3"/>
-      <c r="M74" s="3"/>
-      <c r="N74" s="3"/>
-      <c r="O74" s="3"/>
-      <c r="P74" s="3"/>
-      <c r="Q74" s="3"/>
-    </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M75" s="5" t="s">
+      <c r="B75" s="2"/>
+      <c r="C75" s="2"/>
+      <c r="D75" s="2"/>
+      <c r="E75" s="3"/>
+      <c r="F75" s="3"/>
+      <c r="G75" s="3"/>
+      <c r="H75" s="3"/>
+      <c r="I75" s="3"/>
+      <c r="J75" s="3"/>
+      <c r="K75" s="3"/>
+      <c r="L75" s="3"/>
+      <c r="M75" s="3"/>
+      <c r="N75" s="3"/>
+      <c r="O75" s="3"/>
+      <c r="P75" s="3"/>
+      <c r="Q75" s="3"/>
+    </row>
+    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M76" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="N75" s="5">
+      <c r="N76" s="5">
         <v>100</v>
       </c>
-      <c r="O75" s="5" t="s">
+      <c r="O76" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P75" s="5" t="s">
+      <c r="P76" s="5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="I76" t="s">
-        <v>49</v>
-      </c>
-      <c r="M76" t="s">
-        <v>88</v>
-      </c>
-      <c r="N76" s="11">
-        <v>0</v>
-      </c>
-      <c r="O76" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="P76" s="5"/>
     </row>
     <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I77" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="M77" t="s">
         <v>88</v>
       </c>
-      <c r="N77" s="9">
-        <v>0</v>
-      </c>
-      <c r="O77" t="s">
+      <c r="N77" s="11">
+        <v>0</v>
+      </c>
+      <c r="O77" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="P77" s="9" t="s">
-        <v>89</v>
-      </c>
+      <c r="P77" s="5"/>
     </row>
     <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I78" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="M78" t="s">
         <v>88</v>
       </c>
       <c r="N78" s="9">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="O78" t="s">
         <v>82</v>
       </c>
       <c r="P78" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="I79" t="s">
+        <v>40</v>
+      </c>
+      <c r="M79" t="s">
+        <v>88</v>
+      </c>
+      <c r="N79" s="9">
+        <v>50</v>
+      </c>
+      <c r="O79" t="s">
+        <v>82</v>
+      </c>
+      <c r="P79" s="9" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N79" s="9"/>
-      <c r="P79" s="9"/>
-    </row>
     <row r="80" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="J80" t="s">
-        <v>60</v>
-      </c>
-      <c r="M80" t="s">
-        <v>88</v>
-      </c>
-      <c r="N80" s="9">
-        <v>80</v>
-      </c>
-      <c r="O80" t="s">
-        <v>82</v>
-      </c>
+      <c r="N80" s="9"/>
       <c r="P80" s="9"/>
     </row>
     <row r="81" spans="3:16" x14ac:dyDescent="0.25">
       <c r="J81" t="s">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="M81" t="s">
         <v>88</v>
       </c>
       <c r="N81" s="9">
-        <v>42</v>
+        <v>80</v>
       </c>
       <c r="O81" t="s">
         <v>82</v>
@@ -4390,13 +4418,13 @@
     </row>
     <row r="82" spans="3:16" x14ac:dyDescent="0.25">
       <c r="J82" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="M82" t="s">
         <v>88</v>
       </c>
       <c r="N82" s="9">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="O82" t="s">
         <v>82</v>
@@ -4405,7 +4433,7 @@
     </row>
     <row r="83" spans="3:16" x14ac:dyDescent="0.25">
       <c r="J83" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="M83" t="s">
         <v>88</v>
@@ -4420,7 +4448,7 @@
     </row>
     <row r="84" spans="3:16" x14ac:dyDescent="0.25">
       <c r="J84" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="M84" t="s">
         <v>88</v>
@@ -4435,7 +4463,7 @@
     </row>
     <row r="85" spans="3:16" x14ac:dyDescent="0.25">
       <c r="J85" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M85" t="s">
         <v>88</v>
@@ -4450,7 +4478,7 @@
     </row>
     <row r="86" spans="3:16" x14ac:dyDescent="0.25">
       <c r="J86" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M86" t="s">
         <v>88</v>
@@ -4465,7 +4493,7 @@
     </row>
     <row r="87" spans="3:16" x14ac:dyDescent="0.25">
       <c r="J87" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="M87" t="s">
         <v>88</v>
@@ -4480,7 +4508,7 @@
     </row>
     <row r="88" spans="3:16" x14ac:dyDescent="0.25">
       <c r="J88" t="s">
-        <v>193</v>
+        <v>76</v>
       </c>
       <c r="M88" t="s">
         <v>88</v>
@@ -4494,25 +4522,22 @@
       <c r="P88" s="9"/>
     </row>
     <row r="89" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="N89" s="9"/>
+      <c r="J89" t="s">
+        <v>193</v>
+      </c>
+      <c r="M89" t="s">
+        <v>88</v>
+      </c>
+      <c r="N89" s="9">
+        <v>0</v>
+      </c>
+      <c r="O89" t="s">
+        <v>82</v>
+      </c>
       <c r="P89" s="9"/>
     </row>
     <row r="90" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="C90" t="s">
-        <v>644</v>
-      </c>
-      <c r="J90" t="s">
-        <v>60</v>
-      </c>
-      <c r="M90" t="s">
-        <v>88</v>
-      </c>
-      <c r="N90" s="9">
-        <v>85</v>
-      </c>
-      <c r="O90" t="s">
-        <v>82</v>
-      </c>
+      <c r="N90" s="9"/>
       <c r="P90" s="9"/>
     </row>
     <row r="91" spans="3:16" x14ac:dyDescent="0.25">
@@ -4520,13 +4545,13 @@
         <v>644</v>
       </c>
       <c r="J91" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="M91" t="s">
         <v>88</v>
       </c>
       <c r="N91" s="9">
-        <v>4</v>
+        <v>85</v>
       </c>
       <c r="O91" t="s">
         <v>82</v>
@@ -4538,13 +4563,13 @@
         <v>644</v>
       </c>
       <c r="J92" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="M92" t="s">
         <v>88</v>
       </c>
       <c r="N92" s="9">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="O92" t="s">
         <v>82</v>
@@ -4556,27 +4581,25 @@
         <v>644</v>
       </c>
       <c r="J93" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="M93" t="s">
         <v>88</v>
       </c>
       <c r="N93" s="9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O93" t="s">
         <v>82</v>
       </c>
-      <c r="P93" s="9" t="s">
-        <v>645</v>
-      </c>
+      <c r="P93" s="9"/>
     </row>
     <row r="94" spans="3:16" x14ac:dyDescent="0.25">
       <c r="C94" t="s">
         <v>644</v>
       </c>
       <c r="J94" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M94" t="s">
         <v>88</v>
@@ -4587,14 +4610,16 @@
       <c r="O94" t="s">
         <v>82</v>
       </c>
-      <c r="P94" s="9"/>
+      <c r="P94" s="9" t="s">
+        <v>645</v>
+      </c>
     </row>
     <row r="95" spans="3:16" x14ac:dyDescent="0.25">
       <c r="C95" t="s">
         <v>644</v>
       </c>
       <c r="J95" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="M95" t="s">
         <v>88</v>
@@ -4608,68 +4633,54 @@
       <c r="P95" s="9"/>
     </row>
     <row r="96" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="N96" s="9"/>
+      <c r="C96" t="s">
+        <v>644</v>
+      </c>
+      <c r="J96" t="s">
+        <v>74</v>
+      </c>
+      <c r="M96" t="s">
+        <v>88</v>
+      </c>
+      <c r="N96" s="9">
+        <v>0</v>
+      </c>
+      <c r="O96" t="s">
+        <v>82</v>
+      </c>
       <c r="P96" s="9"/>
     </row>
     <row r="97" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A97" s="2" t="s">
+      <c r="N97" s="9"/>
+      <c r="P97" s="9"/>
+    </row>
+    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A98" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B97" s="2"/>
-      <c r="C97" s="2"/>
-      <c r="D97" s="2"/>
-      <c r="E97" s="3"/>
-      <c r="F97" s="3"/>
-      <c r="G97" s="3"/>
-      <c r="H97" s="3"/>
-      <c r="I97" s="3"/>
-      <c r="J97" s="3"/>
-      <c r="K97" s="3"/>
-      <c r="L97" s="3"/>
-      <c r="M97" s="3"/>
-      <c r="N97" s="3"/>
-      <c r="O97" s="3"/>
-      <c r="P97" s="3"/>
-      <c r="Q97" s="3"/>
-    </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>92</v>
-      </c>
-      <c r="B99" t="s">
-        <v>93</v>
-      </c>
-      <c r="E99" t="s">
-        <v>94</v>
-      </c>
-      <c r="H99" t="s">
-        <v>95</v>
-      </c>
-      <c r="I99" t="s">
-        <v>34</v>
-      </c>
-      <c r="M99" t="s">
-        <v>96</v>
-      </c>
-      <c r="N99" s="11">
-        <v>28</v>
-      </c>
-      <c r="O99" t="s">
-        <v>82</v>
-      </c>
-      <c r="P99" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q99" t="s">
-        <v>98</v>
-      </c>
+      <c r="B98" s="2"/>
+      <c r="C98" s="2"/>
+      <c r="D98" s="2"/>
+      <c r="E98" s="3"/>
+      <c r="F98" s="3"/>
+      <c r="G98" s="3"/>
+      <c r="H98" s="3"/>
+      <c r="I98" s="3"/>
+      <c r="J98" s="3"/>
+      <c r="K98" s="3"/>
+      <c r="L98" s="3"/>
+      <c r="M98" s="3"/>
+      <c r="N98" s="3"/>
+      <c r="O98" s="3"/>
+      <c r="P98" s="3"/>
+      <c r="Q98" s="3"/>
     </row>
     <row r="100" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>92</v>
       </c>
       <c r="B100" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="E100" t="s">
         <v>94</v>
@@ -4684,12 +4695,14 @@
         <v>96</v>
       </c>
       <c r="N100" s="11">
-        <v>100</v>
+        <v>28</v>
       </c>
       <c r="O100" t="s">
         <v>82</v>
       </c>
-      <c r="P100" s="11"/>
+      <c r="P100" s="11" t="s">
+        <v>97</v>
+      </c>
       <c r="Q100" t="s">
         <v>98</v>
       </c>
@@ -4702,7 +4715,7 @@
         <v>99</v>
       </c>
       <c r="E101" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="H101" t="s">
         <v>95</v>
@@ -4713,16 +4726,13 @@
       <c r="M101" t="s">
         <v>96</v>
       </c>
-      <c r="N101" s="13">
-        <f>N100</f>
+      <c r="N101" s="11">
         <v>100</v>
       </c>
       <c r="O101" t="s">
         <v>82</v>
       </c>
-      <c r="P101" s="11" t="s">
-        <v>101</v>
-      </c>
+      <c r="P101" s="11"/>
       <c r="Q101" t="s">
         <v>98</v>
       </c>
@@ -4731,6 +4741,12 @@
       <c r="A102" t="s">
         <v>92</v>
       </c>
+      <c r="B102" t="s">
+        <v>99</v>
+      </c>
+      <c r="E102" t="s">
+        <v>100</v>
+      </c>
       <c r="H102" t="s">
         <v>95</v>
       </c>
@@ -4740,20 +4756,23 @@
       <c r="M102" t="s">
         <v>96</v>
       </c>
-      <c r="N102" s="11">
-        <v>80</v>
+      <c r="N102" s="13">
+        <f>N101</f>
+        <v>100</v>
       </c>
       <c r="O102" t="s">
         <v>82</v>
       </c>
-      <c r="P102" s="11"/>
+      <c r="P102" s="11" t="s">
+        <v>101</v>
+      </c>
       <c r="Q102" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="103" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="H103" t="s">
         <v>95</v>
@@ -4765,19 +4784,19 @@
         <v>96</v>
       </c>
       <c r="N103" s="11">
-        <v>14.5</v>
+        <v>80</v>
       </c>
       <c r="O103" t="s">
         <v>82</v>
       </c>
-      <c r="P103" s="9"/>
+      <c r="P103" s="11"/>
       <c r="Q103" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="104" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H104" t="s">
         <v>95</v>
@@ -4789,23 +4808,20 @@
         <v>96</v>
       </c>
       <c r="N104" s="11">
-        <v>100</v>
+        <v>14.5</v>
       </c>
       <c r="O104" t="s">
         <v>82</v>
       </c>
       <c r="P104" s="9"/>
       <c r="Q104" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="105" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>104</v>
       </c>
-      <c r="D105" t="s">
-        <v>106</v>
-      </c>
       <c r="H105" t="s">
         <v>95</v>
       </c>
@@ -4816,7 +4832,7 @@
         <v>96</v>
       </c>
       <c r="N105" s="11">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="O105" t="s">
         <v>82</v>
@@ -4833,9 +4849,6 @@
       <c r="D106" t="s">
         <v>106</v>
       </c>
-      <c r="E106" t="s">
-        <v>107</v>
-      </c>
       <c r="H106" t="s">
         <v>95</v>
       </c>
@@ -4846,7 +4859,7 @@
         <v>96</v>
       </c>
       <c r="N106" s="11">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="O106" t="s">
         <v>82</v>
@@ -4857,47 +4870,63 @@
       </c>
     </row>
     <row r="107" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N107" s="9"/>
+      <c r="A107" t="s">
+        <v>104</v>
+      </c>
+      <c r="D107" t="s">
+        <v>106</v>
+      </c>
+      <c r="E107" t="s">
+        <v>107</v>
+      </c>
+      <c r="H107" t="s">
+        <v>95</v>
+      </c>
+      <c r="I107" t="s">
+        <v>34</v>
+      </c>
+      <c r="M107" t="s">
+        <v>96</v>
+      </c>
+      <c r="N107" s="11">
+        <v>69</v>
+      </c>
+      <c r="O107" t="s">
+        <v>82</v>
+      </c>
       <c r="P107" s="9"/>
+      <c r="Q107" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="108" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A108" s="2" t="s">
+      <c r="N108" s="9"/>
+      <c r="P108" s="9"/>
+    </row>
+    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A109" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B108" s="2"/>
-      <c r="C108" s="2"/>
-      <c r="D108" s="2"/>
-      <c r="E108" s="3"/>
-      <c r="F108" s="3"/>
-      <c r="G108" s="3"/>
-      <c r="H108" s="3"/>
-      <c r="I108" s="3"/>
-      <c r="J108" s="3"/>
-      <c r="K108" s="3"/>
-      <c r="L108" s="3"/>
-      <c r="M108" s="3"/>
-      <c r="N108" s="3"/>
-      <c r="O108" s="3"/>
-      <c r="P108" s="3"/>
-      <c r="Q108" s="3"/>
-    </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M109" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="N109" s="5">
-        <v>0</v>
-      </c>
-      <c r="O109" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="P109" s="5" t="s">
-        <v>25</v>
-      </c>
+      <c r="B109" s="2"/>
+      <c r="C109" s="2"/>
+      <c r="D109" s="2"/>
+      <c r="E109" s="3"/>
+      <c r="F109" s="3"/>
+      <c r="G109" s="3"/>
+      <c r="H109" s="3"/>
+      <c r="I109" s="3"/>
+      <c r="J109" s="3"/>
+      <c r="K109" s="3"/>
+      <c r="L109" s="3"/>
+      <c r="M109" s="3"/>
+      <c r="N109" s="3"/>
+      <c r="O109" s="3"/>
+      <c r="P109" s="3"/>
+      <c r="Q109" s="3"/>
     </row>
     <row r="110" spans="1:17" x14ac:dyDescent="0.25">
       <c r="M110" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N110" s="5">
         <v>0</v>
@@ -4910,39 +4939,29 @@
       </c>
     </row>
     <row r="111" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>92</v>
-      </c>
-      <c r="B111" t="s">
-        <v>93</v>
-      </c>
-      <c r="E111" t="s">
-        <v>94</v>
-      </c>
-      <c r="G111" t="s">
-        <v>111</v>
-      </c>
-      <c r="M111" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="N111" s="11">
-        <f>(0.8*20+0.2*2)</f>
-        <v>16.399999999999999</v>
-      </c>
-      <c r="O111" s="11" t="s">
+      <c r="M111" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="N111" s="5">
+        <v>0</v>
+      </c>
+      <c r="O111" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P111" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q111" t="s">
-        <v>103</v>
+      <c r="P111" s="5" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="112" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>92</v>
       </c>
+      <c r="B112" t="s">
+        <v>93</v>
+      </c>
+      <c r="E112" t="s">
+        <v>94</v>
+      </c>
       <c r="G112" t="s">
         <v>111</v>
       </c>
@@ -4950,37 +4969,38 @@
         <v>109</v>
       </c>
       <c r="N112" s="11">
+        <f>(0.8*20+0.2*2)</f>
+        <v>16.399999999999999</v>
+      </c>
+      <c r="O112" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="P112" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q112" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>92</v>
+      </c>
+      <c r="G113" t="s">
+        <v>111</v>
+      </c>
+      <c r="M113" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="N113" s="11">
         <f>(0.6*20+0.4*2)</f>
         <v>12.8</v>
       </c>
-      <c r="O112" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="P112" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q112" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>104</v>
-      </c>
-      <c r="G113" t="s">
-        <v>111</v>
-      </c>
-      <c r="M113" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="N113" s="11">
-        <v>2</v>
-      </c>
       <c r="O113" s="11" t="s">
         <v>82</v>
       </c>
       <c r="P113" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="Q113" t="s">
         <v>103</v>
@@ -4988,7 +5008,7 @@
     </row>
     <row r="114" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G114" t="s">
         <v>111</v>
@@ -5010,46 +5030,43 @@
       </c>
     </row>
     <row r="115" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M115" s="11"/>
-      <c r="N115" s="11"/>
-      <c r="O115" s="11"/>
-      <c r="P115" s="11"/>
+      <c r="A115" t="s">
+        <v>102</v>
+      </c>
+      <c r="G115" t="s">
+        <v>111</v>
+      </c>
+      <c r="M115" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="N115" s="11">
+        <v>2</v>
+      </c>
+      <c r="O115" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="P115" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q115" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="116" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>92</v>
-      </c>
-      <c r="B116" t="s">
-        <v>93</v>
-      </c>
-      <c r="E116" t="s">
-        <v>94</v>
-      </c>
-      <c r="G116" t="s">
-        <v>111</v>
-      </c>
-      <c r="M116" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="N116" s="11">
-        <v>5</v>
-      </c>
-      <c r="O116" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="P116" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="Q116" t="s">
-        <v>103</v>
-      </c>
+      <c r="M116" s="11"/>
+      <c r="N116" s="11"/>
+      <c r="O116" s="11"/>
+      <c r="P116" s="11"/>
     </row>
     <row r="117" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>92</v>
       </c>
+      <c r="B117" t="s">
+        <v>93</v>
+      </c>
       <c r="E117" t="s">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="G117" t="s">
         <v>111</v>
@@ -5074,6 +5091,9 @@
       <c r="A118" t="s">
         <v>92</v>
       </c>
+      <c r="E118" t="s">
+        <v>116</v>
+      </c>
       <c r="G118" t="s">
         <v>111</v>
       </c>
@@ -5081,43 +5101,45 @@
         <v>110</v>
       </c>
       <c r="N118" s="11">
+        <v>5</v>
+      </c>
+      <c r="O118" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="P118" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q118" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>92</v>
+      </c>
+      <c r="G119" t="s">
+        <v>111</v>
+      </c>
+      <c r="M119" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="N119" s="11">
         <f>0.9*5+0.1*15</f>
         <v>6</v>
       </c>
-      <c r="O118" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="P118" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="Q118" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>104</v>
-      </c>
-      <c r="G119" t="s">
-        <v>111</v>
-      </c>
-      <c r="M119" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="N119" s="11">
-        <v>15</v>
-      </c>
       <c r="O119" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="P119" s="11"/>
+      <c r="P119" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="Q119" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="120" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G120" t="s">
         <v>111</v>
@@ -5137,67 +5159,51 @@
       </c>
     </row>
     <row r="121" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M121" s="11"/>
-      <c r="N121" s="11"/>
-      <c r="O121" s="11"/>
+      <c r="A121" t="s">
+        <v>102</v>
+      </c>
+      <c r="G121" t="s">
+        <v>111</v>
+      </c>
+      <c r="M121" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="N121" s="11">
+        <v>15</v>
+      </c>
+      <c r="O121" s="11" t="s">
+        <v>82</v>
+      </c>
       <c r="P121" s="11"/>
+      <c r="Q121" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="122" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A122" s="14"/>
-      <c r="B122" s="14"/>
-      <c r="E122" s="14"/>
-      <c r="G122" t="s">
-        <v>30</v>
-      </c>
-      <c r="M122" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="N122" s="11">
-        <v>5</v>
-      </c>
-      <c r="O122" s="11" t="s">
-        <v>82</v>
-      </c>
+      <c r="M122" s="11"/>
+      <c r="N122" s="11"/>
+      <c r="O122" s="11"/>
       <c r="P122" s="11"/>
-      <c r="Q122" t="s">
-        <v>103</v>
-      </c>
     </row>
     <row r="123" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A123" s="14" t="str">
-        <f>A116</f>
-        <v>cattle</v>
-      </c>
-      <c r="B123" s="14" t="str">
-        <f>B116</f>
-        <v>dairy</v>
-      </c>
-      <c r="E123" s="14" t="str">
-        <f>E116</f>
-        <v>cows</v>
-      </c>
+      <c r="A123" s="14"/>
+      <c r="B123" s="14"/>
+      <c r="E123" s="14"/>
       <c r="G123" t="s">
         <v>30</v>
       </c>
-      <c r="M123" s="14" t="str">
-        <f t="shared" ref="M123:Q125" si="0">M116</f>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N123" s="14">
-        <f t="shared" si="0"/>
+      <c r="M123" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="N123" s="11">
         <v>5</v>
       </c>
-      <c r="O123" s="14" t="str">
-        <f t="shared" si="0"/>
-        <v>%</v>
-      </c>
-      <c r="P123" s="14" t="str">
-        <f t="shared" si="0"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="Q123" s="14" t="str">
-        <f t="shared" si="0"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
+      <c r="O123" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="P123" s="11"/>
+      <c r="Q123" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="124" spans="1:17" x14ac:dyDescent="0.25">
@@ -5205,15 +5211,19 @@
         <f>A117</f>
         <v>cattle</v>
       </c>
+      <c r="B124" s="14" t="str">
+        <f>B117</f>
+        <v>dairy</v>
+      </c>
       <c r="E124" s="14" t="str">
         <f>E117</f>
-        <v>bulls</v>
+        <v>cows</v>
       </c>
       <c r="G124" t="s">
         <v>30</v>
       </c>
       <c r="M124" s="14" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="M124:Q126" si="0">M117</f>
         <v>feeding_losses</v>
       </c>
       <c r="N124" s="14">
@@ -5238,6 +5248,10 @@
         <f>A118</f>
         <v>cattle</v>
       </c>
+      <c r="E125" s="14" t="str">
+        <f>E118</f>
+        <v>bulls</v>
+      </c>
       <c r="G125" t="s">
         <v>30</v>
       </c>
@@ -5247,7 +5261,7 @@
       </c>
       <c r="N125" s="14">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O125" s="14" t="str">
         <f t="shared" si="0"/>
@@ -5255,7 +5269,7 @@
       </c>
       <c r="P125" s="14" t="str">
         <f t="shared" si="0"/>
-        <v>10% feeding on pasture</v>
+        <v>No feeding on pasture</v>
       </c>
       <c r="Q125" s="14" t="str">
         <f t="shared" si="0"/>
@@ -5265,39 +5279,42 @@
     <row r="126" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A126" s="14" t="str">
         <f>A119</f>
-        <v>sheep</v>
+        <v>cattle</v>
       </c>
       <c r="G126" t="s">
         <v>30</v>
       </c>
       <c r="M126" s="14" t="str">
-        <f t="shared" ref="M126:O127" si="1">M119</f>
+        <f t="shared" si="0"/>
         <v>feeding_losses</v>
       </c>
       <c r="N126" s="14">
-        <f t="shared" si="1"/>
-        <v>15</v>
+        <f t="shared" si="0"/>
+        <v>6</v>
       </c>
       <c r="O126" s="14" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>%</v>
       </c>
-      <c r="P126" s="14"/>
+      <c r="P126" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>10% feeding on pasture</v>
+      </c>
       <c r="Q126" s="14" t="str">
-        <f>Q119</f>
+        <f t="shared" si="0"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="127" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A127" s="14" t="str">
         <f>A120</f>
-        <v>horses</v>
+        <v>sheep</v>
       </c>
       <c r="G127" t="s">
         <v>30</v>
       </c>
       <c r="M127" s="14" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="M127:O128" si="1">M120</f>
         <v>feeding_losses</v>
       </c>
       <c r="N127" s="14">
@@ -5315,66 +5332,55 @@
       </c>
     </row>
     <row r="128" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A128" s="14"/>
-      <c r="M128" s="14"/>
-      <c r="N128" s="14"/>
-      <c r="O128" s="14"/>
+      <c r="A128" s="14" t="str">
+        <f>A121</f>
+        <v>horses</v>
+      </c>
+      <c r="G128" t="s">
+        <v>30</v>
+      </c>
+      <c r="M128" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N128" s="14">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="O128" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
       <c r="P128" s="14"/>
-      <c r="Q128" s="14"/>
+      <c r="Q128" s="14" t="str">
+        <f>Q121</f>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
     </row>
     <row r="129" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="G129" t="s">
-        <v>118</v>
-      </c>
-      <c r="M129" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="N129" s="11">
-        <v>5</v>
-      </c>
-      <c r="O129" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="P129" s="11"/>
-      <c r="Q129" t="s">
-        <v>103</v>
-      </c>
+      <c r="A129" s="14"/>
+      <c r="M129" s="14"/>
+      <c r="N129" s="14"/>
+      <c r="O129" s="14"/>
+      <c r="P129" s="14"/>
+      <c r="Q129" s="14"/>
     </row>
     <row r="130" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A130" s="14" t="str">
-        <f>A116</f>
-        <v>cattle</v>
-      </c>
-      <c r="B130" s="14" t="str">
-        <f>B116</f>
-        <v>dairy</v>
-      </c>
-      <c r="E130" s="14" t="str">
-        <f>E116</f>
-        <v>cows</v>
-      </c>
       <c r="G130" t="s">
         <v>118</v>
       </c>
-      <c r="M130" s="14" t="str">
-        <f t="shared" ref="M130:Q132" si="2">M116</f>
-        <v>feeding_losses</v>
-      </c>
-      <c r="N130" s="14">
-        <f t="shared" si="2"/>
+      <c r="M130" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="N130" s="11">
         <v>5</v>
       </c>
-      <c r="O130" s="14" t="str">
-        <f t="shared" si="2"/>
-        <v>%</v>
-      </c>
-      <c r="P130" s="14" t="str">
-        <f t="shared" si="2"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="Q130" s="14" t="str">
-        <f t="shared" si="2"/>
-        <v>Cederberg &amp; Henriksson (2020)</v>
+      <c r="O130" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="P130" s="11"/>
+      <c r="Q130" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="131" spans="1:17" x14ac:dyDescent="0.25">
@@ -5382,15 +5388,19 @@
         <f>A117</f>
         <v>cattle</v>
       </c>
+      <c r="B131" s="14" t="str">
+        <f>B117</f>
+        <v>dairy</v>
+      </c>
       <c r="E131" s="14" t="str">
         <f>E117</f>
-        <v>bulls</v>
+        <v>cows</v>
       </c>
       <c r="G131" t="s">
         <v>118</v>
       </c>
       <c r="M131" s="14" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="M131:Q133" si="2">M117</f>
         <v>feeding_losses</v>
       </c>
       <c r="N131" s="14">
@@ -5415,6 +5425,10 @@
         <f>A118</f>
         <v>cattle</v>
       </c>
+      <c r="E132" s="14" t="str">
+        <f>E118</f>
+        <v>bulls</v>
+      </c>
       <c r="G132" t="s">
         <v>118</v>
       </c>
@@ -5424,7 +5438,7 @@
       </c>
       <c r="N132" s="14">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O132" s="14" t="str">
         <f t="shared" si="2"/>
@@ -5432,7 +5446,7 @@
       </c>
       <c r="P132" s="14" t="str">
         <f t="shared" si="2"/>
-        <v>10% feeding on pasture</v>
+        <v>No feeding on pasture</v>
       </c>
       <c r="Q132" s="14" t="str">
         <f t="shared" si="2"/>
@@ -5442,39 +5456,42 @@
     <row r="133" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A133" s="14" t="str">
         <f>A119</f>
-        <v>sheep</v>
+        <v>cattle</v>
       </c>
       <c r="G133" t="s">
         <v>118</v>
       </c>
       <c r="M133" s="14" t="str">
-        <f t="shared" ref="M133:O134" si="3">M119</f>
+        <f t="shared" si="2"/>
         <v>feeding_losses</v>
       </c>
       <c r="N133" s="14">
-        <f t="shared" si="3"/>
-        <v>15</v>
+        <f t="shared" si="2"/>
+        <v>6</v>
       </c>
       <c r="O133" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>%</v>
       </c>
-      <c r="P133" s="11"/>
+      <c r="P133" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>10% feeding on pasture</v>
+      </c>
       <c r="Q133" s="14" t="str">
-        <f>Q119</f>
+        <f t="shared" si="2"/>
         <v>Cederberg &amp; Henriksson (2020)</v>
       </c>
     </row>
     <row r="134" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A134" s="14" t="str">
         <f>A120</f>
-        <v>horses</v>
+        <v>sheep</v>
       </c>
       <c r="G134" t="s">
         <v>118</v>
       </c>
       <c r="M134" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="M134:O135" si="3">M120</f>
         <v>feeding_losses</v>
       </c>
       <c r="N134" s="14">
@@ -5492,21 +5509,34 @@
       </c>
     </row>
     <row r="135" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N135" s="9"/>
+      <c r="A135" s="14" t="str">
+        <f>A121</f>
+        <v>horses</v>
+      </c>
+      <c r="G135" t="s">
+        <v>118</v>
+      </c>
+      <c r="M135" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="N135" s="14">
+        <f t="shared" si="3"/>
+        <v>15</v>
+      </c>
+      <c r="O135" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>%</v>
+      </c>
       <c r="P135" s="11"/>
+      <c r="Q135" s="14" t="str">
+        <f>Q121</f>
+        <v>Cederberg &amp; Henriksson (2020)</v>
+      </c>
     </row>
     <row r="136" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A136" s="9"/>
-      <c r="G136" t="s">
-        <v>119</v>
-      </c>
-      <c r="M136" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="N136" s="11"/>
-      <c r="P136" s="9" t="s">
-        <v>120</v>
-      </c>
+      <c r="N136" s="9"/>
+      <c r="P136" s="11"/>
     </row>
     <row r="137" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A137" s="9"/>
@@ -5514,40 +5544,40 @@
         <v>119</v>
       </c>
       <c r="M137" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="N137" s="11">
-        <v>2</v>
-      </c>
-      <c r="O137" s="11" t="s">
-        <v>82</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="N137" s="11"/>
       <c r="P137" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="Q137" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="138" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A138" s="9"/>
-      <c r="M138" s="11"/>
-      <c r="N138" s="11"/>
-      <c r="O138" s="11"/>
-      <c r="P138" s="9"/>
+      <c r="G138" t="s">
+        <v>119</v>
+      </c>
+      <c r="M138" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="N138" s="11">
+        <v>2</v>
+      </c>
+      <c r="O138" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="P138" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q138" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="139" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A139" s="9"/>
-      <c r="G139" t="s">
-        <v>123</v>
-      </c>
-      <c r="M139" s="11" t="s">
-        <v>109</v>
-      </c>
+      <c r="M139" s="11"/>
       <c r="N139" s="11"/>
-      <c r="P139" s="9" t="s">
-        <v>120</v>
-      </c>
+      <c r="O139" s="11"/>
+      <c r="P139" s="9"/>
     </row>
     <row r="140" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A140" s="9"/>
@@ -5555,111 +5585,106 @@
         <v>123</v>
       </c>
       <c r="M140" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="N140" s="11"/>
+      <c r="P140" s="9" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A141" s="9"/>
+      <c r="G141" t="s">
+        <v>123</v>
+      </c>
+      <c r="M141" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="N140" s="11">
+      <c r="N141" s="11">
         <v>3</v>
       </c>
-      <c r="O140" s="11" t="s">
+      <c r="O141" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="P140" s="9" t="s">
+      <c r="P141" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="Q140" t="s">
+      <c r="Q141" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N141" s="9"/>
-      <c r="P141" s="11"/>
-    </row>
     <row r="142" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A142" s="2" t="s">
+      <c r="N142" s="9"/>
+      <c r="P142" s="11"/>
+    </row>
+    <row r="143" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A143" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B142" s="2"/>
-      <c r="C142" s="2"/>
-      <c r="D142" s="2"/>
-      <c r="E142" s="3"/>
-      <c r="F142" s="3"/>
-      <c r="G142" s="3"/>
-      <c r="H142" s="3"/>
-      <c r="I142" s="3"/>
-      <c r="J142" s="3"/>
-      <c r="K142" s="3"/>
-      <c r="L142" s="3"/>
-      <c r="M142" s="3"/>
-      <c r="N142" s="3"/>
-      <c r="O142" s="3"/>
-      <c r="P142" s="3"/>
-      <c r="Q142" s="3"/>
-    </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A143" t="s">
+      <c r="B143" s="2"/>
+      <c r="C143" s="2"/>
+      <c r="D143" s="2"/>
+      <c r="E143" s="3"/>
+      <c r="F143" s="3"/>
+      <c r="G143" s="3"/>
+      <c r="H143" s="3"/>
+      <c r="I143" s="3"/>
+      <c r="J143" s="3"/>
+      <c r="K143" s="3"/>
+      <c r="L143" s="3"/>
+      <c r="M143" s="3"/>
+      <c r="N143" s="3"/>
+      <c r="O143" s="3"/>
+      <c r="P143" s="3"/>
+      <c r="Q143" s="3"/>
+    </row>
+    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
         <v>92</v>
       </c>
-      <c r="N143" s="11"/>
-      <c r="P143" s="11" t="s">
+      <c r="N144" s="11"/>
+      <c r="P144" s="11" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A144" s="11" t="s">
+    <row r="145" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A145" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="B144" s="9"/>
-      <c r="C144" s="9"/>
-      <c r="D144" s="9"/>
-      <c r="E144" s="9"/>
-      <c r="F144" s="9"/>
-      <c r="G144" s="9"/>
-      <c r="H144" s="9"/>
-      <c r="I144" s="9"/>
-      <c r="J144" s="9"/>
-      <c r="K144" s="9"/>
-      <c r="L144" s="9"/>
-      <c r="M144" s="11" t="s">
+      <c r="B145" s="9"/>
+      <c r="C145" s="9"/>
+      <c r="D145" s="9"/>
+      <c r="E145" s="9"/>
+      <c r="F145" s="9"/>
+      <c r="G145" s="9"/>
+      <c r="H145" s="9"/>
+      <c r="I145" s="9"/>
+      <c r="J145" s="9"/>
+      <c r="K145" s="9"/>
+      <c r="L145" s="9"/>
+      <c r="M145" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="N144" s="11">
+      <c r="N145" s="11">
         <v>6.7</v>
       </c>
-      <c r="O144" s="11" t="s">
+      <c r="O145" s="11" t="s">
         <v>127</v>
-      </c>
-      <c r="P144" s="9"/>
-      <c r="Q144" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="145" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A145" t="s">
-        <v>102</v>
-      </c>
-      <c r="M145" t="s">
-        <v>129</v>
-      </c>
-      <c r="N145" s="11">
-        <v>18</v>
-      </c>
-      <c r="O145" t="s">
-        <v>130</v>
       </c>
       <c r="P145" s="9"/>
       <c r="Q145" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="146" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>83</v>
+        <v>102</v>
       </c>
       <c r="M146" t="s">
         <v>129</v>
       </c>
       <c r="N146" s="11">
-        <v>1.5</v>
+        <v>18</v>
       </c>
       <c r="O146" t="s">
         <v>130</v>
@@ -5671,13 +5696,13 @@
     </row>
     <row r="147" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="M147" t="s">
         <v>129</v>
       </c>
       <c r="N147" s="11">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="O147" t="s">
         <v>130</v>
@@ -5688,28 +5713,28 @@
       </c>
     </row>
     <row r="148" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N148" s="11"/>
+      <c r="A148" t="s">
+        <v>84</v>
+      </c>
+      <c r="M148" t="s">
+        <v>129</v>
+      </c>
+      <c r="N148" s="11">
+        <v>0</v>
+      </c>
+      <c r="O148" t="s">
+        <v>130</v>
+      </c>
       <c r="P148" s="9"/>
+      <c r="Q148" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="149" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M149" t="s">
-        <v>132</v>
-      </c>
-      <c r="N149" s="11">
-        <v>1</v>
-      </c>
-      <c r="O149" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="P149" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="Q149" s="11"/>
+      <c r="N149" s="11"/>
+      <c r="P149" s="9"/>
     </row>
     <row r="150" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A150" t="s">
-        <v>92</v>
-      </c>
       <c r="M150" t="s">
         <v>132</v>
       </c>
@@ -5719,19 +5744,15 @@
       <c r="O150" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="P150" s="11"/>
+      <c r="P150" s="11" t="s">
+        <v>134</v>
+      </c>
       <c r="Q150" s="11"/>
     </row>
     <row r="151" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>92</v>
       </c>
-      <c r="B151" t="s">
-        <v>93</v>
-      </c>
-      <c r="E151" t="s">
-        <v>94</v>
-      </c>
       <c r="M151" t="s">
         <v>132</v>
       </c>
@@ -5752,7 +5773,7 @@
         <v>93</v>
       </c>
       <c r="E152" t="s">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="M152" t="s">
         <v>132</v>
@@ -5771,7 +5792,7 @@
         <v>92</v>
       </c>
       <c r="B153" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="E153" t="s">
         <v>116</v>
@@ -5789,38 +5810,60 @@
       <c r="Q153" s="11"/>
     </row>
     <row r="154" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N154" s="9"/>
-      <c r="P154" s="9"/>
+      <c r="A154" t="s">
+        <v>92</v>
+      </c>
+      <c r="B154" t="s">
+        <v>99</v>
+      </c>
+      <c r="E154" t="s">
+        <v>116</v>
+      </c>
+      <c r="M154" t="s">
+        <v>132</v>
+      </c>
+      <c r="N154" s="11">
+        <v>1</v>
+      </c>
+      <c r="O154" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="P154" s="11"/>
+      <c r="Q154" s="11"/>
     </row>
     <row r="155" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A155" s="2" t="s">
+      <c r="N155" s="9"/>
+      <c r="P155" s="9"/>
+    </row>
+    <row r="156" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A156" s="2" t="s">
         <v>647</v>
       </c>
-      <c r="B155" s="2"/>
-      <c r="C155" s="2"/>
-      <c r="D155" s="2"/>
-      <c r="E155" s="3"/>
-      <c r="F155" s="3"/>
-      <c r="G155" s="3"/>
-      <c r="H155" s="3"/>
-      <c r="I155" s="3"/>
-      <c r="J155" s="3"/>
-      <c r="K155" s="3"/>
-      <c r="L155" s="3"/>
-      <c r="M155" s="3"/>
-      <c r="N155" s="3"/>
-      <c r="O155" s="3"/>
-      <c r="P155" s="3"/>
-      <c r="Q155" s="3"/>
-    </row>
-    <row r="156" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="M156" t="s">
+      <c r="B156" s="2"/>
+      <c r="C156" s="2"/>
+      <c r="D156" s="2"/>
+      <c r="E156" s="3"/>
+      <c r="F156" s="3"/>
+      <c r="G156" s="3"/>
+      <c r="H156" s="3"/>
+      <c r="I156" s="3"/>
+      <c r="J156" s="3"/>
+      <c r="K156" s="3"/>
+      <c r="L156" s="3"/>
+      <c r="M156" s="3"/>
+      <c r="N156" s="3"/>
+      <c r="O156" s="3"/>
+      <c r="P156" s="3"/>
+      <c r="Q156" s="3"/>
+    </row>
+    <row r="157" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M157" t="s">
         <v>135</v>
       </c>
-      <c r="N156" s="11" t="s">
+      <c r="N157" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="P156" t="s">
+      <c r="P157" t="s">
         <v>648</v>
       </c>
     </row>

</xml_diff>